<commit_message>
Mise à jour depuis Excel — 2026-09-18T09:13:59.736Z
</commit_message>
<xml_diff>
--- a/comparatif.xlsx
+++ b/comparatif.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30431"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30516"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nge1-my.sharepoint.com/personal/fabienne_cohanoff_nge_fr/Documents/Documents/FAMILLE/POMPES/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nge1.sharepoint.com/sites/FR_SADE_DAM/Documents partages/01 - Achats/Achats Production/Pompes &amp; Instrum/Pompes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{80DDC44F-6169-4D5B-B16F-52915D55FDA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C868B7AA-C382-4258-B0FF-FC718A978C12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{723C6001-552E-447F-BEBB-92F546F7738F}"/>
+    <workbookView xWindow="7716" yWindow="12852" windowWidth="23256" windowHeight="12456" xr2:uid="{723C6001-552E-447F-BEBB-92F546F7738F}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="285">
   <si>
     <t>Eau potable et irrigation</t>
   </si>
@@ -940,21 +940,6 @@
   </si>
   <si>
     <t>TSURUMI</t>
-  </si>
-  <si>
-    <t>ATEX</t>
-  </si>
-  <si>
-    <t>HMT</t>
-  </si>
-  <si>
-    <t>PUISSANCE</t>
-  </si>
-  <si>
-    <t>DN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MOTEUR </t>
   </si>
 </sst>
 </file>
@@ -2296,7 +2281,7 @@
     <col min="33" max="16384" width="11.42578125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" ht="12.6" thickBot="1"/>
+    <row r="1" spans="1:32" ht="12.75" thickBot="1"/>
     <row r="2" spans="1:32" s="70" customFormat="1" ht="23.25" customHeight="1" thickBot="1">
       <c r="A2" s="68"/>
       <c r="B2" s="69"/>
@@ -5843,34 +5828,9 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9695ECB-13A0-4CDA-8A65-46AFD650B789}">
-  <dimension ref="B4:F23"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
+  <dimension ref="F23"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <sheetData>
-    <row r="4" spans="2:2">
-      <c r="B4" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="5" spans="2:2">
-      <c r="B5" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="6" spans="2:2">
-      <c r="B6" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="7" spans="2:2">
-      <c r="B7" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="8" spans="2:2">
-      <c r="B8" t="s">
-        <v>289</v>
-      </c>
-    </row>
     <row r="23" spans="6:6">
       <c r="F23">
         <f>4.5*7*22</f>
@@ -5882,8 +5842,296 @@
 </worksheet>
 </file>
 
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101004976F38B5FA2A5428FEEC343358A0CB6" ma:contentTypeVersion="19" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="d78edfbf191a497d28ab4f4b405a2c3f">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xmlns:ns3="c4b3ccb6-1a3d-47c8-9c28-87cc19c94359" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="79eaa508d83d12f280b303d7506ce0b5" ns2:_="" ns3:_="">
+    <xsd:import namespace="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5"/>
+    <xsd:import namespace="c4b3ccb6-1a3d-47c8-9c28-87cc19c94359"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:CloudMigratorOriginId" minOccurs="0"/>
+                <xsd:element ref="ns2:FileHash" minOccurs="0"/>
+                <xsd:element ref="ns2:CloudMigratorVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:UniqueSourceRef" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:nombre" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="CloudMigratorOriginId" ma:index="8" nillable="true" ma:displayName="CloudMigratorOriginId" ma:description="" ma:internalName="CloudMigratorOriginId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="FileHash" ma:index="9" nillable="true" ma:displayName="FileHash" ma:description="" ma:internalName="FileHash">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="CloudMigratorVersion" ma:index="10" nillable="true" ma:displayName="CloudMigratorVersion" ma:description="" ma:internalName="CloudMigratorVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="UniqueSourceRef" ma:index="11" nillable="true" ma:displayName="UniqueSourceRef" ma:description="" ma:internalName="UniqueSourceRef">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="13" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="14" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="15" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="16" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:description="" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="22" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Balises d’images" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="2de30655-58d6-405c-b76f-318c55c6c931" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="24" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="nombre" ma:index="25" nillable="true" ma:displayName="nombre" ma:format="Dropdown" ma:internalName="nombre" ma:percentage="FALSE">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Number"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="26" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="c4b3ccb6-1a3d-47c8-9c28-87cc19c94359" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="23" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{d5604f43-09db-4a5b-a1b4-d25d7657b1fa}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="c4b3ccb6-1a3d-47c8-9c28-87cc19c94359">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Type de contenu"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Titre"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <FileHash xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
+    <nombre xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
+    <CloudMigratorVersion xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <CloudMigratorOriginId xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
+    <TaxCatchAll xmlns="c4b3ccb6-1a3d-47c8-9c28-87cc19c94359" xsi:nil="true"/>
+    <UniqueSourceRef xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2B67381A-06A2-445B-9B84-A17F50FAEFF2}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DFA46023-FA4E-40CC-AE09-8D10AF59D952}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CC74D80B-69A9-4194-90FE-61316E92C740}"/>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{3e7a5884-aef9-4d53-85a1-19dae5fd11e1}" enabled="1" method="Standard" siteId="{7d7ef55b-d006-4101-afe3-f2bbfa26e84b}" removed="0"/>
+  <clbl:label id="{7d7ef55b-d006-4101-afe3-f2bbfa26e84b}" enabled="0" method="" siteId="{7d7ef55b-d006-4101-afe3-f2bbfa26e84b}" removed="1"/>
 </clbl:labelList>
 </file>
</xml_diff>

<commit_message>
Mise à jour depuis Excel — 2026-09-18T09:16:52.468Z
</commit_message>
<xml_diff>
--- a/comparatif.xlsx
+++ b/comparatif.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nge1.sharepoint.com/sites/FR_SADE_DAM/Documents partages/01 - Achats/Achats Production/Pompes &amp; Instrum/Pompes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C868B7AA-C382-4258-B0FF-FC718A978C12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{36A0A010-C73D-49F2-8250-986B5CF995C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="7716" yWindow="12852" windowWidth="23256" windowHeight="12456" xr2:uid="{723C6001-552E-447F-BEBB-92F546F7738F}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="286">
   <si>
     <t>Eau potable et irrigation</t>
   </si>
@@ -87,10 +87,13 @@
     <t>Pompes immergées</t>
   </si>
   <si>
+    <t>De surcroit</t>
+  </si>
+  <si>
+    <t>Immergées</t>
+  </si>
+  <si>
     <t>De surface</t>
-  </si>
-  <si>
-    <t>Immergées</t>
   </si>
   <si>
     <t>Types</t>
@@ -2366,7 +2369,7 @@
       </c>
       <c r="P3" s="101"/>
       <c r="Q3" s="100" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="R3" s="101"/>
       <c r="S3" s="101"/>
@@ -2386,67 +2389,67 @@
     </row>
     <row r="4" spans="1:32" s="80" customFormat="1" ht="57.75" customHeight="1" thickBot="1">
       <c r="B4" s="81" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C4" s="82" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D4" s="82" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E4" s="82" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F4" s="82" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G4" s="82" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H4" s="82" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I4" s="82" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J4" s="82" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K4" s="82" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L4" s="82" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="M4" s="82" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="N4" s="82" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="O4" s="82" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="P4" s="82" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q4" s="82" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R4" s="82" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="S4" s="82" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="T4" s="82" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="U4" s="83" t="s">
         <v>15</v>
       </c>
       <c r="V4" s="83" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="W4" s="107"/>
       <c r="X4" s="99"/>
@@ -2494,136 +2497,136 @@
     </row>
     <row r="6" spans="1:32" s="74" customFormat="1" ht="52.9" customHeight="1">
       <c r="B6" s="84" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C6" s="77" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D6" s="77" t="s">
+        <v>38</v>
+      </c>
+      <c r="E6" s="77" t="s">
+        <v>39</v>
+      </c>
+      <c r="F6" s="77" t="s">
+        <v>38</v>
+      </c>
+      <c r="G6" s="77" t="s">
+        <v>40</v>
+      </c>
+      <c r="H6" s="77" t="s">
+        <v>38</v>
+      </c>
+      <c r="I6" s="77" t="s">
+        <v>41</v>
+      </c>
+      <c r="J6" s="77" t="s">
+        <v>38</v>
+      </c>
+      <c r="K6" s="77" t="s">
+        <v>38</v>
+      </c>
+      <c r="L6" s="77" t="s">
         <v>37</v>
       </c>
-      <c r="E6" s="77" t="s">
+      <c r="M6" s="77" t="s">
         <v>38</v>
       </c>
-      <c r="F6" s="77" t="s">
-        <v>37</v>
-      </c>
-      <c r="G6" s="77" t="s">
-        <v>39</v>
-      </c>
-      <c r="H6" s="77" t="s">
-        <v>37</v>
-      </c>
-      <c r="I6" s="77" t="s">
-        <v>40</v>
-      </c>
-      <c r="J6" s="77" t="s">
-        <v>37</v>
-      </c>
-      <c r="K6" s="77" t="s">
-        <v>37</v>
-      </c>
-      <c r="L6" s="77" t="s">
-        <v>36</v>
-      </c>
-      <c r="M6" s="77" t="s">
-        <v>37</v>
-      </c>
       <c r="N6" s="77" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="O6" s="77" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="P6" s="77" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q6" s="77" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="R6" s="77" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="S6" s="77" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="T6" s="77" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="U6" s="77" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="V6" s="77" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="W6" s="77"/>
       <c r="X6" s="77" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Y6" s="77" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Z6" s="77"/>
       <c r="AA6" s="77"/>
       <c r="AB6" s="77"/>
       <c r="AC6" s="78"/>
       <c r="AD6" s="79" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AE6" s="79" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="AF6" s="76" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:32" s="1" customFormat="1" ht="18" customHeight="1">
       <c r="A7" s="95" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B7" s="116" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E7" s="11"/>
       <c r="F7" s="11" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G7" s="11"/>
       <c r="H7" s="11" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I7" s="11" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J7" s="11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="K7" s="11"/>
       <c r="L7" s="11"/>
       <c r="M7" s="11"/>
       <c r="N7" s="11" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="O7" s="11" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="P7" s="11"/>
       <c r="Q7" s="11" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R7" s="11"/>
       <c r="S7" s="11" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="T7" s="11"/>
       <c r="U7" s="11" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="V7" s="11"/>
       <c r="W7" s="11"/>
@@ -2641,53 +2644,53 @@
       <c r="A8" s="96"/>
       <c r="B8" s="114"/>
       <c r="C8" s="11" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F8" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="G8" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G8" s="11" t="s">
-        <v>59</v>
-      </c>
       <c r="H8" s="11" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I8" s="11"/>
       <c r="J8" s="11" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="K8" s="11" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="L8" s="11"/>
       <c r="M8" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="N8" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="N8" s="11" t="s">
-        <v>62</v>
-      </c>
       <c r="O8" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="P8" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="Q8" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="R8" s="11"/>
       <c r="S8" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="T8" s="11"/>
       <c r="U8" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="V8" s="11"/>
       <c r="W8" s="11"/>
@@ -2710,27 +2713,27 @@
       <c r="F9" s="11"/>
       <c r="G9" s="11"/>
       <c r="H9" s="11" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I9" s="11"/>
       <c r="J9" s="11"/>
       <c r="K9" s="11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="L9" s="11" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="M9" s="11" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="N9" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="O9" s="11" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="P9" s="11" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q9" s="11"/>
       <c r="R9" s="11"/>
@@ -2758,18 +2761,18 @@
       <c r="F10" s="11"/>
       <c r="G10" s="11"/>
       <c r="H10" s="11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I10" s="11"/>
       <c r="J10" s="11"/>
       <c r="K10" s="11"/>
       <c r="L10" s="11" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="M10" s="11"/>
       <c r="N10" s="11"/>
       <c r="O10" s="11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="P10" s="11"/>
       <c r="Q10" s="11"/>
@@ -2802,20 +2805,20 @@
       <c r="J11" s="52"/>
       <c r="K11" s="52"/>
       <c r="L11" s="52" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="M11" s="52"/>
       <c r="N11" s="52" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O11" s="52"/>
       <c r="P11" s="52"/>
       <c r="Q11" s="52" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="R11" s="52"/>
       <c r="S11" s="52" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="T11" s="52"/>
       <c r="U11" s="52"/>
@@ -2834,88 +2837,88 @@
     <row r="12" spans="1:32" ht="18" customHeight="1">
       <c r="A12" s="96"/>
       <c r="B12" s="113" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C12" s="61" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D12" s="62" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E12" s="63" t="s">
+        <v>78</v>
+      </c>
+      <c r="F12" s="62" t="s">
         <v>77</v>
       </c>
-      <c r="F12" s="62" t="s">
-        <v>76</v>
-      </c>
       <c r="G12" s="62" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H12" s="62" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I12" s="61" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J12" s="61" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="K12" s="37" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="L12" s="61" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="M12" s="62" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="N12" s="61" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="O12" s="61" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="P12" s="37" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q12" s="61" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="R12" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="S12" s="61" t="s">
         <v>85</v>
       </c>
-      <c r="S12" s="61" t="s">
-        <v>84</v>
-      </c>
       <c r="T12" s="61" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="U12" s="61" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="V12" s="62" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="W12" s="61" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="X12" s="62" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="Y12" s="61" t="s">
+        <v>88</v>
+      </c>
+      <c r="Z12" s="61" t="s">
         <v>87</v>
       </c>
-      <c r="Z12" s="61" t="s">
-        <v>86</v>
-      </c>
       <c r="AA12" s="61" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="AB12" s="37" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AC12" s="61" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="AD12" s="20"/>
       <c r="AE12" s="20"/>
@@ -2925,69 +2928,69 @@
       <c r="A13" s="96"/>
       <c r="B13" s="114"/>
       <c r="C13" s="11" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D13" s="4"/>
       <c r="E13" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
       <c r="I13" s="11" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J13" s="11" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="K13" s="11" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="L13" s="11" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="M13" s="4"/>
       <c r="N13" s="11" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="O13" s="11" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="P13" s="4"/>
       <c r="Q13" s="11" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="R13" s="11" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="S13" s="11" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="T13" s="11" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="U13" s="12" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="V13" s="4"/>
       <c r="W13" s="11" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="X13" s="4"/>
       <c r="Y13" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="Z13" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="Z13" s="11" t="s">
-        <v>97</v>
-      </c>
       <c r="AA13" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AB13" s="12" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AC13" s="11" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="AD13" s="10"/>
       <c r="AE13" s="10"/>
@@ -2997,62 +3000,62 @@
       <c r="A14" s="96"/>
       <c r="B14" s="114"/>
       <c r="C14" s="11" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D14" s="4"/>
       <c r="E14" s="4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
       <c r="I14" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J14" s="11" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K14" s="11" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="L14" s="11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M14" s="4"/>
       <c r="N14" s="11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="O14" s="11" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="P14" s="4"/>
       <c r="Q14" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="R14" s="11" t="s">
         <v>98</v>
-      </c>
-      <c r="R14" s="11" t="s">
-        <v>97</v>
       </c>
       <c r="S14" s="4"/>
       <c r="T14" s="11" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="U14" s="11" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="V14" s="4"/>
       <c r="W14" s="11" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="X14" s="4"/>
       <c r="Y14" s="4"/>
       <c r="Z14" s="11" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="AA14" s="12" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AC14" s="11" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="AD14" s="10"/>
       <c r="AE14" s="10"/>
@@ -3062,57 +3065,57 @@
       <c r="A15" s="96"/>
       <c r="B15" s="114"/>
       <c r="C15" s="11" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D15" s="4"/>
       <c r="E15" s="4" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
       <c r="I15" s="4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J15" s="11" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="K15" s="11" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4"/>
       <c r="N15" s="4"/>
       <c r="O15" s="11" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="P15" s="4"/>
       <c r="Q15" s="4" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="R15" s="11" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="S15" s="4"/>
       <c r="T15" s="4"/>
       <c r="U15" s="11" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="V15" s="4"/>
       <c r="W15" s="11" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="X15" s="4"/>
       <c r="Y15" s="4"/>
       <c r="Z15" s="11" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="AA15" s="11" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AB15" s="11"/>
       <c r="AC15" s="11" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AD15" s="10"/>
       <c r="AE15" s="10"/>
@@ -3122,7 +3125,7 @@
       <c r="A16" s="96"/>
       <c r="B16" s="114"/>
       <c r="C16" s="11" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
@@ -3130,45 +3133,45 @@
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
       <c r="I16" s="4" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="J16" s="11" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="K16" s="11" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4"/>
       <c r="N16" s="4"/>
       <c r="O16" s="11" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="P16" s="4"/>
       <c r="Q16" s="4"/>
       <c r="R16" s="11" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="S16" s="4"/>
       <c r="T16" s="4"/>
       <c r="U16" s="11" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="V16" s="4"/>
       <c r="W16" s="11" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="X16" s="4"/>
       <c r="Y16" s="4"/>
       <c r="Z16" s="11" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AA16" s="11" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="AB16" s="11"/>
       <c r="AC16" s="11" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="AD16" s="10"/>
       <c r="AE16" s="10"/>
@@ -3185,38 +3188,38 @@
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
       <c r="J17" s="11" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K17" s="4"/>
       <c r="L17" s="4"/>
       <c r="M17" s="4"/>
       <c r="N17" s="4"/>
       <c r="O17" s="11" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="P17" s="4"/>
       <c r="Q17" s="4"/>
       <c r="R17" s="11" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="S17" s="4"/>
       <c r="T17" s="4"/>
       <c r="U17" s="11" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="V17" s="4"/>
       <c r="W17" s="12" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="X17" s="4"/>
       <c r="Y17" s="4"/>
       <c r="Z17" s="4"/>
       <c r="AA17" s="11" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AB17" s="11"/>
       <c r="AC17" s="11" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="AD17" s="10"/>
       <c r="AE17" s="10"/>
@@ -3233,34 +3236,34 @@
       <c r="H18" s="32"/>
       <c r="I18" s="32"/>
       <c r="J18" s="52" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="K18" s="32"/>
       <c r="L18" s="32"/>
       <c r="M18" s="32"/>
       <c r="N18" s="32"/>
       <c r="O18" s="52" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="P18" s="32"/>
       <c r="Q18" s="32"/>
       <c r="R18" s="64" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="S18" s="32"/>
       <c r="T18" s="32"/>
       <c r="U18" s="52" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="V18" s="32"/>
       <c r="W18" s="64" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="X18" s="32"/>
       <c r="Y18" s="32"/>
       <c r="Z18" s="32"/>
       <c r="AA18" s="52" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="AB18" s="52"/>
       <c r="AC18" s="52"/>
@@ -3270,75 +3273,75 @@
     </row>
     <row r="19" spans="1:155" s="3" customFormat="1" ht="89.45" customHeight="1" thickBot="1">
       <c r="A19" s="56" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B19" s="85" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C19" s="43"/>
       <c r="D19" s="43"/>
       <c r="E19" s="44" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F19" s="44" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="G19" s="44" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H19" s="43"/>
       <c r="I19" s="44" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="J19" s="43" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K19" s="43" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="L19" s="43" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="M19" s="43" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="N19" s="43"/>
       <c r="O19" s="44" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="P19" s="44" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="Q19" s="44" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="R19" s="57" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="S19" s="58" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="T19" s="57"/>
       <c r="U19" s="58" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="V19" s="57"/>
       <c r="W19" s="59" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="X19" s="57"/>
       <c r="Y19" s="58" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="Z19" s="57"/>
       <c r="AA19" s="58" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="AB19" s="58" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="AC19" s="58" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="AD19" s="57"/>
       <c r="AE19" s="57"/>
@@ -3347,245 +3350,245 @@
     <row r="20" spans="1:155" s="1" customFormat="1" ht="36" customHeight="1">
       <c r="A20" s="21"/>
       <c r="B20" s="110" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C20" s="22" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D20" s="22" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E20" s="22" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F20" s="22" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G20" s="22" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H20" s="22" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I20" s="22" t="s">
+        <v>152</v>
+      </c>
+      <c r="J20" s="22" t="s">
+        <v>153</v>
+      </c>
+      <c r="K20" s="22" t="s">
+        <v>154</v>
+      </c>
+      <c r="L20" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="M20" s="22" t="s">
+        <v>156</v>
+      </c>
+      <c r="N20" s="22" t="s">
+        <v>157</v>
+      </c>
+      <c r="O20" s="22" t="s">
+        <v>158</v>
+      </c>
+      <c r="P20" s="22" t="s">
+        <v>159</v>
+      </c>
+      <c r="Q20" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="R20" s="22" t="s">
         <v>151</v>
       </c>
-      <c r="J20" s="22" t="s">
-        <v>152</v>
-      </c>
-      <c r="K20" s="22" t="s">
-        <v>153</v>
-      </c>
-      <c r="L20" s="22" t="s">
-        <v>154</v>
-      </c>
-      <c r="M20" s="22" t="s">
-        <v>155</v>
-      </c>
-      <c r="N20" s="22" t="s">
-        <v>156</v>
-      </c>
-      <c r="O20" s="22" t="s">
-        <v>157</v>
-      </c>
-      <c r="P20" s="22" t="s">
-        <v>158</v>
-      </c>
-      <c r="Q20" s="22" t="s">
-        <v>159</v>
-      </c>
-      <c r="R20" s="22" t="s">
-        <v>150</v>
-      </c>
       <c r="S20" s="22" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="T20" s="22" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="U20" s="22" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="V20" s="22" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="W20" s="22" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="X20" s="22" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="Y20" s="22" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="Z20" s="22" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="AA20" s="22" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="AB20" s="22" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="AC20" s="22" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="AD20" s="22" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="AE20" s="22" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="AF20" s="23" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="21" spans="1:155" ht="18" customHeight="1">
       <c r="A21" s="24"/>
       <c r="B21" s="111"/>
       <c r="C21" s="25" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D21" s="25" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E21" s="25" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F21" s="25" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
       <c r="I21" s="13" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="J21" s="13" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="K21" s="13" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="L21" s="14"/>
       <c r="M21" s="13" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="N21" s="13" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="O21" s="13" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="P21" s="13" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="Q21" s="13" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="R21" s="14"/>
       <c r="S21" s="13" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="T21" s="14"/>
       <c r="U21" s="4"/>
       <c r="V21" s="4"/>
       <c r="W21" s="13" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="X21" s="4"/>
       <c r="Y21" s="13" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="Z21" s="13" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AA21" s="4"/>
       <c r="AB21" s="4"/>
       <c r="AC21" s="4"/>
       <c r="AD21" s="13" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="AE21" s="13" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="AF21" s="26" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="22" spans="1:155" ht="18" customHeight="1">
       <c r="A22" s="24"/>
       <c r="B22" s="111"/>
       <c r="C22" s="25" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D22" s="25" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="E22" s="25" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
       <c r="I22" s="14"/>
       <c r="J22" s="13" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="K22" s="14"/>
       <c r="L22" s="13" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="M22" s="13" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="N22" s="13" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="O22" s="13" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P22" s="13" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="Q22" s="13" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="R22" s="14"/>
       <c r="S22" s="13" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="T22" s="14"/>
       <c r="U22" s="4"/>
       <c r="V22" s="4"/>
       <c r="W22" s="13" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="X22" s="4"/>
       <c r="Y22" s="13" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="Z22" s="13"/>
       <c r="AA22" s="4"/>
       <c r="AB22" s="4"/>
       <c r="AC22" s="4"/>
       <c r="AD22" s="13" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="AE22" s="13" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="AF22" s="26" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="23" spans="1:155" ht="18" customHeight="1">
       <c r="A23" s="24"/>
       <c r="B23" s="111"/>
       <c r="C23" s="25" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D23" s="25" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E23" s="4"/>
       <c r="F23" s="4"/>
@@ -3593,51 +3596,51 @@
       <c r="H23" s="4"/>
       <c r="I23" s="14"/>
       <c r="J23" s="13" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K23" s="14"/>
       <c r="L23" s="13" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="M23" s="13" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="N23" s="13" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="O23" s="13" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="P23" s="14"/>
       <c r="Q23" s="13" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="R23" s="14"/>
       <c r="S23" s="13" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="T23" s="14"/>
       <c r="U23" s="4"/>
       <c r="V23" s="4"/>
       <c r="W23" s="13" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="X23" s="4"/>
       <c r="Y23" s="13" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="Z23" s="14"/>
       <c r="AA23" s="4"/>
       <c r="AB23" s="4"/>
       <c r="AC23" s="4"/>
       <c r="AD23" s="13" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AE23" s="13" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AF23" s="26" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="24" spans="1:155" ht="18" customHeight="1">
@@ -3651,48 +3654,48 @@
       <c r="H24" s="4"/>
       <c r="I24" s="14"/>
       <c r="J24" s="13" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="K24" s="14"/>
       <c r="L24" s="13" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M24" s="13" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="N24" s="13" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="O24" s="13" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="P24" s="14"/>
       <c r="Q24" s="13" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="R24" s="14"/>
       <c r="S24" s="13" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="T24" s="14"/>
       <c r="U24" s="4"/>
       <c r="V24" s="4"/>
       <c r="W24" s="13" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="X24" s="4"/>
       <c r="Y24" s="13" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="Z24" s="14"/>
       <c r="AA24" s="4"/>
       <c r="AB24" s="4"/>
       <c r="AC24" s="4"/>
       <c r="AD24" s="13" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AE24" s="13" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AF24" s="27"/>
     </row>
@@ -3707,44 +3710,44 @@
       <c r="H25" s="4"/>
       <c r="I25" s="14"/>
       <c r="J25" s="13" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="K25" s="14"/>
       <c r="L25" s="13" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="M25" s="14"/>
       <c r="N25" s="14"/>
       <c r="O25" s="13" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="P25" s="14"/>
       <c r="Q25" s="13" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="R25" s="14"/>
       <c r="S25" s="13" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="T25" s="14"/>
       <c r="U25" s="4"/>
       <c r="V25" s="4"/>
       <c r="W25" s="13" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="X25" s="4"/>
       <c r="Y25" s="13" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="Z25" s="14"/>
       <c r="AA25" s="4"/>
       <c r="AB25" s="4"/>
       <c r="AC25" s="4"/>
       <c r="AD25" s="13" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="AE25" s="13" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="AF25" s="27"/>
     </row>
@@ -3759,24 +3762,24 @@
       <c r="H26" s="6"/>
       <c r="I26" s="17"/>
       <c r="J26" s="18" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="K26" s="17"/>
       <c r="L26" s="18" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="M26" s="17"/>
       <c r="N26" s="17"/>
       <c r="O26" s="18" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="P26" s="17"/>
       <c r="Q26" s="18" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="R26" s="17"/>
       <c r="S26" s="18" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="T26" s="17"/>
       <c r="U26" s="6"/>
@@ -3784,14 +3787,14 @@
       <c r="W26" s="6"/>
       <c r="X26" s="6"/>
       <c r="Y26" s="18" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="Z26" s="17"/>
       <c r="AA26" s="6"/>
       <c r="AB26" s="6"/>
       <c r="AC26" s="6"/>
       <c r="AD26" s="18" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="AE26" s="17"/>
       <c r="AF26" s="29"/>
@@ -3822,14 +3825,14 @@
       <c r="W27" s="32"/>
       <c r="X27" s="32"/>
       <c r="Y27" s="33" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="Z27" s="34"/>
       <c r="AA27" s="32"/>
       <c r="AB27" s="32"/>
       <c r="AC27" s="32"/>
       <c r="AD27" s="33" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="AE27" s="34"/>
       <c r="AF27" s="35"/>
@@ -3960,72 +3963,72 @@
     <row r="28" spans="1:155" s="10" customFormat="1" ht="36" customHeight="1">
       <c r="A28" s="21"/>
       <c r="B28" s="117" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C28" s="36" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D28" s="36" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E28" s="36" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F28" s="36" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="G28" s="36" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="H28" s="37"/>
       <c r="I28" s="36" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="J28" s="36" t="s">
+        <v>228</v>
+      </c>
+      <c r="K28" s="36" t="s">
+        <v>229</v>
+      </c>
+      <c r="L28" s="36" t="s">
+        <v>230</v>
+      </c>
+      <c r="M28" s="36" t="s">
+        <v>231</v>
+      </c>
+      <c r="N28" s="36" t="s">
+        <v>232</v>
+      </c>
+      <c r="O28" s="36" t="s">
+        <v>233</v>
+      </c>
+      <c r="P28" s="36" t="s">
+        <v>234</v>
+      </c>
+      <c r="Q28" s="36" t="s">
+        <v>235</v>
+      </c>
+      <c r="R28" s="36" t="s">
         <v>227</v>
       </c>
-      <c r="K28" s="36" t="s">
-        <v>228</v>
-      </c>
-      <c r="L28" s="36" t="s">
-        <v>229</v>
-      </c>
-      <c r="M28" s="36" t="s">
-        <v>230</v>
-      </c>
-      <c r="N28" s="36" t="s">
-        <v>231</v>
-      </c>
-      <c r="O28" s="36" t="s">
-        <v>232</v>
-      </c>
-      <c r="P28" s="36" t="s">
+      <c r="S28" s="36" t="s">
         <v>233</v>
-      </c>
-      <c r="Q28" s="36" t="s">
-        <v>234</v>
-      </c>
-      <c r="R28" s="36" t="s">
-        <v>226</v>
-      </c>
-      <c r="S28" s="36" t="s">
-        <v>232</v>
       </c>
       <c r="T28" s="37"/>
       <c r="U28" s="36" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="V28" s="37"/>
       <c r="W28" s="36" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="X28" s="37"/>
       <c r="Y28" s="37"/>
       <c r="Z28" s="36" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="AA28" s="37" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="AB28" s="37"/>
       <c r="AC28" s="37"/>
@@ -4160,60 +4163,60 @@
       <c r="A29" s="24"/>
       <c r="B29" s="118"/>
       <c r="C29" s="13" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D29" s="13" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E29" s="4"/>
       <c r="F29" s="13" t="s">
+        <v>240</v>
+      </c>
+      <c r="G29" s="13" t="s">
         <v>239</v>
-      </c>
-      <c r="G29" s="13" t="s">
-        <v>238</v>
       </c>
       <c r="H29" s="4"/>
       <c r="I29" s="4"/>
       <c r="J29" s="13" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="K29" s="13" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="L29" s="13" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="M29" s="13" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="N29" s="13" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="O29" s="13" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="P29" s="13" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="Q29" s="13" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="R29" s="14"/>
       <c r="S29" s="13" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="T29" s="4"/>
       <c r="U29" s="13" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="V29" s="4"/>
       <c r="W29" s="13" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="X29" s="4"/>
       <c r="Y29" s="4"/>
       <c r="Z29" s="13" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="AA29" s="4"/>
       <c r="AB29" s="4"/>
@@ -4347,51 +4350,51 @@
       <c r="A30" s="24"/>
       <c r="B30" s="118"/>
       <c r="C30" s="13" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D30" s="13" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E30" s="4"/>
       <c r="F30" s="13" t="s">
+        <v>252</v>
+      </c>
+      <c r="G30" s="13" t="s">
         <v>251</v>
-      </c>
-      <c r="G30" s="13" t="s">
-        <v>250</v>
       </c>
       <c r="H30" s="4"/>
       <c r="I30" s="4"/>
       <c r="J30" s="13" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="K30" s="13" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="L30" s="13" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="M30" s="14"/>
       <c r="N30" s="13" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="O30" s="13" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="P30" s="14"/>
       <c r="Q30" s="13" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="R30" s="14"/>
       <c r="S30" s="13" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="T30" s="4"/>
       <c r="U30" s="13" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="V30" s="4"/>
       <c r="W30" s="13" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="X30" s="4"/>
       <c r="Y30" s="4"/>
@@ -4528,15 +4531,15 @@
       <c r="A31" s="24"/>
       <c r="B31" s="118"/>
       <c r="C31" s="13" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D31" s="13" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E31" s="4"/>
       <c r="F31" s="4"/>
       <c r="G31" s="13" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="H31" s="4"/>
       <c r="I31" s="4"/>
@@ -4546,21 +4549,21 @@
       <c r="M31" s="14"/>
       <c r="N31" s="14"/>
       <c r="O31" s="13" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="P31" s="14"/>
       <c r="Q31" s="14"/>
       <c r="R31" s="14"/>
       <c r="S31" s="13" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="T31" s="4"/>
       <c r="U31" s="13" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="V31" s="4"/>
       <c r="W31" s="13" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="X31" s="4"/>
       <c r="Y31" s="4"/>
@@ -4697,15 +4700,15 @@
       <c r="A32" s="24"/>
       <c r="B32" s="118"/>
       <c r="C32" s="13" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D32" s="13" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E32" s="4"/>
       <c r="F32" s="4"/>
       <c r="G32" s="13" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="H32" s="4"/>
       <c r="I32" s="4"/>
@@ -4715,21 +4718,21 @@
       <c r="M32" s="14"/>
       <c r="N32" s="14"/>
       <c r="O32" s="13" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="P32" s="14"/>
       <c r="Q32" s="14"/>
       <c r="R32" s="14"/>
       <c r="S32" s="13" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="T32" s="4"/>
       <c r="U32" s="13" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="V32" s="4"/>
       <c r="W32" s="13" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="X32" s="4"/>
       <c r="Y32" s="4"/>
@@ -4866,15 +4869,15 @@
       <c r="A33" s="30"/>
       <c r="B33" s="119"/>
       <c r="C33" s="33" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D33" s="33" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E33" s="32"/>
       <c r="F33" s="32"/>
       <c r="G33" s="33" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="H33" s="32"/>
       <c r="I33" s="32"/>
@@ -5028,7 +5031,7 @@
     <row r="34" spans="1:155" ht="18" customHeight="1" thickBot="1">
       <c r="A34" s="42"/>
       <c r="B34" s="66" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C34" s="43"/>
       <c r="D34" s="43"/>
@@ -5052,10 +5055,10 @@
       <c r="V34" s="43"/>
       <c r="W34" s="43"/>
       <c r="X34" s="44" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="Y34" s="44" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="Z34" s="43"/>
       <c r="AA34" s="43"/>
@@ -5068,7 +5071,7 @@
     <row r="35" spans="1:155" ht="18" customHeight="1">
       <c r="A35" s="19"/>
       <c r="B35" s="51" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C35" s="8"/>
       <c r="D35" s="8"/>
@@ -5090,14 +5093,14 @@
       <c r="T35" s="8"/>
       <c r="U35" s="8"/>
       <c r="V35" s="8" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="W35" s="8"/>
       <c r="X35" s="8" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="Y35" s="8" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="Z35" s="8"/>
       <c r="AA35" s="8"/>
@@ -5110,7 +5113,7 @@
     <row r="36" spans="1:155" ht="18" customHeight="1" thickBot="1">
       <c r="A36" s="15"/>
       <c r="B36" s="67" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C36" s="6"/>
       <c r="D36" s="6"/>
@@ -5125,29 +5128,29 @@
       <c r="M36" s="6"/>
       <c r="N36" s="6"/>
       <c r="O36" s="6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="P36" s="6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="Q36" s="6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="R36" s="6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="S36" s="6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="T36" s="6"/>
       <c r="U36" s="6"/>
       <c r="V36" s="6"/>
       <c r="W36" s="6"/>
       <c r="X36" s="6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="Y36" s="6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="Z36" s="6"/>
       <c r="AA36" s="6"/>
@@ -5160,7 +5163,7 @@
     <row r="37" spans="1:155" ht="18" customHeight="1" thickBot="1">
       <c r="A37" s="42"/>
       <c r="B37" s="66" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C37" s="43"/>
       <c r="D37" s="43"/>
@@ -5184,7 +5187,7 @@
       <c r="V37" s="43"/>
       <c r="W37" s="43"/>
       <c r="X37" s="49" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="Y37" s="43"/>
       <c r="Z37" s="43"/>
@@ -5193,35 +5196,35 @@
       <c r="AC37" s="43"/>
       <c r="AD37" s="46"/>
       <c r="AE37" s="44" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AF37" s="50" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="38" spans="1:155" ht="18" customHeight="1">
       <c r="A38" s="19"/>
       <c r="B38" s="51" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D38" s="8" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="E38" s="8"/>
       <c r="F38" s="8"/>
       <c r="G38" s="8" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="H38" s="8"/>
       <c r="I38" s="8"/>
       <c r="J38" s="8" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="K38" s="8" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="L38" s="8"/>
       <c r="M38" s="8"/>
@@ -5237,7 +5240,7 @@
       <c r="W38" s="8"/>
       <c r="X38" s="8"/>
       <c r="Y38" s="8" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="Z38" s="8"/>
       <c r="AA38" s="8"/>
@@ -5250,7 +5253,7 @@
     <row r="39" spans="1:155" ht="18" customHeight="1">
       <c r="A39" s="9"/>
       <c r="B39" s="12" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C39" s="4"/>
       <c r="D39" s="4"/>
@@ -5261,7 +5264,7 @@
       <c r="I39" s="4"/>
       <c r="J39" s="4"/>
       <c r="K39" s="4" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="L39" s="4"/>
       <c r="M39" s="4"/>
@@ -5269,24 +5272,24 @@
       <c r="O39" s="4"/>
       <c r="P39" s="4"/>
       <c r="Q39" s="4" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="R39" s="4" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="S39" s="4"/>
       <c r="T39" s="4"/>
       <c r="U39" s="4"/>
       <c r="V39" s="4" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="W39" s="4"/>
       <c r="X39" s="4"/>
       <c r="Y39" s="4" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="Z39" s="4" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="AA39" s="4"/>
       <c r="AB39" s="4"/>
@@ -5298,7 +5301,7 @@
     <row r="40" spans="1:155" ht="18" customHeight="1">
       <c r="A40" s="9"/>
       <c r="B40" s="12" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C40" s="4"/>
       <c r="D40" s="4"/>
@@ -5323,11 +5326,11 @@
       <c r="W40" s="4"/>
       <c r="X40" s="4"/>
       <c r="Y40" s="4" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="Z40" s="4"/>
       <c r="AA40" s="4" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="AB40" s="4"/>
       <c r="AC40" s="4"/>
@@ -5338,7 +5341,7 @@
     <row r="41" spans="1:155" ht="18" customHeight="1">
       <c r="A41" s="9"/>
       <c r="B41" s="12" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C41" s="4"/>
       <c r="D41" s="4"/>
@@ -5374,14 +5377,14 @@
     <row r="42" spans="1:155" ht="18" customHeight="1">
       <c r="A42" s="9"/>
       <c r="B42" s="12" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C42" s="4"/>
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="H42" s="4"/>
       <c r="I42" s="4"/>
@@ -5412,7 +5415,7 @@
     <row r="43" spans="1:155" ht="18" customHeight="1">
       <c r="A43" s="9"/>
       <c r="B43" s="12" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C43" s="4"/>
       <c r="D43" s="4"/>
@@ -5440,7 +5443,7 @@
       <c r="Z43" s="10"/>
       <c r="AA43" s="10"/>
       <c r="AB43" s="10" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="AC43" s="10"/>
       <c r="AD43" s="10"/>
@@ -5449,7 +5452,7 @@
     <row r="44" spans="1:155" ht="18" customHeight="1">
       <c r="A44" s="9"/>
       <c r="B44" s="12" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C44" s="4"/>
       <c r="D44" s="4"/>
@@ -5484,7 +5487,7 @@
     <row r="45" spans="1:155" ht="18" customHeight="1">
       <c r="A45" s="9"/>
       <c r="B45" s="12" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C45" s="4"/>
       <c r="D45" s="4"/>
@@ -5519,7 +5522,7 @@
     <row r="46" spans="1:155" ht="18" customHeight="1">
       <c r="A46" s="9"/>
       <c r="B46" s="12" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C46" s="4"/>
       <c r="D46" s="4"/>
@@ -5554,7 +5557,7 @@
     <row r="47" spans="1:155" ht="18" customHeight="1">
       <c r="A47" s="9"/>
       <c r="B47" s="12" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C47" s="4"/>
       <c r="D47" s="4"/>

</xml_diff>

<commit_message>
Mise à jour depuis Excel — 2026-09-18T09:21:37.157Z
</commit_message>
<xml_diff>
--- a/comparatif.xlsx
+++ b/comparatif.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nge1.sharepoint.com/sites/FR_SADE_DAM/Documents partages/01 - Achats/Achats Production/Pompes &amp; Instrum/Pompes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{36A0A010-C73D-49F2-8250-986B5CF995C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{37FDA403-DBA7-4B2E-BE07-2EFF4B991CF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="7716" yWindow="12852" windowWidth="23256" windowHeight="12456" xr2:uid="{723C6001-552E-447F-BEBB-92F546F7738F}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Feuil2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Feuil1!$A$2:$AF$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Feuil1!$A$2:$AF$34</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="289">
   <si>
     <t>Eau potable et irrigation</t>
   </si>
@@ -87,13 +87,10 @@
     <t>Pompes immergées</t>
   </si>
   <si>
-    <t>De surcroit</t>
+    <t>De surface</t>
   </si>
   <si>
     <t>Immergées</t>
-  </si>
-  <si>
-    <t>De surface</t>
   </si>
   <si>
     <t>Types</t>
@@ -152,6 +149,21 @@
   <si>
     <t xml:space="preserve"> Volumétrique
 cela veut il dire extérieure ?</t>
+  </si>
+  <si>
+    <t>Couleur</t>
+  </si>
+  <si>
+    <t>jaune</t>
+  </si>
+  <si>
+    <t>bleu</t>
+  </si>
+  <si>
+    <t>Vertical turbine</t>
+  </si>
+  <si>
+    <t>rouge</t>
   </si>
   <si>
     <t>Application</t>
@@ -754,9 +766,6 @@
   </si>
   <si>
     <t>sub TWI 4/6/8 , Actun ZETOS K8/10/12, EMU</t>
-  </si>
-  <si>
-    <t>Vertical turbine</t>
   </si>
   <si>
     <t>SCP, Atmos Tera SCH
@@ -1585,7 +1594,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="120">
+  <cellXfs count="121">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1921,6 +1930,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2267,7 +2279,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:EY60"/>
+  <dimension ref="A1:EY61"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="7.140625" style="1" customWidth="1"/>
@@ -2369,7 +2381,7 @@
       </c>
       <c r="P3" s="101"/>
       <c r="Q3" s="100" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="R3" s="101"/>
       <c r="S3" s="101"/>
@@ -2389,67 +2401,67 @@
     </row>
     <row r="4" spans="1:32" s="80" customFormat="1" ht="57.75" customHeight="1" thickBot="1">
       <c r="B4" s="81" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="82" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="82" t="s">
+      <c r="D4" s="82" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="82" t="s">
+      <c r="E4" s="82" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="82" t="s">
+      <c r="F4" s="82" t="s">
         <v>20</v>
       </c>
-      <c r="F4" s="82" t="s">
+      <c r="G4" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="G4" s="82" t="s">
+      <c r="H4" s="82" t="s">
         <v>22</v>
       </c>
-      <c r="H4" s="82" t="s">
+      <c r="I4" s="82" t="s">
         <v>23</v>
       </c>
-      <c r="I4" s="82" t="s">
+      <c r="J4" s="82" t="s">
         <v>24</v>
       </c>
-      <c r="J4" s="82" t="s">
+      <c r="K4" s="82" t="s">
         <v>25</v>
       </c>
-      <c r="K4" s="82" t="s">
+      <c r="L4" s="82" t="s">
         <v>26</v>
       </c>
-      <c r="L4" s="82" t="s">
+      <c r="M4" s="82" t="s">
         <v>27</v>
       </c>
-      <c r="M4" s="82" t="s">
+      <c r="N4" s="82" t="s">
+        <v>27</v>
+      </c>
+      <c r="O4" s="82" t="s">
         <v>28</v>
       </c>
-      <c r="N4" s="82" t="s">
-        <v>28</v>
-      </c>
-      <c r="O4" s="82" t="s">
+      <c r="P4" s="82" t="s">
         <v>29</v>
       </c>
-      <c r="P4" s="82" t="s">
+      <c r="Q4" s="82" t="s">
         <v>30</v>
       </c>
-      <c r="Q4" s="82" t="s">
+      <c r="R4" s="82" t="s">
         <v>31</v>
       </c>
-      <c r="R4" s="82" t="s">
+      <c r="S4" s="82" t="s">
         <v>32</v>
       </c>
-      <c r="S4" s="82" t="s">
+      <c r="T4" s="82" t="s">
         <v>33</v>
-      </c>
-      <c r="T4" s="82" t="s">
-        <v>34</v>
       </c>
       <c r="U4" s="83" t="s">
         <v>15</v>
       </c>
       <c r="V4" s="83" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="W4" s="107"/>
       <c r="X4" s="99"/>
@@ -2462,235 +2474,248 @@
       <c r="AE4" s="93"/>
       <c r="AF4" s="94"/>
     </row>
-    <row r="5" spans="1:32" s="80" customFormat="1" ht="10.15" customHeight="1" thickBot="1">
-      <c r="B5" s="87"/>
-      <c r="C5" s="88"/>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="88"/>
-      <c r="K5" s="88"/>
-      <c r="L5" s="88"/>
-      <c r="M5" s="88"/>
-      <c r="N5" s="88"/>
-      <c r="O5" s="88"/>
-      <c r="P5" s="88"/>
-      <c r="Q5" s="88"/>
-      <c r="R5" s="88"/>
-      <c r="S5" s="88"/>
-      <c r="T5" s="88"/>
-      <c r="U5" s="89"/>
-      <c r="V5" s="89"/>
-      <c r="W5" s="86"/>
+    <row r="5" spans="1:32" s="80" customFormat="1" ht="57.75" customHeight="1">
+      <c r="B5" s="87" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" s="88" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" s="88" t="s">
+        <v>37</v>
+      </c>
+      <c r="E5" s="88" t="s">
+        <v>38</v>
+      </c>
+      <c r="F5" s="88" t="s">
+        <v>39</v>
+      </c>
+      <c r="G5" s="88" t="s">
+        <v>36</v>
+      </c>
+      <c r="H5" s="88" t="s">
+        <v>37</v>
+      </c>
+      <c r="I5" s="88" t="s">
+        <v>38</v>
+      </c>
+      <c r="J5" s="88" t="s">
+        <v>39</v>
+      </c>
+      <c r="K5" s="88" t="s">
+        <v>36</v>
+      </c>
+      <c r="L5" s="88" t="s">
+        <v>37</v>
+      </c>
+      <c r="M5" s="88" t="s">
+        <v>38</v>
+      </c>
+      <c r="N5" s="88" t="s">
+        <v>39</v>
+      </c>
+      <c r="O5" s="88" t="s">
+        <v>36</v>
+      </c>
+      <c r="P5" s="88" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q5" s="88" t="s">
+        <v>38</v>
+      </c>
+      <c r="R5" s="88" t="s">
+        <v>39</v>
+      </c>
+      <c r="S5" s="88" t="s">
+        <v>36</v>
+      </c>
+      <c r="T5" s="88" t="s">
+        <v>37</v>
+      </c>
+      <c r="U5" s="88" t="s">
+        <v>38</v>
+      </c>
+      <c r="V5" s="88" t="s">
+        <v>39</v>
+      </c>
+      <c r="W5" s="88" t="s">
+        <v>36</v>
+      </c>
       <c r="X5" s="86"/>
       <c r="Y5" s="86"/>
       <c r="Z5" s="86"/>
       <c r="AA5" s="86"/>
       <c r="AB5" s="86"/>
       <c r="AC5" s="90"/>
-      <c r="AD5" s="91"/>
-      <c r="AE5" s="91"/>
-      <c r="AF5" s="91"/>
+      <c r="AD5" s="120"/>
+      <c r="AE5" s="120"/>
+      <c r="AF5" s="120"/>
     </row>
-    <row r="6" spans="1:32" s="74" customFormat="1" ht="52.9" customHeight="1">
-      <c r="B6" s="84" t="s">
-        <v>36</v>
-      </c>
-      <c r="C6" s="77" t="s">
-        <v>37</v>
-      </c>
-      <c r="D6" s="77" t="s">
-        <v>38</v>
-      </c>
-      <c r="E6" s="77" t="s">
-        <v>39</v>
-      </c>
-      <c r="F6" s="77" t="s">
-        <v>38</v>
-      </c>
-      <c r="G6" s="77" t="s">
+    <row r="6" spans="1:32" s="80" customFormat="1" ht="10.15" customHeight="1" thickBot="1">
+      <c r="B6" s="87"/>
+      <c r="C6" s="88"/>
+      <c r="D6" s="88"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="88"/>
+      <c r="G6" s="88"/>
+      <c r="H6" s="88"/>
+      <c r="I6" s="88"/>
+      <c r="J6" s="88"/>
+      <c r="K6" s="88"/>
+      <c r="L6" s="88"/>
+      <c r="M6" s="88"/>
+      <c r="N6" s="88"/>
+      <c r="O6" s="88"/>
+      <c r="P6" s="88"/>
+      <c r="Q6" s="88"/>
+      <c r="R6" s="88"/>
+      <c r="S6" s="88"/>
+      <c r="T6" s="88"/>
+      <c r="U6" s="89"/>
+      <c r="V6" s="89"/>
+      <c r="W6" s="86"/>
+      <c r="X6" s="86"/>
+      <c r="Y6" s="86"/>
+      <c r="Z6" s="86"/>
+      <c r="AA6" s="86"/>
+      <c r="AB6" s="86"/>
+      <c r="AC6" s="90"/>
+      <c r="AD6" s="91"/>
+      <c r="AE6" s="91"/>
+      <c r="AF6" s="91"/>
+    </row>
+    <row r="7" spans="1:32" s="74" customFormat="1" ht="52.9" customHeight="1">
+      <c r="B7" s="84" t="s">
         <v>40</v>
       </c>
-      <c r="H6" s="77" t="s">
-        <v>38</v>
-      </c>
-      <c r="I6" s="77" t="s">
+      <c r="C7" s="77" t="s">
         <v>41</v>
       </c>
-      <c r="J6" s="77" t="s">
-        <v>38</v>
-      </c>
-      <c r="K6" s="77" t="s">
-        <v>38</v>
-      </c>
-      <c r="L6" s="77" t="s">
-        <v>37</v>
-      </c>
-      <c r="M6" s="77" t="s">
-        <v>38</v>
-      </c>
-      <c r="N6" s="77" t="s">
+      <c r="D7" s="77" t="s">
         <v>42</v>
       </c>
-      <c r="O6" s="77" t="s">
+      <c r="E7" s="77" t="s">
         <v>43</v>
       </c>
-      <c r="P6" s="77" t="s">
-        <v>43</v>
-      </c>
-      <c r="Q6" s="77" t="s">
-        <v>43</v>
-      </c>
-      <c r="R6" s="77" t="s">
-        <v>43</v>
-      </c>
-      <c r="S6" s="77" t="s">
-        <v>43</v>
-      </c>
-      <c r="T6" s="77" t="s">
-        <v>43</v>
-      </c>
-      <c r="U6" s="77" t="s">
-        <v>43</v>
-      </c>
-      <c r="V6" s="77" t="s">
-        <v>43</v>
-      </c>
-      <c r="W6" s="77"/>
-      <c r="X6" s="77" t="s">
+      <c r="F7" s="77" t="s">
+        <v>42</v>
+      </c>
+      <c r="G7" s="77" t="s">
         <v>44</v>
       </c>
-      <c r="Y6" s="77" t="s">
+      <c r="H7" s="77" t="s">
+        <v>42</v>
+      </c>
+      <c r="I7" s="77" t="s">
         <v>45</v>
       </c>
-      <c r="Z6" s="77"/>
-      <c r="AA6" s="77"/>
-      <c r="AB6" s="77"/>
-      <c r="AC6" s="78"/>
-      <c r="AD6" s="79" t="s">
+      <c r="J7" s="77" t="s">
+        <v>42</v>
+      </c>
+      <c r="K7" s="77" t="s">
+        <v>42</v>
+      </c>
+      <c r="L7" s="77" t="s">
+        <v>41</v>
+      </c>
+      <c r="M7" s="77" t="s">
+        <v>42</v>
+      </c>
+      <c r="N7" s="77" t="s">
         <v>46</v>
       </c>
-      <c r="AE6" s="79" t="s">
+      <c r="O7" s="77" t="s">
         <v>47</v>
       </c>
-      <c r="AF6" s="76" t="s">
+      <c r="P7" s="77" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q7" s="77" t="s">
+        <v>47</v>
+      </c>
+      <c r="R7" s="77" t="s">
+        <v>47</v>
+      </c>
+      <c r="S7" s="77" t="s">
+        <v>47</v>
+      </c>
+      <c r="T7" s="77" t="s">
+        <v>47</v>
+      </c>
+      <c r="U7" s="77" t="s">
+        <v>47</v>
+      </c>
+      <c r="V7" s="77" t="s">
+        <v>47</v>
+      </c>
+      <c r="W7" s="77"/>
+      <c r="X7" s="77" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="7" spans="1:32" s="1" customFormat="1" ht="18" customHeight="1">
-      <c r="A7" s="95" t="s">
+      <c r="Y7" s="77" t="s">
         <v>49</v>
       </c>
-      <c r="B7" s="116" t="s">
+      <c r="Z7" s="77"/>
+      <c r="AA7" s="77"/>
+      <c r="AB7" s="77"/>
+      <c r="AC7" s="78"/>
+      <c r="AD7" s="79" t="s">
         <v>50</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="AE7" s="79" t="s">
         <v>51</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="AF7" s="76" t="s">
         <v>52</v>
       </c>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="I7" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="J7" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="K7" s="11"/>
-      <c r="L7" s="11"/>
-      <c r="M7" s="11"/>
-      <c r="N7" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="O7" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="P7" s="11"/>
-      <c r="Q7" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="R7" s="11"/>
-      <c r="S7" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="T7" s="11"/>
-      <c r="U7" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="V7" s="11"/>
-      <c r="W7" s="11"/>
-      <c r="X7" s="11"/>
-      <c r="Y7" s="11"/>
-      <c r="Z7" s="11"/>
-      <c r="AA7" s="11"/>
-      <c r="AB7" s="5"/>
-      <c r="AC7" s="54"/>
-      <c r="AD7" s="76"/>
-      <c r="AE7" s="76"/>
-      <c r="AF7" s="76"/>
     </row>
     <row r="8" spans="1:32" s="1" customFormat="1" ht="18" customHeight="1">
-      <c r="A8" s="96"/>
-      <c r="B8" s="114"/>
+      <c r="A8" s="95" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" s="116" t="s">
+        <v>54</v>
+      </c>
       <c r="C8" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8" s="11"/>
+      <c r="F8" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="G8" s="11"/>
+      <c r="H8" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="I8" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="E8" s="11" t="s">
+      <c r="J8" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="K8" s="11"/>
+      <c r="L8" s="11"/>
+      <c r="M8" s="11"/>
+      <c r="N8" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="F8" s="11" t="s">
+      <c r="O8" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="G8" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="H8" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="I8" s="11"/>
-      <c r="J8" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="K8" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="L8" s="11"/>
-      <c r="M8" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="N8" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="O8" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="P8" s="11" t="s">
-        <v>65</v>
-      </c>
+      <c r="P8" s="11"/>
       <c r="Q8" s="11" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="R8" s="11"/>
       <c r="S8" s="11" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="T8" s="11"/>
       <c r="U8" s="11" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="V8" s="11"/>
       <c r="W8" s="11"/>
@@ -2707,39 +2732,55 @@
     <row r="9" spans="1:32" s="1" customFormat="1" ht="18" customHeight="1">
       <c r="A9" s="96"/>
       <c r="B9" s="114"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
+      <c r="C9" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="G9" s="11" t="s">
+        <v>64</v>
+      </c>
       <c r="H9" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I9" s="11"/>
+      <c r="J9" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="K9" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="I9" s="11"/>
-      <c r="J9" s="11"/>
-      <c r="K9" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="L9" s="11" t="s">
-        <v>64</v>
-      </c>
+      <c r="L9" s="11"/>
       <c r="M9" s="11" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="N9" s="11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="O9" s="11" t="s">
         <v>69</v>
       </c>
       <c r="P9" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="Q9" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="Q9" s="11"/>
       <c r="R9" s="11"/>
-      <c r="S9" s="11"/>
+      <c r="S9" s="11" t="s">
+        <v>70</v>
+      </c>
       <c r="T9" s="11"/>
-      <c r="U9" s="11"/>
+      <c r="U9" s="11" t="s">
+        <v>69</v>
+      </c>
       <c r="V9" s="11"/>
       <c r="W9" s="11"/>
       <c r="X9" s="11"/>
@@ -2765,16 +2806,24 @@
       </c>
       <c r="I10" s="11"/>
       <c r="J10" s="11"/>
-      <c r="K10" s="11"/>
+      <c r="K10" s="11" t="s">
+        <v>56</v>
+      </c>
       <c r="L10" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="M10" s="11"/>
-      <c r="N10" s="11"/>
+        <v>68</v>
+      </c>
+      <c r="M10" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="N10" s="11" t="s">
+        <v>72</v>
+      </c>
       <c r="O10" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="P10" s="11"/>
+        <v>73</v>
+      </c>
+      <c r="P10" s="11" t="s">
+        <v>74</v>
+      </c>
       <c r="Q10" s="11"/>
       <c r="R10" s="11"/>
       <c r="S10" s="11"/>
@@ -2792,270 +2841,245 @@
       <c r="AE10" s="76"/>
       <c r="AF10" s="76"/>
     </row>
-    <row r="11" spans="1:32" s="1" customFormat="1" ht="18" customHeight="1" thickBot="1">
+    <row r="11" spans="1:32" s="1" customFormat="1" ht="18" customHeight="1">
       <c r="A11" s="96"/>
-      <c r="B11" s="115"/>
-      <c r="C11" s="52"/>
-      <c r="D11" s="52"/>
-      <c r="E11" s="52"/>
-      <c r="F11" s="52"/>
-      <c r="G11" s="52"/>
-      <c r="H11" s="52"/>
-      <c r="I11" s="52"/>
-      <c r="J11" s="52"/>
-      <c r="K11" s="52"/>
-      <c r="L11" s="52" t="s">
+      <c r="B11" s="114"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="I11" s="11"/>
+      <c r="J11" s="11"/>
+      <c r="K11" s="11"/>
+      <c r="L11" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="M11" s="52"/>
-      <c r="N11" s="52" t="s">
-        <v>73</v>
-      </c>
-      <c r="O11" s="52"/>
-      <c r="P11" s="52"/>
-      <c r="Q11" s="52" t="s">
-        <v>74</v>
-      </c>
-      <c r="R11" s="52"/>
-      <c r="S11" s="52" t="s">
-        <v>74</v>
-      </c>
-      <c r="T11" s="52"/>
-      <c r="U11" s="52"/>
-      <c r="V11" s="52"/>
-      <c r="W11" s="52"/>
-      <c r="X11" s="52"/>
-      <c r="Y11" s="52"/>
-      <c r="Z11" s="52"/>
-      <c r="AA11" s="52"/>
-      <c r="AB11" s="53"/>
-      <c r="AC11" s="55"/>
+      <c r="M11" s="11"/>
+      <c r="N11" s="11"/>
+      <c r="O11" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="P11" s="11"/>
+      <c r="Q11" s="11"/>
+      <c r="R11" s="11"/>
+      <c r="S11" s="11"/>
+      <c r="T11" s="11"/>
+      <c r="U11" s="11"/>
+      <c r="V11" s="11"/>
+      <c r="W11" s="11"/>
+      <c r="X11" s="11"/>
+      <c r="Y11" s="11"/>
+      <c r="Z11" s="11"/>
+      <c r="AA11" s="11"/>
+      <c r="AB11" s="5"/>
+      <c r="AC11" s="54"/>
       <c r="AD11" s="76"/>
       <c r="AE11" s="76"/>
       <c r="AF11" s="76"/>
     </row>
-    <row r="12" spans="1:32" ht="18" customHeight="1">
+    <row r="12" spans="1:32" s="1" customFormat="1" ht="18" customHeight="1">
       <c r="A12" s="96"/>
-      <c r="B12" s="113" t="s">
-        <v>75</v>
-      </c>
-      <c r="C12" s="61" t="s">
-        <v>76</v>
-      </c>
-      <c r="D12" s="62" t="s">
+      <c r="B12" s="115"/>
+      <c r="C12" s="52"/>
+      <c r="D12" s="52"/>
+      <c r="E12" s="52"/>
+      <c r="F12" s="52"/>
+      <c r="G12" s="52"/>
+      <c r="H12" s="52"/>
+      <c r="I12" s="52"/>
+      <c r="J12" s="52"/>
+      <c r="K12" s="52"/>
+      <c r="L12" s="52" t="s">
+        <v>67</v>
+      </c>
+      <c r="M12" s="52"/>
+      <c r="N12" s="52" t="s">
         <v>77</v>
       </c>
-      <c r="E12" s="63" t="s">
+      <c r="O12" s="52"/>
+      <c r="P12" s="52"/>
+      <c r="Q12" s="52" t="s">
         <v>78</v>
       </c>
-      <c r="F12" s="62" t="s">
-        <v>77</v>
-      </c>
-      <c r="G12" s="62" t="s">
-        <v>77</v>
-      </c>
-      <c r="H12" s="62" t="s">
-        <v>77</v>
-      </c>
-      <c r="I12" s="61" t="s">
-        <v>79</v>
-      </c>
-      <c r="J12" s="61" t="s">
-        <v>80</v>
-      </c>
-      <c r="K12" s="37" t="s">
-        <v>81</v>
-      </c>
-      <c r="L12" s="61" t="s">
-        <v>82</v>
-      </c>
-      <c r="M12" s="62" t="s">
-        <v>77</v>
-      </c>
-      <c r="N12" s="61" t="s">
-        <v>83</v>
-      </c>
-      <c r="O12" s="61" t="s">
-        <v>84</v>
-      </c>
-      <c r="P12" s="37" t="s">
-        <v>85</v>
-      </c>
-      <c r="Q12" s="61" t="s">
-        <v>85</v>
-      </c>
-      <c r="R12" s="37" t="s">
-        <v>86</v>
-      </c>
-      <c r="S12" s="61" t="s">
-        <v>85</v>
-      </c>
-      <c r="T12" s="61" t="s">
-        <v>85</v>
-      </c>
-      <c r="U12" s="61" t="s">
-        <v>85</v>
-      </c>
-      <c r="V12" s="62" t="s">
-        <v>77</v>
-      </c>
-      <c r="W12" s="61" t="s">
-        <v>87</v>
-      </c>
-      <c r="X12" s="62" t="s">
-        <v>77</v>
-      </c>
-      <c r="Y12" s="61" t="s">
-        <v>88</v>
-      </c>
-      <c r="Z12" s="61" t="s">
-        <v>87</v>
-      </c>
-      <c r="AA12" s="61" t="s">
-        <v>85</v>
-      </c>
-      <c r="AB12" s="37" t="s">
-        <v>89</v>
-      </c>
-      <c r="AC12" s="61" t="s">
-        <v>90</v>
-      </c>
-      <c r="AD12" s="20"/>
-      <c r="AE12" s="20"/>
-      <c r="AF12" s="75"/>
+      <c r="R12" s="52"/>
+      <c r="S12" s="52" t="s">
+        <v>78</v>
+      </c>
+      <c r="T12" s="52"/>
+      <c r="U12" s="52"/>
+      <c r="V12" s="52"/>
+      <c r="W12" s="52"/>
+      <c r="X12" s="52"/>
+      <c r="Y12" s="52"/>
+      <c r="Z12" s="52"/>
+      <c r="AA12" s="52"/>
+      <c r="AB12" s="53"/>
+      <c r="AC12" s="55"/>
+      <c r="AD12" s="76"/>
+      <c r="AE12" s="76"/>
+      <c r="AF12" s="76"/>
     </row>
     <row r="13" spans="1:32" ht="18" customHeight="1">
       <c r="A13" s="96"/>
-      <c r="B13" s="114"/>
-      <c r="C13" s="11" t="s">
+      <c r="B13" s="113" t="s">
+        <v>79</v>
+      </c>
+      <c r="C13" s="61" t="s">
+        <v>80</v>
+      </c>
+      <c r="D13" s="62" t="s">
+        <v>81</v>
+      </c>
+      <c r="E13" s="63" t="s">
+        <v>82</v>
+      </c>
+      <c r="F13" s="62" t="s">
+        <v>81</v>
+      </c>
+      <c r="G13" s="62" t="s">
+        <v>81</v>
+      </c>
+      <c r="H13" s="62" t="s">
+        <v>81</v>
+      </c>
+      <c r="I13" s="61" t="s">
+        <v>83</v>
+      </c>
+      <c r="J13" s="61" t="s">
+        <v>84</v>
+      </c>
+      <c r="K13" s="37" t="s">
+        <v>85</v>
+      </c>
+      <c r="L13" s="61" t="s">
+        <v>86</v>
+      </c>
+      <c r="M13" s="62" t="s">
+        <v>81</v>
+      </c>
+      <c r="N13" s="61" t="s">
+        <v>87</v>
+      </c>
+      <c r="O13" s="61" t="s">
+        <v>88</v>
+      </c>
+      <c r="P13" s="37" t="s">
+        <v>89</v>
+      </c>
+      <c r="Q13" s="61" t="s">
+        <v>89</v>
+      </c>
+      <c r="R13" s="37" t="s">
+        <v>90</v>
+      </c>
+      <c r="S13" s="61" t="s">
+        <v>89</v>
+      </c>
+      <c r="T13" s="61" t="s">
+        <v>89</v>
+      </c>
+      <c r="U13" s="61" t="s">
+        <v>89</v>
+      </c>
+      <c r="V13" s="62" t="s">
+        <v>81</v>
+      </c>
+      <c r="W13" s="61" t="s">
         <v>91</v>
       </c>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4" t="s">
+      <c r="X13" s="62" t="s">
+        <v>81</v>
+      </c>
+      <c r="Y13" s="61" t="s">
         <v>92</v>
       </c>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-      <c r="I13" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="J13" s="11" t="s">
+      <c r="Z13" s="61" t="s">
+        <v>91</v>
+      </c>
+      <c r="AA13" s="61" t="s">
+        <v>89</v>
+      </c>
+      <c r="AB13" s="37" t="s">
         <v>93</v>
       </c>
-      <c r="K13" s="11" t="s">
+      <c r="AC13" s="61" t="s">
         <v>94</v>
       </c>
-      <c r="L13" s="11" t="s">
-        <v>95</v>
-      </c>
-      <c r="M13" s="4"/>
-      <c r="N13" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="O13" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="P13" s="4"/>
-      <c r="Q13" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="R13" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="S13" s="11" t="s">
-        <v>97</v>
-      </c>
-      <c r="T13" s="11" t="s">
-        <v>97</v>
-      </c>
-      <c r="U13" s="12" t="s">
-        <v>89</v>
-      </c>
-      <c r="V13" s="4"/>
-      <c r="W13" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="X13" s="4"/>
-      <c r="Y13" s="12" t="s">
-        <v>99</v>
-      </c>
-      <c r="Z13" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="AA13" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="AB13" s="12" t="s">
-        <v>100</v>
-      </c>
-      <c r="AC13" s="11" t="s">
-        <v>101</v>
-      </c>
-      <c r="AD13" s="10"/>
-      <c r="AE13" s="10"/>
-      <c r="AF13" s="40"/>
+      <c r="AD13" s="20"/>
+      <c r="AE13" s="20"/>
+      <c r="AF13" s="75"/>
     </row>
     <row r="14" spans="1:32" ht="18" customHeight="1">
       <c r="A14" s="96"/>
       <c r="B14" s="114"/>
       <c r="C14" s="11" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="D14" s="4"/>
       <c r="E14" s="4" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
-      <c r="I14" s="4" t="s">
-        <v>92</v>
+      <c r="I14" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="J14" s="11" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="K14" s="11" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="L14" s="11" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="M14" s="4"/>
       <c r="N14" s="11" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="O14" s="11" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="P14" s="4"/>
-      <c r="Q14" s="12" t="s">
-        <v>99</v>
+      <c r="Q14" s="11" t="s">
+        <v>90</v>
       </c>
       <c r="R14" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="S14" s="4"/>
+        <v>91</v>
+      </c>
+      <c r="S14" s="11" t="s">
+        <v>101</v>
+      </c>
       <c r="T14" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="U14" s="11" t="s">
-        <v>98</v>
+        <v>101</v>
+      </c>
+      <c r="U14" s="12" t="s">
+        <v>93</v>
       </c>
       <c r="V14" s="4"/>
       <c r="W14" s="11" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="X14" s="4"/>
-      <c r="Y14" s="4"/>
+      <c r="Y14" s="12" t="s">
+        <v>103</v>
+      </c>
       <c r="Z14" s="11" t="s">
-        <v>108</v>
-      </c>
-      <c r="AA14" s="12" t="s">
-        <v>100</v>
+        <v>102</v>
+      </c>
+      <c r="AA14" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="AB14" s="12" t="s">
+        <v>104</v>
       </c>
       <c r="AC14" s="11" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="AD14" s="10"/>
       <c r="AE14" s="10"/>
@@ -3065,57 +3089,62 @@
       <c r="A15" s="96"/>
       <c r="B15" s="114"/>
       <c r="C15" s="11" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="D15" s="4"/>
       <c r="E15" s="4" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
       <c r="I15" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="J15" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="K15" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="L15" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="M15" s="4"/>
+      <c r="N15" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="O15" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="P15" s="4"/>
+      <c r="Q15" s="12" t="s">
         <v>103</v>
       </c>
-      <c r="J15" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="K15" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="L15" s="4"/>
-      <c r="M15" s="4"/>
-      <c r="N15" s="4"/>
-      <c r="O15" s="11" t="s">
-        <v>97</v>
-      </c>
-      <c r="P15" s="4"/>
-      <c r="Q15" s="4" t="s">
-        <v>113</v>
-      </c>
       <c r="R15" s="11" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="S15" s="4"/>
-      <c r="T15" s="4"/>
+      <c r="T15" s="11" t="s">
+        <v>90</v>
+      </c>
       <c r="U15" s="11" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="V15" s="4"/>
       <c r="W15" s="11" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="X15" s="4"/>
       <c r="Y15" s="4"/>
       <c r="Z15" s="11" t="s">
-        <v>114</v>
-      </c>
-      <c r="AA15" s="11" t="s">
-        <v>97</v>
-      </c>
-      <c r="AB15" s="11"/>
+        <v>112</v>
+      </c>
+      <c r="AA15" s="12" t="s">
+        <v>104</v>
+      </c>
       <c r="AC15" s="11" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="AD15" s="10"/>
       <c r="AE15" s="10"/>
@@ -3125,53 +3154,57 @@
       <c r="A16" s="96"/>
       <c r="B16" s="114"/>
       <c r="C16" s="11" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
+      <c r="E16" s="4" t="s">
+        <v>115</v>
+      </c>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
       <c r="I16" s="4" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="J16" s="11" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="K16" s="11" t="s">
-        <v>118</v>
+        <v>86</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4"/>
       <c r="N16" s="4"/>
       <c r="O16" s="11" t="s">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="P16" s="4"/>
-      <c r="Q16" s="4"/>
+      <c r="Q16" s="4" t="s">
+        <v>117</v>
+      </c>
       <c r="R16" s="11" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="S16" s="4"/>
       <c r="T16" s="4"/>
       <c r="U16" s="11" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="V16" s="4"/>
       <c r="W16" s="11" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="X16" s="4"/>
       <c r="Y16" s="4"/>
       <c r="Z16" s="11" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AA16" s="11" t="s">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="AB16" s="11"/>
       <c r="AC16" s="11" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AD16" s="10"/>
       <c r="AE16" s="10"/>
@@ -3180,524 +3213,524 @@
     <row r="17" spans="1:155" ht="18" customHeight="1">
       <c r="A17" s="96"/>
       <c r="B17" s="114"/>
-      <c r="C17" s="4"/>
+      <c r="C17" s="11" t="s">
+        <v>120</v>
+      </c>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
-      <c r="I17" s="4"/>
+      <c r="I17" s="4" t="s">
+        <v>115</v>
+      </c>
       <c r="J17" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="K17" s="4"/>
+      <c r="K17" s="11" t="s">
+        <v>122</v>
+      </c>
       <c r="L17" s="4"/>
       <c r="M17" s="4"/>
       <c r="N17" s="4"/>
       <c r="O17" s="11" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="P17" s="4"/>
       <c r="Q17" s="4"/>
       <c r="R17" s="11" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="S17" s="4"/>
       <c r="T17" s="4"/>
       <c r="U17" s="11" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="V17" s="4"/>
-      <c r="W17" s="12" t="s">
-        <v>99</v>
+      <c r="W17" s="11" t="s">
+        <v>123</v>
       </c>
       <c r="X17" s="4"/>
       <c r="Y17" s="4"/>
-      <c r="Z17" s="4"/>
+      <c r="Z17" s="11" t="s">
+        <v>123</v>
+      </c>
       <c r="AA17" s="11" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="AB17" s="11"/>
       <c r="AC17" s="11" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="AD17" s="10"/>
       <c r="AE17" s="10"/>
       <c r="AF17" s="40"/>
     </row>
-    <row r="18" spans="1:155" ht="18" customHeight="1" thickBot="1">
-      <c r="A18" s="97"/>
-      <c r="B18" s="115"/>
-      <c r="C18" s="32"/>
-      <c r="D18" s="32"/>
-      <c r="E18" s="32"/>
-      <c r="F18" s="32"/>
-      <c r="G18" s="32"/>
-      <c r="H18" s="32"/>
-      <c r="I18" s="32"/>
-      <c r="J18" s="52" t="s">
+    <row r="18" spans="1:155" ht="18" customHeight="1">
+      <c r="A18" s="96"/>
+      <c r="B18" s="114"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="4"/>
+      <c r="H18" s="4"/>
+      <c r="I18" s="4"/>
+      <c r="J18" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="K18" s="4"/>
+      <c r="L18" s="4"/>
+      <c r="M18" s="4"/>
+      <c r="N18" s="4"/>
+      <c r="O18" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="P18" s="4"/>
+      <c r="Q18" s="4"/>
+      <c r="R18" s="11" t="s">
         <v>123</v>
       </c>
-      <c r="K18" s="32"/>
-      <c r="L18" s="32"/>
-      <c r="M18" s="32"/>
-      <c r="N18" s="32"/>
-      <c r="O18" s="52" t="s">
-        <v>108</v>
-      </c>
-      <c r="P18" s="32"/>
-      <c r="Q18" s="32"/>
-      <c r="R18" s="64" t="s">
-        <v>99</v>
-      </c>
-      <c r="S18" s="32"/>
-      <c r="T18" s="32"/>
-      <c r="U18" s="52" t="s">
-        <v>88</v>
-      </c>
-      <c r="V18" s="32"/>
-      <c r="W18" s="64" t="s">
-        <v>124</v>
-      </c>
-      <c r="X18" s="32"/>
-      <c r="Y18" s="32"/>
-      <c r="Z18" s="32"/>
-      <c r="AA18" s="52" t="s">
-        <v>108</v>
-      </c>
-      <c r="AB18" s="52"/>
-      <c r="AC18" s="52"/>
-      <c r="AD18" s="31"/>
-      <c r="AE18" s="31"/>
-      <c r="AF18" s="41"/>
+      <c r="S18" s="4"/>
+      <c r="T18" s="4"/>
+      <c r="U18" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="V18" s="4"/>
+      <c r="W18" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="X18" s="4"/>
+      <c r="Y18" s="4"/>
+      <c r="Z18" s="4"/>
+      <c r="AA18" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="AB18" s="11"/>
+      <c r="AC18" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="AD18" s="10"/>
+      <c r="AE18" s="10"/>
+      <c r="AF18" s="40"/>
     </row>
-    <row r="19" spans="1:155" s="3" customFormat="1" ht="89.45" customHeight="1" thickBot="1">
-      <c r="A19" s="56" t="s">
-        <v>125</v>
-      </c>
-      <c r="B19" s="85" t="s">
-        <v>126</v>
-      </c>
-      <c r="C19" s="43"/>
-      <c r="D19" s="43"/>
-      <c r="E19" s="44" t="s">
+    <row r="19" spans="1:155" ht="18" customHeight="1">
+      <c r="A19" s="97"/>
+      <c r="B19" s="115"/>
+      <c r="C19" s="32"/>
+      <c r="D19" s="32"/>
+      <c r="E19" s="32"/>
+      <c r="F19" s="32"/>
+      <c r="G19" s="32"/>
+      <c r="H19" s="32"/>
+      <c r="I19" s="32"/>
+      <c r="J19" s="52" t="s">
         <v>127</v>
       </c>
-      <c r="F19" s="44" t="s">
+      <c r="K19" s="32"/>
+      <c r="L19" s="32"/>
+      <c r="M19" s="32"/>
+      <c r="N19" s="32"/>
+      <c r="O19" s="52" t="s">
+        <v>112</v>
+      </c>
+      <c r="P19" s="32"/>
+      <c r="Q19" s="32"/>
+      <c r="R19" s="64" t="s">
+        <v>103</v>
+      </c>
+      <c r="S19" s="32"/>
+      <c r="T19" s="32"/>
+      <c r="U19" s="52" t="s">
+        <v>92</v>
+      </c>
+      <c r="V19" s="32"/>
+      <c r="W19" s="64" t="s">
         <v>128</v>
       </c>
-      <c r="G19" s="44" t="s">
+      <c r="X19" s="32"/>
+      <c r="Y19" s="32"/>
+      <c r="Z19" s="32"/>
+      <c r="AA19" s="52" t="s">
+        <v>112</v>
+      </c>
+      <c r="AB19" s="52"/>
+      <c r="AC19" s="52"/>
+      <c r="AD19" s="31"/>
+      <c r="AE19" s="31"/>
+      <c r="AF19" s="41"/>
+    </row>
+    <row r="20" spans="1:155" s="3" customFormat="1" ht="89.45" customHeight="1">
+      <c r="A20" s="56" t="s">
         <v>129</v>
       </c>
-      <c r="H19" s="43"/>
-      <c r="I19" s="44" t="s">
+      <c r="B20" s="85" t="s">
         <v>130</v>
       </c>
-      <c r="J19" s="43" t="s">
+      <c r="C20" s="43"/>
+      <c r="D20" s="43"/>
+      <c r="E20" s="44" t="s">
         <v>131</v>
       </c>
-      <c r="K19" s="43" t="s">
+      <c r="F20" s="44" t="s">
         <v>132</v>
       </c>
-      <c r="L19" s="43" t="s">
+      <c r="G20" s="44" t="s">
         <v>133</v>
       </c>
-      <c r="M19" s="43" t="s">
+      <c r="H20" s="43"/>
+      <c r="I20" s="44" t="s">
         <v>134</v>
       </c>
-      <c r="N19" s="43"/>
-      <c r="O19" s="44" t="s">
+      <c r="J20" s="43" t="s">
         <v>135</v>
       </c>
-      <c r="P19" s="44" t="s">
+      <c r="K20" s="43" t="s">
         <v>136</v>
       </c>
-      <c r="Q19" s="44" t="s">
+      <c r="L20" s="43" t="s">
         <v>137</v>
       </c>
-      <c r="R19" s="57" t="s">
+      <c r="M20" s="43" t="s">
         <v>138</v>
       </c>
-      <c r="S19" s="58" t="s">
+      <c r="N20" s="43"/>
+      <c r="O20" s="44" t="s">
         <v>139</v>
       </c>
-      <c r="T19" s="57"/>
-      <c r="U19" s="58" t="s">
+      <c r="P20" s="44" t="s">
         <v>140</v>
       </c>
-      <c r="V19" s="57"/>
-      <c r="W19" s="59" t="s">
+      <c r="Q20" s="44" t="s">
         <v>141</v>
       </c>
-      <c r="X19" s="57"/>
-      <c r="Y19" s="58" t="s">
+      <c r="R20" s="57" t="s">
         <v>142</v>
       </c>
-      <c r="Z19" s="57"/>
-      <c r="AA19" s="58" t="s">
+      <c r="S20" s="58" t="s">
         <v>143</v>
       </c>
-      <c r="AB19" s="58" t="s">
+      <c r="T20" s="57"/>
+      <c r="U20" s="58" t="s">
         <v>144</v>
       </c>
-      <c r="AC19" s="58" t="s">
+      <c r="V20" s="57"/>
+      <c r="W20" s="59" t="s">
         <v>145</v>
       </c>
-      <c r="AD19" s="57"/>
-      <c r="AE19" s="57"/>
-      <c r="AF19" s="60"/>
+      <c r="X20" s="57"/>
+      <c r="Y20" s="58" t="s">
+        <v>146</v>
+      </c>
+      <c r="Z20" s="57"/>
+      <c r="AA20" s="58" t="s">
+        <v>147</v>
+      </c>
+      <c r="AB20" s="58" t="s">
+        <v>148</v>
+      </c>
+      <c r="AC20" s="58" t="s">
+        <v>149</v>
+      </c>
+      <c r="AD20" s="57"/>
+      <c r="AE20" s="57"/>
+      <c r="AF20" s="60"/>
     </row>
-    <row r="20" spans="1:155" s="1" customFormat="1" ht="36" customHeight="1">
-      <c r="A20" s="21"/>
-      <c r="B20" s="110" t="s">
-        <v>146</v>
-      </c>
-      <c r="C20" s="22" t="s">
-        <v>147</v>
-      </c>
-      <c r="D20" s="22" t="s">
-        <v>148</v>
-      </c>
-      <c r="E20" s="22" t="s">
-        <v>149</v>
-      </c>
-      <c r="F20" s="22" t="s">
+    <row r="21" spans="1:155" s="1" customFormat="1" ht="36" customHeight="1">
+      <c r="A21" s="21"/>
+      <c r="B21" s="110" t="s">
         <v>150</v>
       </c>
-      <c r="G20" s="22" t="s">
+      <c r="C21" s="22" t="s">
         <v>151</v>
       </c>
-      <c r="H20" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="I20" s="22" t="s">
+      <c r="D21" s="22" t="s">
         <v>152</v>
       </c>
-      <c r="J20" s="22" t="s">
+      <c r="E21" s="22" t="s">
         <v>153</v>
       </c>
-      <c r="K20" s="22" t="s">
+      <c r="F21" s="22" t="s">
         <v>154</v>
       </c>
-      <c r="L20" s="22" t="s">
+      <c r="G21" s="22" t="s">
         <v>155</v>
       </c>
-      <c r="M20" s="22" t="s">
+      <c r="H21" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="I21" s="22" t="s">
         <v>156</v>
       </c>
-      <c r="N20" s="22" t="s">
+      <c r="J21" s="22" t="s">
         <v>157</v>
       </c>
-      <c r="O20" s="22" t="s">
+      <c r="K21" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="P20" s="22" t="s">
+      <c r="L21" s="22" t="s">
         <v>159</v>
       </c>
-      <c r="Q20" s="22" t="s">
+      <c r="M21" s="22" t="s">
         <v>160</v>
       </c>
-      <c r="R20" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="S20" s="22" t="s">
+      <c r="N21" s="22" t="s">
         <v>161</v>
       </c>
-      <c r="T20" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="U20" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="V20" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="W20" s="22" t="s">
+      <c r="O21" s="22" t="s">
         <v>162</v>
       </c>
-      <c r="X20" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="Y20" s="22" t="s">
+      <c r="P21" s="22" t="s">
         <v>163</v>
       </c>
-      <c r="Z20" s="22" t="s">
+      <c r="Q21" s="22" t="s">
         <v>164</v>
       </c>
-      <c r="AA20" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="AB20" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="AC20" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="AD20" s="22" t="s">
+      <c r="R21" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="S21" s="22" t="s">
         <v>165</v>
       </c>
-      <c r="AE20" s="22" t="s">
+      <c r="T21" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="U21" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="V21" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="W21" s="22" t="s">
         <v>166</v>
       </c>
-      <c r="AF20" s="23" t="s">
+      <c r="X21" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="Y21" s="22" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="21" spans="1:155" ht="18" customHeight="1">
-      <c r="A21" s="24"/>
-      <c r="B21" s="111"/>
-      <c r="C21" s="25" t="s">
+      <c r="Z21" s="22" t="s">
         <v>168</v>
       </c>
-      <c r="D21" s="25" t="s">
+      <c r="AA21" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="AB21" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="AC21" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="AD21" s="22" t="s">
         <v>169</v>
       </c>
-      <c r="E21" s="25" t="s">
+      <c r="AE21" s="22" t="s">
         <v>170</v>
       </c>
-      <c r="F21" s="25" t="s">
+      <c r="AF21" s="23" t="s">
         <v>171</v>
-      </c>
-      <c r="G21" s="4"/>
-      <c r="H21" s="4"/>
-      <c r="I21" s="13" t="s">
-        <v>172</v>
-      </c>
-      <c r="J21" s="13" t="s">
-        <v>173</v>
-      </c>
-      <c r="K21" s="13" t="s">
-        <v>174</v>
-      </c>
-      <c r="L21" s="14"/>
-      <c r="M21" s="13" t="s">
-        <v>175</v>
-      </c>
-      <c r="N21" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="O21" s="13" t="s">
-        <v>177</v>
-      </c>
-      <c r="P21" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q21" s="13" t="s">
-        <v>179</v>
-      </c>
-      <c r="R21" s="14"/>
-      <c r="S21" s="13" t="s">
-        <v>179</v>
-      </c>
-      <c r="T21" s="14"/>
-      <c r="U21" s="4"/>
-      <c r="V21" s="4"/>
-      <c r="W21" s="13" t="s">
-        <v>180</v>
-      </c>
-      <c r="X21" s="4"/>
-      <c r="Y21" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="Z21" s="13" t="s">
-        <v>182</v>
-      </c>
-      <c r="AA21" s="4"/>
-      <c r="AB21" s="4"/>
-      <c r="AC21" s="4"/>
-      <c r="AD21" s="13" t="s">
-        <v>183</v>
-      </c>
-      <c r="AE21" s="13" t="s">
-        <v>184</v>
-      </c>
-      <c r="AF21" s="26" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="22" spans="1:155" ht="18" customHeight="1">
       <c r="A22" s="24"/>
       <c r="B22" s="111"/>
       <c r="C22" s="25" t="s">
-        <v>186</v>
+        <v>172</v>
       </c>
       <c r="D22" s="25" t="s">
-        <v>187</v>
+        <v>173</v>
       </c>
       <c r="E22" s="25" t="s">
-        <v>188</v>
-      </c>
-      <c r="F22" s="4"/>
+        <v>174</v>
+      </c>
+      <c r="F22" s="25" t="s">
+        <v>175</v>
+      </c>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
-      <c r="I22" s="14"/>
+      <c r="I22" s="13" t="s">
+        <v>176</v>
+      </c>
       <c r="J22" s="13" t="s">
-        <v>189</v>
-      </c>
-      <c r="K22" s="14"/>
-      <c r="L22" s="13" t="s">
-        <v>190</v>
-      </c>
+        <v>177</v>
+      </c>
+      <c r="K22" s="13" t="s">
+        <v>178</v>
+      </c>
+      <c r="L22" s="14"/>
       <c r="M22" s="13" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="N22" s="13" t="s">
-        <v>191</v>
+        <v>180</v>
       </c>
       <c r="O22" s="13" t="s">
-        <v>192</v>
+        <v>181</v>
       </c>
       <c r="P22" s="13" t="s">
-        <v>193</v>
+        <v>182</v>
       </c>
       <c r="Q22" s="13" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="R22" s="14"/>
       <c r="S22" s="13" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="T22" s="14"/>
       <c r="U22" s="4"/>
       <c r="V22" s="4"/>
       <c r="W22" s="13" t="s">
-        <v>195</v>
+        <v>184</v>
       </c>
       <c r="X22" s="4"/>
       <c r="Y22" s="13" t="s">
-        <v>196</v>
-      </c>
-      <c r="Z22" s="13"/>
+        <v>185</v>
+      </c>
+      <c r="Z22" s="13" t="s">
+        <v>186</v>
+      </c>
       <c r="AA22" s="4"/>
       <c r="AB22" s="4"/>
       <c r="AC22" s="4"/>
       <c r="AD22" s="13" t="s">
-        <v>197</v>
+        <v>187</v>
       </c>
       <c r="AE22" s="13" t="s">
-        <v>198</v>
+        <v>188</v>
       </c>
       <c r="AF22" s="26" t="s">
-        <v>199</v>
+        <v>189</v>
       </c>
     </row>
     <row r="23" spans="1:155" ht="18" customHeight="1">
       <c r="A23" s="24"/>
       <c r="B23" s="111"/>
       <c r="C23" s="25" t="s">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="D23" s="25" t="s">
-        <v>201</v>
-      </c>
-      <c r="E23" s="4"/>
+        <v>191</v>
+      </c>
+      <c r="E23" s="25" t="s">
+        <v>192</v>
+      </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
       <c r="I23" s="14"/>
       <c r="J23" s="13" t="s">
-        <v>176</v>
+        <v>193</v>
       </c>
       <c r="K23" s="14"/>
       <c r="L23" s="13" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="M23" s="13" t="s">
-        <v>191</v>
+        <v>180</v>
       </c>
       <c r="N23" s="13" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="O23" s="13" t="s">
-        <v>204</v>
-      </c>
-      <c r="P23" s="14"/>
+        <v>196</v>
+      </c>
+      <c r="P23" s="13" t="s">
+        <v>197</v>
+      </c>
       <c r="Q23" s="13" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="R23" s="14"/>
       <c r="S23" s="13" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="T23" s="14"/>
       <c r="U23" s="4"/>
       <c r="V23" s="4"/>
       <c r="W23" s="13" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="X23" s="4"/>
       <c r="Y23" s="13" t="s">
-        <v>189</v>
-      </c>
-      <c r="Z23" s="14"/>
+        <v>200</v>
+      </c>
+      <c r="Z23" s="13"/>
       <c r="AA23" s="4"/>
       <c r="AB23" s="4"/>
       <c r="AC23" s="4"/>
       <c r="AD23" s="13" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="AE23" s="13" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="AF23" s="26" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
     </row>
     <row r="24" spans="1:155" ht="18" customHeight="1">
       <c r="A24" s="24"/>
       <c r="B24" s="111"/>
-      <c r="C24" s="4"/>
-      <c r="D24" s="4"/>
+      <c r="C24" s="25" t="s">
+        <v>204</v>
+      </c>
+      <c r="D24" s="25" t="s">
+        <v>205</v>
+      </c>
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
       <c r="I24" s="14"/>
       <c r="J24" s="13" t="s">
-        <v>191</v>
+        <v>180</v>
       </c>
       <c r="K24" s="14"/>
       <c r="L24" s="13" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="M24" s="13" t="s">
-        <v>210</v>
+        <v>195</v>
       </c>
       <c r="N24" s="13" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="O24" s="13" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="P24" s="14"/>
       <c r="Q24" s="13" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="R24" s="14"/>
       <c r="S24" s="13" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="T24" s="14"/>
       <c r="U24" s="4"/>
       <c r="V24" s="4"/>
       <c r="W24" s="13" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="X24" s="4"/>
       <c r="Y24" s="13" t="s">
-        <v>176</v>
+        <v>193</v>
       </c>
       <c r="Z24" s="14"/>
       <c r="AA24" s="4"/>
       <c r="AB24" s="4"/>
       <c r="AC24" s="4"/>
       <c r="AD24" s="13" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="AE24" s="13" t="s">
-        <v>214</v>
-      </c>
-      <c r="AF24" s="27"/>
+        <v>211</v>
+      </c>
+      <c r="AF24" s="26" t="s">
+        <v>212</v>
+      </c>
     </row>
     <row r="25" spans="1:155" ht="18" customHeight="1">
       <c r="A25" s="24"/>
@@ -3710,41 +3743,45 @@
       <c r="H25" s="4"/>
       <c r="I25" s="14"/>
       <c r="J25" s="13" t="s">
-        <v>210</v>
+        <v>195</v>
       </c>
       <c r="K25" s="14"/>
       <c r="L25" s="13" t="s">
+        <v>213</v>
+      </c>
+      <c r="M25" s="13" t="s">
+        <v>214</v>
+      </c>
+      <c r="N25" s="13" t="s">
+        <v>214</v>
+      </c>
+      <c r="O25" s="13" t="s">
         <v>215</v>
-      </c>
-      <c r="M25" s="14"/>
-      <c r="N25" s="14"/>
-      <c r="O25" s="13" t="s">
-        <v>216</v>
       </c>
       <c r="P25" s="14"/>
       <c r="Q25" s="13" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="R25" s="14"/>
       <c r="S25" s="13" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="T25" s="14"/>
       <c r="U25" s="4"/>
       <c r="V25" s="4"/>
       <c r="W25" s="13" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="X25" s="4"/>
       <c r="Y25" s="13" t="s">
-        <v>191</v>
+        <v>180</v>
       </c>
       <c r="Z25" s="14"/>
       <c r="AA25" s="4"/>
       <c r="AB25" s="4"/>
       <c r="AC25" s="4"/>
       <c r="AD25" s="13" t="s">
-        <v>168</v>
+        <v>217</v>
       </c>
       <c r="AE25" s="13" t="s">
         <v>218</v>
@@ -3752,289 +3789,142 @@
       <c r="AF25" s="27"/>
     </row>
     <row r="26" spans="1:155" ht="18" customHeight="1">
-      <c r="A26" s="28"/>
+      <c r="A26" s="24"/>
       <c r="B26" s="111"/>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
-      <c r="E26" s="6"/>
-      <c r="F26" s="6"/>
-      <c r="G26" s="6"/>
-      <c r="H26" s="6"/>
-      <c r="I26" s="17"/>
-      <c r="J26" s="18" t="s">
-        <v>203</v>
-      </c>
-      <c r="K26" s="17"/>
-      <c r="L26" s="18" t="s">
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4"/>
+      <c r="F26" s="4"/>
+      <c r="G26" s="4"/>
+      <c r="H26" s="4"/>
+      <c r="I26" s="14"/>
+      <c r="J26" s="13" t="s">
+        <v>214</v>
+      </c>
+      <c r="K26" s="14"/>
+      <c r="L26" s="13" t="s">
         <v>219</v>
       </c>
-      <c r="M26" s="17"/>
-      <c r="N26" s="17"/>
-      <c r="O26" s="18" t="s">
+      <c r="M26" s="14"/>
+      <c r="N26" s="14"/>
+      <c r="O26" s="13" t="s">
         <v>220</v>
       </c>
-      <c r="P26" s="17"/>
-      <c r="Q26" s="18" t="s">
+      <c r="P26" s="14"/>
+      <c r="Q26" s="13" t="s">
+        <v>220</v>
+      </c>
+      <c r="R26" s="14"/>
+      <c r="S26" s="13" t="s">
+        <v>220</v>
+      </c>
+      <c r="T26" s="14"/>
+      <c r="U26" s="4"/>
+      <c r="V26" s="4"/>
+      <c r="W26" s="13" t="s">
         <v>221</v>
       </c>
-      <c r="R26" s="17"/>
-      <c r="S26" s="18" t="s">
-        <v>221</v>
-      </c>
-      <c r="T26" s="17"/>
-      <c r="U26" s="6"/>
-      <c r="V26" s="6"/>
-      <c r="W26" s="6"/>
-      <c r="X26" s="6"/>
-      <c r="Y26" s="18" t="s">
-        <v>203</v>
-      </c>
-      <c r="Z26" s="17"/>
-      <c r="AA26" s="6"/>
-      <c r="AB26" s="6"/>
-      <c r="AC26" s="6"/>
-      <c r="AD26" s="18" t="s">
-        <v>186</v>
-      </c>
-      <c r="AE26" s="17"/>
-      <c r="AF26" s="29"/>
+      <c r="X26" s="4"/>
+      <c r="Y26" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="Z26" s="14"/>
+      <c r="AA26" s="4"/>
+      <c r="AB26" s="4"/>
+      <c r="AC26" s="4"/>
+      <c r="AD26" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="AE26" s="13" t="s">
+        <v>222</v>
+      </c>
+      <c r="AF26" s="27"/>
     </row>
-    <row r="27" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1" thickBot="1">
-      <c r="A27" s="30"/>
-      <c r="B27" s="112"/>
-      <c r="C27" s="32"/>
-      <c r="D27" s="32"/>
-      <c r="E27" s="32"/>
-      <c r="F27" s="32"/>
-      <c r="G27" s="32"/>
-      <c r="H27" s="32"/>
-      <c r="I27" s="32"/>
-      <c r="J27" s="32"/>
-      <c r="K27" s="32"/>
-      <c r="L27" s="32"/>
-      <c r="M27" s="32"/>
-      <c r="N27" s="32"/>
-      <c r="O27" s="32"/>
-      <c r="P27" s="32"/>
-      <c r="Q27" s="32"/>
-      <c r="R27" s="32"/>
-      <c r="S27" s="32"/>
-      <c r="T27" s="32"/>
-      <c r="U27" s="32"/>
-      <c r="V27" s="32"/>
-      <c r="W27" s="32"/>
-      <c r="X27" s="32"/>
-      <c r="Y27" s="33" t="s">
-        <v>174</v>
-      </c>
-      <c r="Z27" s="34"/>
-      <c r="AA27" s="32"/>
-      <c r="AB27" s="32"/>
-      <c r="AC27" s="32"/>
-      <c r="AD27" s="33" t="s">
-        <v>174</v>
-      </c>
-      <c r="AE27" s="34"/>
-      <c r="AF27" s="35"/>
-      <c r="AG27" s="2"/>
-      <c r="AH27" s="2"/>
-      <c r="AI27" s="2"/>
-      <c r="AJ27" s="2"/>
-      <c r="AK27" s="2"/>
-      <c r="AL27" s="2"/>
-      <c r="AM27" s="2"/>
-      <c r="AN27" s="2"/>
-      <c r="AO27" s="2"/>
-      <c r="AP27" s="2"/>
-      <c r="AQ27" s="2"/>
-      <c r="AR27" s="2"/>
-      <c r="AS27" s="2"/>
-      <c r="AT27" s="2"/>
-      <c r="AU27" s="2"/>
-      <c r="AV27" s="2"/>
-      <c r="AW27" s="2"/>
-      <c r="AX27" s="2"/>
-      <c r="AY27" s="2"/>
-      <c r="AZ27" s="2"/>
-      <c r="BA27" s="2"/>
-      <c r="BB27" s="2"/>
-      <c r="BC27" s="2"/>
-      <c r="BD27" s="2"/>
-      <c r="BE27" s="2"/>
-      <c r="BF27" s="2"/>
-      <c r="BG27" s="2"/>
-      <c r="BH27" s="2"/>
-      <c r="BI27" s="2"/>
-      <c r="BJ27" s="2"/>
-      <c r="BK27" s="2"/>
-      <c r="BL27" s="2"/>
-      <c r="BM27" s="2"/>
-      <c r="BN27" s="2"/>
-      <c r="BO27" s="2"/>
-      <c r="BP27" s="2"/>
-      <c r="BQ27" s="2"/>
-      <c r="BR27" s="2"/>
-      <c r="BS27" s="2"/>
-      <c r="BT27" s="2"/>
-      <c r="BU27" s="2"/>
-      <c r="BV27" s="2"/>
-      <c r="BW27" s="2"/>
-      <c r="BX27" s="2"/>
-      <c r="BY27" s="2"/>
-      <c r="BZ27" s="2"/>
-      <c r="CA27" s="2"/>
-      <c r="CB27" s="2"/>
-      <c r="CC27" s="2"/>
-      <c r="CD27" s="2"/>
-      <c r="CE27" s="2"/>
-      <c r="CF27" s="2"/>
-      <c r="CG27" s="2"/>
-      <c r="CH27" s="2"/>
-      <c r="CI27" s="2"/>
-      <c r="CJ27" s="2"/>
-      <c r="CK27" s="2"/>
-      <c r="CL27" s="2"/>
-      <c r="CM27" s="2"/>
-      <c r="CN27" s="2"/>
-      <c r="CO27" s="2"/>
-      <c r="CP27" s="2"/>
-      <c r="CQ27" s="2"/>
-      <c r="CR27" s="2"/>
-      <c r="CS27" s="2"/>
-      <c r="CT27" s="2"/>
-      <c r="CU27" s="2"/>
-      <c r="CV27" s="2"/>
-      <c r="CW27" s="2"/>
-      <c r="CX27" s="2"/>
-      <c r="CY27" s="2"/>
-      <c r="CZ27" s="2"/>
-      <c r="DA27" s="2"/>
-      <c r="DB27" s="2"/>
-      <c r="DC27" s="2"/>
-      <c r="DD27" s="2"/>
-      <c r="DE27" s="2"/>
-      <c r="DF27" s="2"/>
-      <c r="DG27" s="2"/>
-      <c r="DH27" s="2"/>
-      <c r="DI27" s="2"/>
-      <c r="DJ27" s="2"/>
-      <c r="DK27" s="2"/>
-      <c r="DL27" s="2"/>
-      <c r="DM27" s="2"/>
-      <c r="DN27" s="2"/>
-      <c r="DO27" s="2"/>
-      <c r="DP27" s="2"/>
-      <c r="DQ27" s="2"/>
-      <c r="DR27" s="2"/>
-      <c r="DS27" s="2"/>
-      <c r="DT27" s="2"/>
-      <c r="DU27" s="2"/>
-      <c r="DV27" s="2"/>
-      <c r="DW27" s="2"/>
-      <c r="DX27" s="2"/>
-      <c r="DY27" s="2"/>
-      <c r="DZ27" s="2"/>
-      <c r="EA27" s="2"/>
-      <c r="EB27" s="2"/>
-      <c r="EC27" s="2"/>
-      <c r="ED27" s="2"/>
-      <c r="EE27" s="2"/>
-      <c r="EF27" s="2"/>
-      <c r="EG27" s="2"/>
-      <c r="EH27" s="2"/>
-      <c r="EI27" s="2"/>
-      <c r="EJ27" s="2"/>
-      <c r="EK27" s="2"/>
-      <c r="EL27" s="2"/>
-      <c r="EM27" s="2"/>
-      <c r="EN27" s="2"/>
-      <c r="EO27" s="2"/>
-      <c r="EP27" s="2"/>
-      <c r="EQ27" s="2"/>
-      <c r="ER27" s="2"/>
-      <c r="ES27" s="2"/>
-      <c r="ET27" s="2"/>
-      <c r="EU27" s="2"/>
-      <c r="EV27" s="2"/>
-      <c r="EW27" s="2"/>
-      <c r="EX27" s="2"/>
-      <c r="EY27" s="2"/>
+    <row r="27" spans="1:155" ht="18" customHeight="1">
+      <c r="A27" s="28"/>
+      <c r="B27" s="111"/>
+      <c r="C27" s="6"/>
+      <c r="D27" s="6"/>
+      <c r="E27" s="6"/>
+      <c r="F27" s="6"/>
+      <c r="G27" s="6"/>
+      <c r="H27" s="6"/>
+      <c r="I27" s="17"/>
+      <c r="J27" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="K27" s="17"/>
+      <c r="L27" s="18" t="s">
+        <v>223</v>
+      </c>
+      <c r="M27" s="17"/>
+      <c r="N27" s="17"/>
+      <c r="O27" s="18" t="s">
+        <v>224</v>
+      </c>
+      <c r="P27" s="17"/>
+      <c r="Q27" s="18" t="s">
+        <v>225</v>
+      </c>
+      <c r="R27" s="17"/>
+      <c r="S27" s="18" t="s">
+        <v>225</v>
+      </c>
+      <c r="T27" s="17"/>
+      <c r="U27" s="6"/>
+      <c r="V27" s="6"/>
+      <c r="W27" s="6"/>
+      <c r="X27" s="6"/>
+      <c r="Y27" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="Z27" s="17"/>
+      <c r="AA27" s="6"/>
+      <c r="AB27" s="6"/>
+      <c r="AC27" s="6"/>
+      <c r="AD27" s="18" t="s">
+        <v>190</v>
+      </c>
+      <c r="AE27" s="17"/>
+      <c r="AF27" s="29"/>
     </row>
-    <row r="28" spans="1:155" s="10" customFormat="1" ht="36" customHeight="1">
-      <c r="A28" s="21"/>
-      <c r="B28" s="117" t="s">
-        <v>222</v>
-      </c>
-      <c r="C28" s="36" t="s">
-        <v>223</v>
-      </c>
-      <c r="D28" s="36" t="s">
-        <v>223</v>
-      </c>
-      <c r="E28" s="36" t="s">
-        <v>224</v>
-      </c>
-      <c r="F28" s="36" t="s">
-        <v>225</v>
-      </c>
-      <c r="G28" s="36" t="s">
-        <v>226</v>
-      </c>
-      <c r="H28" s="37"/>
-      <c r="I28" s="36" t="s">
-        <v>227</v>
-      </c>
-      <c r="J28" s="36" t="s">
-        <v>228</v>
-      </c>
-      <c r="K28" s="36" t="s">
-        <v>229</v>
-      </c>
-      <c r="L28" s="36" t="s">
-        <v>230</v>
-      </c>
-      <c r="M28" s="36" t="s">
-        <v>231</v>
-      </c>
-      <c r="N28" s="36" t="s">
-        <v>232</v>
-      </c>
-      <c r="O28" s="36" t="s">
-        <v>233</v>
-      </c>
-      <c r="P28" s="36" t="s">
-        <v>234</v>
-      </c>
-      <c r="Q28" s="36" t="s">
-        <v>235</v>
-      </c>
-      <c r="R28" s="36" t="s">
-        <v>227</v>
-      </c>
-      <c r="S28" s="36" t="s">
-        <v>233</v>
-      </c>
-      <c r="T28" s="37"/>
-      <c r="U28" s="36" t="s">
-        <v>233</v>
-      </c>
-      <c r="V28" s="37"/>
-      <c r="W28" s="36" t="s">
-        <v>236</v>
-      </c>
-      <c r="X28" s="37"/>
-      <c r="Y28" s="37"/>
-      <c r="Z28" s="36" t="s">
-        <v>237</v>
-      </c>
-      <c r="AA28" s="37" t="s">
-        <v>238</v>
-      </c>
-      <c r="AB28" s="37"/>
-      <c r="AC28" s="37"/>
-      <c r="AD28" s="38"/>
-      <c r="AE28" s="38"/>
-      <c r="AF28" s="39"/>
+    <row r="28" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1">
+      <c r="A28" s="30"/>
+      <c r="B28" s="112"/>
+      <c r="C28" s="32"/>
+      <c r="D28" s="32"/>
+      <c r="E28" s="32"/>
+      <c r="F28" s="32"/>
+      <c r="G28" s="32"/>
+      <c r="H28" s="32"/>
+      <c r="I28" s="32"/>
+      <c r="J28" s="32"/>
+      <c r="K28" s="32"/>
+      <c r="L28" s="32"/>
+      <c r="M28" s="32"/>
+      <c r="N28" s="32"/>
+      <c r="O28" s="32"/>
+      <c r="P28" s="32"/>
+      <c r="Q28" s="32"/>
+      <c r="R28" s="32"/>
+      <c r="S28" s="32"/>
+      <c r="T28" s="32"/>
+      <c r="U28" s="32"/>
+      <c r="V28" s="32"/>
+      <c r="W28" s="32"/>
+      <c r="X28" s="32"/>
+      <c r="Y28" s="33" t="s">
+        <v>178</v>
+      </c>
+      <c r="Z28" s="34"/>
+      <c r="AA28" s="32"/>
+      <c r="AB28" s="32"/>
+      <c r="AC28" s="32"/>
+      <c r="AD28" s="33" t="s">
+        <v>178</v>
+      </c>
+      <c r="AE28" s="34"/>
+      <c r="AF28" s="35"/>
       <c r="AG28" s="2"/>
       <c r="AH28" s="2"/>
       <c r="AI28" s="2"/>
@@ -4159,69 +4049,81 @@
       <c r="EX28" s="2"/>
       <c r="EY28" s="2"/>
     </row>
-    <row r="29" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1">
-      <c r="A29" s="24"/>
-      <c r="B29" s="118"/>
-      <c r="C29" s="13" t="s">
+    <row r="29" spans="1:155" s="10" customFormat="1" ht="36" customHeight="1">
+      <c r="A29" s="21"/>
+      <c r="B29" s="117" t="s">
+        <v>226</v>
+      </c>
+      <c r="C29" s="36" t="s">
+        <v>227</v>
+      </c>
+      <c r="D29" s="36" t="s">
+        <v>227</v>
+      </c>
+      <c r="E29" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="F29" s="36" t="s">
+        <v>228</v>
+      </c>
+      <c r="G29" s="36" t="s">
+        <v>229</v>
+      </c>
+      <c r="H29" s="37"/>
+      <c r="I29" s="36" t="s">
+        <v>230</v>
+      </c>
+      <c r="J29" s="36" t="s">
+        <v>231</v>
+      </c>
+      <c r="K29" s="36" t="s">
+        <v>232</v>
+      </c>
+      <c r="L29" s="36" t="s">
+        <v>233</v>
+      </c>
+      <c r="M29" s="36" t="s">
+        <v>234</v>
+      </c>
+      <c r="N29" s="36" t="s">
+        <v>235</v>
+      </c>
+      <c r="O29" s="36" t="s">
+        <v>236</v>
+      </c>
+      <c r="P29" s="36" t="s">
+        <v>237</v>
+      </c>
+      <c r="Q29" s="36" t="s">
+        <v>238</v>
+      </c>
+      <c r="R29" s="36" t="s">
+        <v>230</v>
+      </c>
+      <c r="S29" s="36" t="s">
+        <v>236</v>
+      </c>
+      <c r="T29" s="37"/>
+      <c r="U29" s="36" t="s">
+        <v>236</v>
+      </c>
+      <c r="V29" s="37"/>
+      <c r="W29" s="36" t="s">
         <v>239</v>
       </c>
-      <c r="D29" s="13" t="s">
-        <v>239</v>
-      </c>
-      <c r="E29" s="4"/>
-      <c r="F29" s="13" t="s">
+      <c r="X29" s="37"/>
+      <c r="Y29" s="37"/>
+      <c r="Z29" s="36" t="s">
         <v>240</v>
       </c>
-      <c r="G29" s="13" t="s">
-        <v>239</v>
-      </c>
-      <c r="H29" s="4"/>
-      <c r="I29" s="4"/>
-      <c r="J29" s="13" t="s">
+      <c r="AA29" s="37" t="s">
         <v>241</v>
       </c>
-      <c r="K29" s="13" t="s">
-        <v>242</v>
-      </c>
-      <c r="L29" s="13" t="s">
-        <v>243</v>
-      </c>
-      <c r="M29" s="13" t="s">
-        <v>244</v>
-      </c>
-      <c r="N29" s="13" t="s">
-        <v>245</v>
-      </c>
-      <c r="O29" s="13" t="s">
-        <v>246</v>
-      </c>
-      <c r="P29" s="13" t="s">
-        <v>247</v>
-      </c>
-      <c r="Q29" s="13" t="s">
-        <v>248</v>
-      </c>
-      <c r="R29" s="14"/>
-      <c r="S29" s="13" t="s">
-        <v>246</v>
-      </c>
-      <c r="T29" s="4"/>
-      <c r="U29" s="13" t="s">
-        <v>246</v>
-      </c>
-      <c r="V29" s="4"/>
-      <c r="W29" s="13" t="s">
-        <v>249</v>
-      </c>
-      <c r="X29" s="4"/>
-      <c r="Y29" s="4"/>
-      <c r="Z29" s="13" t="s">
-        <v>250</v>
-      </c>
-      <c r="AA29" s="4"/>
-      <c r="AB29" s="4"/>
-      <c r="AC29" s="4"/>
-      <c r="AF29" s="40"/>
+      <c r="AB29" s="37"/>
+      <c r="AC29" s="37"/>
+      <c r="AD29" s="38"/>
+      <c r="AE29" s="38"/>
+      <c r="AF29" s="39"/>
       <c r="AG29" s="2"/>
       <c r="AH29" s="2"/>
       <c r="AI29" s="2"/>
@@ -4350,55 +4252,61 @@
       <c r="A30" s="24"/>
       <c r="B30" s="118"/>
       <c r="C30" s="13" t="s">
-        <v>251</v>
+        <v>242</v>
       </c>
       <c r="D30" s="13" t="s">
-        <v>251</v>
+        <v>242</v>
       </c>
       <c r="E30" s="4"/>
       <c r="F30" s="13" t="s">
-        <v>252</v>
+        <v>243</v>
       </c>
       <c r="G30" s="13" t="s">
-        <v>251</v>
+        <v>242</v>
       </c>
       <c r="H30" s="4"/>
       <c r="I30" s="4"/>
       <c r="J30" s="13" t="s">
-        <v>253</v>
+        <v>244</v>
       </c>
       <c r="K30" s="13" t="s">
-        <v>254</v>
+        <v>245</v>
       </c>
       <c r="L30" s="13" t="s">
-        <v>255</v>
-      </c>
-      <c r="M30" s="14"/>
+        <v>246</v>
+      </c>
+      <c r="M30" s="13" t="s">
+        <v>247</v>
+      </c>
       <c r="N30" s="13" t="s">
-        <v>256</v>
+        <v>248</v>
       </c>
       <c r="O30" s="13" t="s">
-        <v>257</v>
-      </c>
-      <c r="P30" s="14"/>
+        <v>249</v>
+      </c>
+      <c r="P30" s="13" t="s">
+        <v>250</v>
+      </c>
       <c r="Q30" s="13" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="R30" s="14"/>
       <c r="S30" s="13" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="T30" s="4"/>
       <c r="U30" s="13" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="V30" s="4"/>
       <c r="W30" s="13" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="X30" s="4"/>
       <c r="Y30" s="4"/>
-      <c r="Z30" s="14"/>
+      <c r="Z30" s="13" t="s">
+        <v>253</v>
+      </c>
       <c r="AA30" s="4"/>
       <c r="AB30" s="4"/>
       <c r="AC30" s="4"/>
@@ -4531,35 +4439,47 @@
       <c r="A31" s="24"/>
       <c r="B31" s="118"/>
       <c r="C31" s="13" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="D31" s="13" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="E31" s="4"/>
-      <c r="F31" s="4"/>
+      <c r="F31" s="13" t="s">
+        <v>255</v>
+      </c>
       <c r="G31" s="13" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="H31" s="4"/>
       <c r="I31" s="4"/>
-      <c r="J31" s="14"/>
-      <c r="K31" s="14"/>
-      <c r="L31" s="14"/>
+      <c r="J31" s="13" t="s">
+        <v>256</v>
+      </c>
+      <c r="K31" s="13" t="s">
+        <v>257</v>
+      </c>
+      <c r="L31" s="13" t="s">
+        <v>258</v>
+      </c>
       <c r="M31" s="14"/>
-      <c r="N31" s="14"/>
+      <c r="N31" s="13" t="s">
+        <v>259</v>
+      </c>
       <c r="O31" s="13" t="s">
+        <v>260</v>
+      </c>
+      <c r="P31" s="14"/>
+      <c r="Q31" s="13" t="s">
         <v>261</v>
       </c>
-      <c r="P31" s="14"/>
-      <c r="Q31" s="14"/>
       <c r="R31" s="14"/>
       <c r="S31" s="13" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="T31" s="4"/>
       <c r="U31" s="13" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="V31" s="4"/>
       <c r="W31" s="13" t="s">
@@ -4567,7 +4487,7 @@
       </c>
       <c r="X31" s="4"/>
       <c r="Y31" s="4"/>
-      <c r="Z31" s="4"/>
+      <c r="Z31" s="14"/>
       <c r="AA31" s="4"/>
       <c r="AB31" s="4"/>
       <c r="AC31" s="4"/>
@@ -4865,45 +4785,51 @@
       <c r="EX32" s="2"/>
       <c r="EY32" s="2"/>
     </row>
-    <row r="33" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1" thickBot="1">
-      <c r="A33" s="30"/>
-      <c r="B33" s="119"/>
-      <c r="C33" s="33" t="s">
+    <row r="33" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1">
+      <c r="A33" s="24"/>
+      <c r="B33" s="118"/>
+      <c r="C33" s="13" t="s">
         <v>266</v>
       </c>
-      <c r="D33" s="33" t="s">
+      <c r="D33" s="13" t="s">
         <v>266</v>
       </c>
-      <c r="E33" s="32"/>
-      <c r="F33" s="32"/>
-      <c r="G33" s="33" t="s">
+      <c r="E33" s="4"/>
+      <c r="F33" s="4"/>
+      <c r="G33" s="13" t="s">
         <v>266</v>
       </c>
-      <c r="H33" s="32"/>
-      <c r="I33" s="32"/>
-      <c r="J33" s="34"/>
-      <c r="K33" s="34"/>
-      <c r="L33" s="34"/>
-      <c r="M33" s="34"/>
-      <c r="N33" s="34"/>
-      <c r="O33" s="34"/>
-      <c r="P33" s="34"/>
-      <c r="Q33" s="34"/>
-      <c r="R33" s="34"/>
-      <c r="S33" s="34"/>
-      <c r="T33" s="32"/>
-      <c r="U33" s="34"/>
-      <c r="V33" s="32"/>
-      <c r="W33" s="34"/>
-      <c r="X33" s="32"/>
-      <c r="Y33" s="32"/>
-      <c r="Z33" s="32"/>
-      <c r="AA33" s="32"/>
-      <c r="AB33" s="32"/>
-      <c r="AC33" s="32"/>
-      <c r="AD33" s="31"/>
-      <c r="AE33" s="31"/>
-      <c r="AF33" s="41"/>
+      <c r="H33" s="4"/>
+      <c r="I33" s="4"/>
+      <c r="J33" s="14"/>
+      <c r="K33" s="14"/>
+      <c r="L33" s="14"/>
+      <c r="M33" s="14"/>
+      <c r="N33" s="14"/>
+      <c r="O33" s="13" t="s">
+        <v>267</v>
+      </c>
+      <c r="P33" s="14"/>
+      <c r="Q33" s="14"/>
+      <c r="R33" s="14"/>
+      <c r="S33" s="13" t="s">
+        <v>267</v>
+      </c>
+      <c r="T33" s="4"/>
+      <c r="U33" s="13" t="s">
+        <v>267</v>
+      </c>
+      <c r="V33" s="4"/>
+      <c r="W33" s="13" t="s">
+        <v>268</v>
+      </c>
+      <c r="X33" s="4"/>
+      <c r="Y33" s="4"/>
+      <c r="Z33" s="4"/>
+      <c r="AA33" s="4"/>
+      <c r="AB33" s="4"/>
+      <c r="AC33" s="4"/>
+      <c r="AF33" s="40"/>
       <c r="AG33" s="2"/>
       <c r="AH33" s="2"/>
       <c r="AI33" s="2"/>
@@ -5028,280 +4954,395 @@
       <c r="EX33" s="2"/>
       <c r="EY33" s="2"/>
     </row>
-    <row r="34" spans="1:155" ht="18" customHeight="1" thickBot="1">
-      <c r="A34" s="42"/>
-      <c r="B34" s="66" t="s">
-        <v>267</v>
-      </c>
-      <c r="C34" s="43"/>
-      <c r="D34" s="43"/>
-      <c r="E34" s="43"/>
-      <c r="F34" s="43"/>
-      <c r="G34" s="43"/>
-      <c r="H34" s="43"/>
-      <c r="I34" s="43"/>
-      <c r="J34" s="43"/>
-      <c r="K34" s="43"/>
-      <c r="L34" s="43"/>
-      <c r="M34" s="43"/>
-      <c r="N34" s="43"/>
-      <c r="O34" s="43"/>
-      <c r="P34" s="43"/>
-      <c r="Q34" s="43"/>
-      <c r="R34" s="43"/>
-      <c r="S34" s="43"/>
-      <c r="T34" s="43"/>
-      <c r="U34" s="43"/>
-      <c r="V34" s="43"/>
-      <c r="W34" s="43"/>
-      <c r="X34" s="44" t="s">
-        <v>268</v>
-      </c>
-      <c r="Y34" s="44" t="s">
+    <row r="34" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1">
+      <c r="A34" s="30"/>
+      <c r="B34" s="119"/>
+      <c r="C34" s="33" t="s">
         <v>269</v>
       </c>
-      <c r="Z34" s="43"/>
-      <c r="AA34" s="43"/>
-      <c r="AB34" s="43"/>
-      <c r="AC34" s="45"/>
-      <c r="AD34" s="46"/>
-      <c r="AE34" s="46"/>
-      <c r="AF34" s="47"/>
+      <c r="D34" s="33" t="s">
+        <v>269</v>
+      </c>
+      <c r="E34" s="32"/>
+      <c r="F34" s="32"/>
+      <c r="G34" s="33" t="s">
+        <v>269</v>
+      </c>
+      <c r="H34" s="32"/>
+      <c r="I34" s="32"/>
+      <c r="J34" s="34"/>
+      <c r="K34" s="34"/>
+      <c r="L34" s="34"/>
+      <c r="M34" s="34"/>
+      <c r="N34" s="34"/>
+      <c r="O34" s="34"/>
+      <c r="P34" s="34"/>
+      <c r="Q34" s="34"/>
+      <c r="R34" s="34"/>
+      <c r="S34" s="34"/>
+      <c r="T34" s="32"/>
+      <c r="U34" s="34"/>
+      <c r="V34" s="32"/>
+      <c r="W34" s="34"/>
+      <c r="X34" s="32"/>
+      <c r="Y34" s="32"/>
+      <c r="Z34" s="32"/>
+      <c r="AA34" s="32"/>
+      <c r="AB34" s="32"/>
+      <c r="AC34" s="32"/>
+      <c r="AD34" s="31"/>
+      <c r="AE34" s="31"/>
+      <c r="AF34" s="41"/>
+      <c r="AG34" s="2"/>
+      <c r="AH34" s="2"/>
+      <c r="AI34" s="2"/>
+      <c r="AJ34" s="2"/>
+      <c r="AK34" s="2"/>
+      <c r="AL34" s="2"/>
+      <c r="AM34" s="2"/>
+      <c r="AN34" s="2"/>
+      <c r="AO34" s="2"/>
+      <c r="AP34" s="2"/>
+      <c r="AQ34" s="2"/>
+      <c r="AR34" s="2"/>
+      <c r="AS34" s="2"/>
+      <c r="AT34" s="2"/>
+      <c r="AU34" s="2"/>
+      <c r="AV34" s="2"/>
+      <c r="AW34" s="2"/>
+      <c r="AX34" s="2"/>
+      <c r="AY34" s="2"/>
+      <c r="AZ34" s="2"/>
+      <c r="BA34" s="2"/>
+      <c r="BB34" s="2"/>
+      <c r="BC34" s="2"/>
+      <c r="BD34" s="2"/>
+      <c r="BE34" s="2"/>
+      <c r="BF34" s="2"/>
+      <c r="BG34" s="2"/>
+      <c r="BH34" s="2"/>
+      <c r="BI34" s="2"/>
+      <c r="BJ34" s="2"/>
+      <c r="BK34" s="2"/>
+      <c r="BL34" s="2"/>
+      <c r="BM34" s="2"/>
+      <c r="BN34" s="2"/>
+      <c r="BO34" s="2"/>
+      <c r="BP34" s="2"/>
+      <c r="BQ34" s="2"/>
+      <c r="BR34" s="2"/>
+      <c r="BS34" s="2"/>
+      <c r="BT34" s="2"/>
+      <c r="BU34" s="2"/>
+      <c r="BV34" s="2"/>
+      <c r="BW34" s="2"/>
+      <c r="BX34" s="2"/>
+      <c r="BY34" s="2"/>
+      <c r="BZ34" s="2"/>
+      <c r="CA34" s="2"/>
+      <c r="CB34" s="2"/>
+      <c r="CC34" s="2"/>
+      <c r="CD34" s="2"/>
+      <c r="CE34" s="2"/>
+      <c r="CF34" s="2"/>
+      <c r="CG34" s="2"/>
+      <c r="CH34" s="2"/>
+      <c r="CI34" s="2"/>
+      <c r="CJ34" s="2"/>
+      <c r="CK34" s="2"/>
+      <c r="CL34" s="2"/>
+      <c r="CM34" s="2"/>
+      <c r="CN34" s="2"/>
+      <c r="CO34" s="2"/>
+      <c r="CP34" s="2"/>
+      <c r="CQ34" s="2"/>
+      <c r="CR34" s="2"/>
+      <c r="CS34" s="2"/>
+      <c r="CT34" s="2"/>
+      <c r="CU34" s="2"/>
+      <c r="CV34" s="2"/>
+      <c r="CW34" s="2"/>
+      <c r="CX34" s="2"/>
+      <c r="CY34" s="2"/>
+      <c r="CZ34" s="2"/>
+      <c r="DA34" s="2"/>
+      <c r="DB34" s="2"/>
+      <c r="DC34" s="2"/>
+      <c r="DD34" s="2"/>
+      <c r="DE34" s="2"/>
+      <c r="DF34" s="2"/>
+      <c r="DG34" s="2"/>
+      <c r="DH34" s="2"/>
+      <c r="DI34" s="2"/>
+      <c r="DJ34" s="2"/>
+      <c r="DK34" s="2"/>
+      <c r="DL34" s="2"/>
+      <c r="DM34" s="2"/>
+      <c r="DN34" s="2"/>
+      <c r="DO34" s="2"/>
+      <c r="DP34" s="2"/>
+      <c r="DQ34" s="2"/>
+      <c r="DR34" s="2"/>
+      <c r="DS34" s="2"/>
+      <c r="DT34" s="2"/>
+      <c r="DU34" s="2"/>
+      <c r="DV34" s="2"/>
+      <c r="DW34" s="2"/>
+      <c r="DX34" s="2"/>
+      <c r="DY34" s="2"/>
+      <c r="DZ34" s="2"/>
+      <c r="EA34" s="2"/>
+      <c r="EB34" s="2"/>
+      <c r="EC34" s="2"/>
+      <c r="ED34" s="2"/>
+      <c r="EE34" s="2"/>
+      <c r="EF34" s="2"/>
+      <c r="EG34" s="2"/>
+      <c r="EH34" s="2"/>
+      <c r="EI34" s="2"/>
+      <c r="EJ34" s="2"/>
+      <c r="EK34" s="2"/>
+      <c r="EL34" s="2"/>
+      <c r="EM34" s="2"/>
+      <c r="EN34" s="2"/>
+      <c r="EO34" s="2"/>
+      <c r="EP34" s="2"/>
+      <c r="EQ34" s="2"/>
+      <c r="ER34" s="2"/>
+      <c r="ES34" s="2"/>
+      <c r="ET34" s="2"/>
+      <c r="EU34" s="2"/>
+      <c r="EV34" s="2"/>
+      <c r="EW34" s="2"/>
+      <c r="EX34" s="2"/>
+      <c r="EY34" s="2"/>
     </row>
     <row r="35" spans="1:155" ht="18" customHeight="1">
-      <c r="A35" s="19"/>
-      <c r="B35" s="51" t="s">
+      <c r="A35" s="42"/>
+      <c r="B35" s="66" t="s">
         <v>270</v>
       </c>
-      <c r="C35" s="8"/>
-      <c r="D35" s="8"/>
-      <c r="E35" s="8"/>
-      <c r="F35" s="8"/>
-      <c r="G35" s="8"/>
-      <c r="H35" s="8"/>
-      <c r="I35" s="8"/>
-      <c r="J35" s="8"/>
-      <c r="K35" s="8"/>
-      <c r="L35" s="8"/>
-      <c r="M35" s="8"/>
-      <c r="N35" s="8"/>
-      <c r="O35" s="8"/>
-      <c r="P35" s="8"/>
-      <c r="Q35" s="8"/>
-      <c r="R35" s="8"/>
-      <c r="S35" s="8"/>
-      <c r="T35" s="8"/>
-      <c r="U35" s="8"/>
-      <c r="V35" s="8" t="s">
-        <v>238</v>
-      </c>
-      <c r="W35" s="8"/>
-      <c r="X35" s="8" t="s">
-        <v>238</v>
-      </c>
-      <c r="Y35" s="8" t="s">
-        <v>238</v>
-      </c>
-      <c r="Z35" s="8"/>
-      <c r="AA35" s="8"/>
-      <c r="AB35" s="8"/>
-      <c r="AC35" s="7"/>
-      <c r="AD35" s="20"/>
-      <c r="AE35" s="20"/>
-      <c r="AF35" s="20"/>
+      <c r="C35" s="43"/>
+      <c r="D35" s="43"/>
+      <c r="E35" s="43"/>
+      <c r="F35" s="43"/>
+      <c r="G35" s="43"/>
+      <c r="H35" s="43"/>
+      <c r="I35" s="43"/>
+      <c r="J35" s="43"/>
+      <c r="K35" s="43"/>
+      <c r="L35" s="43"/>
+      <c r="M35" s="43"/>
+      <c r="N35" s="43"/>
+      <c r="O35" s="43"/>
+      <c r="P35" s="43"/>
+      <c r="Q35" s="43"/>
+      <c r="R35" s="43"/>
+      <c r="S35" s="43"/>
+      <c r="T35" s="43"/>
+      <c r="U35" s="43"/>
+      <c r="V35" s="43"/>
+      <c r="W35" s="43"/>
+      <c r="X35" s="44" t="s">
+        <v>271</v>
+      </c>
+      <c r="Y35" s="44" t="s">
+        <v>272</v>
+      </c>
+      <c r="Z35" s="43"/>
+      <c r="AA35" s="43"/>
+      <c r="AB35" s="43"/>
+      <c r="AC35" s="45"/>
+      <c r="AD35" s="46"/>
+      <c r="AE35" s="46"/>
+      <c r="AF35" s="47"/>
     </row>
-    <row r="36" spans="1:155" ht="18" customHeight="1" thickBot="1">
-      <c r="A36" s="15"/>
-      <c r="B36" s="67" t="s">
-        <v>271</v>
-      </c>
-      <c r="C36" s="6"/>
-      <c r="D36" s="6"/>
-      <c r="E36" s="6"/>
-      <c r="F36" s="6"/>
-      <c r="G36" s="6"/>
-      <c r="H36" s="6"/>
-      <c r="I36" s="6"/>
-      <c r="J36" s="6"/>
-      <c r="K36" s="6"/>
-      <c r="L36" s="6"/>
-      <c r="M36" s="6"/>
-      <c r="N36" s="6"/>
-      <c r="O36" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="P36" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="Q36" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="R36" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="S36" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="T36" s="6"/>
-      <c r="U36" s="6"/>
-      <c r="V36" s="6"/>
-      <c r="W36" s="6"/>
-      <c r="X36" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="Y36" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="Z36" s="6"/>
-      <c r="AA36" s="6"/>
-      <c r="AB36" s="6"/>
-      <c r="AC36" s="48"/>
-      <c r="AD36" s="16"/>
-      <c r="AE36" s="16"/>
-      <c r="AF36" s="16"/>
+    <row r="36" spans="1:155" ht="18" customHeight="1">
+      <c r="A36" s="19"/>
+      <c r="B36" s="51" t="s">
+        <v>273</v>
+      </c>
+      <c r="C36" s="8"/>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="8"/>
+      <c r="G36" s="8"/>
+      <c r="H36" s="8"/>
+      <c r="I36" s="8"/>
+      <c r="J36" s="8"/>
+      <c r="K36" s="8"/>
+      <c r="L36" s="8"/>
+      <c r="M36" s="8"/>
+      <c r="N36" s="8"/>
+      <c r="O36" s="8"/>
+      <c r="P36" s="8"/>
+      <c r="Q36" s="8"/>
+      <c r="R36" s="8"/>
+      <c r="S36" s="8"/>
+      <c r="T36" s="8"/>
+      <c r="U36" s="8"/>
+      <c r="V36" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="W36" s="8"/>
+      <c r="X36" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="Y36" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="Z36" s="8"/>
+      <c r="AA36" s="8"/>
+      <c r="AB36" s="8"/>
+      <c r="AC36" s="7"/>
+      <c r="AD36" s="20"/>
+      <c r="AE36" s="20"/>
+      <c r="AF36" s="20"/>
     </row>
-    <row r="37" spans="1:155" ht="18" customHeight="1" thickBot="1">
-      <c r="A37" s="42"/>
-      <c r="B37" s="66" t="s">
-        <v>272</v>
-      </c>
-      <c r="C37" s="43"/>
-      <c r="D37" s="43"/>
-      <c r="E37" s="43"/>
-      <c r="F37" s="43"/>
-      <c r="G37" s="43"/>
-      <c r="H37" s="43"/>
-      <c r="I37" s="43"/>
-      <c r="J37" s="43"/>
-      <c r="K37" s="43"/>
-      <c r="L37" s="43"/>
-      <c r="M37" s="43"/>
-      <c r="N37" s="43"/>
-      <c r="O37" s="43"/>
-      <c r="P37" s="43"/>
-      <c r="Q37" s="43"/>
-      <c r="R37" s="43"/>
-      <c r="S37" s="43"/>
-      <c r="T37" s="43"/>
-      <c r="U37" s="43"/>
-      <c r="V37" s="43"/>
-      <c r="W37" s="43"/>
-      <c r="X37" s="49" t="s">
-        <v>273</v>
-      </c>
-      <c r="Y37" s="43"/>
-      <c r="Z37" s="43"/>
-      <c r="AA37" s="43"/>
-      <c r="AB37" s="43"/>
-      <c r="AC37" s="43"/>
-      <c r="AD37" s="46"/>
-      <c r="AE37" s="44" t="s">
+    <row r="37" spans="1:155" ht="18" customHeight="1">
+      <c r="A37" s="15"/>
+      <c r="B37" s="67" t="s">
         <v>274</v>
       </c>
-      <c r="AF37" s="50" t="s">
-        <v>275</v>
-      </c>
+      <c r="C37" s="6"/>
+      <c r="D37" s="6"/>
+      <c r="E37" s="6"/>
+      <c r="F37" s="6"/>
+      <c r="G37" s="6"/>
+      <c r="H37" s="6"/>
+      <c r="I37" s="6"/>
+      <c r="J37" s="6"/>
+      <c r="K37" s="6"/>
+      <c r="L37" s="6"/>
+      <c r="M37" s="6"/>
+      <c r="N37" s="6"/>
+      <c r="O37" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="P37" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="Q37" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="R37" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="S37" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="T37" s="6"/>
+      <c r="U37" s="6"/>
+      <c r="V37" s="6"/>
+      <c r="W37" s="6"/>
+      <c r="X37" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="Y37" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="Z37" s="6"/>
+      <c r="AA37" s="6"/>
+      <c r="AB37" s="6"/>
+      <c r="AC37" s="48"/>
+      <c r="AD37" s="16"/>
+      <c r="AE37" s="16"/>
+      <c r="AF37" s="16"/>
     </row>
     <row r="38" spans="1:155" ht="18" customHeight="1">
-      <c r="A38" s="19"/>
-      <c r="B38" s="51" t="s">
+      <c r="A38" s="42"/>
+      <c r="B38" s="66" t="s">
+        <v>275</v>
+      </c>
+      <c r="C38" s="43"/>
+      <c r="D38" s="43"/>
+      <c r="E38" s="43"/>
+      <c r="F38" s="43"/>
+      <c r="G38" s="43"/>
+      <c r="H38" s="43"/>
+      <c r="I38" s="43"/>
+      <c r="J38" s="43"/>
+      <c r="K38" s="43"/>
+      <c r="L38" s="43"/>
+      <c r="M38" s="43"/>
+      <c r="N38" s="43"/>
+      <c r="O38" s="43"/>
+      <c r="P38" s="43"/>
+      <c r="Q38" s="43"/>
+      <c r="R38" s="43"/>
+      <c r="S38" s="43"/>
+      <c r="T38" s="43"/>
+      <c r="U38" s="43"/>
+      <c r="V38" s="43"/>
+      <c r="W38" s="43"/>
+      <c r="X38" s="49" t="s">
         <v>276</v>
       </c>
-      <c r="C38" s="8" t="s">
-        <v>238</v>
-      </c>
-      <c r="D38" s="8" t="s">
-        <v>238</v>
-      </c>
-      <c r="E38" s="8"/>
-      <c r="F38" s="8"/>
-      <c r="G38" s="8" t="s">
-        <v>238</v>
-      </c>
-      <c r="H38" s="8"/>
-      <c r="I38" s="8"/>
-      <c r="J38" s="8" t="s">
-        <v>238</v>
-      </c>
-      <c r="K38" s="8" t="s">
-        <v>238</v>
-      </c>
-      <c r="L38" s="8"/>
-      <c r="M38" s="8"/>
-      <c r="N38" s="8"/>
-      <c r="O38" s="8"/>
-      <c r="P38" s="8"/>
-      <c r="Q38" s="8"/>
-      <c r="R38" s="8"/>
-      <c r="S38" s="8"/>
-      <c r="T38" s="8"/>
-      <c r="U38" s="8"/>
-      <c r="V38" s="8"/>
-      <c r="W38" s="8"/>
-      <c r="X38" s="8"/>
-      <c r="Y38" s="8" t="s">
-        <v>238</v>
-      </c>
-      <c r="Z38" s="8"/>
-      <c r="AA38" s="8"/>
-      <c r="AB38" s="8"/>
-      <c r="AC38" s="8"/>
-      <c r="AD38" s="20"/>
-      <c r="AE38" s="20"/>
-      <c r="AF38" s="20"/>
+      <c r="Y38" s="43"/>
+      <c r="Z38" s="43"/>
+      <c r="AA38" s="43"/>
+      <c r="AB38" s="43"/>
+      <c r="AC38" s="43"/>
+      <c r="AD38" s="46"/>
+      <c r="AE38" s="44" t="s">
+        <v>277</v>
+      </c>
+      <c r="AF38" s="50" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="39" spans="1:155" ht="18" customHeight="1">
-      <c r="A39" s="9"/>
-      <c r="B39" s="12" t="s">
-        <v>277</v>
-      </c>
-      <c r="C39" s="4"/>
-      <c r="D39" s="4"/>
-      <c r="E39" s="4"/>
-      <c r="F39" s="4"/>
-      <c r="G39" s="4"/>
-      <c r="H39" s="4"/>
-      <c r="I39" s="4"/>
-      <c r="J39" s="4"/>
-      <c r="K39" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="L39" s="4"/>
-      <c r="M39" s="4"/>
-      <c r="N39" s="4"/>
-      <c r="O39" s="4"/>
-      <c r="P39" s="4"/>
-      <c r="Q39" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="R39" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="S39" s="4"/>
-      <c r="T39" s="4"/>
-      <c r="U39" s="4"/>
-      <c r="V39" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="W39" s="4"/>
-      <c r="X39" s="4"/>
-      <c r="Y39" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="Z39" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="AA39" s="4"/>
-      <c r="AB39" s="4"/>
-      <c r="AC39" s="4"/>
-      <c r="AD39" s="10"/>
-      <c r="AE39" s="10"/>
-      <c r="AF39" s="10"/>
+      <c r="A39" s="19"/>
+      <c r="B39" s="51" t="s">
+        <v>279</v>
+      </c>
+      <c r="C39" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="D39" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="E39" s="8"/>
+      <c r="F39" s="8"/>
+      <c r="G39" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="H39" s="8"/>
+      <c r="I39" s="8"/>
+      <c r="J39" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="K39" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="L39" s="8"/>
+      <c r="M39" s="8"/>
+      <c r="N39" s="8"/>
+      <c r="O39" s="8"/>
+      <c r="P39" s="8"/>
+      <c r="Q39" s="8"/>
+      <c r="R39" s="8"/>
+      <c r="S39" s="8"/>
+      <c r="T39" s="8"/>
+      <c r="U39" s="8"/>
+      <c r="V39" s="8"/>
+      <c r="W39" s="8"/>
+      <c r="X39" s="8"/>
+      <c r="Y39" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="Z39" s="8"/>
+      <c r="AA39" s="8"/>
+      <c r="AB39" s="8"/>
+      <c r="AC39" s="8"/>
+      <c r="AD39" s="20"/>
+      <c r="AE39" s="20"/>
+      <c r="AF39" s="20"/>
     </row>
     <row r="40" spans="1:155" ht="18" customHeight="1">
       <c r="A40" s="9"/>
       <c r="B40" s="12" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C40" s="4"/>
       <c r="D40" s="4"/>
@@ -5311,27 +5352,35 @@
       <c r="H40" s="4"/>
       <c r="I40" s="4"/>
       <c r="J40" s="4"/>
-      <c r="K40" s="4"/>
+      <c r="K40" s="4" t="s">
+        <v>241</v>
+      </c>
       <c r="L40" s="4"/>
       <c r="M40" s="4"/>
       <c r="N40" s="4"/>
       <c r="O40" s="4"/>
       <c r="P40" s="4"/>
-      <c r="Q40" s="4"/>
-      <c r="R40" s="4"/>
+      <c r="Q40" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="R40" s="4" t="s">
+        <v>241</v>
+      </c>
       <c r="S40" s="4"/>
       <c r="T40" s="4"/>
       <c r="U40" s="4"/>
-      <c r="V40" s="4"/>
+      <c r="V40" s="4" t="s">
+        <v>241</v>
+      </c>
       <c r="W40" s="4"/>
       <c r="X40" s="4"/>
       <c r="Y40" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="Z40" s="4"/>
-      <c r="AA40" s="4" t="s">
-        <v>238</v>
-      </c>
+        <v>241</v>
+      </c>
+      <c r="Z40" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="AA40" s="4"/>
       <c r="AB40" s="4"/>
       <c r="AC40" s="4"/>
       <c r="AD40" s="10"/>
@@ -5341,7 +5390,7 @@
     <row r="41" spans="1:155" ht="18" customHeight="1">
       <c r="A41" s="9"/>
       <c r="B41" s="12" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C41" s="4"/>
       <c r="D41" s="4"/>
@@ -5365,9 +5414,13 @@
       <c r="V41" s="4"/>
       <c r="W41" s="4"/>
       <c r="X41" s="4"/>
-      <c r="Y41" s="4"/>
+      <c r="Y41" s="4" t="s">
+        <v>241</v>
+      </c>
       <c r="Z41" s="4"/>
-      <c r="AA41" s="4"/>
+      <c r="AA41" s="4" t="s">
+        <v>241</v>
+      </c>
       <c r="AB41" s="4"/>
       <c r="AC41" s="4"/>
       <c r="AD41" s="10"/>
@@ -5377,15 +5430,13 @@
     <row r="42" spans="1:155" ht="18" customHeight="1">
       <c r="A42" s="9"/>
       <c r="B42" s="12" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C42" s="4"/>
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>
       <c r="F42" s="4"/>
-      <c r="G42" s="4" t="s">
-        <v>238</v>
-      </c>
+      <c r="G42" s="4"/>
       <c r="H42" s="4"/>
       <c r="I42" s="4"/>
       <c r="J42" s="4"/>
@@ -5415,13 +5466,15 @@
     <row r="43" spans="1:155" ht="18" customHeight="1">
       <c r="A43" s="9"/>
       <c r="B43" s="12" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="C43" s="4"/>
       <c r="D43" s="4"/>
       <c r="E43" s="4"/>
       <c r="F43" s="4"/>
-      <c r="G43" s="4"/>
+      <c r="G43" s="4" t="s">
+        <v>241</v>
+      </c>
       <c r="H43" s="4"/>
       <c r="I43" s="4"/>
       <c r="J43" s="4"/>
@@ -5438,21 +5491,20 @@
       <c r="U43" s="4"/>
       <c r="V43" s="4"/>
       <c r="W43" s="4"/>
-      <c r="X43" s="10"/>
-      <c r="Y43" s="10"/>
-      <c r="Z43" s="10"/>
-      <c r="AA43" s="10"/>
-      <c r="AB43" s="10" t="s">
-        <v>238</v>
-      </c>
-      <c r="AC43" s="10"/>
+      <c r="X43" s="4"/>
+      <c r="Y43" s="4"/>
+      <c r="Z43" s="4"/>
+      <c r="AA43" s="4"/>
+      <c r="AB43" s="4"/>
+      <c r="AC43" s="4"/>
       <c r="AD43" s="10"/>
       <c r="AE43" s="10"/>
+      <c r="AF43" s="10"/>
     </row>
     <row r="44" spans="1:155" ht="18" customHeight="1">
       <c r="A44" s="9"/>
       <c r="B44" s="12" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C44" s="4"/>
       <c r="D44" s="4"/>
@@ -5479,7 +5531,9 @@
       <c r="Y44" s="10"/>
       <c r="Z44" s="10"/>
       <c r="AA44" s="10"/>
-      <c r="AB44" s="10"/>
+      <c r="AB44" s="10" t="s">
+        <v>241</v>
+      </c>
       <c r="AC44" s="10"/>
       <c r="AD44" s="10"/>
       <c r="AE44" s="10"/>
@@ -5487,7 +5541,7 @@
     <row r="45" spans="1:155" ht="18" customHeight="1">
       <c r="A45" s="9"/>
       <c r="B45" s="12" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C45" s="4"/>
       <c r="D45" s="4"/>
@@ -5522,7 +5576,7 @@
     <row r="46" spans="1:155" ht="18" customHeight="1">
       <c r="A46" s="9"/>
       <c r="B46" s="12" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="C46" s="4"/>
       <c r="D46" s="4"/>
@@ -5557,7 +5611,7 @@
     <row r="47" spans="1:155" ht="18" customHeight="1">
       <c r="A47" s="9"/>
       <c r="B47" s="12" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C47" s="4"/>
       <c r="D47" s="4"/>
@@ -5589,10 +5643,40 @@
       <c r="AD47" s="10"/>
       <c r="AE47" s="10"/>
     </row>
-    <row r="48" spans="1:155">
-      <c r="X48" s="2"/>
-      <c r="Y48" s="2"/>
-      <c r="Z48" s="2"/>
+    <row r="48" spans="1:155" ht="18" customHeight="1">
+      <c r="A48" s="9"/>
+      <c r="B48" s="12" t="s">
+        <v>288</v>
+      </c>
+      <c r="C48" s="4"/>
+      <c r="D48" s="4"/>
+      <c r="E48" s="4"/>
+      <c r="F48" s="4"/>
+      <c r="G48" s="4"/>
+      <c r="H48" s="4"/>
+      <c r="I48" s="4"/>
+      <c r="J48" s="4"/>
+      <c r="K48" s="4"/>
+      <c r="L48" s="4"/>
+      <c r="M48" s="4"/>
+      <c r="N48" s="4"/>
+      <c r="O48" s="4"/>
+      <c r="P48" s="4"/>
+      <c r="Q48" s="4"/>
+      <c r="R48" s="4"/>
+      <c r="S48" s="4"/>
+      <c r="T48" s="4"/>
+      <c r="U48" s="4"/>
+      <c r="V48" s="4"/>
+      <c r="W48" s="4"/>
+      <c r="X48" s="10"/>
+      <c r="Y48" s="10"/>
+      <c r="Z48" s="10"/>
+      <c r="AA48" s="10"/>
+      <c r="AB48" s="10"/>
+      <c r="AC48" s="10"/>
+      <c r="AD48" s="10"/>
+      <c r="AE48" s="10"/>
     </row>
     <row r="49" spans="24:26">
       <c r="X49" s="2"/>
@@ -5654,8 +5738,13 @@
       <c r="Y60" s="2"/>
       <c r="Z60" s="2"/>
     </row>
+    <row r="61" spans="24:26">
+      <c r="X61" s="2"/>
+      <c r="Y61" s="2"/>
+      <c r="Z61" s="2"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:AF33" xr:uid="{D8B0CA4D-B55F-4AFA-903E-3D529FFFD0A1}">
+  <autoFilter ref="A2:AF34" xr:uid="{D8B0CA4D-B55F-4AFA-903E-3D529FFFD0A1}">
     <filterColumn colId="2" showButton="0"/>
     <filterColumn colId="3" showButton="0"/>
     <filterColumn colId="4" showButton="0"/>
@@ -5675,15 +5764,15 @@
     <filterColumn colId="20" showButton="0"/>
   </autoFilter>
   <mergeCells count="22">
-    <mergeCell ref="B20:B27"/>
-    <mergeCell ref="B12:B18"/>
-    <mergeCell ref="B7:B11"/>
-    <mergeCell ref="B28:B33"/>
+    <mergeCell ref="B21:B28"/>
+    <mergeCell ref="B13:B19"/>
+    <mergeCell ref="B8:B12"/>
+    <mergeCell ref="B29:B34"/>
     <mergeCell ref="AD2:AD4"/>
     <mergeCell ref="Z2:Z4"/>
     <mergeCell ref="AE2:AE4"/>
     <mergeCell ref="AF2:AF4"/>
-    <mergeCell ref="A7:A18"/>
+    <mergeCell ref="A8:A19"/>
     <mergeCell ref="AB2:AB4"/>
     <mergeCell ref="AC2:AC4"/>
     <mergeCell ref="C3:E3"/>
@@ -5699,130 +5788,130 @@
     <mergeCell ref="Y2:Y4"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="C21" r:id="rId1" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/sp?tab=models" xr:uid="{FE987DC0-578A-4A81-AB17-6E49D6983782}"/>
-    <hyperlink ref="C22" r:id="rId2" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/spe?tab=models" xr:uid="{E414E66B-6D50-4BC0-93B6-EEDD71D1D349}"/>
-    <hyperlink ref="C23" r:id="rId3" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/sp-ne?tab=models" xr:uid="{79A82224-5E75-416A-BD5C-1C442DB4F9E7}"/>
-    <hyperlink ref="D21" r:id="rId4" display="https://product-selection.grundfos.com/fr/products/bm?tab=products" xr:uid="{39935FC4-BF60-4ADA-99B8-6280D11B4087}"/>
-    <hyperlink ref="D22" r:id="rId5" display="https://product-selection.grundfos.com/fr/products/bms?tab=products" xr:uid="{201298BF-F5B7-4DD8-896A-A6CFDF20A155}"/>
-    <hyperlink ref="D23" r:id="rId6" display="https://product-selection.grundfos.com/fr/products/bm-hp?tab=products" xr:uid="{0AA34BB7-1783-4351-AB39-2E3E2C9E6D24}"/>
-    <hyperlink ref="E21" r:id="rId7" display="https://product-selection.grundfos.com/fr/products/kpl?tab=models" xr:uid="{02FD05D5-211D-4185-A911-F718E163AF22}"/>
-    <hyperlink ref="E22" r:id="rId8" display="https://product-selection.grundfos.com/fr/products/kwm?tab=documentation" xr:uid="{F11B5E61-F53C-4DA1-93C5-A57D0408930C}"/>
-    <hyperlink ref="F21" r:id="rId9" display="https://product-selection.grundfos.com/fr/products/ls?tab=products" xr:uid="{070C34E9-9C05-4522-9AD2-8E6D82261A9B}"/>
-    <hyperlink ref="J21" r:id="rId10" display="https://product-selection.grundfos.com/fr/products/cm-cme?tab=products" xr:uid="{E79A5B97-E6E0-4649-B070-9A1CF47F88B2}"/>
-    <hyperlink ref="I21" r:id="rId11" display="https://product-selection.grundfos.com/fr/products/cm-cme/cm-self-priming?tab=models" xr:uid="{CFEF6DD3-2F90-4195-BA05-DEE28F55BD3E}"/>
-    <hyperlink ref="J22" r:id="rId12" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nb?tab=documentation" xr:uid="{ABC208A8-FE5B-4CC4-B585-6A3873FA7294}"/>
-    <hyperlink ref="J23" r:id="rId13" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nbe?tab=models" xr:uid="{1D4EF590-19C1-44EB-8B92-46AD5F28F62F}"/>
-    <hyperlink ref="J24" r:id="rId14" display="https://product-selection.grundfos.com/fr/products/nk-nke-nke-series-2000-nk-bare-shaft?tab=products" xr:uid="{76D3161D-F2DD-4CCA-AC1D-AD2E393D8694}"/>
-    <hyperlink ref="J25" r:id="rId15" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft?tab=products" xr:uid="{9CA4757F-439C-4161-8B60-7C14A9EDCA69}"/>
-    <hyperlink ref="J26" r:id="rId16" display="https://product-selection.grundfos.com/fr/products/tp-tpe?tab=products" xr:uid="{0C9A1473-1926-417A-947F-8561754B7D76}"/>
-    <hyperlink ref="N23" r:id="rId17" display="https://product-selection.grundfos.com/fr/products/tp-tpe?tab=products" xr:uid="{7D2D046F-1C95-42DD-8F35-90280675B9EA}"/>
-    <hyperlink ref="N21" r:id="rId18" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nbe?tab=models" xr:uid="{303D01A6-AC7B-42EE-AE09-2A10FBED3940}"/>
-    <hyperlink ref="N22" r:id="rId19" display="https://product-selection.grundfos.com/fr/products/nk-nke-nke-series-2000-nk-bare-shaft?tab=products" xr:uid="{A1442A3E-E286-4D87-BF5A-B52C00F11931}"/>
-    <hyperlink ref="N24" r:id="rId20" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft?tab=products" xr:uid="{91C811C0-E7C2-45CC-8C4A-41851188982F}"/>
-    <hyperlink ref="K21" r:id="rId21" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte?tab=products" xr:uid="{168A97AE-925F-4CB8-99FA-4D28B053F7CB}"/>
-    <hyperlink ref="L22" r:id="rId22" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte/cre?tab=models" xr:uid="{43E68B92-4EB3-4ECE-A299-C7DDCAFB1889}"/>
-    <hyperlink ref="L23" r:id="rId23" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte/crne?tab=models" xr:uid="{9DD9406E-F477-49F6-BA29-841ED00CE74B}"/>
-    <hyperlink ref="M21" r:id="rId24" display="https://product-selection.grundfos.com/fr/products/cm-cme/cme?tab=models" xr:uid="{CB210458-379C-4663-B0FD-73E843090C67}"/>
-    <hyperlink ref="M22" r:id="rId25" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nbe?tab=models" xr:uid="{3776F606-4CBE-49B1-912C-5B2BC9586206}"/>
-    <hyperlink ref="M23" r:id="rId26" display="https://product-selection.grundfos.com/fr/products/nk-nke-nke-series-2000-nk-bare-shaft?tab=products" xr:uid="{8731A9E7-9B51-450F-BCB5-013214A2B33F}"/>
-    <hyperlink ref="M24" r:id="rId27" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft?tab=products" xr:uid="{EDB8C821-F675-4CE1-B7B0-0FAF39DCEFD4}"/>
-    <hyperlink ref="L25" r:id="rId28" display="https://product-selection.grundfos.com/fr/products/hydro-multi-e?tab=models" xr:uid="{5995DFA3-65AE-4378-BD2E-CDA4F6FA5ED7}"/>
-    <hyperlink ref="L26" r:id="rId29" display="https://product-selection.grundfos.com/fr/products/hydro-mpc?tab=products" xr:uid="{2E37CE89-9B22-43AA-B967-C6F20A25613F}"/>
-    <hyperlink ref="L24" r:id="rId30" display="https://product-selection.grundfos.com/fr/products/hydro-solo-e?tab=models" xr:uid="{5A1F2584-1AA0-4C8B-A55D-39C825C8A3F8}"/>
-    <hyperlink ref="O21" r:id="rId31" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/sl1?tab=models" xr:uid="{9C7E88DB-59BA-4B5C-8769-45D64CC97D40}"/>
-    <hyperlink ref="O22" r:id="rId32" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/slv?tab=models" xr:uid="{00039B9D-B404-44A8-B557-BBF172D7CD31}"/>
-    <hyperlink ref="O23" r:id="rId33" display="https://product-selection.grundfos.com/fr/products/sesl-9-30-kw?tab=models" xr:uid="{C90FBAD5-7C9C-4429-9BAC-9BE027B562FD}"/>
-    <hyperlink ref="O25" r:id="rId34" display="https://product-selection.grundfos.com/fr/products/s?tab=products" xr:uid="{6F267867-1729-460E-9939-DEBA10D95429}"/>
-    <hyperlink ref="O24" r:id="rId35" display="https://product-selection.grundfos.com/fr/products/sesl-frame-size-56?tab=models" xr:uid="{541D6F69-2D4F-412B-91C7-A0B79C20C0CA}"/>
-    <hyperlink ref="P22" r:id="rId36" display="https://product-selection.grundfos.com/fr/products/unilift-ap/unilift-apg?tab=models" xr:uid="{CF6542DD-C411-4584-A2A2-ADD9BD336104}"/>
-    <hyperlink ref="P21" r:id="rId37" display="https://product-selection.grundfos.com/fr/products/seg?tab=models" xr:uid="{AF847B64-9B08-45DD-8487-57C6900B0D5F}"/>
-    <hyperlink ref="Q21" r:id="rId38" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/se1?tab=models" xr:uid="{D2271F27-967E-46DC-8195-E2EAFD3339EB}"/>
-    <hyperlink ref="Q22" r:id="rId39" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/sev?tab=models" xr:uid="{6D042873-5F32-4A50-8803-93F40528C6A1}"/>
-    <hyperlink ref="Q23" r:id="rId40" display="https://product-selection.grundfos.com/fr/products/sesl-9-30-kw?tab=models" xr:uid="{A344F5B5-8A97-456F-87D5-4C6EFCA52D3A}"/>
-    <hyperlink ref="Q24" r:id="rId41" display="https://product-selection.grundfos.com/fr/products/sesl-frame-size-56?tab=models" xr:uid="{BB0B40A3-A20A-44BC-9FC9-E9EE00FC9F45}"/>
-    <hyperlink ref="Q25" r:id="rId42" display="https://product-selection.grundfos.com/fr/products/s?tab=products" xr:uid="{2E26D22E-3FD7-4718-9B39-661D30AF938C}"/>
-    <hyperlink ref="Q26" r:id="rId43" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft/nkg-supervortex-impeller?tab=explore" xr:uid="{FA539854-B47D-4B47-9F9A-7CE595B28025}"/>
-    <hyperlink ref="S21" r:id="rId44" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/se1?tab=models" xr:uid="{66C50FE8-D6EA-4602-866A-7B3258A9261C}"/>
-    <hyperlink ref="S22" r:id="rId45" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/sev?tab=models" xr:uid="{DEFE3A48-5152-4917-935D-8BAB7D40CDD7}"/>
-    <hyperlink ref="S23" r:id="rId46" display="https://product-selection.grundfos.com/fr/products/sesl-9-30-kw?tab=models" xr:uid="{62BA715F-3850-4F49-A593-7645C6C0C3CC}"/>
-    <hyperlink ref="S24" r:id="rId47" display="https://product-selection.grundfos.com/fr/products/sesl-frame-size-56?tab=models" xr:uid="{F0AA29DC-4DA5-4CA6-94B3-C22351F6904E}"/>
-    <hyperlink ref="S25" r:id="rId48" display="https://product-selection.grundfos.com/fr/products/s?tab=products" xr:uid="{96671AB9-9AEA-4A5F-B84F-E78888F9B311}"/>
-    <hyperlink ref="S26" r:id="rId49" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft/nkg-supervortex-impeller?tab=explore" xr:uid="{8A1CF826-08F5-4AF2-B984-9AA020480952}"/>
-    <hyperlink ref="O26" r:id="rId50" display="https://product-selection.grundfos.com/fr/products/unilift-ap/unilift-ap50b?tab=models" xr:uid="{14E21A07-FF5F-4129-AE6E-260A1AA5098C}"/>
-    <hyperlink ref="W21" r:id="rId51" display="https://product-selection.grundfos.com/fr/products/unilift-ap?tab=products" xr:uid="{FF1F3D5A-16C1-4C5A-8F69-37BEB2C51657}"/>
-    <hyperlink ref="W22" r:id="rId52" display="https://product-selection.grundfos.com/fr/products/unilift-kp?tab=models" xr:uid="{D8B15CDE-A46F-4955-8CE5-B1F2491BDDEE}"/>
-    <hyperlink ref="W23" r:id="rId53" display="https://product-selection.grundfos.com/fr/products/unilift-cc?tab=models" xr:uid="{5DA16314-BD6C-4DB3-8EC0-A99C56D3006D}"/>
-    <hyperlink ref="W24" r:id="rId54" display="https://product-selection.grundfos.com/fr/products/dp?tab=models" xr:uid="{4D82ED98-3DD6-4697-9C9C-A060C7E06489}"/>
-    <hyperlink ref="W25" r:id="rId55" display="https://product-selection.grundfos.com/fr/products/ef?tab=models" xr:uid="{ABDE8970-72CB-4EB8-979F-99183A9FD9D3}"/>
-    <hyperlink ref="Y21" r:id="rId56" display="https://product-selection.grundfos.com/fr/products/mt-tank-mounted-pumps/mtr?tab=models" xr:uid="{D5799B15-EF87-41DF-88D8-05F25935D793}"/>
-    <hyperlink ref="Y22" r:id="rId57" display="https://product-selection.grundfos.com/fr/products/mt-tank-mounted-pumps/mtre?tab=models" xr:uid="{7E2DAAB5-3884-49DD-BF25-FA92C2CE9951}"/>
-    <hyperlink ref="Y23" r:id="rId58" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nb?tab=documentation" xr:uid="{92C19ACB-7462-4938-A66E-478979299908}"/>
-    <hyperlink ref="Y24" r:id="rId59" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nbe?tab=models" xr:uid="{D2CCE95F-A5DF-4715-B3CA-DB297F6DF5C8}"/>
-    <hyperlink ref="Y25" r:id="rId60" display="https://product-selection.grundfos.com/fr/products/nk-nke-nke-series-2000-nk-bare-shaft?tab=products" xr:uid="{EA080A36-FCEB-4D04-B389-F8ABE5514300}"/>
-    <hyperlink ref="Y26" r:id="rId61" display="https://product-selection.grundfos.com/fr/products/tp-tpe?tab=products" xr:uid="{2A2A6B6D-2CAA-4110-9FED-BCA8DC5F1709}"/>
-    <hyperlink ref="Y27" r:id="rId62" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte?tab=products" xr:uid="{D902984C-2BC5-48A4-BF49-DCE4C7E629F6}"/>
-    <hyperlink ref="Z21" r:id="rId63" display="https://product-selection.grundfos.com/fr/products/hydro-en?tab=models" xr:uid="{69CECDCF-71ED-40D6-A274-30663F73D3A6}"/>
-    <hyperlink ref="AD21" r:id="rId64" display="https://product-selection.grundfos.com/fr/products/poweradapt?tab=models" xr:uid="{CBB79406-3EE4-4CC7-BCD3-398882D58A96}"/>
-    <hyperlink ref="AD22" r:id="rId65" display="https://product-selection.grundfos.com/fr/products/rsi?tab=models" xr:uid="{2ECDD4BA-B757-4A11-9F78-EB235920F462}"/>
-    <hyperlink ref="AD23" r:id="rId66" display="https://product-selection.grundfos.com/fr/products/crflex?tab=models" xr:uid="{F1835770-C21F-4E8A-9EBF-7C701B0E9CF4}"/>
-    <hyperlink ref="AD24" r:id="rId67" display="https://product-selection.grundfos.com/fr/products/sqflex?tab=models" xr:uid="{2932EAA4-553E-42B6-AD4B-37D91C9B845C}"/>
-    <hyperlink ref="AD25" r:id="rId68" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/sp?tab=models" xr:uid="{25A70C6E-05E1-4E40-956B-50B78B088135}"/>
-    <hyperlink ref="AD26" r:id="rId69" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/spe?tab=models" xr:uid="{7C346AF6-2EEB-4DFC-A819-DAE2C3B09113}"/>
-    <hyperlink ref="AD27" r:id="rId70" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte?tab=products" xr:uid="{9F4AE584-6CDD-45BE-ABC9-5087AAD766B9}"/>
-    <hyperlink ref="AE21" r:id="rId71" display="https://product-selection.grundfos.com/fr/products/dosing-pumps-digital/dda?tab=models" xr:uid="{68600FE5-FDB0-4237-8B8A-45786462FE8A}"/>
-    <hyperlink ref="AE22" r:id="rId72" display="https://product-selection.grundfos.com/fr/products/dosing-pumps-digital/dme?tab=models" xr:uid="{41502941-2297-46B7-A840-2EF7A24064D7}"/>
-    <hyperlink ref="AE23" r:id="rId73" display="https://product-selection.grundfos.com/fr/products/dosing-pumps-mechanical/dmx?tab=models" xr:uid="{A892A826-C3E1-4B26-9529-8174E76C068D}"/>
-    <hyperlink ref="AE24" r:id="rId74" display="https://product-selection.grundfos.com/fr/products/dosing-pumps-mechanical/dmh?tab=models" xr:uid="{60926621-C7DA-4892-9ACA-4145E303C37B}"/>
-    <hyperlink ref="AE25" r:id="rId75" xr:uid="{EB339B7E-AAB0-4720-A5DC-B7E47BEFE888}"/>
-    <hyperlink ref="AF23" r:id="rId76" display="https://product-selection.grundfos.com/fr/products/disinfection-systems/oxiperm?tab=models" xr:uid="{D1CFBDC1-076A-4661-B343-B5087946D2BF}"/>
-    <hyperlink ref="AF21" r:id="rId77" display="https://product-selection.grundfos.com/fr/products/disinfection-systems/vaccuperm?tab=models" xr:uid="{0E5CA30E-D80E-4BC1-BE8D-5757C0E703F9}"/>
-    <hyperlink ref="AF22" r:id="rId78" display="https://product-selection.grundfos.com/fr/products/disinfection-systems/selcoperm?tab=models" xr:uid="{3FE337C4-03C2-4326-92F3-2ADF14429172}"/>
-    <hyperlink ref="C29" r:id="rId79" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-4" xr:uid="{7CECB146-2C6E-4D8C-8362-B574F0A0B1CD}"/>
-    <hyperlink ref="C30" r:id="rId80" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-6" xr:uid="{77066640-D437-4393-AE04-9291CA2EA2E2}"/>
-    <hyperlink ref="C31" r:id="rId81" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-8" xr:uid="{440D559C-9B55-46F7-B47D-809066594D8E}"/>
-    <hyperlink ref="C32" r:id="rId82" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-actun-zetos" xr:uid="{6B88B868-32F8-4635-8067-C4F8AA30A87A}"/>
-    <hyperlink ref="C33" r:id="rId83" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-14-24" xr:uid="{6AAEB27D-0CD4-409C-9175-B5DC81BA5B91}"/>
-    <hyperlink ref="D29" r:id="rId84" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-4" xr:uid="{70B5668C-6DE4-4721-BD0D-15695ACCFD10}"/>
-    <hyperlink ref="D30" r:id="rId85" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-6" xr:uid="{AB0F5528-0721-49E7-9EB4-443A836A5BE6}"/>
-    <hyperlink ref="D31" r:id="rId86" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-8" xr:uid="{CE5D4CF5-B9AD-4786-AF2A-5CBA0FB4461E}"/>
-    <hyperlink ref="D32" r:id="rId87" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-actun-zetos" xr:uid="{F3302311-60D3-4257-BE0E-8ADCE8FD3F26}"/>
-    <hyperlink ref="D33" r:id="rId88" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-14-24" xr:uid="{C714C692-05B2-43B9-83CE-06CDCF547DAA}"/>
-    <hyperlink ref="F29" r:id="rId89" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-scp" xr:uid="{7BEBF8BE-E457-43DD-A078-9A05C9712ED1}"/>
-    <hyperlink ref="F30" r:id="rId90" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-atmos-tera-sch" xr:uid="{8AC9B5FF-3554-4A3F-9A49-254FDDC1D679}"/>
-    <hyperlink ref="G29" r:id="rId91" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-4" xr:uid="{A6F45EEC-DFC1-4F41-A737-7D50D323F858}"/>
-    <hyperlink ref="G30" r:id="rId92" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-6" xr:uid="{E8092E13-22EC-4AA4-A0E2-CB8C894814DA}"/>
-    <hyperlink ref="G31" r:id="rId93" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-8" xr:uid="{06C47C82-BB6B-4167-9AFC-F87F629A6D2D}"/>
-    <hyperlink ref="G32" r:id="rId94" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-actun-zetos" xr:uid="{7F484481-A382-4AA7-BC6F-9F9E8E881F13}"/>
-    <hyperlink ref="G33" r:id="rId95" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-14-24" xr:uid="{145E082E-ACF5-4C03-95AA-D5FF287B68E9}"/>
-    <hyperlink ref="J29" r:id="rId96" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-medana-ch1-l" xr:uid="{CB6CAFF8-329E-47DC-8F46-39C8BB5E04DD}"/>
-    <hyperlink ref="J30" r:id="rId97" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-zeox-first-h" xr:uid="{2D403080-ECF0-434D-8570-2DCE4384BDB3}"/>
-    <hyperlink ref="K29" r:id="rId98" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-helix-v" xr:uid="{24EB14FB-8853-4DD9-BFF7-D08622F6269E}"/>
-    <hyperlink ref="K30" r:id="rId99" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-helix-first-v" xr:uid="{292648A6-CEF7-4F6A-B9E8-2C2D1935D493}"/>
-    <hyperlink ref="L29" r:id="rId100" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-helix-ve" xr:uid="{CB04A41A-2CE9-45EC-90FB-F63D1D7003E0}"/>
-    <hyperlink ref="L30" r:id="rId101" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-helix2-0-ve" xr:uid="{0D95BEE0-BF20-4117-86C3-9423999074AC}"/>
-    <hyperlink ref="M29" r:id="rId102" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-medana-ch3-le" xr:uid="{E61CDC21-E587-41FD-8720-AA95E8F2BCB8}"/>
-    <hyperlink ref="N29" r:id="rId103" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-isar-modh1-e-2-3" xr:uid="{2D23D0CC-B7DF-4FF1-ABE9-A9C38B0D675F}"/>
-    <hyperlink ref="N30" r:id="rId104" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-siboost2-0-smart-helix-ve" xr:uid="{FFEEE275-2C73-4EC4-B193-CB85762B0142}"/>
-    <hyperlink ref="O29" r:id="rId105" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-pro" xr:uid="{40187CA6-E027-4F57-B695-B124E41E9781}"/>
-    <hyperlink ref="O30" r:id="rId106" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-supra" xr:uid="{6510CD0A-CFE7-486C-91AF-7C7A655B4AFB}"/>
-    <hyperlink ref="O31" r:id="rId107" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-solid" xr:uid="{BDC567B5-AC65-4996-9A0B-1AF09DF2041A}"/>
-    <hyperlink ref="Q29" r:id="rId108" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-bloc" xr:uid="{3980AF89-63D6-4F8A-AA62-E67520B41458}"/>
-    <hyperlink ref="Q30" r:id="rId109" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-norm" xr:uid="{713EE9E0-CE07-4B5A-8098-8828FD7A2BE1}"/>
-    <hyperlink ref="P29" r:id="rId110" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-pro-s" xr:uid="{7EA67BA6-0CB9-4BC2-8D2F-2187D3E3EC87}"/>
-    <hyperlink ref="O32" r:id="rId111" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-fa-configure" xr:uid="{F271E929-C189-489C-95BA-44C8F95B9706}"/>
-    <hyperlink ref="S29" r:id="rId112" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-pro" xr:uid="{4E520461-D8CA-4714-95A3-4A07D979003B}"/>
-    <hyperlink ref="S30" r:id="rId113" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-supra" xr:uid="{7E747CBF-258D-4F97-AE71-AF52B950EDDE}"/>
-    <hyperlink ref="S31" r:id="rId114" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-solid" xr:uid="{90F21445-AD91-480E-9E60-99DEEB471A24}"/>
-    <hyperlink ref="S32" r:id="rId115" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-fa-configure" xr:uid="{CAC9CBDD-5033-4067-92F5-E1A89E7A10BF}"/>
-    <hyperlink ref="U29" r:id="rId116" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-pro" xr:uid="{DED143CB-BC81-4CC1-99AF-6D9EFDCA04A2}"/>
-    <hyperlink ref="U30" r:id="rId117" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-supra" xr:uid="{AD0F4A4E-82E3-443D-B5CE-BB1383456F96}"/>
-    <hyperlink ref="U31" r:id="rId118" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-solid" xr:uid="{F30C0BD2-ACC1-498E-B06C-26D556B514B6}"/>
-    <hyperlink ref="U32" r:id="rId119" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-fa-configure" xr:uid="{FC92FF04-817E-49C9-B9E1-3FED19E3DBAA}"/>
-    <hyperlink ref="W29" r:id="rId120" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-drain-tm-tmw-tmr-32" xr:uid="{0F177732-3552-46D9-B2A1-0858315CC611}"/>
-    <hyperlink ref="W30" r:id="rId121" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-padus-uni" xr:uid="{31C21B43-5DBE-431A-A886-4FBC3A6BE491}"/>
-    <hyperlink ref="W31" r:id="rId122" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-padus-mini3" xr:uid="{D91894CF-CB16-4C43-980E-41E743666848}"/>
-    <hyperlink ref="W32" r:id="rId123" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-padus-pro" xr:uid="{79DE7E3B-A7A2-4098-B5DF-694F7F93640D}"/>
-    <hyperlink ref="Z29" r:id="rId124" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-cof-helix" xr:uid="{2E5216D3-37DA-48CB-ABA0-7C21064BB2D3}"/>
+    <hyperlink ref="C22" r:id="rId1" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/sp?tab=models" xr:uid="{FE987DC0-578A-4A81-AB17-6E49D6983782}"/>
+    <hyperlink ref="C23" r:id="rId2" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/spe?tab=models" xr:uid="{E414E66B-6D50-4BC0-93B6-EEDD71D1D349}"/>
+    <hyperlink ref="C24" r:id="rId3" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/sp-ne?tab=models" xr:uid="{79A82224-5E75-416A-BD5C-1C442DB4F9E7}"/>
+    <hyperlink ref="D22" r:id="rId4" display="https://product-selection.grundfos.com/fr/products/bm?tab=products" xr:uid="{39935FC4-BF60-4ADA-99B8-6280D11B4087}"/>
+    <hyperlink ref="D23" r:id="rId5" display="https://product-selection.grundfos.com/fr/products/bms?tab=products" xr:uid="{201298BF-F5B7-4DD8-896A-A6CFDF20A155}"/>
+    <hyperlink ref="D24" r:id="rId6" display="https://product-selection.grundfos.com/fr/products/bm-hp?tab=products" xr:uid="{0AA34BB7-1783-4351-AB39-2E3E2C9E6D24}"/>
+    <hyperlink ref="E22" r:id="rId7" display="https://product-selection.grundfos.com/fr/products/kpl?tab=models" xr:uid="{02FD05D5-211D-4185-A911-F718E163AF22}"/>
+    <hyperlink ref="E23" r:id="rId8" display="https://product-selection.grundfos.com/fr/products/kwm?tab=documentation" xr:uid="{F11B5E61-F53C-4DA1-93C5-A57D0408930C}"/>
+    <hyperlink ref="F22" r:id="rId9" display="https://product-selection.grundfos.com/fr/products/ls?tab=products" xr:uid="{070C34E9-9C05-4522-9AD2-8E6D82261A9B}"/>
+    <hyperlink ref="J22" r:id="rId10" display="https://product-selection.grundfos.com/fr/products/cm-cme?tab=products" xr:uid="{E79A5B97-E6E0-4649-B070-9A1CF47F88B2}"/>
+    <hyperlink ref="I22" r:id="rId11" display="https://product-selection.grundfos.com/fr/products/cm-cme/cm-self-priming?tab=models" xr:uid="{CFEF6DD3-2F90-4195-BA05-DEE28F55BD3E}"/>
+    <hyperlink ref="J23" r:id="rId12" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nb?tab=documentation" xr:uid="{ABC208A8-FE5B-4CC4-B585-6A3873FA7294}"/>
+    <hyperlink ref="J24" r:id="rId13" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nbe?tab=models" xr:uid="{1D4EF590-19C1-44EB-8B92-46AD5F28F62F}"/>
+    <hyperlink ref="J25" r:id="rId14" display="https://product-selection.grundfos.com/fr/products/nk-nke-nke-series-2000-nk-bare-shaft?tab=products" xr:uid="{76D3161D-F2DD-4CCA-AC1D-AD2E393D8694}"/>
+    <hyperlink ref="J26" r:id="rId15" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft?tab=products" xr:uid="{9CA4757F-439C-4161-8B60-7C14A9EDCA69}"/>
+    <hyperlink ref="J27" r:id="rId16" display="https://product-selection.grundfos.com/fr/products/tp-tpe?tab=products" xr:uid="{0C9A1473-1926-417A-947F-8561754B7D76}"/>
+    <hyperlink ref="N24" r:id="rId17" display="https://product-selection.grundfos.com/fr/products/tp-tpe?tab=products" xr:uid="{7D2D046F-1C95-42DD-8F35-90280675B9EA}"/>
+    <hyperlink ref="N22" r:id="rId18" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nbe?tab=models" xr:uid="{303D01A6-AC7B-42EE-AE09-2A10FBED3940}"/>
+    <hyperlink ref="N23" r:id="rId19" display="https://product-selection.grundfos.com/fr/products/nk-nke-nke-series-2000-nk-bare-shaft?tab=products" xr:uid="{A1442A3E-E286-4D87-BF5A-B52C00F11931}"/>
+    <hyperlink ref="N25" r:id="rId20" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft?tab=products" xr:uid="{91C811C0-E7C2-45CC-8C4A-41851188982F}"/>
+    <hyperlink ref="K22" r:id="rId21" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte?tab=products" xr:uid="{168A97AE-925F-4CB8-99FA-4D28B053F7CB}"/>
+    <hyperlink ref="L23" r:id="rId22" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte/cre?tab=models" xr:uid="{43E68B92-4EB3-4ECE-A299-C7DDCAFB1889}"/>
+    <hyperlink ref="L24" r:id="rId23" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte/crne?tab=models" xr:uid="{9DD9406E-F477-49F6-BA29-841ED00CE74B}"/>
+    <hyperlink ref="M22" r:id="rId24" display="https://product-selection.grundfos.com/fr/products/cm-cme/cme?tab=models" xr:uid="{CB210458-379C-4663-B0FD-73E843090C67}"/>
+    <hyperlink ref="M23" r:id="rId25" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nbe?tab=models" xr:uid="{3776F606-4CBE-49B1-912C-5B2BC9586206}"/>
+    <hyperlink ref="M24" r:id="rId26" display="https://product-selection.grundfos.com/fr/products/nk-nke-nke-series-2000-nk-bare-shaft?tab=products" xr:uid="{8731A9E7-9B51-450F-BCB5-013214A2B33F}"/>
+    <hyperlink ref="M25" r:id="rId27" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft?tab=products" xr:uid="{EDB8C821-F675-4CE1-B7B0-0FAF39DCEFD4}"/>
+    <hyperlink ref="L26" r:id="rId28" display="https://product-selection.grundfos.com/fr/products/hydro-multi-e?tab=models" xr:uid="{5995DFA3-65AE-4378-BD2E-CDA4F6FA5ED7}"/>
+    <hyperlink ref="L27" r:id="rId29" display="https://product-selection.grundfos.com/fr/products/hydro-mpc?tab=products" xr:uid="{2E37CE89-9B22-43AA-B967-C6F20A25613F}"/>
+    <hyperlink ref="L25" r:id="rId30" display="https://product-selection.grundfos.com/fr/products/hydro-solo-e?tab=models" xr:uid="{5A1F2584-1AA0-4C8B-A55D-39C825C8A3F8}"/>
+    <hyperlink ref="O22" r:id="rId31" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/sl1?tab=models" xr:uid="{9C7E88DB-59BA-4B5C-8769-45D64CC97D40}"/>
+    <hyperlink ref="O23" r:id="rId32" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/slv?tab=models" xr:uid="{00039B9D-B404-44A8-B557-BBF172D7CD31}"/>
+    <hyperlink ref="O24" r:id="rId33" display="https://product-selection.grundfos.com/fr/products/sesl-9-30-kw?tab=models" xr:uid="{C90FBAD5-7C9C-4429-9BAC-9BE027B562FD}"/>
+    <hyperlink ref="O26" r:id="rId34" display="https://product-selection.grundfos.com/fr/products/s?tab=products" xr:uid="{6F267867-1729-460E-9939-DEBA10D95429}"/>
+    <hyperlink ref="O25" r:id="rId35" display="https://product-selection.grundfos.com/fr/products/sesl-frame-size-56?tab=models" xr:uid="{541D6F69-2D4F-412B-91C7-A0B79C20C0CA}"/>
+    <hyperlink ref="P23" r:id="rId36" display="https://product-selection.grundfos.com/fr/products/unilift-ap/unilift-apg?tab=models" xr:uid="{CF6542DD-C411-4584-A2A2-ADD9BD336104}"/>
+    <hyperlink ref="P22" r:id="rId37" display="https://product-selection.grundfos.com/fr/products/seg?tab=models" xr:uid="{AF847B64-9B08-45DD-8487-57C6900B0D5F}"/>
+    <hyperlink ref="Q22" r:id="rId38" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/se1?tab=models" xr:uid="{D2271F27-967E-46DC-8195-E2EAFD3339EB}"/>
+    <hyperlink ref="Q23" r:id="rId39" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/sev?tab=models" xr:uid="{6D042873-5F32-4A50-8803-93F40528C6A1}"/>
+    <hyperlink ref="Q24" r:id="rId40" display="https://product-selection.grundfos.com/fr/products/sesl-9-30-kw?tab=models" xr:uid="{A344F5B5-8A97-456F-87D5-4C6EFCA52D3A}"/>
+    <hyperlink ref="Q25" r:id="rId41" display="https://product-selection.grundfos.com/fr/products/sesl-frame-size-56?tab=models" xr:uid="{BB0B40A3-A20A-44BC-9FC9-E9EE00FC9F45}"/>
+    <hyperlink ref="Q26" r:id="rId42" display="https://product-selection.grundfos.com/fr/products/s?tab=products" xr:uid="{2E26D22E-3FD7-4718-9B39-661D30AF938C}"/>
+    <hyperlink ref="Q27" r:id="rId43" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft/nkg-supervortex-impeller?tab=explore" xr:uid="{FA539854-B47D-4B47-9F9A-7CE595B28025}"/>
+    <hyperlink ref="S22" r:id="rId44" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/se1?tab=models" xr:uid="{66C50FE8-D6EA-4602-866A-7B3258A9261C}"/>
+    <hyperlink ref="S23" r:id="rId45" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/sev?tab=models" xr:uid="{DEFE3A48-5152-4917-935D-8BAB7D40CDD7}"/>
+    <hyperlink ref="S24" r:id="rId46" display="https://product-selection.grundfos.com/fr/products/sesl-9-30-kw?tab=models" xr:uid="{62BA715F-3850-4F49-A593-7645C6C0C3CC}"/>
+    <hyperlink ref="S25" r:id="rId47" display="https://product-selection.grundfos.com/fr/products/sesl-frame-size-56?tab=models" xr:uid="{F0AA29DC-4DA5-4CA6-94B3-C22351F6904E}"/>
+    <hyperlink ref="S26" r:id="rId48" display="https://product-selection.grundfos.com/fr/products/s?tab=products" xr:uid="{96671AB9-9AEA-4A5F-B84F-E78888F9B311}"/>
+    <hyperlink ref="S27" r:id="rId49" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft/nkg-supervortex-impeller?tab=explore" xr:uid="{8A1CF826-08F5-4AF2-B984-9AA020480952}"/>
+    <hyperlink ref="O27" r:id="rId50" display="https://product-selection.grundfos.com/fr/products/unilift-ap/unilift-ap50b?tab=models" xr:uid="{14E21A07-FF5F-4129-AE6E-260A1AA5098C}"/>
+    <hyperlink ref="W22" r:id="rId51" display="https://product-selection.grundfos.com/fr/products/unilift-ap?tab=products" xr:uid="{FF1F3D5A-16C1-4C5A-8F69-37BEB2C51657}"/>
+    <hyperlink ref="W23" r:id="rId52" display="https://product-selection.grundfos.com/fr/products/unilift-kp?tab=models" xr:uid="{D8B15CDE-A46F-4955-8CE5-B1F2491BDDEE}"/>
+    <hyperlink ref="W24" r:id="rId53" display="https://product-selection.grundfos.com/fr/products/unilift-cc?tab=models" xr:uid="{5DA16314-BD6C-4DB3-8EC0-A99C56D3006D}"/>
+    <hyperlink ref="W25" r:id="rId54" display="https://product-selection.grundfos.com/fr/products/dp?tab=models" xr:uid="{4D82ED98-3DD6-4697-9C9C-A060C7E06489}"/>
+    <hyperlink ref="W26" r:id="rId55" display="https://product-selection.grundfos.com/fr/products/ef?tab=models" xr:uid="{ABDE8970-72CB-4EB8-979F-99183A9FD9D3}"/>
+    <hyperlink ref="Y22" r:id="rId56" display="https://product-selection.grundfos.com/fr/products/mt-tank-mounted-pumps/mtr?tab=models" xr:uid="{D5799B15-EF87-41DF-88D8-05F25935D793}"/>
+    <hyperlink ref="Y23" r:id="rId57" display="https://product-selection.grundfos.com/fr/products/mt-tank-mounted-pumps/mtre?tab=models" xr:uid="{7E2DAAB5-3884-49DD-BF25-FA92C2CE9951}"/>
+    <hyperlink ref="Y24" r:id="rId58" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nb?tab=documentation" xr:uid="{92C19ACB-7462-4938-A66E-478979299908}"/>
+    <hyperlink ref="Y25" r:id="rId59" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nbe?tab=models" xr:uid="{D2CCE95F-A5DF-4715-B3CA-DB297F6DF5C8}"/>
+    <hyperlink ref="Y26" r:id="rId60" display="https://product-selection.grundfos.com/fr/products/nk-nke-nke-series-2000-nk-bare-shaft?tab=products" xr:uid="{EA080A36-FCEB-4D04-B389-F8ABE5514300}"/>
+    <hyperlink ref="Y27" r:id="rId61" display="https://product-selection.grundfos.com/fr/products/tp-tpe?tab=products" xr:uid="{2A2A6B6D-2CAA-4110-9FED-BCA8DC5F1709}"/>
+    <hyperlink ref="Y28" r:id="rId62" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte?tab=products" xr:uid="{D902984C-2BC5-48A4-BF49-DCE4C7E629F6}"/>
+    <hyperlink ref="Z22" r:id="rId63" display="https://product-selection.grundfos.com/fr/products/hydro-en?tab=models" xr:uid="{69CECDCF-71ED-40D6-A274-30663F73D3A6}"/>
+    <hyperlink ref="AD22" r:id="rId64" display="https://product-selection.grundfos.com/fr/products/poweradapt?tab=models" xr:uid="{CBB79406-3EE4-4CC7-BCD3-398882D58A96}"/>
+    <hyperlink ref="AD23" r:id="rId65" display="https://product-selection.grundfos.com/fr/products/rsi?tab=models" xr:uid="{2ECDD4BA-B757-4A11-9F78-EB235920F462}"/>
+    <hyperlink ref="AD24" r:id="rId66" display="https://product-selection.grundfos.com/fr/products/crflex?tab=models" xr:uid="{F1835770-C21F-4E8A-9EBF-7C701B0E9CF4}"/>
+    <hyperlink ref="AD25" r:id="rId67" display="https://product-selection.grundfos.com/fr/products/sqflex?tab=models" xr:uid="{2932EAA4-553E-42B6-AD4B-37D91C9B845C}"/>
+    <hyperlink ref="AD26" r:id="rId68" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/sp?tab=models" xr:uid="{25A70C6E-05E1-4E40-956B-50B78B088135}"/>
+    <hyperlink ref="AD27" r:id="rId69" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/spe?tab=models" xr:uid="{7C346AF6-2EEB-4DFC-A819-DAE2C3B09113}"/>
+    <hyperlink ref="AD28" r:id="rId70" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte?tab=products" xr:uid="{9F4AE584-6CDD-45BE-ABC9-5087AAD766B9}"/>
+    <hyperlink ref="AE22" r:id="rId71" display="https://product-selection.grundfos.com/fr/products/dosing-pumps-digital/dda?tab=models" xr:uid="{68600FE5-FDB0-4237-8B8A-45786462FE8A}"/>
+    <hyperlink ref="AE23" r:id="rId72" display="https://product-selection.grundfos.com/fr/products/dosing-pumps-digital/dme?tab=models" xr:uid="{41502941-2297-46B7-A840-2EF7A24064D7}"/>
+    <hyperlink ref="AE24" r:id="rId73" display="https://product-selection.grundfos.com/fr/products/dosing-pumps-mechanical/dmx?tab=models" xr:uid="{A892A826-C3E1-4B26-9529-8174E76C068D}"/>
+    <hyperlink ref="AE25" r:id="rId74" display="https://product-selection.grundfos.com/fr/products/dosing-pumps-mechanical/dmh?tab=models" xr:uid="{60926621-C7DA-4892-9ACA-4145E303C37B}"/>
+    <hyperlink ref="AE26" r:id="rId75" xr:uid="{EB339B7E-AAB0-4720-A5DC-B7E47BEFE888}"/>
+    <hyperlink ref="AF24" r:id="rId76" display="https://product-selection.grundfos.com/fr/products/disinfection-systems/oxiperm?tab=models" xr:uid="{D1CFBDC1-076A-4661-B343-B5087946D2BF}"/>
+    <hyperlink ref="AF22" r:id="rId77" display="https://product-selection.grundfos.com/fr/products/disinfection-systems/vaccuperm?tab=models" xr:uid="{0E5CA30E-D80E-4BC1-BE8D-5757C0E703F9}"/>
+    <hyperlink ref="AF23" r:id="rId78" display="https://product-selection.grundfos.com/fr/products/disinfection-systems/selcoperm?tab=models" xr:uid="{3FE337C4-03C2-4326-92F3-2ADF14429172}"/>
+    <hyperlink ref="C30" r:id="rId79" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-4" xr:uid="{7CECB146-2C6E-4D8C-8362-B574F0A0B1CD}"/>
+    <hyperlink ref="C31" r:id="rId80" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-6" xr:uid="{77066640-D437-4393-AE04-9291CA2EA2E2}"/>
+    <hyperlink ref="C32" r:id="rId81" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-8" xr:uid="{440D559C-9B55-46F7-B47D-809066594D8E}"/>
+    <hyperlink ref="C33" r:id="rId82" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-actun-zetos" xr:uid="{6B88B868-32F8-4635-8067-C4F8AA30A87A}"/>
+    <hyperlink ref="C34" r:id="rId83" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-14-24" xr:uid="{6AAEB27D-0CD4-409C-9175-B5DC81BA5B91}"/>
+    <hyperlink ref="D30" r:id="rId84" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-4" xr:uid="{70B5668C-6DE4-4721-BD0D-15695ACCFD10}"/>
+    <hyperlink ref="D31" r:id="rId85" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-6" xr:uid="{AB0F5528-0721-49E7-9EB4-443A836A5BE6}"/>
+    <hyperlink ref="D32" r:id="rId86" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-8" xr:uid="{CE5D4CF5-B9AD-4786-AF2A-5CBA0FB4461E}"/>
+    <hyperlink ref="D33" r:id="rId87" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-actun-zetos" xr:uid="{F3302311-60D3-4257-BE0E-8ADCE8FD3F26}"/>
+    <hyperlink ref="D34" r:id="rId88" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-14-24" xr:uid="{C714C692-05B2-43B9-83CE-06CDCF547DAA}"/>
+    <hyperlink ref="F30" r:id="rId89" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-scp" xr:uid="{7BEBF8BE-E457-43DD-A078-9A05C9712ED1}"/>
+    <hyperlink ref="F31" r:id="rId90" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-atmos-tera-sch" xr:uid="{8AC9B5FF-3554-4A3F-9A49-254FDDC1D679}"/>
+    <hyperlink ref="G30" r:id="rId91" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-4" xr:uid="{A6F45EEC-DFC1-4F41-A737-7D50D323F858}"/>
+    <hyperlink ref="G31" r:id="rId92" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-6" xr:uid="{E8092E13-22EC-4AA4-A0E2-CB8C894814DA}"/>
+    <hyperlink ref="G32" r:id="rId93" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-8" xr:uid="{06C47C82-BB6B-4167-9AFC-F87F629A6D2D}"/>
+    <hyperlink ref="G33" r:id="rId94" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-actun-zetos" xr:uid="{7F484481-A382-4AA7-BC6F-9F9E8E881F13}"/>
+    <hyperlink ref="G34" r:id="rId95" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-14-24" xr:uid="{145E082E-ACF5-4C03-95AA-D5FF287B68E9}"/>
+    <hyperlink ref="J30" r:id="rId96" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-medana-ch1-l" xr:uid="{CB6CAFF8-329E-47DC-8F46-39C8BB5E04DD}"/>
+    <hyperlink ref="J31" r:id="rId97" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-zeox-first-h" xr:uid="{2D403080-ECF0-434D-8570-2DCE4384BDB3}"/>
+    <hyperlink ref="K30" r:id="rId98" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-helix-v" xr:uid="{24EB14FB-8853-4DD9-BFF7-D08622F6269E}"/>
+    <hyperlink ref="K31" r:id="rId99" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-helix-first-v" xr:uid="{292648A6-CEF7-4F6A-B9E8-2C2D1935D493}"/>
+    <hyperlink ref="L30" r:id="rId100" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-helix-ve" xr:uid="{CB04A41A-2CE9-45EC-90FB-F63D1D7003E0}"/>
+    <hyperlink ref="L31" r:id="rId101" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-helix2-0-ve" xr:uid="{0D95BEE0-BF20-4117-86C3-9423999074AC}"/>
+    <hyperlink ref="M30" r:id="rId102" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-medana-ch3-le" xr:uid="{E61CDC21-E587-41FD-8720-AA95E8F2BCB8}"/>
+    <hyperlink ref="N30" r:id="rId103" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-isar-modh1-e-2-3" xr:uid="{2D23D0CC-B7DF-4FF1-ABE9-A9C38B0D675F}"/>
+    <hyperlink ref="N31" r:id="rId104" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-siboost2-0-smart-helix-ve" xr:uid="{FFEEE275-2C73-4EC4-B193-CB85762B0142}"/>
+    <hyperlink ref="O30" r:id="rId105" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-pro" xr:uid="{40187CA6-E027-4F57-B695-B124E41E9781}"/>
+    <hyperlink ref="O31" r:id="rId106" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-supra" xr:uid="{6510CD0A-CFE7-486C-91AF-7C7A655B4AFB}"/>
+    <hyperlink ref="O32" r:id="rId107" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-solid" xr:uid="{BDC567B5-AC65-4996-9A0B-1AF09DF2041A}"/>
+    <hyperlink ref="Q30" r:id="rId108" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-bloc" xr:uid="{3980AF89-63D6-4F8A-AA62-E67520B41458}"/>
+    <hyperlink ref="Q31" r:id="rId109" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-norm" xr:uid="{713EE9E0-CE07-4B5A-8098-8828FD7A2BE1}"/>
+    <hyperlink ref="P30" r:id="rId110" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-pro-s" xr:uid="{7EA67BA6-0CB9-4BC2-8D2F-2187D3E3EC87}"/>
+    <hyperlink ref="O33" r:id="rId111" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-fa-configure" xr:uid="{F271E929-C189-489C-95BA-44C8F95B9706}"/>
+    <hyperlink ref="S30" r:id="rId112" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-pro" xr:uid="{4E520461-D8CA-4714-95A3-4A07D979003B}"/>
+    <hyperlink ref="S31" r:id="rId113" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-supra" xr:uid="{7E747CBF-258D-4F97-AE71-AF52B950EDDE}"/>
+    <hyperlink ref="S32" r:id="rId114" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-solid" xr:uid="{90F21445-AD91-480E-9E60-99DEEB471A24}"/>
+    <hyperlink ref="S33" r:id="rId115" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-fa-configure" xr:uid="{CAC9CBDD-5033-4067-92F5-E1A89E7A10BF}"/>
+    <hyperlink ref="U30" r:id="rId116" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-pro" xr:uid="{DED143CB-BC81-4CC1-99AF-6D9EFDCA04A2}"/>
+    <hyperlink ref="U31" r:id="rId117" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-supra" xr:uid="{AD0F4A4E-82E3-443D-B5CE-BB1383456F96}"/>
+    <hyperlink ref="U32" r:id="rId118" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-solid" xr:uid="{F30C0BD2-ACC1-498E-B06C-26D556B514B6}"/>
+    <hyperlink ref="U33" r:id="rId119" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-fa-configure" xr:uid="{FC92FF04-817E-49C9-B9E1-3FED19E3DBAA}"/>
+    <hyperlink ref="W30" r:id="rId120" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-drain-tm-tmw-tmr-32" xr:uid="{0F177732-3552-46D9-B2A1-0858315CC611}"/>
+    <hyperlink ref="W31" r:id="rId121" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-padus-uni" xr:uid="{31C21B43-5DBE-431A-A886-4FBC3A6BE491}"/>
+    <hyperlink ref="W32" r:id="rId122" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-padus-mini3" xr:uid="{D91894CF-CB16-4C43-980E-41E743666848}"/>
+    <hyperlink ref="W33" r:id="rId123" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-padus-pro" xr:uid="{79DE7E3B-A7A2-4098-B5DF-694F7F93640D}"/>
+    <hyperlink ref="Z30" r:id="rId124" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-cof-helix" xr:uid="{2E5216D3-37DA-48CB-ABA0-7C21064BB2D3}"/>
   </hyperlinks>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="8" scale="83" orientation="landscape" r:id="rId125"/>

</xml_diff>

<commit_message>
Mise à jour depuis Excel — 2026-09-18T09:32:46.536Z
</commit_message>
<xml_diff>
--- a/comparatif.xlsx
+++ b/comparatif.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nge1.sharepoint.com/sites/FR_SADE_DAM/Documents partages/01 - Achats/Achats Production/Pompes &amp; Instrum/Pompes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{37FDA403-DBA7-4B2E-BE07-2EFF4B991CF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6A66B74A-82F5-418B-B656-D58A0D28BDBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="7716" yWindow="12852" windowWidth="23256" windowHeight="12456" xr2:uid="{723C6001-552E-447F-BEBB-92F546F7738F}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Feuil2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Feuil1!$A$2:$AF$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Feuil1!$A$2:$AF$33</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="286">
   <si>
     <t>Eau potable et irrigation</t>
   </si>
@@ -87,10 +87,13 @@
     <t>Pompes immergées</t>
   </si>
   <si>
+    <t>cantine</t>
+  </si>
+  <si>
+    <t>Immergées</t>
+  </si>
+  <si>
     <t>De surface</t>
-  </si>
-  <si>
-    <t>Immergées</t>
   </si>
   <si>
     <t>Types</t>
@@ -149,21 +152,6 @@
   <si>
     <t xml:space="preserve"> Volumétrique
 cela veut il dire extérieure ?</t>
-  </si>
-  <si>
-    <t>Couleur</t>
-  </si>
-  <si>
-    <t>jaune</t>
-  </si>
-  <si>
-    <t>bleu</t>
-  </si>
-  <si>
-    <t>Vertical turbine</t>
-  </si>
-  <si>
-    <t>rouge</t>
   </si>
   <si>
     <t>Application</t>
@@ -766,6 +754,9 @@
   </si>
   <si>
     <t>sub TWI 4/6/8 , Actun ZETOS K8/10/12, EMU</t>
+  </si>
+  <si>
+    <t>Vertical turbine</t>
   </si>
   <si>
     <t>SCP, Atmos Tera SCH
@@ -1594,7 +1585,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="121">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1930,9 +1921,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2279,7 +2267,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:EY61"/>
+  <dimension ref="A1:EY60"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="7.140625" style="1" customWidth="1"/>
@@ -2381,7 +2369,7 @@
       </c>
       <c r="P3" s="101"/>
       <c r="Q3" s="100" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="R3" s="101"/>
       <c r="S3" s="101"/>
@@ -2401,67 +2389,67 @@
     </row>
     <row r="4" spans="1:32" s="80" customFormat="1" ht="57.75" customHeight="1" thickBot="1">
       <c r="B4" s="81" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C4" s="82" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D4" s="82" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E4" s="82" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F4" s="82" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G4" s="82" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H4" s="82" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I4" s="82" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J4" s="82" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K4" s="82" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L4" s="82" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="M4" s="82" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="N4" s="82" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="O4" s="82" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="P4" s="82" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q4" s="82" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R4" s="82" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="S4" s="82" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="T4" s="82" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="U4" s="83" t="s">
         <v>15</v>
       </c>
       <c r="V4" s="83" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="W4" s="107"/>
       <c r="X4" s="99"/>
@@ -2474,248 +2462,235 @@
       <c r="AE4" s="93"/>
       <c r="AF4" s="94"/>
     </row>
-    <row r="5" spans="1:32" s="80" customFormat="1" ht="57.75" customHeight="1">
-      <c r="B5" s="87" t="s">
-        <v>35</v>
-      </c>
-      <c r="C5" s="88" t="s">
-        <v>36</v>
-      </c>
-      <c r="D5" s="88" t="s">
-        <v>37</v>
-      </c>
-      <c r="E5" s="88" t="s">
-        <v>38</v>
-      </c>
-      <c r="F5" s="88" t="s">
-        <v>39</v>
-      </c>
-      <c r="G5" s="88" t="s">
-        <v>36</v>
-      </c>
-      <c r="H5" s="88" t="s">
-        <v>37</v>
-      </c>
-      <c r="I5" s="88" t="s">
-        <v>38</v>
-      </c>
-      <c r="J5" s="88" t="s">
-        <v>39</v>
-      </c>
-      <c r="K5" s="88" t="s">
-        <v>36</v>
-      </c>
-      <c r="L5" s="88" t="s">
-        <v>37</v>
-      </c>
-      <c r="M5" s="88" t="s">
-        <v>38</v>
-      </c>
-      <c r="N5" s="88" t="s">
-        <v>39</v>
-      </c>
-      <c r="O5" s="88" t="s">
-        <v>36</v>
-      </c>
-      <c r="P5" s="88" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q5" s="88" t="s">
-        <v>38</v>
-      </c>
-      <c r="R5" s="88" t="s">
-        <v>39</v>
-      </c>
-      <c r="S5" s="88" t="s">
-        <v>36</v>
-      </c>
-      <c r="T5" s="88" t="s">
-        <v>37</v>
-      </c>
-      <c r="U5" s="88" t="s">
-        <v>38</v>
-      </c>
-      <c r="V5" s="88" t="s">
-        <v>39</v>
-      </c>
-      <c r="W5" s="88" t="s">
-        <v>36</v>
-      </c>
+    <row r="5" spans="1:32" s="80" customFormat="1" ht="10.15" customHeight="1" thickBot="1">
+      <c r="B5" s="87"/>
+      <c r="C5" s="88"/>
+      <c r="D5" s="88"/>
+      <c r="E5" s="88"/>
+      <c r="F5" s="88"/>
+      <c r="G5" s="88"/>
+      <c r="H5" s="88"/>
+      <c r="I5" s="88"/>
+      <c r="J5" s="88"/>
+      <c r="K5" s="88"/>
+      <c r="L5" s="88"/>
+      <c r="M5" s="88"/>
+      <c r="N5" s="88"/>
+      <c r="O5" s="88"/>
+      <c r="P5" s="88"/>
+      <c r="Q5" s="88"/>
+      <c r="R5" s="88"/>
+      <c r="S5" s="88"/>
+      <c r="T5" s="88"/>
+      <c r="U5" s="89"/>
+      <c r="V5" s="89"/>
+      <c r="W5" s="86"/>
       <c r="X5" s="86"/>
       <c r="Y5" s="86"/>
       <c r="Z5" s="86"/>
       <c r="AA5" s="86"/>
       <c r="AB5" s="86"/>
       <c r="AC5" s="90"/>
-      <c r="AD5" s="120"/>
-      <c r="AE5" s="120"/>
-      <c r="AF5" s="120"/>
+      <c r="AD5" s="91"/>
+      <c r="AE5" s="91"/>
+      <c r="AF5" s="91"/>
     </row>
-    <row r="6" spans="1:32" s="80" customFormat="1" ht="10.15" customHeight="1" thickBot="1">
-      <c r="B6" s="87"/>
-      <c r="C6" s="88"/>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="88"/>
-      <c r="K6" s="88"/>
-      <c r="L6" s="88"/>
-      <c r="M6" s="88"/>
-      <c r="N6" s="88"/>
-      <c r="O6" s="88"/>
-      <c r="P6" s="88"/>
-      <c r="Q6" s="88"/>
-      <c r="R6" s="88"/>
-      <c r="S6" s="88"/>
-      <c r="T6" s="88"/>
-      <c r="U6" s="89"/>
-      <c r="V6" s="89"/>
-      <c r="W6" s="86"/>
-      <c r="X6" s="86"/>
-      <c r="Y6" s="86"/>
-      <c r="Z6" s="86"/>
-      <c r="AA6" s="86"/>
-      <c r="AB6" s="86"/>
-      <c r="AC6" s="90"/>
-      <c r="AD6" s="91"/>
-      <c r="AE6" s="91"/>
-      <c r="AF6" s="91"/>
+    <row r="6" spans="1:32" s="74" customFormat="1" ht="52.9" customHeight="1">
+      <c r="B6" s="84" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" s="77" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" s="77" t="s">
+        <v>38</v>
+      </c>
+      <c r="E6" s="77" t="s">
+        <v>39</v>
+      </c>
+      <c r="F6" s="77" t="s">
+        <v>38</v>
+      </c>
+      <c r="G6" s="77" t="s">
+        <v>40</v>
+      </c>
+      <c r="H6" s="77" t="s">
+        <v>38</v>
+      </c>
+      <c r="I6" s="77" t="s">
+        <v>41</v>
+      </c>
+      <c r="J6" s="77" t="s">
+        <v>38</v>
+      </c>
+      <c r="K6" s="77" t="s">
+        <v>38</v>
+      </c>
+      <c r="L6" s="77" t="s">
+        <v>37</v>
+      </c>
+      <c r="M6" s="77" t="s">
+        <v>38</v>
+      </c>
+      <c r="N6" s="77" t="s">
+        <v>42</v>
+      </c>
+      <c r="O6" s="77" t="s">
+        <v>43</v>
+      </c>
+      <c r="P6" s="77" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q6" s="77" t="s">
+        <v>43</v>
+      </c>
+      <c r="R6" s="77" t="s">
+        <v>43</v>
+      </c>
+      <c r="S6" s="77" t="s">
+        <v>43</v>
+      </c>
+      <c r="T6" s="77" t="s">
+        <v>43</v>
+      </c>
+      <c r="U6" s="77" t="s">
+        <v>43</v>
+      </c>
+      <c r="V6" s="77" t="s">
+        <v>43</v>
+      </c>
+      <c r="W6" s="77"/>
+      <c r="X6" s="77" t="s">
+        <v>44</v>
+      </c>
+      <c r="Y6" s="77" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z6" s="77"/>
+      <c r="AA6" s="77"/>
+      <c r="AB6" s="77"/>
+      <c r="AC6" s="78"/>
+      <c r="AD6" s="79" t="s">
+        <v>46</v>
+      </c>
+      <c r="AE6" s="79" t="s">
+        <v>47</v>
+      </c>
+      <c r="AF6" s="76" t="s">
+        <v>48</v>
+      </c>
     </row>
-    <row r="7" spans="1:32" s="74" customFormat="1" ht="52.9" customHeight="1">
-      <c r="B7" s="84" t="s">
-        <v>40</v>
-      </c>
-      <c r="C7" s="77" t="s">
-        <v>41</v>
-      </c>
-      <c r="D7" s="77" t="s">
-        <v>42</v>
-      </c>
-      <c r="E7" s="77" t="s">
-        <v>43</v>
-      </c>
-      <c r="F7" s="77" t="s">
-        <v>42</v>
-      </c>
-      <c r="G7" s="77" t="s">
-        <v>44</v>
-      </c>
-      <c r="H7" s="77" t="s">
-        <v>42</v>
-      </c>
-      <c r="I7" s="77" t="s">
-        <v>45</v>
-      </c>
-      <c r="J7" s="77" t="s">
-        <v>42</v>
-      </c>
-      <c r="K7" s="77" t="s">
-        <v>42</v>
-      </c>
-      <c r="L7" s="77" t="s">
-        <v>41</v>
-      </c>
-      <c r="M7" s="77" t="s">
-        <v>42</v>
-      </c>
-      <c r="N7" s="77" t="s">
-        <v>46</v>
-      </c>
-      <c r="O7" s="77" t="s">
-        <v>47</v>
-      </c>
-      <c r="P7" s="77" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q7" s="77" t="s">
-        <v>47</v>
-      </c>
-      <c r="R7" s="77" t="s">
-        <v>47</v>
-      </c>
-      <c r="S7" s="77" t="s">
-        <v>47</v>
-      </c>
-      <c r="T7" s="77" t="s">
-        <v>47</v>
-      </c>
-      <c r="U7" s="77" t="s">
-        <v>47</v>
-      </c>
-      <c r="V7" s="77" t="s">
-        <v>47</v>
-      </c>
-      <c r="W7" s="77"/>
-      <c r="X7" s="77" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y7" s="77" t="s">
+    <row r="7" spans="1:32" s="1" customFormat="1" ht="18" customHeight="1">
+      <c r="A7" s="95" t="s">
         <v>49</v>
       </c>
-      <c r="Z7" s="77"/>
-      <c r="AA7" s="77"/>
-      <c r="AB7" s="77"/>
-      <c r="AC7" s="78"/>
-      <c r="AD7" s="79" t="s">
+      <c r="B7" s="116" t="s">
         <v>50</v>
       </c>
-      <c r="AE7" s="79" t="s">
+      <c r="C7" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="AF7" s="76" t="s">
+      <c r="D7" s="11" t="s">
         <v>52</v>
       </c>
+      <c r="E7" s="11"/>
+      <c r="F7" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="I7" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="J7" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="K7" s="11"/>
+      <c r="L7" s="11"/>
+      <c r="M7" s="11"/>
+      <c r="N7" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="O7" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="P7" s="11"/>
+      <c r="Q7" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="R7" s="11"/>
+      <c r="S7" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="T7" s="11"/>
+      <c r="U7" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="V7" s="11"/>
+      <c r="W7" s="11"/>
+      <c r="X7" s="11"/>
+      <c r="Y7" s="11"/>
+      <c r="Z7" s="11"/>
+      <c r="AA7" s="11"/>
+      <c r="AB7" s="5"/>
+      <c r="AC7" s="54"/>
+      <c r="AD7" s="76"/>
+      <c r="AE7" s="76"/>
+      <c r="AF7" s="76"/>
     </row>
     <row r="8" spans="1:32" s="1" customFormat="1" ht="18" customHeight="1">
-      <c r="A8" s="95" t="s">
-        <v>53</v>
-      </c>
-      <c r="B8" s="116" t="s">
-        <v>54</v>
-      </c>
+      <c r="A8" s="96"/>
+      <c r="B8" s="114"/>
       <c r="C8" s="11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="E8" s="11"/>
+        <v>59</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>60</v>
+      </c>
       <c r="F8" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="G8" s="11"/>
+        <v>61</v>
+      </c>
+      <c r="G8" s="11" t="s">
+        <v>60</v>
+      </c>
       <c r="H8" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="I8" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="I8" s="11"/>
+      <c r="J8" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="J8" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="K8" s="11"/>
+      <c r="K8" s="11" t="s">
+        <v>63</v>
+      </c>
       <c r="L8" s="11"/>
-      <c r="M8" s="11"/>
+      <c r="M8" s="11" t="s">
+        <v>64</v>
+      </c>
       <c r="N8" s="11" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="O8" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="P8" s="11"/>
+        <v>65</v>
+      </c>
+      <c r="P8" s="11" t="s">
+        <v>65</v>
+      </c>
       <c r="Q8" s="11" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="R8" s="11"/>
       <c r="S8" s="11" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="T8" s="11"/>
       <c r="U8" s="11" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="V8" s="11"/>
       <c r="W8" s="11"/>
@@ -2732,55 +2707,39 @@
     <row r="9" spans="1:32" s="1" customFormat="1" ht="18" customHeight="1">
       <c r="A9" s="96"/>
       <c r="B9" s="114"/>
-      <c r="C9" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="E9" s="11" t="s">
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="I9" s="11"/>
+      <c r="J9" s="11"/>
+      <c r="K9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="L9" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="F9" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="G9" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="H9" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="I9" s="11"/>
-      <c r="J9" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="K9" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="L9" s="11"/>
       <c r="M9" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="N9" s="11" t="s">
         <v>68</v>
-      </c>
-      <c r="N9" s="11" t="s">
-        <v>67</v>
       </c>
       <c r="O9" s="11" t="s">
         <v>69</v>
       </c>
       <c r="P9" s="11" t="s">
-        <v>69</v>
-      </c>
-      <c r="Q9" s="11" t="s">
         <v>70</v>
       </c>
+      <c r="Q9" s="11"/>
       <c r="R9" s="11"/>
-      <c r="S9" s="11" t="s">
-        <v>70</v>
-      </c>
+      <c r="S9" s="11"/>
       <c r="T9" s="11"/>
-      <c r="U9" s="11" t="s">
-        <v>69</v>
-      </c>
+      <c r="U9" s="11"/>
       <c r="V9" s="11"/>
       <c r="W9" s="11"/>
       <c r="X9" s="11"/>
@@ -2806,24 +2765,16 @@
       </c>
       <c r="I10" s="11"/>
       <c r="J10" s="11"/>
-      <c r="K10" s="11" t="s">
-        <v>56</v>
-      </c>
+      <c r="K10" s="11"/>
       <c r="L10" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="M10" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="N10" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="M10" s="11"/>
+      <c r="N10" s="11"/>
+      <c r="O10" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="O10" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="P10" s="11" t="s">
-        <v>74</v>
-      </c>
+      <c r="P10" s="11"/>
       <c r="Q10" s="11"/>
       <c r="R10" s="11"/>
       <c r="S10" s="11"/>
@@ -2843,243 +2794,268 @@
     </row>
     <row r="11" spans="1:32" s="1" customFormat="1" ht="18" customHeight="1">
       <c r="A11" s="96"/>
-      <c r="B11" s="114"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="I11" s="11"/>
-      <c r="J11" s="11"/>
-      <c r="K11" s="11"/>
-      <c r="L11" s="11" t="s">
+      <c r="B11" s="115"/>
+      <c r="C11" s="52"/>
+      <c r="D11" s="52"/>
+      <c r="E11" s="52"/>
+      <c r="F11" s="52"/>
+      <c r="G11" s="52"/>
+      <c r="H11" s="52"/>
+      <c r="I11" s="52"/>
+      <c r="J11" s="52"/>
+      <c r="K11" s="52"/>
+      <c r="L11" s="52" t="s">
         <v>63</v>
       </c>
-      <c r="M11" s="11"/>
-      <c r="N11" s="11"/>
-      <c r="O11" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="P11" s="11"/>
-      <c r="Q11" s="11"/>
-      <c r="R11" s="11"/>
-      <c r="S11" s="11"/>
-      <c r="T11" s="11"/>
-      <c r="U11" s="11"/>
-      <c r="V11" s="11"/>
-      <c r="W11" s="11"/>
-      <c r="X11" s="11"/>
-      <c r="Y11" s="11"/>
-      <c r="Z11" s="11"/>
-      <c r="AA11" s="11"/>
-      <c r="AB11" s="5"/>
-      <c r="AC11" s="54"/>
+      <c r="M11" s="52"/>
+      <c r="N11" s="52" t="s">
+        <v>73</v>
+      </c>
+      <c r="O11" s="52"/>
+      <c r="P11" s="52"/>
+      <c r="Q11" s="52" t="s">
+        <v>74</v>
+      </c>
+      <c r="R11" s="52"/>
+      <c r="S11" s="52" t="s">
+        <v>74</v>
+      </c>
+      <c r="T11" s="52"/>
+      <c r="U11" s="52"/>
+      <c r="V11" s="52"/>
+      <c r="W11" s="52"/>
+      <c r="X11" s="52"/>
+      <c r="Y11" s="52"/>
+      <c r="Z11" s="52"/>
+      <c r="AA11" s="52"/>
+      <c r="AB11" s="53"/>
+      <c r="AC11" s="55"/>
       <c r="AD11" s="76"/>
       <c r="AE11" s="76"/>
       <c r="AF11" s="76"/>
     </row>
-    <row r="12" spans="1:32" s="1" customFormat="1" ht="18" customHeight="1">
+    <row r="12" spans="1:32" ht="18" customHeight="1">
       <c r="A12" s="96"/>
-      <c r="B12" s="115"/>
-      <c r="C12" s="52"/>
-      <c r="D12" s="52"/>
-      <c r="E12" s="52"/>
-      <c r="F12" s="52"/>
-      <c r="G12" s="52"/>
-      <c r="H12" s="52"/>
-      <c r="I12" s="52"/>
-      <c r="J12" s="52"/>
-      <c r="K12" s="52"/>
-      <c r="L12" s="52" t="s">
-        <v>67</v>
-      </c>
-      <c r="M12" s="52"/>
-      <c r="N12" s="52" t="s">
+      <c r="B12" s="113" t="s">
+        <v>75</v>
+      </c>
+      <c r="C12" s="61" t="s">
+        <v>76</v>
+      </c>
+      <c r="D12" s="62" t="s">
         <v>77</v>
       </c>
-      <c r="O12" s="52"/>
-      <c r="P12" s="52"/>
-      <c r="Q12" s="52" t="s">
+      <c r="E12" s="63" t="s">
         <v>78</v>
       </c>
-      <c r="R12" s="52"/>
-      <c r="S12" s="52" t="s">
-        <v>78</v>
-      </c>
-      <c r="T12" s="52"/>
-      <c r="U12" s="52"/>
-      <c r="V12" s="52"/>
-      <c r="W12" s="52"/>
-      <c r="X12" s="52"/>
-      <c r="Y12" s="52"/>
-      <c r="Z12" s="52"/>
-      <c r="AA12" s="52"/>
-      <c r="AB12" s="53"/>
-      <c r="AC12" s="55"/>
-      <c r="AD12" s="76"/>
-      <c r="AE12" s="76"/>
-      <c r="AF12" s="76"/>
+      <c r="F12" s="62" t="s">
+        <v>77</v>
+      </c>
+      <c r="G12" s="62" t="s">
+        <v>77</v>
+      </c>
+      <c r="H12" s="62" t="s">
+        <v>77</v>
+      </c>
+      <c r="I12" s="61" t="s">
+        <v>79</v>
+      </c>
+      <c r="J12" s="61" t="s">
+        <v>80</v>
+      </c>
+      <c r="K12" s="37" t="s">
+        <v>81</v>
+      </c>
+      <c r="L12" s="61" t="s">
+        <v>82</v>
+      </c>
+      <c r="M12" s="62" t="s">
+        <v>77</v>
+      </c>
+      <c r="N12" s="61" t="s">
+        <v>83</v>
+      </c>
+      <c r="O12" s="61" t="s">
+        <v>84</v>
+      </c>
+      <c r="P12" s="37" t="s">
+        <v>85</v>
+      </c>
+      <c r="Q12" s="61" t="s">
+        <v>85</v>
+      </c>
+      <c r="R12" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="S12" s="61" t="s">
+        <v>85</v>
+      </c>
+      <c r="T12" s="61" t="s">
+        <v>85</v>
+      </c>
+      <c r="U12" s="61" t="s">
+        <v>85</v>
+      </c>
+      <c r="V12" s="62" t="s">
+        <v>77</v>
+      </c>
+      <c r="W12" s="61" t="s">
+        <v>87</v>
+      </c>
+      <c r="X12" s="62" t="s">
+        <v>77</v>
+      </c>
+      <c r="Y12" s="61" t="s">
+        <v>88</v>
+      </c>
+      <c r="Z12" s="61" t="s">
+        <v>87</v>
+      </c>
+      <c r="AA12" s="61" t="s">
+        <v>85</v>
+      </c>
+      <c r="AB12" s="37" t="s">
+        <v>89</v>
+      </c>
+      <c r="AC12" s="61" t="s">
+        <v>90</v>
+      </c>
+      <c r="AD12" s="20"/>
+      <c r="AE12" s="20"/>
+      <c r="AF12" s="75"/>
     </row>
     <row r="13" spans="1:32" ht="18" customHeight="1">
       <c r="A13" s="96"/>
-      <c r="B13" s="113" t="s">
-        <v>79</v>
-      </c>
-      <c r="C13" s="61" t="s">
-        <v>80</v>
-      </c>
-      <c r="D13" s="62" t="s">
-        <v>81</v>
-      </c>
-      <c r="E13" s="63" t="s">
-        <v>82</v>
-      </c>
-      <c r="F13" s="62" t="s">
-        <v>81</v>
-      </c>
-      <c r="G13" s="62" t="s">
-        <v>81</v>
-      </c>
-      <c r="H13" s="62" t="s">
-        <v>81</v>
-      </c>
-      <c r="I13" s="61" t="s">
-        <v>83</v>
-      </c>
-      <c r="J13" s="61" t="s">
-        <v>84</v>
-      </c>
-      <c r="K13" s="37" t="s">
+      <c r="B13" s="114"/>
+      <c r="C13" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
+      <c r="I13" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="J13" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="K13" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="L13" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="M13" s="4"/>
+      <c r="N13" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="O13" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="L13" s="61" t="s">
+      <c r="P13" s="4"/>
+      <c r="Q13" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="M13" s="62" t="s">
-        <v>81</v>
-      </c>
-      <c r="N13" s="61" t="s">
+      <c r="R13" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="O13" s="61" t="s">
-        <v>88</v>
-      </c>
-      <c r="P13" s="37" t="s">
+      <c r="S13" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="T13" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="U13" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="Q13" s="61" t="s">
+      <c r="V13" s="4"/>
+      <c r="W13" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="X13" s="4"/>
+      <c r="Y13" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="Z13" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="AA13" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="R13" s="37" t="s">
-        <v>90</v>
-      </c>
-      <c r="S13" s="61" t="s">
-        <v>89</v>
-      </c>
-      <c r="T13" s="61" t="s">
-        <v>89</v>
-      </c>
-      <c r="U13" s="61" t="s">
-        <v>89</v>
-      </c>
-      <c r="V13" s="62" t="s">
-        <v>81</v>
-      </c>
-      <c r="W13" s="61" t="s">
-        <v>91</v>
-      </c>
-      <c r="X13" s="62" t="s">
-        <v>81</v>
-      </c>
-      <c r="Y13" s="61" t="s">
-        <v>92</v>
-      </c>
-      <c r="Z13" s="61" t="s">
-        <v>91</v>
-      </c>
-      <c r="AA13" s="61" t="s">
-        <v>89</v>
-      </c>
-      <c r="AB13" s="37" t="s">
-        <v>93</v>
-      </c>
-      <c r="AC13" s="61" t="s">
-        <v>94</v>
-      </c>
-      <c r="AD13" s="20"/>
-      <c r="AE13" s="20"/>
-      <c r="AF13" s="75"/>
+      <c r="AB13" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="AC13" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="AD13" s="10"/>
+      <c r="AE13" s="10"/>
+      <c r="AF13" s="40"/>
     </row>
     <row r="14" spans="1:32" ht="18" customHeight="1">
       <c r="A14" s="96"/>
       <c r="B14" s="114"/>
       <c r="C14" s="11" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="D14" s="4"/>
       <c r="E14" s="4" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
-      <c r="I14" s="11" t="s">
-        <v>82</v>
+      <c r="I14" s="4" t="s">
+        <v>92</v>
       </c>
       <c r="J14" s="11" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="K14" s="11" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="L14" s="11" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="M14" s="4"/>
       <c r="N14" s="11" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="O14" s="11" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="P14" s="4"/>
-      <c r="Q14" s="11" t="s">
-        <v>90</v>
+      <c r="Q14" s="12" t="s">
+        <v>99</v>
       </c>
       <c r="R14" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="S14" s="11" t="s">
-        <v>101</v>
-      </c>
+        <v>98</v>
+      </c>
+      <c r="S14" s="4"/>
       <c r="T14" s="11" t="s">
-        <v>101</v>
-      </c>
-      <c r="U14" s="12" t="s">
-        <v>93</v>
+        <v>86</v>
+      </c>
+      <c r="U14" s="11" t="s">
+        <v>98</v>
       </c>
       <c r="V14" s="4"/>
       <c r="W14" s="11" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="X14" s="4"/>
-      <c r="Y14" s="12" t="s">
-        <v>103</v>
-      </c>
+      <c r="Y14" s="4"/>
       <c r="Z14" s="11" t="s">
-        <v>102</v>
-      </c>
-      <c r="AA14" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="AB14" s="12" t="s">
-        <v>104</v>
+        <v>108</v>
+      </c>
+      <c r="AA14" s="12" t="s">
+        <v>100</v>
       </c>
       <c r="AC14" s="11" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="AD14" s="10"/>
       <c r="AE14" s="10"/>
@@ -3089,62 +3065,57 @@
       <c r="A15" s="96"/>
       <c r="B15" s="114"/>
       <c r="C15" s="11" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="D15" s="4"/>
       <c r="E15" s="4" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
       <c r="I15" s="4" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="J15" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="K15" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="L15" s="4"/>
+      <c r="M15" s="4"/>
+      <c r="N15" s="4"/>
+      <c r="O15" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="P15" s="4"/>
+      <c r="Q15" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="R15" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="K15" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="L15" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="M15" s="4"/>
-      <c r="N15" s="11" t="s">
-        <v>111</v>
-      </c>
-      <c r="O15" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="P15" s="4"/>
-      <c r="Q15" s="12" t="s">
-        <v>103</v>
-      </c>
-      <c r="R15" s="11" t="s">
-        <v>102</v>
-      </c>
       <c r="S15" s="4"/>
-      <c r="T15" s="11" t="s">
-        <v>90</v>
-      </c>
+      <c r="T15" s="4"/>
       <c r="U15" s="11" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="V15" s="4"/>
       <c r="W15" s="11" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="X15" s="4"/>
       <c r="Y15" s="4"/>
       <c r="Z15" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="AA15" s="12" t="s">
-        <v>104</v>
-      </c>
+        <v>114</v>
+      </c>
+      <c r="AA15" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="AB15" s="11"/>
       <c r="AC15" s="11" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="AD15" s="10"/>
       <c r="AE15" s="10"/>
@@ -3154,57 +3125,53 @@
       <c r="A16" s="96"/>
       <c r="B16" s="114"/>
       <c r="C16" s="11" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D16" s="4"/>
-      <c r="E16" s="4" t="s">
-        <v>115</v>
-      </c>
+      <c r="E16" s="4"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
       <c r="I16" s="4" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="J16" s="11" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="K16" s="11" t="s">
-        <v>86</v>
+        <v>118</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4"/>
       <c r="N16" s="4"/>
       <c r="O16" s="11" t="s">
-        <v>101</v>
+        <v>87</v>
       </c>
       <c r="P16" s="4"/>
-      <c r="Q16" s="4" t="s">
-        <v>117</v>
-      </c>
+      <c r="Q16" s="4"/>
       <c r="R16" s="11" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="S16" s="4"/>
       <c r="T16" s="4"/>
       <c r="U16" s="11" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="V16" s="4"/>
       <c r="W16" s="11" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="X16" s="4"/>
       <c r="Y16" s="4"/>
       <c r="Z16" s="11" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AA16" s="11" t="s">
-        <v>101</v>
+        <v>87</v>
       </c>
       <c r="AB16" s="11"/>
       <c r="AC16" s="11" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="AD16" s="10"/>
       <c r="AE16" s="10"/>
@@ -3213,524 +3180,524 @@
     <row r="17" spans="1:155" ht="18" customHeight="1">
       <c r="A17" s="96"/>
       <c r="B17" s="114"/>
-      <c r="C17" s="11" t="s">
-        <v>120</v>
-      </c>
+      <c r="C17" s="4"/>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
-      <c r="I17" s="4" t="s">
-        <v>115</v>
-      </c>
+      <c r="I17" s="4"/>
       <c r="J17" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="K17" s="11" t="s">
-        <v>122</v>
-      </c>
+      <c r="K17" s="4"/>
       <c r="L17" s="4"/>
       <c r="M17" s="4"/>
       <c r="N17" s="4"/>
       <c r="O17" s="11" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="P17" s="4"/>
       <c r="Q17" s="4"/>
       <c r="R17" s="11" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="S17" s="4"/>
       <c r="T17" s="4"/>
       <c r="U17" s="11" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="V17" s="4"/>
-      <c r="W17" s="11" t="s">
-        <v>123</v>
+      <c r="W17" s="12" t="s">
+        <v>99</v>
       </c>
       <c r="X17" s="4"/>
       <c r="Y17" s="4"/>
-      <c r="Z17" s="11" t="s">
-        <v>123</v>
-      </c>
+      <c r="Z17" s="4"/>
       <c r="AA17" s="11" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="AB17" s="11"/>
       <c r="AC17" s="11" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="AD17" s="10"/>
       <c r="AE17" s="10"/>
       <c r="AF17" s="40"/>
     </row>
     <row r="18" spans="1:155" ht="18" customHeight="1">
-      <c r="A18" s="96"/>
-      <c r="B18" s="114"/>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
-      <c r="H18" s="4"/>
-      <c r="I18" s="4"/>
-      <c r="J18" s="11" t="s">
+      <c r="A18" s="97"/>
+      <c r="B18" s="115"/>
+      <c r="C18" s="32"/>
+      <c r="D18" s="32"/>
+      <c r="E18" s="32"/>
+      <c r="F18" s="32"/>
+      <c r="G18" s="32"/>
+      <c r="H18" s="32"/>
+      <c r="I18" s="32"/>
+      <c r="J18" s="52" t="s">
+        <v>123</v>
+      </c>
+      <c r="K18" s="32"/>
+      <c r="L18" s="32"/>
+      <c r="M18" s="32"/>
+      <c r="N18" s="32"/>
+      <c r="O18" s="52" t="s">
+        <v>108</v>
+      </c>
+      <c r="P18" s="32"/>
+      <c r="Q18" s="32"/>
+      <c r="R18" s="64" t="s">
+        <v>99</v>
+      </c>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="52" t="s">
+        <v>88</v>
+      </c>
+      <c r="V18" s="32"/>
+      <c r="W18" s="64" t="s">
+        <v>124</v>
+      </c>
+      <c r="X18" s="32"/>
+      <c r="Y18" s="32"/>
+      <c r="Z18" s="32"/>
+      <c r="AA18" s="52" t="s">
+        <v>108</v>
+      </c>
+      <c r="AB18" s="52"/>
+      <c r="AC18" s="52"/>
+      <c r="AD18" s="31"/>
+      <c r="AE18" s="31"/>
+      <c r="AF18" s="41"/>
+    </row>
+    <row r="19" spans="1:155" s="3" customFormat="1" ht="89.45" customHeight="1">
+      <c r="A19" s="56" t="s">
         <v>125</v>
       </c>
-      <c r="K18" s="4"/>
-      <c r="L18" s="4"/>
-      <c r="M18" s="4"/>
-      <c r="N18" s="4"/>
-      <c r="O18" s="11" t="s">
-        <v>102</v>
-      </c>
-      <c r="P18" s="4"/>
-      <c r="Q18" s="4"/>
-      <c r="R18" s="11" t="s">
-        <v>123</v>
-      </c>
-      <c r="S18" s="4"/>
-      <c r="T18" s="4"/>
-      <c r="U18" s="11" t="s">
-        <v>123</v>
-      </c>
-      <c r="V18" s="4"/>
-      <c r="W18" s="12" t="s">
-        <v>103</v>
-      </c>
-      <c r="X18" s="4"/>
-      <c r="Y18" s="4"/>
-      <c r="Z18" s="4"/>
-      <c r="AA18" s="11" t="s">
-        <v>102</v>
-      </c>
-      <c r="AB18" s="11"/>
-      <c r="AC18" s="11" t="s">
+      <c r="B19" s="85" t="s">
         <v>126</v>
       </c>
-      <c r="AD18" s="10"/>
-      <c r="AE18" s="10"/>
-      <c r="AF18" s="40"/>
+      <c r="C19" s="43"/>
+      <c r="D19" s="43"/>
+      <c r="E19" s="44" t="s">
+        <v>127</v>
+      </c>
+      <c r="F19" s="44" t="s">
+        <v>128</v>
+      </c>
+      <c r="G19" s="44" t="s">
+        <v>129</v>
+      </c>
+      <c r="H19" s="43"/>
+      <c r="I19" s="44" t="s">
+        <v>130</v>
+      </c>
+      <c r="J19" s="43" t="s">
+        <v>131</v>
+      </c>
+      <c r="K19" s="43" t="s">
+        <v>132</v>
+      </c>
+      <c r="L19" s="43" t="s">
+        <v>133</v>
+      </c>
+      <c r="M19" s="43" t="s">
+        <v>134</v>
+      </c>
+      <c r="N19" s="43"/>
+      <c r="O19" s="44" t="s">
+        <v>135</v>
+      </c>
+      <c r="P19" s="44" t="s">
+        <v>136</v>
+      </c>
+      <c r="Q19" s="44" t="s">
+        <v>137</v>
+      </c>
+      <c r="R19" s="57" t="s">
+        <v>138</v>
+      </c>
+      <c r="S19" s="58" t="s">
+        <v>139</v>
+      </c>
+      <c r="T19" s="57"/>
+      <c r="U19" s="58" t="s">
+        <v>140</v>
+      </c>
+      <c r="V19" s="57"/>
+      <c r="W19" s="59" t="s">
+        <v>141</v>
+      </c>
+      <c r="X19" s="57"/>
+      <c r="Y19" s="58" t="s">
+        <v>142</v>
+      </c>
+      <c r="Z19" s="57"/>
+      <c r="AA19" s="58" t="s">
+        <v>143</v>
+      </c>
+      <c r="AB19" s="58" t="s">
+        <v>144</v>
+      </c>
+      <c r="AC19" s="58" t="s">
+        <v>145</v>
+      </c>
+      <c r="AD19" s="57"/>
+      <c r="AE19" s="57"/>
+      <c r="AF19" s="60"/>
     </row>
-    <row r="19" spans="1:155" ht="18" customHeight="1">
-      <c r="A19" s="97"/>
-      <c r="B19" s="115"/>
-      <c r="C19" s="32"/>
-      <c r="D19" s="32"/>
-      <c r="E19" s="32"/>
-      <c r="F19" s="32"/>
-      <c r="G19" s="32"/>
-      <c r="H19" s="32"/>
-      <c r="I19" s="32"/>
-      <c r="J19" s="52" t="s">
-        <v>127</v>
-      </c>
-      <c r="K19" s="32"/>
-      <c r="L19" s="32"/>
-      <c r="M19" s="32"/>
-      <c r="N19" s="32"/>
-      <c r="O19" s="52" t="s">
-        <v>112</v>
-      </c>
-      <c r="P19" s="32"/>
-      <c r="Q19" s="32"/>
-      <c r="R19" s="64" t="s">
-        <v>103</v>
-      </c>
-      <c r="S19" s="32"/>
-      <c r="T19" s="32"/>
-      <c r="U19" s="52" t="s">
-        <v>92</v>
-      </c>
-      <c r="V19" s="32"/>
-      <c r="W19" s="64" t="s">
-        <v>128</v>
-      </c>
-      <c r="X19" s="32"/>
-      <c r="Y19" s="32"/>
-      <c r="Z19" s="32"/>
-      <c r="AA19" s="52" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB19" s="52"/>
-      <c r="AC19" s="52"/>
-      <c r="AD19" s="31"/>
-      <c r="AE19" s="31"/>
-      <c r="AF19" s="41"/>
+    <row r="20" spans="1:155" s="1" customFormat="1" ht="36" customHeight="1">
+      <c r="A20" s="21"/>
+      <c r="B20" s="110" t="s">
+        <v>146</v>
+      </c>
+      <c r="C20" s="22" t="s">
+        <v>147</v>
+      </c>
+      <c r="D20" s="22" t="s">
+        <v>148</v>
+      </c>
+      <c r="E20" s="22" t="s">
+        <v>149</v>
+      </c>
+      <c r="F20" s="22" t="s">
+        <v>150</v>
+      </c>
+      <c r="G20" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="H20" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="I20" s="22" t="s">
+        <v>152</v>
+      </c>
+      <c r="J20" s="22" t="s">
+        <v>153</v>
+      </c>
+      <c r="K20" s="22" t="s">
+        <v>154</v>
+      </c>
+      <c r="L20" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="M20" s="22" t="s">
+        <v>156</v>
+      </c>
+      <c r="N20" s="22" t="s">
+        <v>157</v>
+      </c>
+      <c r="O20" s="22" t="s">
+        <v>158</v>
+      </c>
+      <c r="P20" s="22" t="s">
+        <v>159</v>
+      </c>
+      <c r="Q20" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="R20" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="S20" s="22" t="s">
+        <v>161</v>
+      </c>
+      <c r="T20" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="U20" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="V20" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="W20" s="22" t="s">
+        <v>162</v>
+      </c>
+      <c r="X20" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="Y20" s="22" t="s">
+        <v>163</v>
+      </c>
+      <c r="Z20" s="22" t="s">
+        <v>164</v>
+      </c>
+      <c r="AA20" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="AB20" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="AC20" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="AD20" s="22" t="s">
+        <v>165</v>
+      </c>
+      <c r="AE20" s="22" t="s">
+        <v>166</v>
+      </c>
+      <c r="AF20" s="23" t="s">
+        <v>167</v>
+      </c>
     </row>
-    <row r="20" spans="1:155" s="3" customFormat="1" ht="89.45" customHeight="1">
-      <c r="A20" s="56" t="s">
-        <v>129</v>
-      </c>
-      <c r="B20" s="85" t="s">
-        <v>130</v>
-      </c>
-      <c r="C20" s="43"/>
-      <c r="D20" s="43"/>
-      <c r="E20" s="44" t="s">
-        <v>131</v>
-      </c>
-      <c r="F20" s="44" t="s">
-        <v>132</v>
-      </c>
-      <c r="G20" s="44" t="s">
-        <v>133</v>
-      </c>
-      <c r="H20" s="43"/>
-      <c r="I20" s="44" t="s">
-        <v>134</v>
-      </c>
-      <c r="J20" s="43" t="s">
-        <v>135</v>
-      </c>
-      <c r="K20" s="43" t="s">
-        <v>136</v>
-      </c>
-      <c r="L20" s="43" t="s">
-        <v>137</v>
-      </c>
-      <c r="M20" s="43" t="s">
-        <v>138</v>
-      </c>
-      <c r="N20" s="43"/>
-      <c r="O20" s="44" t="s">
-        <v>139</v>
-      </c>
-      <c r="P20" s="44" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q20" s="44" t="s">
-        <v>141</v>
-      </c>
-      <c r="R20" s="57" t="s">
-        <v>142</v>
-      </c>
-      <c r="S20" s="58" t="s">
-        <v>143</v>
-      </c>
-      <c r="T20" s="57"/>
-      <c r="U20" s="58" t="s">
-        <v>144</v>
-      </c>
-      <c r="V20" s="57"/>
-      <c r="W20" s="59" t="s">
-        <v>145</v>
-      </c>
-      <c r="X20" s="57"/>
-      <c r="Y20" s="58" t="s">
-        <v>146</v>
-      </c>
-      <c r="Z20" s="57"/>
-      <c r="AA20" s="58" t="s">
-        <v>147</v>
-      </c>
-      <c r="AB20" s="58" t="s">
-        <v>148</v>
-      </c>
-      <c r="AC20" s="58" t="s">
-        <v>149</v>
-      </c>
-      <c r="AD20" s="57"/>
-      <c r="AE20" s="57"/>
-      <c r="AF20" s="60"/>
-    </row>
-    <row r="21" spans="1:155" s="1" customFormat="1" ht="36" customHeight="1">
-      <c r="A21" s="21"/>
-      <c r="B21" s="110" t="s">
-        <v>150</v>
-      </c>
-      <c r="C21" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="D21" s="22" t="s">
-        <v>152</v>
-      </c>
-      <c r="E21" s="22" t="s">
-        <v>153</v>
-      </c>
-      <c r="F21" s="22" t="s">
-        <v>154</v>
-      </c>
-      <c r="G21" s="22" t="s">
-        <v>155</v>
-      </c>
-      <c r="H21" s="22" t="s">
-        <v>155</v>
-      </c>
-      <c r="I21" s="22" t="s">
-        <v>156</v>
-      </c>
-      <c r="J21" s="22" t="s">
-        <v>157</v>
-      </c>
-      <c r="K21" s="22" t="s">
-        <v>158</v>
-      </c>
-      <c r="L21" s="22" t="s">
-        <v>159</v>
-      </c>
-      <c r="M21" s="22" t="s">
-        <v>160</v>
-      </c>
-      <c r="N21" s="22" t="s">
-        <v>161</v>
-      </c>
-      <c r="O21" s="22" t="s">
-        <v>162</v>
-      </c>
-      <c r="P21" s="22" t="s">
-        <v>163</v>
-      </c>
-      <c r="Q21" s="22" t="s">
-        <v>164</v>
-      </c>
-      <c r="R21" s="22" t="s">
-        <v>155</v>
-      </c>
-      <c r="S21" s="22" t="s">
-        <v>165</v>
-      </c>
-      <c r="T21" s="22" t="s">
-        <v>155</v>
-      </c>
-      <c r="U21" s="22" t="s">
-        <v>155</v>
-      </c>
-      <c r="V21" s="22" t="s">
-        <v>155</v>
-      </c>
-      <c r="W21" s="22" t="s">
-        <v>166</v>
-      </c>
-      <c r="X21" s="22" t="s">
-        <v>155</v>
-      </c>
-      <c r="Y21" s="22" t="s">
-        <v>167</v>
-      </c>
-      <c r="Z21" s="22" t="s">
+    <row r="21" spans="1:155" ht="18" customHeight="1">
+      <c r="A21" s="24"/>
+      <c r="B21" s="111"/>
+      <c r="C21" s="25" t="s">
         <v>168</v>
       </c>
-      <c r="AA21" s="22" t="s">
-        <v>155</v>
-      </c>
-      <c r="AB21" s="22" t="s">
-        <v>155</v>
-      </c>
-      <c r="AC21" s="22" t="s">
-        <v>155</v>
-      </c>
-      <c r="AD21" s="22" t="s">
+      <c r="D21" s="25" t="s">
         <v>169</v>
       </c>
-      <c r="AE21" s="22" t="s">
+      <c r="E21" s="25" t="s">
         <v>170</v>
       </c>
-      <c r="AF21" s="23" t="s">
+      <c r="F21" s="25" t="s">
         <v>171</v>
+      </c>
+      <c r="G21" s="4"/>
+      <c r="H21" s="4"/>
+      <c r="I21" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="J21" s="13" t="s">
+        <v>173</v>
+      </c>
+      <c r="K21" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="L21" s="14"/>
+      <c r="M21" s="13" t="s">
+        <v>175</v>
+      </c>
+      <c r="N21" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="O21" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="P21" s="13" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q21" s="13" t="s">
+        <v>179</v>
+      </c>
+      <c r="R21" s="14"/>
+      <c r="S21" s="13" t="s">
+        <v>179</v>
+      </c>
+      <c r="T21" s="14"/>
+      <c r="U21" s="4"/>
+      <c r="V21" s="4"/>
+      <c r="W21" s="13" t="s">
+        <v>180</v>
+      </c>
+      <c r="X21" s="4"/>
+      <c r="Y21" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="Z21" s="13" t="s">
+        <v>182</v>
+      </c>
+      <c r="AA21" s="4"/>
+      <c r="AB21" s="4"/>
+      <c r="AC21" s="4"/>
+      <c r="AD21" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="AE21" s="13" t="s">
+        <v>184</v>
+      </c>
+      <c r="AF21" s="26" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="22" spans="1:155" ht="18" customHeight="1">
       <c r="A22" s="24"/>
       <c r="B22" s="111"/>
       <c r="C22" s="25" t="s">
-        <v>172</v>
+        <v>186</v>
       </c>
       <c r="D22" s="25" t="s">
-        <v>173</v>
+        <v>187</v>
       </c>
       <c r="E22" s="25" t="s">
-        <v>174</v>
-      </c>
-      <c r="F22" s="25" t="s">
-        <v>175</v>
-      </c>
+        <v>188</v>
+      </c>
+      <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
-      <c r="I22" s="13" t="s">
+      <c r="I22" s="14"/>
+      <c r="J22" s="13" t="s">
+        <v>189</v>
+      </c>
+      <c r="K22" s="14"/>
+      <c r="L22" s="13" t="s">
+        <v>190</v>
+      </c>
+      <c r="M22" s="13" t="s">
         <v>176</v>
       </c>
-      <c r="J22" s="13" t="s">
-        <v>177</v>
-      </c>
-      <c r="K22" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="L22" s="14"/>
-      <c r="M22" s="13" t="s">
-        <v>179</v>
-      </c>
       <c r="N22" s="13" t="s">
-        <v>180</v>
+        <v>191</v>
       </c>
       <c r="O22" s="13" t="s">
-        <v>181</v>
+        <v>192</v>
       </c>
       <c r="P22" s="13" t="s">
-        <v>182</v>
+        <v>193</v>
       </c>
       <c r="Q22" s="13" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="R22" s="14"/>
       <c r="S22" s="13" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="T22" s="14"/>
       <c r="U22" s="4"/>
       <c r="V22" s="4"/>
       <c r="W22" s="13" t="s">
-        <v>184</v>
+        <v>195</v>
       </c>
       <c r="X22" s="4"/>
       <c r="Y22" s="13" t="s">
-        <v>185</v>
-      </c>
-      <c r="Z22" s="13" t="s">
-        <v>186</v>
-      </c>
+        <v>196</v>
+      </c>
+      <c r="Z22" s="13"/>
       <c r="AA22" s="4"/>
       <c r="AB22" s="4"/>
       <c r="AC22" s="4"/>
       <c r="AD22" s="13" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
       <c r="AE22" s="13" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
       <c r="AF22" s="26" t="s">
-        <v>189</v>
+        <v>199</v>
       </c>
     </row>
     <row r="23" spans="1:155" ht="18" customHeight="1">
       <c r="A23" s="24"/>
       <c r="B23" s="111"/>
       <c r="C23" s="25" t="s">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="D23" s="25" t="s">
-        <v>191</v>
-      </c>
-      <c r="E23" s="25" t="s">
-        <v>192</v>
-      </c>
+        <v>201</v>
+      </c>
+      <c r="E23" s="4"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
       <c r="I23" s="14"/>
       <c r="J23" s="13" t="s">
-        <v>193</v>
+        <v>176</v>
       </c>
       <c r="K23" s="14"/>
       <c r="L23" s="13" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="M23" s="13" t="s">
-        <v>180</v>
+        <v>191</v>
       </c>
       <c r="N23" s="13" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="O23" s="13" t="s">
-        <v>196</v>
-      </c>
-      <c r="P23" s="13" t="s">
-        <v>197</v>
-      </c>
+        <v>204</v>
+      </c>
+      <c r="P23" s="14"/>
       <c r="Q23" s="13" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="R23" s="14"/>
       <c r="S23" s="13" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="T23" s="14"/>
       <c r="U23" s="4"/>
       <c r="V23" s="4"/>
       <c r="W23" s="13" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="X23" s="4"/>
       <c r="Y23" s="13" t="s">
-        <v>200</v>
-      </c>
-      <c r="Z23" s="13"/>
+        <v>189</v>
+      </c>
+      <c r="Z23" s="14"/>
       <c r="AA23" s="4"/>
       <c r="AB23" s="4"/>
       <c r="AC23" s="4"/>
       <c r="AD23" s="13" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="AE23" s="13" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="AF23" s="26" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
     </row>
     <row r="24" spans="1:155" ht="18" customHeight="1">
       <c r="A24" s="24"/>
       <c r="B24" s="111"/>
-      <c r="C24" s="25" t="s">
-        <v>204</v>
-      </c>
-      <c r="D24" s="25" t="s">
-        <v>205</v>
-      </c>
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
       <c r="I24" s="14"/>
       <c r="J24" s="13" t="s">
-        <v>180</v>
+        <v>191</v>
       </c>
       <c r="K24" s="14"/>
       <c r="L24" s="13" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="M24" s="13" t="s">
-        <v>195</v>
+        <v>210</v>
       </c>
       <c r="N24" s="13" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="O24" s="13" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="P24" s="14"/>
       <c r="Q24" s="13" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="R24" s="14"/>
       <c r="S24" s="13" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="T24" s="14"/>
       <c r="U24" s="4"/>
       <c r="V24" s="4"/>
       <c r="W24" s="13" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="X24" s="4"/>
       <c r="Y24" s="13" t="s">
-        <v>193</v>
+        <v>176</v>
       </c>
       <c r="Z24" s="14"/>
       <c r="AA24" s="4"/>
       <c r="AB24" s="4"/>
       <c r="AC24" s="4"/>
       <c r="AD24" s="13" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="AE24" s="13" t="s">
-        <v>211</v>
-      </c>
-      <c r="AF24" s="26" t="s">
-        <v>212</v>
-      </c>
+        <v>214</v>
+      </c>
+      <c r="AF24" s="27"/>
     </row>
     <row r="25" spans="1:155" ht="18" customHeight="1">
       <c r="A25" s="24"/>
@@ -3743,45 +3710,41 @@
       <c r="H25" s="4"/>
       <c r="I25" s="14"/>
       <c r="J25" s="13" t="s">
-        <v>195</v>
+        <v>210</v>
       </c>
       <c r="K25" s="14"/>
       <c r="L25" s="13" t="s">
-        <v>213</v>
-      </c>
-      <c r="M25" s="13" t="s">
-        <v>214</v>
-      </c>
-      <c r="N25" s="13" t="s">
-        <v>214</v>
-      </c>
+        <v>215</v>
+      </c>
+      <c r="M25" s="14"/>
+      <c r="N25" s="14"/>
       <c r="O25" s="13" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="P25" s="14"/>
       <c r="Q25" s="13" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="R25" s="14"/>
       <c r="S25" s="13" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="T25" s="14"/>
       <c r="U25" s="4"/>
       <c r="V25" s="4"/>
       <c r="W25" s="13" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="X25" s="4"/>
       <c r="Y25" s="13" t="s">
-        <v>180</v>
+        <v>191</v>
       </c>
       <c r="Z25" s="14"/>
       <c r="AA25" s="4"/>
       <c r="AB25" s="4"/>
       <c r="AC25" s="4"/>
       <c r="AD25" s="13" t="s">
-        <v>217</v>
+        <v>168</v>
       </c>
       <c r="AE25" s="13" t="s">
         <v>218</v>
@@ -3789,142 +3752,289 @@
       <c r="AF25" s="27"/>
     </row>
     <row r="26" spans="1:155" ht="18" customHeight="1">
-      <c r="A26" s="24"/>
+      <c r="A26" s="28"/>
       <c r="B26" s="111"/>
-      <c r="C26" s="4"/>
-      <c r="D26" s="4"/>
-      <c r="E26" s="4"/>
-      <c r="F26" s="4"/>
-      <c r="G26" s="4"/>
-      <c r="H26" s="4"/>
-      <c r="I26" s="14"/>
-      <c r="J26" s="13" t="s">
-        <v>214</v>
-      </c>
-      <c r="K26" s="14"/>
-      <c r="L26" s="13" t="s">
+      <c r="C26" s="6"/>
+      <c r="D26" s="6"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="6"/>
+      <c r="G26" s="6"/>
+      <c r="H26" s="6"/>
+      <c r="I26" s="17"/>
+      <c r="J26" s="18" t="s">
+        <v>203</v>
+      </c>
+      <c r="K26" s="17"/>
+      <c r="L26" s="18" t="s">
         <v>219</v>
       </c>
-      <c r="M26" s="14"/>
-      <c r="N26" s="14"/>
-      <c r="O26" s="13" t="s">
+      <c r="M26" s="17"/>
+      <c r="N26" s="17"/>
+      <c r="O26" s="18" t="s">
         <v>220</v>
       </c>
-      <c r="P26" s="14"/>
-      <c r="Q26" s="13" t="s">
-        <v>220</v>
-      </c>
-      <c r="R26" s="14"/>
-      <c r="S26" s="13" t="s">
-        <v>220</v>
-      </c>
-      <c r="T26" s="14"/>
-      <c r="U26" s="4"/>
-      <c r="V26" s="4"/>
-      <c r="W26" s="13" t="s">
+      <c r="P26" s="17"/>
+      <c r="Q26" s="18" t="s">
         <v>221</v>
       </c>
-      <c r="X26" s="4"/>
-      <c r="Y26" s="13" t="s">
-        <v>195</v>
-      </c>
-      <c r="Z26" s="14"/>
-      <c r="AA26" s="4"/>
-      <c r="AB26" s="4"/>
-      <c r="AC26" s="4"/>
-      <c r="AD26" s="13" t="s">
-        <v>172</v>
-      </c>
-      <c r="AE26" s="13" t="s">
+      <c r="R26" s="17"/>
+      <c r="S26" s="18" t="s">
+        <v>221</v>
+      </c>
+      <c r="T26" s="17"/>
+      <c r="U26" s="6"/>
+      <c r="V26" s="6"/>
+      <c r="W26" s="6"/>
+      <c r="X26" s="6"/>
+      <c r="Y26" s="18" t="s">
+        <v>203</v>
+      </c>
+      <c r="Z26" s="17"/>
+      <c r="AA26" s="6"/>
+      <c r="AB26" s="6"/>
+      <c r="AC26" s="6"/>
+      <c r="AD26" s="18" t="s">
+        <v>186</v>
+      </c>
+      <c r="AE26" s="17"/>
+      <c r="AF26" s="29"/>
+    </row>
+    <row r="27" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1">
+      <c r="A27" s="30"/>
+      <c r="B27" s="112"/>
+      <c r="C27" s="32"/>
+      <c r="D27" s="32"/>
+      <c r="E27" s="32"/>
+      <c r="F27" s="32"/>
+      <c r="G27" s="32"/>
+      <c r="H27" s="32"/>
+      <c r="I27" s="32"/>
+      <c r="J27" s="32"/>
+      <c r="K27" s="32"/>
+      <c r="L27" s="32"/>
+      <c r="M27" s="32"/>
+      <c r="N27" s="32"/>
+      <c r="O27" s="32"/>
+      <c r="P27" s="32"/>
+      <c r="Q27" s="32"/>
+      <c r="R27" s="32"/>
+      <c r="S27" s="32"/>
+      <c r="T27" s="32"/>
+      <c r="U27" s="32"/>
+      <c r="V27" s="32"/>
+      <c r="W27" s="32"/>
+      <c r="X27" s="32"/>
+      <c r="Y27" s="33" t="s">
+        <v>174</v>
+      </c>
+      <c r="Z27" s="34"/>
+      <c r="AA27" s="32"/>
+      <c r="AB27" s="32"/>
+      <c r="AC27" s="32"/>
+      <c r="AD27" s="33" t="s">
+        <v>174</v>
+      </c>
+      <c r="AE27" s="34"/>
+      <c r="AF27" s="35"/>
+      <c r="AG27" s="2"/>
+      <c r="AH27" s="2"/>
+      <c r="AI27" s="2"/>
+      <c r="AJ27" s="2"/>
+      <c r="AK27" s="2"/>
+      <c r="AL27" s="2"/>
+      <c r="AM27" s="2"/>
+      <c r="AN27" s="2"/>
+      <c r="AO27" s="2"/>
+      <c r="AP27" s="2"/>
+      <c r="AQ27" s="2"/>
+      <c r="AR27" s="2"/>
+      <c r="AS27" s="2"/>
+      <c r="AT27" s="2"/>
+      <c r="AU27" s="2"/>
+      <c r="AV27" s="2"/>
+      <c r="AW27" s="2"/>
+      <c r="AX27" s="2"/>
+      <c r="AY27" s="2"/>
+      <c r="AZ27" s="2"/>
+      <c r="BA27" s="2"/>
+      <c r="BB27" s="2"/>
+      <c r="BC27" s="2"/>
+      <c r="BD27" s="2"/>
+      <c r="BE27" s="2"/>
+      <c r="BF27" s="2"/>
+      <c r="BG27" s="2"/>
+      <c r="BH27" s="2"/>
+      <c r="BI27" s="2"/>
+      <c r="BJ27" s="2"/>
+      <c r="BK27" s="2"/>
+      <c r="BL27" s="2"/>
+      <c r="BM27" s="2"/>
+      <c r="BN27" s="2"/>
+      <c r="BO27" s="2"/>
+      <c r="BP27" s="2"/>
+      <c r="BQ27" s="2"/>
+      <c r="BR27" s="2"/>
+      <c r="BS27" s="2"/>
+      <c r="BT27" s="2"/>
+      <c r="BU27" s="2"/>
+      <c r="BV27" s="2"/>
+      <c r="BW27" s="2"/>
+      <c r="BX27" s="2"/>
+      <c r="BY27" s="2"/>
+      <c r="BZ27" s="2"/>
+      <c r="CA27" s="2"/>
+      <c r="CB27" s="2"/>
+      <c r="CC27" s="2"/>
+      <c r="CD27" s="2"/>
+      <c r="CE27" s="2"/>
+      <c r="CF27" s="2"/>
+      <c r="CG27" s="2"/>
+      <c r="CH27" s="2"/>
+      <c r="CI27" s="2"/>
+      <c r="CJ27" s="2"/>
+      <c r="CK27" s="2"/>
+      <c r="CL27" s="2"/>
+      <c r="CM27" s="2"/>
+      <c r="CN27" s="2"/>
+      <c r="CO27" s="2"/>
+      <c r="CP27" s="2"/>
+      <c r="CQ27" s="2"/>
+      <c r="CR27" s="2"/>
+      <c r="CS27" s="2"/>
+      <c r="CT27" s="2"/>
+      <c r="CU27" s="2"/>
+      <c r="CV27" s="2"/>
+      <c r="CW27" s="2"/>
+      <c r="CX27" s="2"/>
+      <c r="CY27" s="2"/>
+      <c r="CZ27" s="2"/>
+      <c r="DA27" s="2"/>
+      <c r="DB27" s="2"/>
+      <c r="DC27" s="2"/>
+      <c r="DD27" s="2"/>
+      <c r="DE27" s="2"/>
+      <c r="DF27" s="2"/>
+      <c r="DG27" s="2"/>
+      <c r="DH27" s="2"/>
+      <c r="DI27" s="2"/>
+      <c r="DJ27" s="2"/>
+      <c r="DK27" s="2"/>
+      <c r="DL27" s="2"/>
+      <c r="DM27" s="2"/>
+      <c r="DN27" s="2"/>
+      <c r="DO27" s="2"/>
+      <c r="DP27" s="2"/>
+      <c r="DQ27" s="2"/>
+      <c r="DR27" s="2"/>
+      <c r="DS27" s="2"/>
+      <c r="DT27" s="2"/>
+      <c r="DU27" s="2"/>
+      <c r="DV27" s="2"/>
+      <c r="DW27" s="2"/>
+      <c r="DX27" s="2"/>
+      <c r="DY27" s="2"/>
+      <c r="DZ27" s="2"/>
+      <c r="EA27" s="2"/>
+      <c r="EB27" s="2"/>
+      <c r="EC27" s="2"/>
+      <c r="ED27" s="2"/>
+      <c r="EE27" s="2"/>
+      <c r="EF27" s="2"/>
+      <c r="EG27" s="2"/>
+      <c r="EH27" s="2"/>
+      <c r="EI27" s="2"/>
+      <c r="EJ27" s="2"/>
+      <c r="EK27" s="2"/>
+      <c r="EL27" s="2"/>
+      <c r="EM27" s="2"/>
+      <c r="EN27" s="2"/>
+      <c r="EO27" s="2"/>
+      <c r="EP27" s="2"/>
+      <c r="EQ27" s="2"/>
+      <c r="ER27" s="2"/>
+      <c r="ES27" s="2"/>
+      <c r="ET27" s="2"/>
+      <c r="EU27" s="2"/>
+      <c r="EV27" s="2"/>
+      <c r="EW27" s="2"/>
+      <c r="EX27" s="2"/>
+      <c r="EY27" s="2"/>
+    </row>
+    <row r="28" spans="1:155" s="10" customFormat="1" ht="36" customHeight="1">
+      <c r="A28" s="21"/>
+      <c r="B28" s="117" t="s">
         <v>222</v>
       </c>
-      <c r="AF26" s="27"/>
-    </row>
-    <row r="27" spans="1:155" ht="18" customHeight="1">
-      <c r="A27" s="28"/>
-      <c r="B27" s="111"/>
-      <c r="C27" s="6"/>
-      <c r="D27" s="6"/>
-      <c r="E27" s="6"/>
-      <c r="F27" s="6"/>
-      <c r="G27" s="6"/>
-      <c r="H27" s="6"/>
-      <c r="I27" s="17"/>
-      <c r="J27" s="18" t="s">
-        <v>207</v>
-      </c>
-      <c r="K27" s="17"/>
-      <c r="L27" s="18" t="s">
+      <c r="C28" s="36" t="s">
         <v>223</v>
       </c>
-      <c r="M27" s="17"/>
-      <c r="N27" s="17"/>
-      <c r="O27" s="18" t="s">
+      <c r="D28" s="36" t="s">
+        <v>223</v>
+      </c>
+      <c r="E28" s="36" t="s">
         <v>224</v>
       </c>
-      <c r="P27" s="17"/>
-      <c r="Q27" s="18" t="s">
+      <c r="F28" s="36" t="s">
         <v>225</v>
       </c>
-      <c r="R27" s="17"/>
-      <c r="S27" s="18" t="s">
-        <v>225</v>
-      </c>
-      <c r="T27" s="17"/>
-      <c r="U27" s="6"/>
-      <c r="V27" s="6"/>
-      <c r="W27" s="6"/>
-      <c r="X27" s="6"/>
-      <c r="Y27" s="18" t="s">
-        <v>207</v>
-      </c>
-      <c r="Z27" s="17"/>
-      <c r="AA27" s="6"/>
-      <c r="AB27" s="6"/>
-      <c r="AC27" s="6"/>
-      <c r="AD27" s="18" t="s">
-        <v>190</v>
-      </c>
-      <c r="AE27" s="17"/>
-      <c r="AF27" s="29"/>
-    </row>
-    <row r="28" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1">
-      <c r="A28" s="30"/>
-      <c r="B28" s="112"/>
-      <c r="C28" s="32"/>
-      <c r="D28" s="32"/>
-      <c r="E28" s="32"/>
-      <c r="F28" s="32"/>
-      <c r="G28" s="32"/>
-      <c r="H28" s="32"/>
-      <c r="I28" s="32"/>
-      <c r="J28" s="32"/>
-      <c r="K28" s="32"/>
-      <c r="L28" s="32"/>
-      <c r="M28" s="32"/>
-      <c r="N28" s="32"/>
-      <c r="O28" s="32"/>
-      <c r="P28" s="32"/>
-      <c r="Q28" s="32"/>
-      <c r="R28" s="32"/>
-      <c r="S28" s="32"/>
-      <c r="T28" s="32"/>
-      <c r="U28" s="32"/>
-      <c r="V28" s="32"/>
-      <c r="W28" s="32"/>
-      <c r="X28" s="32"/>
-      <c r="Y28" s="33" t="s">
-        <v>178</v>
-      </c>
-      <c r="Z28" s="34"/>
-      <c r="AA28" s="32"/>
-      <c r="AB28" s="32"/>
-      <c r="AC28" s="32"/>
-      <c r="AD28" s="33" t="s">
-        <v>178</v>
-      </c>
-      <c r="AE28" s="34"/>
-      <c r="AF28" s="35"/>
+      <c r="G28" s="36" t="s">
+        <v>226</v>
+      </c>
+      <c r="H28" s="37"/>
+      <c r="I28" s="36" t="s">
+        <v>227</v>
+      </c>
+      <c r="J28" s="36" t="s">
+        <v>228</v>
+      </c>
+      <c r="K28" s="36" t="s">
+        <v>229</v>
+      </c>
+      <c r="L28" s="36" t="s">
+        <v>230</v>
+      </c>
+      <c r="M28" s="36" t="s">
+        <v>231</v>
+      </c>
+      <c r="N28" s="36" t="s">
+        <v>232</v>
+      </c>
+      <c r="O28" s="36" t="s">
+        <v>233</v>
+      </c>
+      <c r="P28" s="36" t="s">
+        <v>234</v>
+      </c>
+      <c r="Q28" s="36" t="s">
+        <v>235</v>
+      </c>
+      <c r="R28" s="36" t="s">
+        <v>227</v>
+      </c>
+      <c r="S28" s="36" t="s">
+        <v>233</v>
+      </c>
+      <c r="T28" s="37"/>
+      <c r="U28" s="36" t="s">
+        <v>233</v>
+      </c>
+      <c r="V28" s="37"/>
+      <c r="W28" s="36" t="s">
+        <v>236</v>
+      </c>
+      <c r="X28" s="37"/>
+      <c r="Y28" s="37"/>
+      <c r="Z28" s="36" t="s">
+        <v>237</v>
+      </c>
+      <c r="AA28" s="37" t="s">
+        <v>238</v>
+      </c>
+      <c r="AB28" s="37"/>
+      <c r="AC28" s="37"/>
+      <c r="AD28" s="38"/>
+      <c r="AE28" s="38"/>
+      <c r="AF28" s="39"/>
       <c r="AG28" s="2"/>
       <c r="AH28" s="2"/>
       <c r="AI28" s="2"/>
@@ -4049,81 +4159,69 @@
       <c r="EX28" s="2"/>
       <c r="EY28" s="2"/>
     </row>
-    <row r="29" spans="1:155" s="10" customFormat="1" ht="36" customHeight="1">
-      <c r="A29" s="21"/>
-      <c r="B29" s="117" t="s">
-        <v>226</v>
-      </c>
-      <c r="C29" s="36" t="s">
-        <v>227</v>
-      </c>
-      <c r="D29" s="36" t="s">
-        <v>227</v>
-      </c>
-      <c r="E29" s="36" t="s">
-        <v>38</v>
-      </c>
-      <c r="F29" s="36" t="s">
-        <v>228</v>
-      </c>
-      <c r="G29" s="36" t="s">
-        <v>229</v>
-      </c>
-      <c r="H29" s="37"/>
-      <c r="I29" s="36" t="s">
-        <v>230</v>
-      </c>
-      <c r="J29" s="36" t="s">
-        <v>231</v>
-      </c>
-      <c r="K29" s="36" t="s">
-        <v>232</v>
-      </c>
-      <c r="L29" s="36" t="s">
-        <v>233</v>
-      </c>
-      <c r="M29" s="36" t="s">
-        <v>234</v>
-      </c>
-      <c r="N29" s="36" t="s">
-        <v>235</v>
-      </c>
-      <c r="O29" s="36" t="s">
-        <v>236</v>
-      </c>
-      <c r="P29" s="36" t="s">
-        <v>237</v>
-      </c>
-      <c r="Q29" s="36" t="s">
-        <v>238</v>
-      </c>
-      <c r="R29" s="36" t="s">
-        <v>230</v>
-      </c>
-      <c r="S29" s="36" t="s">
-        <v>236</v>
-      </c>
-      <c r="T29" s="37"/>
-      <c r="U29" s="36" t="s">
-        <v>236</v>
-      </c>
-      <c r="V29" s="37"/>
-      <c r="W29" s="36" t="s">
+    <row r="29" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1">
+      <c r="A29" s="24"/>
+      <c r="B29" s="118"/>
+      <c r="C29" s="13" t="s">
         <v>239</v>
       </c>
-      <c r="X29" s="37"/>
-      <c r="Y29" s="37"/>
-      <c r="Z29" s="36" t="s">
+      <c r="D29" s="13" t="s">
+        <v>239</v>
+      </c>
+      <c r="E29" s="4"/>
+      <c r="F29" s="13" t="s">
         <v>240</v>
       </c>
-      <c r="AA29" s="37" t="s">
+      <c r="G29" s="13" t="s">
+        <v>239</v>
+      </c>
+      <c r="H29" s="4"/>
+      <c r="I29" s="4"/>
+      <c r="J29" s="13" t="s">
         <v>241</v>
       </c>
-      <c r="AB29" s="37"/>
-      <c r="AC29" s="37"/>
-      <c r="AD29" s="38"/>
-      <c r="AE29" s="38"/>
-      <c r="AF29" s="39"/>
+      <c r="K29" s="13" t="s">
+        <v>242</v>
+      </c>
+      <c r="L29" s="13" t="s">
+        <v>243</v>
+      </c>
+      <c r="M29" s="13" t="s">
+        <v>244</v>
+      </c>
+      <c r="N29" s="13" t="s">
+        <v>245</v>
+      </c>
+      <c r="O29" s="13" t="s">
+        <v>246</v>
+      </c>
+      <c r="P29" s="13" t="s">
+        <v>247</v>
+      </c>
+      <c r="Q29" s="13" t="s">
+        <v>248</v>
+      </c>
+      <c r="R29" s="14"/>
+      <c r="S29" s="13" t="s">
+        <v>246</v>
+      </c>
+      <c r="T29" s="4"/>
+      <c r="U29" s="13" t="s">
+        <v>246</v>
+      </c>
+      <c r="V29" s="4"/>
+      <c r="W29" s="13" t="s">
+        <v>249</v>
+      </c>
+      <c r="X29" s="4"/>
+      <c r="Y29" s="4"/>
+      <c r="Z29" s="13" t="s">
+        <v>250</v>
+      </c>
+      <c r="AA29" s="4"/>
+      <c r="AB29" s="4"/>
+      <c r="AC29" s="4"/>
+      <c r="AF29" s="40"/>
       <c r="AG29" s="2"/>
       <c r="AH29" s="2"/>
       <c r="AI29" s="2"/>
@@ -4252,61 +4350,55 @@
       <c r="A30" s="24"/>
       <c r="B30" s="118"/>
       <c r="C30" s="13" t="s">
-        <v>242</v>
+        <v>251</v>
       </c>
       <c r="D30" s="13" t="s">
-        <v>242</v>
+        <v>251</v>
       </c>
       <c r="E30" s="4"/>
       <c r="F30" s="13" t="s">
-        <v>243</v>
+        <v>252</v>
       </c>
       <c r="G30" s="13" t="s">
-        <v>242</v>
+        <v>251</v>
       </c>
       <c r="H30" s="4"/>
       <c r="I30" s="4"/>
       <c r="J30" s="13" t="s">
-        <v>244</v>
+        <v>253</v>
       </c>
       <c r="K30" s="13" t="s">
-        <v>245</v>
+        <v>254</v>
       </c>
       <c r="L30" s="13" t="s">
-        <v>246</v>
-      </c>
-      <c r="M30" s="13" t="s">
-        <v>247</v>
-      </c>
+        <v>255</v>
+      </c>
+      <c r="M30" s="14"/>
       <c r="N30" s="13" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="O30" s="13" t="s">
-        <v>249</v>
-      </c>
-      <c r="P30" s="13" t="s">
-        <v>250</v>
-      </c>
+        <v>257</v>
+      </c>
+      <c r="P30" s="14"/>
       <c r="Q30" s="13" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="R30" s="14"/>
       <c r="S30" s="13" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="T30" s="4"/>
       <c r="U30" s="13" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="V30" s="4"/>
       <c r="W30" s="13" t="s">
-        <v>252</v>
+        <v>259</v>
       </c>
       <c r="X30" s="4"/>
       <c r="Y30" s="4"/>
-      <c r="Z30" s="13" t="s">
-        <v>253</v>
-      </c>
+      <c r="Z30" s="14"/>
       <c r="AA30" s="4"/>
       <c r="AB30" s="4"/>
       <c r="AC30" s="4"/>
@@ -4439,47 +4531,35 @@
       <c r="A31" s="24"/>
       <c r="B31" s="118"/>
       <c r="C31" s="13" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="D31" s="13" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="E31" s="4"/>
-      <c r="F31" s="13" t="s">
-        <v>255</v>
-      </c>
+      <c r="F31" s="4"/>
       <c r="G31" s="13" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="H31" s="4"/>
       <c r="I31" s="4"/>
-      <c r="J31" s="13" t="s">
-        <v>256</v>
-      </c>
-      <c r="K31" s="13" t="s">
-        <v>257</v>
-      </c>
-      <c r="L31" s="13" t="s">
-        <v>258</v>
-      </c>
+      <c r="J31" s="14"/>
+      <c r="K31" s="14"/>
+      <c r="L31" s="14"/>
       <c r="M31" s="14"/>
-      <c r="N31" s="13" t="s">
-        <v>259</v>
-      </c>
+      <c r="N31" s="14"/>
       <c r="O31" s="13" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="P31" s="14"/>
-      <c r="Q31" s="13" t="s">
-        <v>261</v>
-      </c>
+      <c r="Q31" s="14"/>
       <c r="R31" s="14"/>
       <c r="S31" s="13" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="T31" s="4"/>
       <c r="U31" s="13" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="V31" s="4"/>
       <c r="W31" s="13" t="s">
@@ -4487,7 +4567,7 @@
       </c>
       <c r="X31" s="4"/>
       <c r="Y31" s="4"/>
-      <c r="Z31" s="14"/>
+      <c r="Z31" s="4"/>
       <c r="AA31" s="4"/>
       <c r="AB31" s="4"/>
       <c r="AC31" s="4"/>
@@ -4786,50 +4866,44 @@
       <c r="EY32" s="2"/>
     </row>
     <row r="33" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1">
-      <c r="A33" s="24"/>
-      <c r="B33" s="118"/>
-      <c r="C33" s="13" t="s">
+      <c r="A33" s="30"/>
+      <c r="B33" s="119"/>
+      <c r="C33" s="33" t="s">
         <v>266</v>
       </c>
-      <c r="D33" s="13" t="s">
+      <c r="D33" s="33" t="s">
         <v>266</v>
       </c>
-      <c r="E33" s="4"/>
-      <c r="F33" s="4"/>
-      <c r="G33" s="13" t="s">
+      <c r="E33" s="32"/>
+      <c r="F33" s="32"/>
+      <c r="G33" s="33" t="s">
         <v>266</v>
       </c>
-      <c r="H33" s="4"/>
-      <c r="I33" s="4"/>
-      <c r="J33" s="14"/>
-      <c r="K33" s="14"/>
-      <c r="L33" s="14"/>
-      <c r="M33" s="14"/>
-      <c r="N33" s="14"/>
-      <c r="O33" s="13" t="s">
-        <v>267</v>
-      </c>
-      <c r="P33" s="14"/>
-      <c r="Q33" s="14"/>
-      <c r="R33" s="14"/>
-      <c r="S33" s="13" t="s">
-        <v>267</v>
-      </c>
-      <c r="T33" s="4"/>
-      <c r="U33" s="13" t="s">
-        <v>267</v>
-      </c>
-      <c r="V33" s="4"/>
-      <c r="W33" s="13" t="s">
-        <v>268</v>
-      </c>
-      <c r="X33" s="4"/>
-      <c r="Y33" s="4"/>
-      <c r="Z33" s="4"/>
-      <c r="AA33" s="4"/>
-      <c r="AB33" s="4"/>
-      <c r="AC33" s="4"/>
-      <c r="AF33" s="40"/>
+      <c r="H33" s="32"/>
+      <c r="I33" s="32"/>
+      <c r="J33" s="34"/>
+      <c r="K33" s="34"/>
+      <c r="L33" s="34"/>
+      <c r="M33" s="34"/>
+      <c r="N33" s="34"/>
+      <c r="O33" s="34"/>
+      <c r="P33" s="34"/>
+      <c r="Q33" s="34"/>
+      <c r="R33" s="34"/>
+      <c r="S33" s="34"/>
+      <c r="T33" s="32"/>
+      <c r="U33" s="34"/>
+      <c r="V33" s="32"/>
+      <c r="W33" s="34"/>
+      <c r="X33" s="32"/>
+      <c r="Y33" s="32"/>
+      <c r="Z33" s="32"/>
+      <c r="AA33" s="32"/>
+      <c r="AB33" s="32"/>
+      <c r="AC33" s="32"/>
+      <c r="AD33" s="31"/>
+      <c r="AE33" s="31"/>
+      <c r="AF33" s="41"/>
       <c r="AG33" s="2"/>
       <c r="AH33" s="2"/>
       <c r="AI33" s="2"/>
@@ -4954,395 +5028,280 @@
       <c r="EX33" s="2"/>
       <c r="EY33" s="2"/>
     </row>
-    <row r="34" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1">
-      <c r="A34" s="30"/>
-      <c r="B34" s="119"/>
-      <c r="C34" s="33" t="s">
+    <row r="34" spans="1:155" ht="18" customHeight="1">
+      <c r="A34" s="42"/>
+      <c r="B34" s="66" t="s">
+        <v>267</v>
+      </c>
+      <c r="C34" s="43"/>
+      <c r="D34" s="43"/>
+      <c r="E34" s="43"/>
+      <c r="F34" s="43"/>
+      <c r="G34" s="43"/>
+      <c r="H34" s="43"/>
+      <c r="I34" s="43"/>
+      <c r="J34" s="43"/>
+      <c r="K34" s="43"/>
+      <c r="L34" s="43"/>
+      <c r="M34" s="43"/>
+      <c r="N34" s="43"/>
+      <c r="O34" s="43"/>
+      <c r="P34" s="43"/>
+      <c r="Q34" s="43"/>
+      <c r="R34" s="43"/>
+      <c r="S34" s="43"/>
+      <c r="T34" s="43"/>
+      <c r="U34" s="43"/>
+      <c r="V34" s="43"/>
+      <c r="W34" s="43"/>
+      <c r="X34" s="44" t="s">
+        <v>268</v>
+      </c>
+      <c r="Y34" s="44" t="s">
         <v>269</v>
       </c>
-      <c r="D34" s="33" t="s">
-        <v>269</v>
-      </c>
-      <c r="E34" s="32"/>
-      <c r="F34" s="32"/>
-      <c r="G34" s="33" t="s">
-        <v>269</v>
-      </c>
-      <c r="H34" s="32"/>
-      <c r="I34" s="32"/>
-      <c r="J34" s="34"/>
-      <c r="K34" s="34"/>
-      <c r="L34" s="34"/>
-      <c r="M34" s="34"/>
-      <c r="N34" s="34"/>
-      <c r="O34" s="34"/>
-      <c r="P34" s="34"/>
-      <c r="Q34" s="34"/>
-      <c r="R34" s="34"/>
-      <c r="S34" s="34"/>
-      <c r="T34" s="32"/>
-      <c r="U34" s="34"/>
-      <c r="V34" s="32"/>
-      <c r="W34" s="34"/>
-      <c r="X34" s="32"/>
-      <c r="Y34" s="32"/>
-      <c r="Z34" s="32"/>
-      <c r="AA34" s="32"/>
-      <c r="AB34" s="32"/>
-      <c r="AC34" s="32"/>
-      <c r="AD34" s="31"/>
-      <c r="AE34" s="31"/>
-      <c r="AF34" s="41"/>
-      <c r="AG34" s="2"/>
-      <c r="AH34" s="2"/>
-      <c r="AI34" s="2"/>
-      <c r="AJ34" s="2"/>
-      <c r="AK34" s="2"/>
-      <c r="AL34" s="2"/>
-      <c r="AM34" s="2"/>
-      <c r="AN34" s="2"/>
-      <c r="AO34" s="2"/>
-      <c r="AP34" s="2"/>
-      <c r="AQ34" s="2"/>
-      <c r="AR34" s="2"/>
-      <c r="AS34" s="2"/>
-      <c r="AT34" s="2"/>
-      <c r="AU34" s="2"/>
-      <c r="AV34" s="2"/>
-      <c r="AW34" s="2"/>
-      <c r="AX34" s="2"/>
-      <c r="AY34" s="2"/>
-      <c r="AZ34" s="2"/>
-      <c r="BA34" s="2"/>
-      <c r="BB34" s="2"/>
-      <c r="BC34" s="2"/>
-      <c r="BD34" s="2"/>
-      <c r="BE34" s="2"/>
-      <c r="BF34" s="2"/>
-      <c r="BG34" s="2"/>
-      <c r="BH34" s="2"/>
-      <c r="BI34" s="2"/>
-      <c r="BJ34" s="2"/>
-      <c r="BK34" s="2"/>
-      <c r="BL34" s="2"/>
-      <c r="BM34" s="2"/>
-      <c r="BN34" s="2"/>
-      <c r="BO34" s="2"/>
-      <c r="BP34" s="2"/>
-      <c r="BQ34" s="2"/>
-      <c r="BR34" s="2"/>
-      <c r="BS34" s="2"/>
-      <c r="BT34" s="2"/>
-      <c r="BU34" s="2"/>
-      <c r="BV34" s="2"/>
-      <c r="BW34" s="2"/>
-      <c r="BX34" s="2"/>
-      <c r="BY34" s="2"/>
-      <c r="BZ34" s="2"/>
-      <c r="CA34" s="2"/>
-      <c r="CB34" s="2"/>
-      <c r="CC34" s="2"/>
-      <c r="CD34" s="2"/>
-      <c r="CE34" s="2"/>
-      <c r="CF34" s="2"/>
-      <c r="CG34" s="2"/>
-      <c r="CH34" s="2"/>
-      <c r="CI34" s="2"/>
-      <c r="CJ34" s="2"/>
-      <c r="CK34" s="2"/>
-      <c r="CL34" s="2"/>
-      <c r="CM34" s="2"/>
-      <c r="CN34" s="2"/>
-      <c r="CO34" s="2"/>
-      <c r="CP34" s="2"/>
-      <c r="CQ34" s="2"/>
-      <c r="CR34" s="2"/>
-      <c r="CS34" s="2"/>
-      <c r="CT34" s="2"/>
-      <c r="CU34" s="2"/>
-      <c r="CV34" s="2"/>
-      <c r="CW34" s="2"/>
-      <c r="CX34" s="2"/>
-      <c r="CY34" s="2"/>
-      <c r="CZ34" s="2"/>
-      <c r="DA34" s="2"/>
-      <c r="DB34" s="2"/>
-      <c r="DC34" s="2"/>
-      <c r="DD34" s="2"/>
-      <c r="DE34" s="2"/>
-      <c r="DF34" s="2"/>
-      <c r="DG34" s="2"/>
-      <c r="DH34" s="2"/>
-      <c r="DI34" s="2"/>
-      <c r="DJ34" s="2"/>
-      <c r="DK34" s="2"/>
-      <c r="DL34" s="2"/>
-      <c r="DM34" s="2"/>
-      <c r="DN34" s="2"/>
-      <c r="DO34" s="2"/>
-      <c r="DP34" s="2"/>
-      <c r="DQ34" s="2"/>
-      <c r="DR34" s="2"/>
-      <c r="DS34" s="2"/>
-      <c r="DT34" s="2"/>
-      <c r="DU34" s="2"/>
-      <c r="DV34" s="2"/>
-      <c r="DW34" s="2"/>
-      <c r="DX34" s="2"/>
-      <c r="DY34" s="2"/>
-      <c r="DZ34" s="2"/>
-      <c r="EA34" s="2"/>
-      <c r="EB34" s="2"/>
-      <c r="EC34" s="2"/>
-      <c r="ED34" s="2"/>
-      <c r="EE34" s="2"/>
-      <c r="EF34" s="2"/>
-      <c r="EG34" s="2"/>
-      <c r="EH34" s="2"/>
-      <c r="EI34" s="2"/>
-      <c r="EJ34" s="2"/>
-      <c r="EK34" s="2"/>
-      <c r="EL34" s="2"/>
-      <c r="EM34" s="2"/>
-      <c r="EN34" s="2"/>
-      <c r="EO34" s="2"/>
-      <c r="EP34" s="2"/>
-      <c r="EQ34" s="2"/>
-      <c r="ER34" s="2"/>
-      <c r="ES34" s="2"/>
-      <c r="ET34" s="2"/>
-      <c r="EU34" s="2"/>
-      <c r="EV34" s="2"/>
-      <c r="EW34" s="2"/>
-      <c r="EX34" s="2"/>
-      <c r="EY34" s="2"/>
+      <c r="Z34" s="43"/>
+      <c r="AA34" s="43"/>
+      <c r="AB34" s="43"/>
+      <c r="AC34" s="45"/>
+      <c r="AD34" s="46"/>
+      <c r="AE34" s="46"/>
+      <c r="AF34" s="47"/>
     </row>
     <row r="35" spans="1:155" ht="18" customHeight="1">
-      <c r="A35" s="42"/>
-      <c r="B35" s="66" t="s">
+      <c r="A35" s="19"/>
+      <c r="B35" s="51" t="s">
         <v>270</v>
       </c>
-      <c r="C35" s="43"/>
-      <c r="D35" s="43"/>
-      <c r="E35" s="43"/>
-      <c r="F35" s="43"/>
-      <c r="G35" s="43"/>
-      <c r="H35" s="43"/>
-      <c r="I35" s="43"/>
-      <c r="J35" s="43"/>
-      <c r="K35" s="43"/>
-      <c r="L35" s="43"/>
-      <c r="M35" s="43"/>
-      <c r="N35" s="43"/>
-      <c r="O35" s="43"/>
-      <c r="P35" s="43"/>
-      <c r="Q35" s="43"/>
-      <c r="R35" s="43"/>
-      <c r="S35" s="43"/>
-      <c r="T35" s="43"/>
-      <c r="U35" s="43"/>
-      <c r="V35" s="43"/>
-      <c r="W35" s="43"/>
-      <c r="X35" s="44" t="s">
-        <v>271</v>
-      </c>
-      <c r="Y35" s="44" t="s">
-        <v>272</v>
-      </c>
-      <c r="Z35" s="43"/>
-      <c r="AA35" s="43"/>
-      <c r="AB35" s="43"/>
-      <c r="AC35" s="45"/>
-      <c r="AD35" s="46"/>
-      <c r="AE35" s="46"/>
-      <c r="AF35" s="47"/>
+      <c r="C35" s="8"/>
+      <c r="D35" s="8"/>
+      <c r="E35" s="8"/>
+      <c r="F35" s="8"/>
+      <c r="G35" s="8"/>
+      <c r="H35" s="8"/>
+      <c r="I35" s="8"/>
+      <c r="J35" s="8"/>
+      <c r="K35" s="8"/>
+      <c r="L35" s="8"/>
+      <c r="M35" s="8"/>
+      <c r="N35" s="8"/>
+      <c r="O35" s="8"/>
+      <c r="P35" s="8"/>
+      <c r="Q35" s="8"/>
+      <c r="R35" s="8"/>
+      <c r="S35" s="8"/>
+      <c r="T35" s="8"/>
+      <c r="U35" s="8"/>
+      <c r="V35" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="W35" s="8"/>
+      <c r="X35" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="Y35" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="Z35" s="8"/>
+      <c r="AA35" s="8"/>
+      <c r="AB35" s="8"/>
+      <c r="AC35" s="7"/>
+      <c r="AD35" s="20"/>
+      <c r="AE35" s="20"/>
+      <c r="AF35" s="20"/>
     </row>
     <row r="36" spans="1:155" ht="18" customHeight="1">
-      <c r="A36" s="19"/>
-      <c r="B36" s="51" t="s">
-        <v>273</v>
-      </c>
-      <c r="C36" s="8"/>
-      <c r="D36" s="8"/>
-      <c r="E36" s="8"/>
-      <c r="F36" s="8"/>
-      <c r="G36" s="8"/>
-      <c r="H36" s="8"/>
-      <c r="I36" s="8"/>
-      <c r="J36" s="8"/>
-      <c r="K36" s="8"/>
-      <c r="L36" s="8"/>
-      <c r="M36" s="8"/>
-      <c r="N36" s="8"/>
-      <c r="O36" s="8"/>
-      <c r="P36" s="8"/>
-      <c r="Q36" s="8"/>
-      <c r="R36" s="8"/>
-      <c r="S36" s="8"/>
-      <c r="T36" s="8"/>
-      <c r="U36" s="8"/>
-      <c r="V36" s="8" t="s">
-        <v>241</v>
-      </c>
-      <c r="W36" s="8"/>
-      <c r="X36" s="8" t="s">
-        <v>241</v>
-      </c>
-      <c r="Y36" s="8" t="s">
-        <v>241</v>
-      </c>
-      <c r="Z36" s="8"/>
-      <c r="AA36" s="8"/>
-      <c r="AB36" s="8"/>
-      <c r="AC36" s="7"/>
-      <c r="AD36" s="20"/>
-      <c r="AE36" s="20"/>
-      <c r="AF36" s="20"/>
+      <c r="A36" s="15"/>
+      <c r="B36" s="67" t="s">
+        <v>271</v>
+      </c>
+      <c r="C36" s="6"/>
+      <c r="D36" s="6"/>
+      <c r="E36" s="6"/>
+      <c r="F36" s="6"/>
+      <c r="G36" s="6"/>
+      <c r="H36" s="6"/>
+      <c r="I36" s="6"/>
+      <c r="J36" s="6"/>
+      <c r="K36" s="6"/>
+      <c r="L36" s="6"/>
+      <c r="M36" s="6"/>
+      <c r="N36" s="6"/>
+      <c r="O36" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="P36" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="Q36" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="R36" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="S36" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="T36" s="6"/>
+      <c r="U36" s="6"/>
+      <c r="V36" s="6"/>
+      <c r="W36" s="6"/>
+      <c r="X36" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="Y36" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="Z36" s="6"/>
+      <c r="AA36" s="6"/>
+      <c r="AB36" s="6"/>
+      <c r="AC36" s="48"/>
+      <c r="AD36" s="16"/>
+      <c r="AE36" s="16"/>
+      <c r="AF36" s="16"/>
     </row>
     <row r="37" spans="1:155" ht="18" customHeight="1">
-      <c r="A37" s="15"/>
-      <c r="B37" s="67" t="s">
+      <c r="A37" s="42"/>
+      <c r="B37" s="66" t="s">
+        <v>272</v>
+      </c>
+      <c r="C37" s="43"/>
+      <c r="D37" s="43"/>
+      <c r="E37" s="43"/>
+      <c r="F37" s="43"/>
+      <c r="G37" s="43"/>
+      <c r="H37" s="43"/>
+      <c r="I37" s="43"/>
+      <c r="J37" s="43"/>
+      <c r="K37" s="43"/>
+      <c r="L37" s="43"/>
+      <c r="M37" s="43"/>
+      <c r="N37" s="43"/>
+      <c r="O37" s="43"/>
+      <c r="P37" s="43"/>
+      <c r="Q37" s="43"/>
+      <c r="R37" s="43"/>
+      <c r="S37" s="43"/>
+      <c r="T37" s="43"/>
+      <c r="U37" s="43"/>
+      <c r="V37" s="43"/>
+      <c r="W37" s="43"/>
+      <c r="X37" s="49" t="s">
+        <v>273</v>
+      </c>
+      <c r="Y37" s="43"/>
+      <c r="Z37" s="43"/>
+      <c r="AA37" s="43"/>
+      <c r="AB37" s="43"/>
+      <c r="AC37" s="43"/>
+      <c r="AD37" s="46"/>
+      <c r="AE37" s="44" t="s">
         <v>274</v>
       </c>
-      <c r="C37" s="6"/>
-      <c r="D37" s="6"/>
-      <c r="E37" s="6"/>
-      <c r="F37" s="6"/>
-      <c r="G37" s="6"/>
-      <c r="H37" s="6"/>
-      <c r="I37" s="6"/>
-      <c r="J37" s="6"/>
-      <c r="K37" s="6"/>
-      <c r="L37" s="6"/>
-      <c r="M37" s="6"/>
-      <c r="N37" s="6"/>
-      <c r="O37" s="6" t="s">
-        <v>241</v>
-      </c>
-      <c r="P37" s="6" t="s">
-        <v>241</v>
-      </c>
-      <c r="Q37" s="6" t="s">
-        <v>241</v>
-      </c>
-      <c r="R37" s="6" t="s">
-        <v>241</v>
-      </c>
-      <c r="S37" s="6" t="s">
-        <v>241</v>
-      </c>
-      <c r="T37" s="6"/>
-      <c r="U37" s="6"/>
-      <c r="V37" s="6"/>
-      <c r="W37" s="6"/>
-      <c r="X37" s="6" t="s">
-        <v>241</v>
-      </c>
-      <c r="Y37" s="6" t="s">
-        <v>241</v>
-      </c>
-      <c r="Z37" s="6"/>
-      <c r="AA37" s="6"/>
-      <c r="AB37" s="6"/>
-      <c r="AC37" s="48"/>
-      <c r="AD37" s="16"/>
-      <c r="AE37" s="16"/>
-      <c r="AF37" s="16"/>
+      <c r="AF37" s="50" t="s">
+        <v>275</v>
+      </c>
     </row>
     <row r="38" spans="1:155" ht="18" customHeight="1">
-      <c r="A38" s="42"/>
-      <c r="B38" s="66" t="s">
-        <v>275</v>
-      </c>
-      <c r="C38" s="43"/>
-      <c r="D38" s="43"/>
-      <c r="E38" s="43"/>
-      <c r="F38" s="43"/>
-      <c r="G38" s="43"/>
-      <c r="H38" s="43"/>
-      <c r="I38" s="43"/>
-      <c r="J38" s="43"/>
-      <c r="K38" s="43"/>
-      <c r="L38" s="43"/>
-      <c r="M38" s="43"/>
-      <c r="N38" s="43"/>
-      <c r="O38" s="43"/>
-      <c r="P38" s="43"/>
-      <c r="Q38" s="43"/>
-      <c r="R38" s="43"/>
-      <c r="S38" s="43"/>
-      <c r="T38" s="43"/>
-      <c r="U38" s="43"/>
-      <c r="V38" s="43"/>
-      <c r="W38" s="43"/>
-      <c r="X38" s="49" t="s">
+      <c r="A38" s="19"/>
+      <c r="B38" s="51" t="s">
         <v>276</v>
       </c>
-      <c r="Y38" s="43"/>
-      <c r="Z38" s="43"/>
-      <c r="AA38" s="43"/>
-      <c r="AB38" s="43"/>
-      <c r="AC38" s="43"/>
-      <c r="AD38" s="46"/>
-      <c r="AE38" s="44" t="s">
-        <v>277</v>
-      </c>
-      <c r="AF38" s="50" t="s">
-        <v>278</v>
-      </c>
+      <c r="C38" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="D38" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="E38" s="8"/>
+      <c r="F38" s="8"/>
+      <c r="G38" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="H38" s="8"/>
+      <c r="I38" s="8"/>
+      <c r="J38" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="K38" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="L38" s="8"/>
+      <c r="M38" s="8"/>
+      <c r="N38" s="8"/>
+      <c r="O38" s="8"/>
+      <c r="P38" s="8"/>
+      <c r="Q38" s="8"/>
+      <c r="R38" s="8"/>
+      <c r="S38" s="8"/>
+      <c r="T38" s="8"/>
+      <c r="U38" s="8"/>
+      <c r="V38" s="8"/>
+      <c r="W38" s="8"/>
+      <c r="X38" s="8"/>
+      <c r="Y38" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="Z38" s="8"/>
+      <c r="AA38" s="8"/>
+      <c r="AB38" s="8"/>
+      <c r="AC38" s="8"/>
+      <c r="AD38" s="20"/>
+      <c r="AE38" s="20"/>
+      <c r="AF38" s="20"/>
     </row>
     <row r="39" spans="1:155" ht="18" customHeight="1">
-      <c r="A39" s="19"/>
-      <c r="B39" s="51" t="s">
-        <v>279</v>
-      </c>
-      <c r="C39" s="8" t="s">
-        <v>241</v>
-      </c>
-      <c r="D39" s="8" t="s">
-        <v>241</v>
-      </c>
-      <c r="E39" s="8"/>
-      <c r="F39" s="8"/>
-      <c r="G39" s="8" t="s">
-        <v>241</v>
-      </c>
-      <c r="H39" s="8"/>
-      <c r="I39" s="8"/>
-      <c r="J39" s="8" t="s">
-        <v>241</v>
-      </c>
-      <c r="K39" s="8" t="s">
-        <v>241</v>
-      </c>
-      <c r="L39" s="8"/>
-      <c r="M39" s="8"/>
-      <c r="N39" s="8"/>
-      <c r="O39" s="8"/>
-      <c r="P39" s="8"/>
-      <c r="Q39" s="8"/>
-      <c r="R39" s="8"/>
-      <c r="S39" s="8"/>
-      <c r="T39" s="8"/>
-      <c r="U39" s="8"/>
-      <c r="V39" s="8"/>
-      <c r="W39" s="8"/>
-      <c r="X39" s="8"/>
-      <c r="Y39" s="8" t="s">
-        <v>241</v>
-      </c>
-      <c r="Z39" s="8"/>
-      <c r="AA39" s="8"/>
-      <c r="AB39" s="8"/>
-      <c r="AC39" s="8"/>
-      <c r="AD39" s="20"/>
-      <c r="AE39" s="20"/>
-      <c r="AF39" s="20"/>
+      <c r="A39" s="9"/>
+      <c r="B39" s="12" t="s">
+        <v>277</v>
+      </c>
+      <c r="C39" s="4"/>
+      <c r="D39" s="4"/>
+      <c r="E39" s="4"/>
+      <c r="F39" s="4"/>
+      <c r="G39" s="4"/>
+      <c r="H39" s="4"/>
+      <c r="I39" s="4"/>
+      <c r="J39" s="4"/>
+      <c r="K39" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="L39" s="4"/>
+      <c r="M39" s="4"/>
+      <c r="N39" s="4"/>
+      <c r="O39" s="4"/>
+      <c r="P39" s="4"/>
+      <c r="Q39" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="R39" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="S39" s="4"/>
+      <c r="T39" s="4"/>
+      <c r="U39" s="4"/>
+      <c r="V39" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="W39" s="4"/>
+      <c r="X39" s="4"/>
+      <c r="Y39" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="Z39" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="AA39" s="4"/>
+      <c r="AB39" s="4"/>
+      <c r="AC39" s="4"/>
+      <c r="AD39" s="10"/>
+      <c r="AE39" s="10"/>
+      <c r="AF39" s="10"/>
     </row>
     <row r="40" spans="1:155" ht="18" customHeight="1">
       <c r="A40" s="9"/>
       <c r="B40" s="12" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C40" s="4"/>
       <c r="D40" s="4"/>
@@ -5352,35 +5311,27 @@
       <c r="H40" s="4"/>
       <c r="I40" s="4"/>
       <c r="J40" s="4"/>
-      <c r="K40" s="4" t="s">
-        <v>241</v>
-      </c>
+      <c r="K40" s="4"/>
       <c r="L40" s="4"/>
       <c r="M40" s="4"/>
       <c r="N40" s="4"/>
       <c r="O40" s="4"/>
       <c r="P40" s="4"/>
-      <c r="Q40" s="4" t="s">
-        <v>241</v>
-      </c>
-      <c r="R40" s="4" t="s">
-        <v>241</v>
-      </c>
+      <c r="Q40" s="4"/>
+      <c r="R40" s="4"/>
       <c r="S40" s="4"/>
       <c r="T40" s="4"/>
       <c r="U40" s="4"/>
-      <c r="V40" s="4" t="s">
-        <v>241</v>
-      </c>
+      <c r="V40" s="4"/>
       <c r="W40" s="4"/>
       <c r="X40" s="4"/>
       <c r="Y40" s="4" t="s">
-        <v>241</v>
-      </c>
-      <c r="Z40" s="4" t="s">
-        <v>241</v>
-      </c>
-      <c r="AA40" s="4"/>
+        <v>238</v>
+      </c>
+      <c r="Z40" s="4"/>
+      <c r="AA40" s="4" t="s">
+        <v>238</v>
+      </c>
       <c r="AB40" s="4"/>
       <c r="AC40" s="4"/>
       <c r="AD40" s="10"/>
@@ -5390,7 +5341,7 @@
     <row r="41" spans="1:155" ht="18" customHeight="1">
       <c r="A41" s="9"/>
       <c r="B41" s="12" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C41" s="4"/>
       <c r="D41" s="4"/>
@@ -5414,13 +5365,9 @@
       <c r="V41" s="4"/>
       <c r="W41" s="4"/>
       <c r="X41" s="4"/>
-      <c r="Y41" s="4" t="s">
-        <v>241</v>
-      </c>
+      <c r="Y41" s="4"/>
       <c r="Z41" s="4"/>
-      <c r="AA41" s="4" t="s">
-        <v>241</v>
-      </c>
+      <c r="AA41" s="4"/>
       <c r="AB41" s="4"/>
       <c r="AC41" s="4"/>
       <c r="AD41" s="10"/>
@@ -5430,13 +5377,15 @@
     <row r="42" spans="1:155" ht="18" customHeight="1">
       <c r="A42" s="9"/>
       <c r="B42" s="12" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C42" s="4"/>
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>
       <c r="F42" s="4"/>
-      <c r="G42" s="4"/>
+      <c r="G42" s="4" t="s">
+        <v>238</v>
+      </c>
       <c r="H42" s="4"/>
       <c r="I42" s="4"/>
       <c r="J42" s="4"/>
@@ -5466,15 +5415,13 @@
     <row r="43" spans="1:155" ht="18" customHeight="1">
       <c r="A43" s="9"/>
       <c r="B43" s="12" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C43" s="4"/>
       <c r="D43" s="4"/>
       <c r="E43" s="4"/>
       <c r="F43" s="4"/>
-      <c r="G43" s="4" t="s">
-        <v>241</v>
-      </c>
+      <c r="G43" s="4"/>
       <c r="H43" s="4"/>
       <c r="I43" s="4"/>
       <c r="J43" s="4"/>
@@ -5491,20 +5438,21 @@
       <c r="U43" s="4"/>
       <c r="V43" s="4"/>
       <c r="W43" s="4"/>
-      <c r="X43" s="4"/>
-      <c r="Y43" s="4"/>
-      <c r="Z43" s="4"/>
-      <c r="AA43" s="4"/>
-      <c r="AB43" s="4"/>
-      <c r="AC43" s="4"/>
+      <c r="X43" s="10"/>
+      <c r="Y43" s="10"/>
+      <c r="Z43" s="10"/>
+      <c r="AA43" s="10"/>
+      <c r="AB43" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="AC43" s="10"/>
       <c r="AD43" s="10"/>
       <c r="AE43" s="10"/>
-      <c r="AF43" s="10"/>
     </row>
     <row r="44" spans="1:155" ht="18" customHeight="1">
       <c r="A44" s="9"/>
       <c r="B44" s="12" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="C44" s="4"/>
       <c r="D44" s="4"/>
@@ -5531,9 +5479,7 @@
       <c r="Y44" s="10"/>
       <c r="Z44" s="10"/>
       <c r="AA44" s="10"/>
-      <c r="AB44" s="10" t="s">
-        <v>241</v>
-      </c>
+      <c r="AB44" s="10"/>
       <c r="AC44" s="10"/>
       <c r="AD44" s="10"/>
       <c r="AE44" s="10"/>
@@ -5541,7 +5487,7 @@
     <row r="45" spans="1:155" ht="18" customHeight="1">
       <c r="A45" s="9"/>
       <c r="B45" s="12" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C45" s="4"/>
       <c r="D45" s="4"/>
@@ -5576,7 +5522,7 @@
     <row r="46" spans="1:155" ht="18" customHeight="1">
       <c r="A46" s="9"/>
       <c r="B46" s="12" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C46" s="4"/>
       <c r="D46" s="4"/>
@@ -5611,7 +5557,7 @@
     <row r="47" spans="1:155" ht="18" customHeight="1">
       <c r="A47" s="9"/>
       <c r="B47" s="12" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C47" s="4"/>
       <c r="D47" s="4"/>
@@ -5643,40 +5589,10 @@
       <c r="AD47" s="10"/>
       <c r="AE47" s="10"/>
     </row>
-    <row r="48" spans="1:155" ht="18" customHeight="1">
-      <c r="A48" s="9"/>
-      <c r="B48" s="12" t="s">
-        <v>288</v>
-      </c>
-      <c r="C48" s="4"/>
-      <c r="D48" s="4"/>
-      <c r="E48" s="4"/>
-      <c r="F48" s="4"/>
-      <c r="G48" s="4"/>
-      <c r="H48" s="4"/>
-      <c r="I48" s="4"/>
-      <c r="J48" s="4"/>
-      <c r="K48" s="4"/>
-      <c r="L48" s="4"/>
-      <c r="M48" s="4"/>
-      <c r="N48" s="4"/>
-      <c r="O48" s="4"/>
-      <c r="P48" s="4"/>
-      <c r="Q48" s="4"/>
-      <c r="R48" s="4"/>
-      <c r="S48" s="4"/>
-      <c r="T48" s="4"/>
-      <c r="U48" s="4"/>
-      <c r="V48" s="4"/>
-      <c r="W48" s="4"/>
-      <c r="X48" s="10"/>
-      <c r="Y48" s="10"/>
-      <c r="Z48" s="10"/>
-      <c r="AA48" s="10"/>
-      <c r="AB48" s="10"/>
-      <c r="AC48" s="10"/>
-      <c r="AD48" s="10"/>
-      <c r="AE48" s="10"/>
+    <row r="48" spans="1:155">
+      <c r="X48" s="2"/>
+      <c r="Y48" s="2"/>
+      <c r="Z48" s="2"/>
     </row>
     <row r="49" spans="24:26">
       <c r="X49" s="2"/>
@@ -5738,13 +5654,8 @@
       <c r="Y60" s="2"/>
       <c r="Z60" s="2"/>
     </row>
-    <row r="61" spans="24:26">
-      <c r="X61" s="2"/>
-      <c r="Y61" s="2"/>
-      <c r="Z61" s="2"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A2:AF34" xr:uid="{D8B0CA4D-B55F-4AFA-903E-3D529FFFD0A1}">
+  <autoFilter ref="A2:AF33" xr:uid="{D8B0CA4D-B55F-4AFA-903E-3D529FFFD0A1}">
     <filterColumn colId="2" showButton="0"/>
     <filterColumn colId="3" showButton="0"/>
     <filterColumn colId="4" showButton="0"/>
@@ -5764,15 +5675,15 @@
     <filterColumn colId="20" showButton="0"/>
   </autoFilter>
   <mergeCells count="22">
-    <mergeCell ref="B21:B28"/>
-    <mergeCell ref="B13:B19"/>
-    <mergeCell ref="B8:B12"/>
-    <mergeCell ref="B29:B34"/>
+    <mergeCell ref="B20:B27"/>
+    <mergeCell ref="B12:B18"/>
+    <mergeCell ref="B7:B11"/>
+    <mergeCell ref="B28:B33"/>
     <mergeCell ref="AD2:AD4"/>
     <mergeCell ref="Z2:Z4"/>
     <mergeCell ref="AE2:AE4"/>
     <mergeCell ref="AF2:AF4"/>
-    <mergeCell ref="A8:A19"/>
+    <mergeCell ref="A7:A18"/>
     <mergeCell ref="AB2:AB4"/>
     <mergeCell ref="AC2:AC4"/>
     <mergeCell ref="C3:E3"/>
@@ -5788,130 +5699,130 @@
     <mergeCell ref="Y2:Y4"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="C22" r:id="rId1" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/sp?tab=models" xr:uid="{FE987DC0-578A-4A81-AB17-6E49D6983782}"/>
-    <hyperlink ref="C23" r:id="rId2" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/spe?tab=models" xr:uid="{E414E66B-6D50-4BC0-93B6-EEDD71D1D349}"/>
-    <hyperlink ref="C24" r:id="rId3" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/sp-ne?tab=models" xr:uid="{79A82224-5E75-416A-BD5C-1C442DB4F9E7}"/>
-    <hyperlink ref="D22" r:id="rId4" display="https://product-selection.grundfos.com/fr/products/bm?tab=products" xr:uid="{39935FC4-BF60-4ADA-99B8-6280D11B4087}"/>
-    <hyperlink ref="D23" r:id="rId5" display="https://product-selection.grundfos.com/fr/products/bms?tab=products" xr:uid="{201298BF-F5B7-4DD8-896A-A6CFDF20A155}"/>
-    <hyperlink ref="D24" r:id="rId6" display="https://product-selection.grundfos.com/fr/products/bm-hp?tab=products" xr:uid="{0AA34BB7-1783-4351-AB39-2E3E2C9E6D24}"/>
-    <hyperlink ref="E22" r:id="rId7" display="https://product-selection.grundfos.com/fr/products/kpl?tab=models" xr:uid="{02FD05D5-211D-4185-A911-F718E163AF22}"/>
-    <hyperlink ref="E23" r:id="rId8" display="https://product-selection.grundfos.com/fr/products/kwm?tab=documentation" xr:uid="{F11B5E61-F53C-4DA1-93C5-A57D0408930C}"/>
-    <hyperlink ref="F22" r:id="rId9" display="https://product-selection.grundfos.com/fr/products/ls?tab=products" xr:uid="{070C34E9-9C05-4522-9AD2-8E6D82261A9B}"/>
-    <hyperlink ref="J22" r:id="rId10" display="https://product-selection.grundfos.com/fr/products/cm-cme?tab=products" xr:uid="{E79A5B97-E6E0-4649-B070-9A1CF47F88B2}"/>
-    <hyperlink ref="I22" r:id="rId11" display="https://product-selection.grundfos.com/fr/products/cm-cme/cm-self-priming?tab=models" xr:uid="{CFEF6DD3-2F90-4195-BA05-DEE28F55BD3E}"/>
-    <hyperlink ref="J23" r:id="rId12" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nb?tab=documentation" xr:uid="{ABC208A8-FE5B-4CC4-B585-6A3873FA7294}"/>
-    <hyperlink ref="J24" r:id="rId13" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nbe?tab=models" xr:uid="{1D4EF590-19C1-44EB-8B92-46AD5F28F62F}"/>
-    <hyperlink ref="J25" r:id="rId14" display="https://product-selection.grundfos.com/fr/products/nk-nke-nke-series-2000-nk-bare-shaft?tab=products" xr:uid="{76D3161D-F2DD-4CCA-AC1D-AD2E393D8694}"/>
-    <hyperlink ref="J26" r:id="rId15" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft?tab=products" xr:uid="{9CA4757F-439C-4161-8B60-7C14A9EDCA69}"/>
-    <hyperlink ref="J27" r:id="rId16" display="https://product-selection.grundfos.com/fr/products/tp-tpe?tab=products" xr:uid="{0C9A1473-1926-417A-947F-8561754B7D76}"/>
-    <hyperlink ref="N24" r:id="rId17" display="https://product-selection.grundfos.com/fr/products/tp-tpe?tab=products" xr:uid="{7D2D046F-1C95-42DD-8F35-90280675B9EA}"/>
-    <hyperlink ref="N22" r:id="rId18" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nbe?tab=models" xr:uid="{303D01A6-AC7B-42EE-AE09-2A10FBED3940}"/>
-    <hyperlink ref="N23" r:id="rId19" display="https://product-selection.grundfos.com/fr/products/nk-nke-nke-series-2000-nk-bare-shaft?tab=products" xr:uid="{A1442A3E-E286-4D87-BF5A-B52C00F11931}"/>
-    <hyperlink ref="N25" r:id="rId20" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft?tab=products" xr:uid="{91C811C0-E7C2-45CC-8C4A-41851188982F}"/>
-    <hyperlink ref="K22" r:id="rId21" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte?tab=products" xr:uid="{168A97AE-925F-4CB8-99FA-4D28B053F7CB}"/>
-    <hyperlink ref="L23" r:id="rId22" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte/cre?tab=models" xr:uid="{43E68B92-4EB3-4ECE-A299-C7DDCAFB1889}"/>
-    <hyperlink ref="L24" r:id="rId23" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte/crne?tab=models" xr:uid="{9DD9406E-F477-49F6-BA29-841ED00CE74B}"/>
-    <hyperlink ref="M22" r:id="rId24" display="https://product-selection.grundfos.com/fr/products/cm-cme/cme?tab=models" xr:uid="{CB210458-379C-4663-B0FD-73E843090C67}"/>
-    <hyperlink ref="M23" r:id="rId25" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nbe?tab=models" xr:uid="{3776F606-4CBE-49B1-912C-5B2BC9586206}"/>
-    <hyperlink ref="M24" r:id="rId26" display="https://product-selection.grundfos.com/fr/products/nk-nke-nke-series-2000-nk-bare-shaft?tab=products" xr:uid="{8731A9E7-9B51-450F-BCB5-013214A2B33F}"/>
-    <hyperlink ref="M25" r:id="rId27" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft?tab=products" xr:uid="{EDB8C821-F675-4CE1-B7B0-0FAF39DCEFD4}"/>
-    <hyperlink ref="L26" r:id="rId28" display="https://product-selection.grundfos.com/fr/products/hydro-multi-e?tab=models" xr:uid="{5995DFA3-65AE-4378-BD2E-CDA4F6FA5ED7}"/>
-    <hyperlink ref="L27" r:id="rId29" display="https://product-selection.grundfos.com/fr/products/hydro-mpc?tab=products" xr:uid="{2E37CE89-9B22-43AA-B967-C6F20A25613F}"/>
-    <hyperlink ref="L25" r:id="rId30" display="https://product-selection.grundfos.com/fr/products/hydro-solo-e?tab=models" xr:uid="{5A1F2584-1AA0-4C8B-A55D-39C825C8A3F8}"/>
-    <hyperlink ref="O22" r:id="rId31" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/sl1?tab=models" xr:uid="{9C7E88DB-59BA-4B5C-8769-45D64CC97D40}"/>
-    <hyperlink ref="O23" r:id="rId32" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/slv?tab=models" xr:uid="{00039B9D-B404-44A8-B557-BBF172D7CD31}"/>
-    <hyperlink ref="O24" r:id="rId33" display="https://product-selection.grundfos.com/fr/products/sesl-9-30-kw?tab=models" xr:uid="{C90FBAD5-7C9C-4429-9BAC-9BE027B562FD}"/>
-    <hyperlink ref="O26" r:id="rId34" display="https://product-selection.grundfos.com/fr/products/s?tab=products" xr:uid="{6F267867-1729-460E-9939-DEBA10D95429}"/>
-    <hyperlink ref="O25" r:id="rId35" display="https://product-selection.grundfos.com/fr/products/sesl-frame-size-56?tab=models" xr:uid="{541D6F69-2D4F-412B-91C7-A0B79C20C0CA}"/>
-    <hyperlink ref="P23" r:id="rId36" display="https://product-selection.grundfos.com/fr/products/unilift-ap/unilift-apg?tab=models" xr:uid="{CF6542DD-C411-4584-A2A2-ADD9BD336104}"/>
-    <hyperlink ref="P22" r:id="rId37" display="https://product-selection.grundfos.com/fr/products/seg?tab=models" xr:uid="{AF847B64-9B08-45DD-8487-57C6900B0D5F}"/>
-    <hyperlink ref="Q22" r:id="rId38" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/se1?tab=models" xr:uid="{D2271F27-967E-46DC-8195-E2EAFD3339EB}"/>
-    <hyperlink ref="Q23" r:id="rId39" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/sev?tab=models" xr:uid="{6D042873-5F32-4A50-8803-93F40528C6A1}"/>
-    <hyperlink ref="Q24" r:id="rId40" display="https://product-selection.grundfos.com/fr/products/sesl-9-30-kw?tab=models" xr:uid="{A344F5B5-8A97-456F-87D5-4C6EFCA52D3A}"/>
-    <hyperlink ref="Q25" r:id="rId41" display="https://product-selection.grundfos.com/fr/products/sesl-frame-size-56?tab=models" xr:uid="{BB0B40A3-A20A-44BC-9FC9-E9EE00FC9F45}"/>
-    <hyperlink ref="Q26" r:id="rId42" display="https://product-selection.grundfos.com/fr/products/s?tab=products" xr:uid="{2E26D22E-3FD7-4718-9B39-661D30AF938C}"/>
-    <hyperlink ref="Q27" r:id="rId43" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft/nkg-supervortex-impeller?tab=explore" xr:uid="{FA539854-B47D-4B47-9F9A-7CE595B28025}"/>
-    <hyperlink ref="S22" r:id="rId44" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/se1?tab=models" xr:uid="{66C50FE8-D6EA-4602-866A-7B3258A9261C}"/>
-    <hyperlink ref="S23" r:id="rId45" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/sev?tab=models" xr:uid="{DEFE3A48-5152-4917-935D-8BAB7D40CDD7}"/>
-    <hyperlink ref="S24" r:id="rId46" display="https://product-selection.grundfos.com/fr/products/sesl-9-30-kw?tab=models" xr:uid="{62BA715F-3850-4F49-A593-7645C6C0C3CC}"/>
-    <hyperlink ref="S25" r:id="rId47" display="https://product-selection.grundfos.com/fr/products/sesl-frame-size-56?tab=models" xr:uid="{F0AA29DC-4DA5-4CA6-94B3-C22351F6904E}"/>
-    <hyperlink ref="S26" r:id="rId48" display="https://product-selection.grundfos.com/fr/products/s?tab=products" xr:uid="{96671AB9-9AEA-4A5F-B84F-E78888F9B311}"/>
-    <hyperlink ref="S27" r:id="rId49" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft/nkg-supervortex-impeller?tab=explore" xr:uid="{8A1CF826-08F5-4AF2-B984-9AA020480952}"/>
-    <hyperlink ref="O27" r:id="rId50" display="https://product-selection.grundfos.com/fr/products/unilift-ap/unilift-ap50b?tab=models" xr:uid="{14E21A07-FF5F-4129-AE6E-260A1AA5098C}"/>
-    <hyperlink ref="W22" r:id="rId51" display="https://product-selection.grundfos.com/fr/products/unilift-ap?tab=products" xr:uid="{FF1F3D5A-16C1-4C5A-8F69-37BEB2C51657}"/>
-    <hyperlink ref="W23" r:id="rId52" display="https://product-selection.grundfos.com/fr/products/unilift-kp?tab=models" xr:uid="{D8B15CDE-A46F-4955-8CE5-B1F2491BDDEE}"/>
-    <hyperlink ref="W24" r:id="rId53" display="https://product-selection.grundfos.com/fr/products/unilift-cc?tab=models" xr:uid="{5DA16314-BD6C-4DB3-8EC0-A99C56D3006D}"/>
-    <hyperlink ref="W25" r:id="rId54" display="https://product-selection.grundfos.com/fr/products/dp?tab=models" xr:uid="{4D82ED98-3DD6-4697-9C9C-A060C7E06489}"/>
-    <hyperlink ref="W26" r:id="rId55" display="https://product-selection.grundfos.com/fr/products/ef?tab=models" xr:uid="{ABDE8970-72CB-4EB8-979F-99183A9FD9D3}"/>
-    <hyperlink ref="Y22" r:id="rId56" display="https://product-selection.grundfos.com/fr/products/mt-tank-mounted-pumps/mtr?tab=models" xr:uid="{D5799B15-EF87-41DF-88D8-05F25935D793}"/>
-    <hyperlink ref="Y23" r:id="rId57" display="https://product-selection.grundfos.com/fr/products/mt-tank-mounted-pumps/mtre?tab=models" xr:uid="{7E2DAAB5-3884-49DD-BF25-FA92C2CE9951}"/>
-    <hyperlink ref="Y24" r:id="rId58" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nb?tab=documentation" xr:uid="{92C19ACB-7462-4938-A66E-478979299908}"/>
-    <hyperlink ref="Y25" r:id="rId59" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nbe?tab=models" xr:uid="{D2CCE95F-A5DF-4715-B3CA-DB297F6DF5C8}"/>
-    <hyperlink ref="Y26" r:id="rId60" display="https://product-selection.grundfos.com/fr/products/nk-nke-nke-series-2000-nk-bare-shaft?tab=products" xr:uid="{EA080A36-FCEB-4D04-B389-F8ABE5514300}"/>
-    <hyperlink ref="Y27" r:id="rId61" display="https://product-selection.grundfos.com/fr/products/tp-tpe?tab=products" xr:uid="{2A2A6B6D-2CAA-4110-9FED-BCA8DC5F1709}"/>
-    <hyperlink ref="Y28" r:id="rId62" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte?tab=products" xr:uid="{D902984C-2BC5-48A4-BF49-DCE4C7E629F6}"/>
-    <hyperlink ref="Z22" r:id="rId63" display="https://product-selection.grundfos.com/fr/products/hydro-en?tab=models" xr:uid="{69CECDCF-71ED-40D6-A274-30663F73D3A6}"/>
-    <hyperlink ref="AD22" r:id="rId64" display="https://product-selection.grundfos.com/fr/products/poweradapt?tab=models" xr:uid="{CBB79406-3EE4-4CC7-BCD3-398882D58A96}"/>
-    <hyperlink ref="AD23" r:id="rId65" display="https://product-selection.grundfos.com/fr/products/rsi?tab=models" xr:uid="{2ECDD4BA-B757-4A11-9F78-EB235920F462}"/>
-    <hyperlink ref="AD24" r:id="rId66" display="https://product-selection.grundfos.com/fr/products/crflex?tab=models" xr:uid="{F1835770-C21F-4E8A-9EBF-7C701B0E9CF4}"/>
-    <hyperlink ref="AD25" r:id="rId67" display="https://product-selection.grundfos.com/fr/products/sqflex?tab=models" xr:uid="{2932EAA4-553E-42B6-AD4B-37D91C9B845C}"/>
-    <hyperlink ref="AD26" r:id="rId68" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/sp?tab=models" xr:uid="{25A70C6E-05E1-4E40-956B-50B78B088135}"/>
-    <hyperlink ref="AD27" r:id="rId69" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/spe?tab=models" xr:uid="{7C346AF6-2EEB-4DFC-A819-DAE2C3B09113}"/>
-    <hyperlink ref="AD28" r:id="rId70" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte?tab=products" xr:uid="{9F4AE584-6CDD-45BE-ABC9-5087AAD766B9}"/>
-    <hyperlink ref="AE22" r:id="rId71" display="https://product-selection.grundfos.com/fr/products/dosing-pumps-digital/dda?tab=models" xr:uid="{68600FE5-FDB0-4237-8B8A-45786462FE8A}"/>
-    <hyperlink ref="AE23" r:id="rId72" display="https://product-selection.grundfos.com/fr/products/dosing-pumps-digital/dme?tab=models" xr:uid="{41502941-2297-46B7-A840-2EF7A24064D7}"/>
-    <hyperlink ref="AE24" r:id="rId73" display="https://product-selection.grundfos.com/fr/products/dosing-pumps-mechanical/dmx?tab=models" xr:uid="{A892A826-C3E1-4B26-9529-8174E76C068D}"/>
-    <hyperlink ref="AE25" r:id="rId74" display="https://product-selection.grundfos.com/fr/products/dosing-pumps-mechanical/dmh?tab=models" xr:uid="{60926621-C7DA-4892-9ACA-4145E303C37B}"/>
-    <hyperlink ref="AE26" r:id="rId75" xr:uid="{EB339B7E-AAB0-4720-A5DC-B7E47BEFE888}"/>
-    <hyperlink ref="AF24" r:id="rId76" display="https://product-selection.grundfos.com/fr/products/disinfection-systems/oxiperm?tab=models" xr:uid="{D1CFBDC1-076A-4661-B343-B5087946D2BF}"/>
-    <hyperlink ref="AF22" r:id="rId77" display="https://product-selection.grundfos.com/fr/products/disinfection-systems/vaccuperm?tab=models" xr:uid="{0E5CA30E-D80E-4BC1-BE8D-5757C0E703F9}"/>
-    <hyperlink ref="AF23" r:id="rId78" display="https://product-selection.grundfos.com/fr/products/disinfection-systems/selcoperm?tab=models" xr:uid="{3FE337C4-03C2-4326-92F3-2ADF14429172}"/>
-    <hyperlink ref="C30" r:id="rId79" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-4" xr:uid="{7CECB146-2C6E-4D8C-8362-B574F0A0B1CD}"/>
-    <hyperlink ref="C31" r:id="rId80" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-6" xr:uid="{77066640-D437-4393-AE04-9291CA2EA2E2}"/>
-    <hyperlink ref="C32" r:id="rId81" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-8" xr:uid="{440D559C-9B55-46F7-B47D-809066594D8E}"/>
-    <hyperlink ref="C33" r:id="rId82" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-actun-zetos" xr:uid="{6B88B868-32F8-4635-8067-C4F8AA30A87A}"/>
-    <hyperlink ref="C34" r:id="rId83" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-14-24" xr:uid="{6AAEB27D-0CD4-409C-9175-B5DC81BA5B91}"/>
-    <hyperlink ref="D30" r:id="rId84" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-4" xr:uid="{70B5668C-6DE4-4721-BD0D-15695ACCFD10}"/>
-    <hyperlink ref="D31" r:id="rId85" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-6" xr:uid="{AB0F5528-0721-49E7-9EB4-443A836A5BE6}"/>
-    <hyperlink ref="D32" r:id="rId86" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-8" xr:uid="{CE5D4CF5-B9AD-4786-AF2A-5CBA0FB4461E}"/>
-    <hyperlink ref="D33" r:id="rId87" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-actun-zetos" xr:uid="{F3302311-60D3-4257-BE0E-8ADCE8FD3F26}"/>
-    <hyperlink ref="D34" r:id="rId88" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-14-24" xr:uid="{C714C692-05B2-43B9-83CE-06CDCF547DAA}"/>
-    <hyperlink ref="F30" r:id="rId89" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-scp" xr:uid="{7BEBF8BE-E457-43DD-A078-9A05C9712ED1}"/>
-    <hyperlink ref="F31" r:id="rId90" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-atmos-tera-sch" xr:uid="{8AC9B5FF-3554-4A3F-9A49-254FDDC1D679}"/>
-    <hyperlink ref="G30" r:id="rId91" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-4" xr:uid="{A6F45EEC-DFC1-4F41-A737-7D50D323F858}"/>
-    <hyperlink ref="G31" r:id="rId92" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-6" xr:uid="{E8092E13-22EC-4AA4-A0E2-CB8C894814DA}"/>
-    <hyperlink ref="G32" r:id="rId93" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-8" xr:uid="{06C47C82-BB6B-4167-9AFC-F87F629A6D2D}"/>
-    <hyperlink ref="G33" r:id="rId94" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-actun-zetos" xr:uid="{7F484481-A382-4AA7-BC6F-9F9E8E881F13}"/>
-    <hyperlink ref="G34" r:id="rId95" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-14-24" xr:uid="{145E082E-ACF5-4C03-95AA-D5FF287B68E9}"/>
-    <hyperlink ref="J30" r:id="rId96" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-medana-ch1-l" xr:uid="{CB6CAFF8-329E-47DC-8F46-39C8BB5E04DD}"/>
-    <hyperlink ref="J31" r:id="rId97" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-zeox-first-h" xr:uid="{2D403080-ECF0-434D-8570-2DCE4384BDB3}"/>
-    <hyperlink ref="K30" r:id="rId98" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-helix-v" xr:uid="{24EB14FB-8853-4DD9-BFF7-D08622F6269E}"/>
-    <hyperlink ref="K31" r:id="rId99" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-helix-first-v" xr:uid="{292648A6-CEF7-4F6A-B9E8-2C2D1935D493}"/>
-    <hyperlink ref="L30" r:id="rId100" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-helix-ve" xr:uid="{CB04A41A-2CE9-45EC-90FB-F63D1D7003E0}"/>
-    <hyperlink ref="L31" r:id="rId101" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-helix2-0-ve" xr:uid="{0D95BEE0-BF20-4117-86C3-9423999074AC}"/>
-    <hyperlink ref="M30" r:id="rId102" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-medana-ch3-le" xr:uid="{E61CDC21-E587-41FD-8720-AA95E8F2BCB8}"/>
-    <hyperlink ref="N30" r:id="rId103" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-isar-modh1-e-2-3" xr:uid="{2D23D0CC-B7DF-4FF1-ABE9-A9C38B0D675F}"/>
-    <hyperlink ref="N31" r:id="rId104" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-siboost2-0-smart-helix-ve" xr:uid="{FFEEE275-2C73-4EC4-B193-CB85762B0142}"/>
-    <hyperlink ref="O30" r:id="rId105" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-pro" xr:uid="{40187CA6-E027-4F57-B695-B124E41E9781}"/>
-    <hyperlink ref="O31" r:id="rId106" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-supra" xr:uid="{6510CD0A-CFE7-486C-91AF-7C7A655B4AFB}"/>
-    <hyperlink ref="O32" r:id="rId107" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-solid" xr:uid="{BDC567B5-AC65-4996-9A0B-1AF09DF2041A}"/>
-    <hyperlink ref="Q30" r:id="rId108" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-bloc" xr:uid="{3980AF89-63D6-4F8A-AA62-E67520B41458}"/>
-    <hyperlink ref="Q31" r:id="rId109" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-norm" xr:uid="{713EE9E0-CE07-4B5A-8098-8828FD7A2BE1}"/>
-    <hyperlink ref="P30" r:id="rId110" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-pro-s" xr:uid="{7EA67BA6-0CB9-4BC2-8D2F-2187D3E3EC87}"/>
-    <hyperlink ref="O33" r:id="rId111" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-fa-configure" xr:uid="{F271E929-C189-489C-95BA-44C8F95B9706}"/>
-    <hyperlink ref="S30" r:id="rId112" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-pro" xr:uid="{4E520461-D8CA-4714-95A3-4A07D979003B}"/>
-    <hyperlink ref="S31" r:id="rId113" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-supra" xr:uid="{7E747CBF-258D-4F97-AE71-AF52B950EDDE}"/>
-    <hyperlink ref="S32" r:id="rId114" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-solid" xr:uid="{90F21445-AD91-480E-9E60-99DEEB471A24}"/>
-    <hyperlink ref="S33" r:id="rId115" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-fa-configure" xr:uid="{CAC9CBDD-5033-4067-92F5-E1A89E7A10BF}"/>
-    <hyperlink ref="U30" r:id="rId116" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-pro" xr:uid="{DED143CB-BC81-4CC1-99AF-6D9EFDCA04A2}"/>
-    <hyperlink ref="U31" r:id="rId117" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-supra" xr:uid="{AD0F4A4E-82E3-443D-B5CE-BB1383456F96}"/>
-    <hyperlink ref="U32" r:id="rId118" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-solid" xr:uid="{F30C0BD2-ACC1-498E-B06C-26D556B514B6}"/>
-    <hyperlink ref="U33" r:id="rId119" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-fa-configure" xr:uid="{FC92FF04-817E-49C9-B9E1-3FED19E3DBAA}"/>
-    <hyperlink ref="W30" r:id="rId120" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-drain-tm-tmw-tmr-32" xr:uid="{0F177732-3552-46D9-B2A1-0858315CC611}"/>
-    <hyperlink ref="W31" r:id="rId121" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-padus-uni" xr:uid="{31C21B43-5DBE-431A-A886-4FBC3A6BE491}"/>
-    <hyperlink ref="W32" r:id="rId122" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-padus-mini3" xr:uid="{D91894CF-CB16-4C43-980E-41E743666848}"/>
-    <hyperlink ref="W33" r:id="rId123" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-padus-pro" xr:uid="{79DE7E3B-A7A2-4098-B5DF-694F7F93640D}"/>
-    <hyperlink ref="Z30" r:id="rId124" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-cof-helix" xr:uid="{2E5216D3-37DA-48CB-ABA0-7C21064BB2D3}"/>
+    <hyperlink ref="C21" r:id="rId1" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/sp?tab=models" xr:uid="{FE987DC0-578A-4A81-AB17-6E49D6983782}"/>
+    <hyperlink ref="C22" r:id="rId2" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/spe?tab=models" xr:uid="{E414E66B-6D50-4BC0-93B6-EEDD71D1D349}"/>
+    <hyperlink ref="C23" r:id="rId3" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/sp-ne?tab=models" xr:uid="{79A82224-5E75-416A-BD5C-1C442DB4F9E7}"/>
+    <hyperlink ref="D21" r:id="rId4" display="https://product-selection.grundfos.com/fr/products/bm?tab=products" xr:uid="{39935FC4-BF60-4ADA-99B8-6280D11B4087}"/>
+    <hyperlink ref="D22" r:id="rId5" display="https://product-selection.grundfos.com/fr/products/bms?tab=products" xr:uid="{201298BF-F5B7-4DD8-896A-A6CFDF20A155}"/>
+    <hyperlink ref="D23" r:id="rId6" display="https://product-selection.grundfos.com/fr/products/bm-hp?tab=products" xr:uid="{0AA34BB7-1783-4351-AB39-2E3E2C9E6D24}"/>
+    <hyperlink ref="E21" r:id="rId7" display="https://product-selection.grundfos.com/fr/products/kpl?tab=models" xr:uid="{02FD05D5-211D-4185-A911-F718E163AF22}"/>
+    <hyperlink ref="E22" r:id="rId8" display="https://product-selection.grundfos.com/fr/products/kwm?tab=documentation" xr:uid="{F11B5E61-F53C-4DA1-93C5-A57D0408930C}"/>
+    <hyperlink ref="F21" r:id="rId9" display="https://product-selection.grundfos.com/fr/products/ls?tab=products" xr:uid="{070C34E9-9C05-4522-9AD2-8E6D82261A9B}"/>
+    <hyperlink ref="J21" r:id="rId10" display="https://product-selection.grundfos.com/fr/products/cm-cme?tab=products" xr:uid="{E79A5B97-E6E0-4649-B070-9A1CF47F88B2}"/>
+    <hyperlink ref="I21" r:id="rId11" display="https://product-selection.grundfos.com/fr/products/cm-cme/cm-self-priming?tab=models" xr:uid="{CFEF6DD3-2F90-4195-BA05-DEE28F55BD3E}"/>
+    <hyperlink ref="J22" r:id="rId12" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nb?tab=documentation" xr:uid="{ABC208A8-FE5B-4CC4-B585-6A3873FA7294}"/>
+    <hyperlink ref="J23" r:id="rId13" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nbe?tab=models" xr:uid="{1D4EF590-19C1-44EB-8B92-46AD5F28F62F}"/>
+    <hyperlink ref="J24" r:id="rId14" display="https://product-selection.grundfos.com/fr/products/nk-nke-nke-series-2000-nk-bare-shaft?tab=products" xr:uid="{76D3161D-F2DD-4CCA-AC1D-AD2E393D8694}"/>
+    <hyperlink ref="J25" r:id="rId15" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft?tab=products" xr:uid="{9CA4757F-439C-4161-8B60-7C14A9EDCA69}"/>
+    <hyperlink ref="J26" r:id="rId16" display="https://product-selection.grundfos.com/fr/products/tp-tpe?tab=products" xr:uid="{0C9A1473-1926-417A-947F-8561754B7D76}"/>
+    <hyperlink ref="N23" r:id="rId17" display="https://product-selection.grundfos.com/fr/products/tp-tpe?tab=products" xr:uid="{7D2D046F-1C95-42DD-8F35-90280675B9EA}"/>
+    <hyperlink ref="N21" r:id="rId18" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nbe?tab=models" xr:uid="{303D01A6-AC7B-42EE-AE09-2A10FBED3940}"/>
+    <hyperlink ref="N22" r:id="rId19" display="https://product-selection.grundfos.com/fr/products/nk-nke-nke-series-2000-nk-bare-shaft?tab=products" xr:uid="{A1442A3E-E286-4D87-BF5A-B52C00F11931}"/>
+    <hyperlink ref="N24" r:id="rId20" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft?tab=products" xr:uid="{91C811C0-E7C2-45CC-8C4A-41851188982F}"/>
+    <hyperlink ref="K21" r:id="rId21" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte?tab=products" xr:uid="{168A97AE-925F-4CB8-99FA-4D28B053F7CB}"/>
+    <hyperlink ref="L22" r:id="rId22" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte/cre?tab=models" xr:uid="{43E68B92-4EB3-4ECE-A299-C7DDCAFB1889}"/>
+    <hyperlink ref="L23" r:id="rId23" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte/crne?tab=models" xr:uid="{9DD9406E-F477-49F6-BA29-841ED00CE74B}"/>
+    <hyperlink ref="M21" r:id="rId24" display="https://product-selection.grundfos.com/fr/products/cm-cme/cme?tab=models" xr:uid="{CB210458-379C-4663-B0FD-73E843090C67}"/>
+    <hyperlink ref="M22" r:id="rId25" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nbe?tab=models" xr:uid="{3776F606-4CBE-49B1-912C-5B2BC9586206}"/>
+    <hyperlink ref="M23" r:id="rId26" display="https://product-selection.grundfos.com/fr/products/nk-nke-nke-series-2000-nk-bare-shaft?tab=products" xr:uid="{8731A9E7-9B51-450F-BCB5-013214A2B33F}"/>
+    <hyperlink ref="M24" r:id="rId27" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft?tab=products" xr:uid="{EDB8C821-F675-4CE1-B7B0-0FAF39DCEFD4}"/>
+    <hyperlink ref="L25" r:id="rId28" display="https://product-selection.grundfos.com/fr/products/hydro-multi-e?tab=models" xr:uid="{5995DFA3-65AE-4378-BD2E-CDA4F6FA5ED7}"/>
+    <hyperlink ref="L26" r:id="rId29" display="https://product-selection.grundfos.com/fr/products/hydro-mpc?tab=products" xr:uid="{2E37CE89-9B22-43AA-B967-C6F20A25613F}"/>
+    <hyperlink ref="L24" r:id="rId30" display="https://product-selection.grundfos.com/fr/products/hydro-solo-e?tab=models" xr:uid="{5A1F2584-1AA0-4C8B-A55D-39C825C8A3F8}"/>
+    <hyperlink ref="O21" r:id="rId31" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/sl1?tab=models" xr:uid="{9C7E88DB-59BA-4B5C-8769-45D64CC97D40}"/>
+    <hyperlink ref="O22" r:id="rId32" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/slv?tab=models" xr:uid="{00039B9D-B404-44A8-B557-BBF172D7CD31}"/>
+    <hyperlink ref="O23" r:id="rId33" display="https://product-selection.grundfos.com/fr/products/sesl-9-30-kw?tab=models" xr:uid="{C90FBAD5-7C9C-4429-9BAC-9BE027B562FD}"/>
+    <hyperlink ref="O25" r:id="rId34" display="https://product-selection.grundfos.com/fr/products/s?tab=products" xr:uid="{6F267867-1729-460E-9939-DEBA10D95429}"/>
+    <hyperlink ref="O24" r:id="rId35" display="https://product-selection.grundfos.com/fr/products/sesl-frame-size-56?tab=models" xr:uid="{541D6F69-2D4F-412B-91C7-A0B79C20C0CA}"/>
+    <hyperlink ref="P22" r:id="rId36" display="https://product-selection.grundfos.com/fr/products/unilift-ap/unilift-apg?tab=models" xr:uid="{CF6542DD-C411-4584-A2A2-ADD9BD336104}"/>
+    <hyperlink ref="P21" r:id="rId37" display="https://product-selection.grundfos.com/fr/products/seg?tab=models" xr:uid="{AF847B64-9B08-45DD-8487-57C6900B0D5F}"/>
+    <hyperlink ref="Q21" r:id="rId38" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/se1?tab=models" xr:uid="{D2271F27-967E-46DC-8195-E2EAFD3339EB}"/>
+    <hyperlink ref="Q22" r:id="rId39" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/sev?tab=models" xr:uid="{6D042873-5F32-4A50-8803-93F40528C6A1}"/>
+    <hyperlink ref="Q23" r:id="rId40" display="https://product-selection.grundfos.com/fr/products/sesl-9-30-kw?tab=models" xr:uid="{A344F5B5-8A97-456F-87D5-4C6EFCA52D3A}"/>
+    <hyperlink ref="Q24" r:id="rId41" display="https://product-selection.grundfos.com/fr/products/sesl-frame-size-56?tab=models" xr:uid="{BB0B40A3-A20A-44BC-9FC9-E9EE00FC9F45}"/>
+    <hyperlink ref="Q25" r:id="rId42" display="https://product-selection.grundfos.com/fr/products/s?tab=products" xr:uid="{2E26D22E-3FD7-4718-9B39-661D30AF938C}"/>
+    <hyperlink ref="Q26" r:id="rId43" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft/nkg-supervortex-impeller?tab=explore" xr:uid="{FA539854-B47D-4B47-9F9A-7CE595B28025}"/>
+    <hyperlink ref="S21" r:id="rId44" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/se1?tab=models" xr:uid="{66C50FE8-D6EA-4602-866A-7B3258A9261C}"/>
+    <hyperlink ref="S22" r:id="rId45" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/sev?tab=models" xr:uid="{DEFE3A48-5152-4917-935D-8BAB7D40CDD7}"/>
+    <hyperlink ref="S23" r:id="rId46" display="https://product-selection.grundfos.com/fr/products/sesl-9-30-kw?tab=models" xr:uid="{62BA715F-3850-4F49-A593-7645C6C0C3CC}"/>
+    <hyperlink ref="S24" r:id="rId47" display="https://product-selection.grundfos.com/fr/products/sesl-frame-size-56?tab=models" xr:uid="{F0AA29DC-4DA5-4CA6-94B3-C22351F6904E}"/>
+    <hyperlink ref="S25" r:id="rId48" display="https://product-selection.grundfos.com/fr/products/s?tab=products" xr:uid="{96671AB9-9AEA-4A5F-B84F-E78888F9B311}"/>
+    <hyperlink ref="S26" r:id="rId49" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft/nkg-supervortex-impeller?tab=explore" xr:uid="{8A1CF826-08F5-4AF2-B984-9AA020480952}"/>
+    <hyperlink ref="O26" r:id="rId50" display="https://product-selection.grundfos.com/fr/products/unilift-ap/unilift-ap50b?tab=models" xr:uid="{14E21A07-FF5F-4129-AE6E-260A1AA5098C}"/>
+    <hyperlink ref="W21" r:id="rId51" display="https://product-selection.grundfos.com/fr/products/unilift-ap?tab=products" xr:uid="{FF1F3D5A-16C1-4C5A-8F69-37BEB2C51657}"/>
+    <hyperlink ref="W22" r:id="rId52" display="https://product-selection.grundfos.com/fr/products/unilift-kp?tab=models" xr:uid="{D8B15CDE-A46F-4955-8CE5-B1F2491BDDEE}"/>
+    <hyperlink ref="W23" r:id="rId53" display="https://product-selection.grundfos.com/fr/products/unilift-cc?tab=models" xr:uid="{5DA16314-BD6C-4DB3-8EC0-A99C56D3006D}"/>
+    <hyperlink ref="W24" r:id="rId54" display="https://product-selection.grundfos.com/fr/products/dp?tab=models" xr:uid="{4D82ED98-3DD6-4697-9C9C-A060C7E06489}"/>
+    <hyperlink ref="W25" r:id="rId55" display="https://product-selection.grundfos.com/fr/products/ef?tab=models" xr:uid="{ABDE8970-72CB-4EB8-979F-99183A9FD9D3}"/>
+    <hyperlink ref="Y21" r:id="rId56" display="https://product-selection.grundfos.com/fr/products/mt-tank-mounted-pumps/mtr?tab=models" xr:uid="{D5799B15-EF87-41DF-88D8-05F25935D793}"/>
+    <hyperlink ref="Y22" r:id="rId57" display="https://product-selection.grundfos.com/fr/products/mt-tank-mounted-pumps/mtre?tab=models" xr:uid="{7E2DAAB5-3884-49DD-BF25-FA92C2CE9951}"/>
+    <hyperlink ref="Y23" r:id="rId58" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nb?tab=documentation" xr:uid="{92C19ACB-7462-4938-A66E-478979299908}"/>
+    <hyperlink ref="Y24" r:id="rId59" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nbe?tab=models" xr:uid="{D2CCE95F-A5DF-4715-B3CA-DB297F6DF5C8}"/>
+    <hyperlink ref="Y25" r:id="rId60" display="https://product-selection.grundfos.com/fr/products/nk-nke-nke-series-2000-nk-bare-shaft?tab=products" xr:uid="{EA080A36-FCEB-4D04-B389-F8ABE5514300}"/>
+    <hyperlink ref="Y26" r:id="rId61" display="https://product-selection.grundfos.com/fr/products/tp-tpe?tab=products" xr:uid="{2A2A6B6D-2CAA-4110-9FED-BCA8DC5F1709}"/>
+    <hyperlink ref="Y27" r:id="rId62" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte?tab=products" xr:uid="{D902984C-2BC5-48A4-BF49-DCE4C7E629F6}"/>
+    <hyperlink ref="Z21" r:id="rId63" display="https://product-selection.grundfos.com/fr/products/hydro-en?tab=models" xr:uid="{69CECDCF-71ED-40D6-A274-30663F73D3A6}"/>
+    <hyperlink ref="AD21" r:id="rId64" display="https://product-selection.grundfos.com/fr/products/poweradapt?tab=models" xr:uid="{CBB79406-3EE4-4CC7-BCD3-398882D58A96}"/>
+    <hyperlink ref="AD22" r:id="rId65" display="https://product-selection.grundfos.com/fr/products/rsi?tab=models" xr:uid="{2ECDD4BA-B757-4A11-9F78-EB235920F462}"/>
+    <hyperlink ref="AD23" r:id="rId66" display="https://product-selection.grundfos.com/fr/products/crflex?tab=models" xr:uid="{F1835770-C21F-4E8A-9EBF-7C701B0E9CF4}"/>
+    <hyperlink ref="AD24" r:id="rId67" display="https://product-selection.grundfos.com/fr/products/sqflex?tab=models" xr:uid="{2932EAA4-553E-42B6-AD4B-37D91C9B845C}"/>
+    <hyperlink ref="AD25" r:id="rId68" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/sp?tab=models" xr:uid="{25A70C6E-05E1-4E40-956B-50B78B088135}"/>
+    <hyperlink ref="AD26" r:id="rId69" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/spe?tab=models" xr:uid="{7C346AF6-2EEB-4DFC-A819-DAE2C3B09113}"/>
+    <hyperlink ref="AD27" r:id="rId70" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte?tab=products" xr:uid="{9F4AE584-6CDD-45BE-ABC9-5087AAD766B9}"/>
+    <hyperlink ref="AE21" r:id="rId71" display="https://product-selection.grundfos.com/fr/products/dosing-pumps-digital/dda?tab=models" xr:uid="{68600FE5-FDB0-4237-8B8A-45786462FE8A}"/>
+    <hyperlink ref="AE22" r:id="rId72" display="https://product-selection.grundfos.com/fr/products/dosing-pumps-digital/dme?tab=models" xr:uid="{41502941-2297-46B7-A840-2EF7A24064D7}"/>
+    <hyperlink ref="AE23" r:id="rId73" display="https://product-selection.grundfos.com/fr/products/dosing-pumps-mechanical/dmx?tab=models" xr:uid="{A892A826-C3E1-4B26-9529-8174E76C068D}"/>
+    <hyperlink ref="AE24" r:id="rId74" display="https://product-selection.grundfos.com/fr/products/dosing-pumps-mechanical/dmh?tab=models" xr:uid="{60926621-C7DA-4892-9ACA-4145E303C37B}"/>
+    <hyperlink ref="AE25" r:id="rId75" xr:uid="{EB339B7E-AAB0-4720-A5DC-B7E47BEFE888}"/>
+    <hyperlink ref="AF23" r:id="rId76" display="https://product-selection.grundfos.com/fr/products/disinfection-systems/oxiperm?tab=models" xr:uid="{D1CFBDC1-076A-4661-B343-B5087946D2BF}"/>
+    <hyperlink ref="AF21" r:id="rId77" display="https://product-selection.grundfos.com/fr/products/disinfection-systems/vaccuperm?tab=models" xr:uid="{0E5CA30E-D80E-4BC1-BE8D-5757C0E703F9}"/>
+    <hyperlink ref="AF22" r:id="rId78" display="https://product-selection.grundfos.com/fr/products/disinfection-systems/selcoperm?tab=models" xr:uid="{3FE337C4-03C2-4326-92F3-2ADF14429172}"/>
+    <hyperlink ref="C29" r:id="rId79" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-4" xr:uid="{7CECB146-2C6E-4D8C-8362-B574F0A0B1CD}"/>
+    <hyperlink ref="C30" r:id="rId80" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-6" xr:uid="{77066640-D437-4393-AE04-9291CA2EA2E2}"/>
+    <hyperlink ref="C31" r:id="rId81" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-8" xr:uid="{440D559C-9B55-46F7-B47D-809066594D8E}"/>
+    <hyperlink ref="C32" r:id="rId82" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-actun-zetos" xr:uid="{6B88B868-32F8-4635-8067-C4F8AA30A87A}"/>
+    <hyperlink ref="C33" r:id="rId83" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-14-24" xr:uid="{6AAEB27D-0CD4-409C-9175-B5DC81BA5B91}"/>
+    <hyperlink ref="D29" r:id="rId84" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-4" xr:uid="{70B5668C-6DE4-4721-BD0D-15695ACCFD10}"/>
+    <hyperlink ref="D30" r:id="rId85" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-6" xr:uid="{AB0F5528-0721-49E7-9EB4-443A836A5BE6}"/>
+    <hyperlink ref="D31" r:id="rId86" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-8" xr:uid="{CE5D4CF5-B9AD-4786-AF2A-5CBA0FB4461E}"/>
+    <hyperlink ref="D32" r:id="rId87" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-actun-zetos" xr:uid="{F3302311-60D3-4257-BE0E-8ADCE8FD3F26}"/>
+    <hyperlink ref="D33" r:id="rId88" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-14-24" xr:uid="{C714C692-05B2-43B9-83CE-06CDCF547DAA}"/>
+    <hyperlink ref="F29" r:id="rId89" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-scp" xr:uid="{7BEBF8BE-E457-43DD-A078-9A05C9712ED1}"/>
+    <hyperlink ref="F30" r:id="rId90" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-atmos-tera-sch" xr:uid="{8AC9B5FF-3554-4A3F-9A49-254FDDC1D679}"/>
+    <hyperlink ref="G29" r:id="rId91" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-4" xr:uid="{A6F45EEC-DFC1-4F41-A737-7D50D323F858}"/>
+    <hyperlink ref="G30" r:id="rId92" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-6" xr:uid="{E8092E13-22EC-4AA4-A0E2-CB8C894814DA}"/>
+    <hyperlink ref="G31" r:id="rId93" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-8" xr:uid="{06C47C82-BB6B-4167-9AFC-F87F629A6D2D}"/>
+    <hyperlink ref="G32" r:id="rId94" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-actun-zetos" xr:uid="{7F484481-A382-4AA7-BC6F-9F9E8E881F13}"/>
+    <hyperlink ref="G33" r:id="rId95" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-14-24" xr:uid="{145E082E-ACF5-4C03-95AA-D5FF287B68E9}"/>
+    <hyperlink ref="J29" r:id="rId96" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-medana-ch1-l" xr:uid="{CB6CAFF8-329E-47DC-8F46-39C8BB5E04DD}"/>
+    <hyperlink ref="J30" r:id="rId97" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-zeox-first-h" xr:uid="{2D403080-ECF0-434D-8570-2DCE4384BDB3}"/>
+    <hyperlink ref="K29" r:id="rId98" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-helix-v" xr:uid="{24EB14FB-8853-4DD9-BFF7-D08622F6269E}"/>
+    <hyperlink ref="K30" r:id="rId99" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-helix-first-v" xr:uid="{292648A6-CEF7-4F6A-B9E8-2C2D1935D493}"/>
+    <hyperlink ref="L29" r:id="rId100" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-helix-ve" xr:uid="{CB04A41A-2CE9-45EC-90FB-F63D1D7003E0}"/>
+    <hyperlink ref="L30" r:id="rId101" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-helix2-0-ve" xr:uid="{0D95BEE0-BF20-4117-86C3-9423999074AC}"/>
+    <hyperlink ref="M29" r:id="rId102" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-medana-ch3-le" xr:uid="{E61CDC21-E587-41FD-8720-AA95E8F2BCB8}"/>
+    <hyperlink ref="N29" r:id="rId103" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-isar-modh1-e-2-3" xr:uid="{2D23D0CC-B7DF-4FF1-ABE9-A9C38B0D675F}"/>
+    <hyperlink ref="N30" r:id="rId104" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-siboost2-0-smart-helix-ve" xr:uid="{FFEEE275-2C73-4EC4-B193-CB85762B0142}"/>
+    <hyperlink ref="O29" r:id="rId105" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-pro" xr:uid="{40187CA6-E027-4F57-B695-B124E41E9781}"/>
+    <hyperlink ref="O30" r:id="rId106" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-supra" xr:uid="{6510CD0A-CFE7-486C-91AF-7C7A655B4AFB}"/>
+    <hyperlink ref="O31" r:id="rId107" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-solid" xr:uid="{BDC567B5-AC65-4996-9A0B-1AF09DF2041A}"/>
+    <hyperlink ref="Q29" r:id="rId108" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-bloc" xr:uid="{3980AF89-63D6-4F8A-AA62-E67520B41458}"/>
+    <hyperlink ref="Q30" r:id="rId109" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-norm" xr:uid="{713EE9E0-CE07-4B5A-8098-8828FD7A2BE1}"/>
+    <hyperlink ref="P29" r:id="rId110" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-pro-s" xr:uid="{7EA67BA6-0CB9-4BC2-8D2F-2187D3E3EC87}"/>
+    <hyperlink ref="O32" r:id="rId111" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-fa-configure" xr:uid="{F271E929-C189-489C-95BA-44C8F95B9706}"/>
+    <hyperlink ref="S29" r:id="rId112" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-pro" xr:uid="{4E520461-D8CA-4714-95A3-4A07D979003B}"/>
+    <hyperlink ref="S30" r:id="rId113" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-supra" xr:uid="{7E747CBF-258D-4F97-AE71-AF52B950EDDE}"/>
+    <hyperlink ref="S31" r:id="rId114" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-solid" xr:uid="{90F21445-AD91-480E-9E60-99DEEB471A24}"/>
+    <hyperlink ref="S32" r:id="rId115" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-fa-configure" xr:uid="{CAC9CBDD-5033-4067-92F5-E1A89E7A10BF}"/>
+    <hyperlink ref="U29" r:id="rId116" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-pro" xr:uid="{DED143CB-BC81-4CC1-99AF-6D9EFDCA04A2}"/>
+    <hyperlink ref="U30" r:id="rId117" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-supra" xr:uid="{AD0F4A4E-82E3-443D-B5CE-BB1383456F96}"/>
+    <hyperlink ref="U31" r:id="rId118" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-solid" xr:uid="{F30C0BD2-ACC1-498E-B06C-26D556B514B6}"/>
+    <hyperlink ref="U32" r:id="rId119" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-fa-configure" xr:uid="{FC92FF04-817E-49C9-B9E1-3FED19E3DBAA}"/>
+    <hyperlink ref="W29" r:id="rId120" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-drain-tm-tmw-tmr-32" xr:uid="{0F177732-3552-46D9-B2A1-0858315CC611}"/>
+    <hyperlink ref="W30" r:id="rId121" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-padus-uni" xr:uid="{31C21B43-5DBE-431A-A886-4FBC3A6BE491}"/>
+    <hyperlink ref="W31" r:id="rId122" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-padus-mini3" xr:uid="{D91894CF-CB16-4C43-980E-41E743666848}"/>
+    <hyperlink ref="W32" r:id="rId123" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-padus-pro" xr:uid="{79DE7E3B-A7A2-4098-B5DF-694F7F93640D}"/>
+    <hyperlink ref="Z29" r:id="rId124" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-cof-helix" xr:uid="{2E5216D3-37DA-48CB-ABA0-7C21064BB2D3}"/>
   </hyperlinks>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="8" scale="83" orientation="landscape" r:id="rId125"/>

</xml_diff>

<commit_message>
Mise à jour depuis Excel — 2026-09-18T13:27:43.512Z
</commit_message>
<xml_diff>
--- a/comparatif.xlsx
+++ b/comparatif.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nge1.sharepoint.com/sites/FR_SADE_DAM/Documents partages/01 - Achats/Achats Production/Pompes &amp; Instrum/Pompes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6A66B74A-82F5-418B-B656-D58A0D28BDBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8E763BE1-4E20-4EE9-B06A-D9C6C0F5B578}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="7716" yWindow="12852" windowWidth="23256" windowHeight="12456" xr2:uid="{723C6001-552E-447F-BEBB-92F546F7738F}"/>
   </bookViews>
@@ -87,7 +87,7 @@
     <t>Pompes immergées</t>
   </si>
   <si>
-    <t>cantine</t>
+    <t>Surface 1</t>
   </si>
   <si>
     <t>Immergées</t>
@@ -5846,6 +5846,31 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <FileHash xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
+    <nombre xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
+    <CloudMigratorVersion xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <CloudMigratorOriginId xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
+    <TaxCatchAll xmlns="c4b3ccb6-1a3d-47c8-9c28-87cc19c94359" xsi:nil="true"/>
+    <UniqueSourceRef xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101004976F38B5FA2A5428FEEC343358A0CB6" ma:contentTypeVersion="19" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="d78edfbf191a497d28ab4f4b405a2c3f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xmlns:ns3="c4b3ccb6-1a3d-47c8-9c28-87cc19c94359" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="79eaa508d83d12f280b303d7506ce0b5" ns2:_="" ns3:_="">
     <xsd:import namespace="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5"/>
@@ -6096,41 +6121,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <FileHash xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
-    <nombre xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
-    <CloudMigratorVersion xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <CloudMigratorOriginId xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
-    <TaxCatchAll xmlns="c4b3ccb6-1a3d-47c8-9c28-87cc19c94359" xsi:nil="true"/>
-    <UniqueSourceRef xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2B67381A-06A2-445B-9B84-A17F50FAEFF2}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DFA46023-FA4E-40CC-AE09-8D10AF59D952}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DFA46023-FA4E-40CC-AE09-8D10AF59D952}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CC74D80B-69A9-4194-90FE-61316E92C740}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CC74D80B-69A9-4194-90FE-61316E92C740}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2B67381A-06A2-445B-9B84-A17F50FAEFF2}"/>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Mise à jour depuis Excel — 2026-09-21T12:09:33.404Z
</commit_message>
<xml_diff>
--- a/comparatif.xlsx
+++ b/comparatif.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nge1.sharepoint.com/sites/FR_SADE_DAM/Documents partages/01 - Achats/Achats Production/Pompes &amp; Instrum/Pompes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8E763BE1-4E20-4EE9-B06A-D9C6C0F5B578}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{94D0A4EA-9542-40D9-B97B-C7BBE4822744}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="7716" yWindow="12852" windowWidth="23256" windowHeight="12456" xr2:uid="{723C6001-552E-447F-BEBB-92F546F7738F}"/>
   </bookViews>
@@ -87,7 +87,7 @@
     <t>Pompes immergées</t>
   </si>
   <si>
-    <t>Surface 1</t>
+    <t>Surface 2</t>
   </si>
   <si>
     <t>Immergées</t>
@@ -1838,12 +1838,48 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="255"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
@@ -1856,12 +1892,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1891,36 +1921,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="255"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2288,104 +2288,104 @@
     <row r="2" spans="1:32" s="70" customFormat="1" ht="23.25" customHeight="1" thickBot="1">
       <c r="A2" s="68"/>
       <c r="B2" s="69"/>
-      <c r="C2" s="102" t="s">
+      <c r="C2" s="112" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="102"/>
-      <c r="E2" s="102"/>
-      <c r="F2" s="102"/>
-      <c r="G2" s="102"/>
-      <c r="H2" s="102"/>
-      <c r="I2" s="102"/>
-      <c r="J2" s="102"/>
-      <c r="K2" s="102"/>
-      <c r="L2" s="102"/>
-      <c r="M2" s="102"/>
-      <c r="N2" s="102"/>
-      <c r="O2" s="109" t="s">
+      <c r="D2" s="112"/>
+      <c r="E2" s="112"/>
+      <c r="F2" s="112"/>
+      <c r="G2" s="112"/>
+      <c r="H2" s="112"/>
+      <c r="I2" s="112"/>
+      <c r="J2" s="112"/>
+      <c r="K2" s="112"/>
+      <c r="L2" s="112"/>
+      <c r="M2" s="112"/>
+      <c r="N2" s="112"/>
+      <c r="O2" s="119" t="s">
         <v>1</v>
       </c>
-      <c r="P2" s="109"/>
-      <c r="Q2" s="109"/>
-      <c r="R2" s="109"/>
-      <c r="S2" s="109"/>
-      <c r="T2" s="109"/>
-      <c r="U2" s="103" t="s">
+      <c r="P2" s="119"/>
+      <c r="Q2" s="119"/>
+      <c r="R2" s="119"/>
+      <c r="S2" s="119"/>
+      <c r="T2" s="119"/>
+      <c r="U2" s="113" t="s">
         <v>2</v>
       </c>
-      <c r="V2" s="103"/>
-      <c r="W2" s="105" t="s">
+      <c r="V2" s="113"/>
+      <c r="W2" s="115" t="s">
         <v>3</v>
       </c>
-      <c r="X2" s="98" t="s">
+      <c r="X2" s="104" t="s">
         <v>4</v>
       </c>
-      <c r="Y2" s="98" t="s">
+      <c r="Y2" s="104" t="s">
         <v>5</v>
       </c>
-      <c r="Z2" s="98" t="s">
+      <c r="Z2" s="104" t="s">
         <v>6</v>
       </c>
-      <c r="AA2" s="98" t="s">
+      <c r="AA2" s="104" t="s">
         <v>7</v>
       </c>
-      <c r="AB2" s="98" t="s">
+      <c r="AB2" s="104" t="s">
         <v>8</v>
       </c>
-      <c r="AC2" s="98" t="s">
+      <c r="AC2" s="104" t="s">
         <v>9</v>
       </c>
-      <c r="AD2" s="92" t="s">
+      <c r="AD2" s="102" t="s">
         <v>10</v>
       </c>
-      <c r="AE2" s="92" t="s">
+      <c r="AE2" s="102" t="s">
         <v>11</v>
       </c>
-      <c r="AF2" s="92" t="s">
+      <c r="AF2" s="102" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:32" s="70" customFormat="1" ht="23.25" customHeight="1" thickBot="1">
       <c r="A3" s="68"/>
       <c r="B3" s="71"/>
-      <c r="C3" s="100" t="s">
+      <c r="C3" s="110" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="101"/>
-      <c r="E3" s="101"/>
+      <c r="D3" s="111"/>
+      <c r="E3" s="111"/>
       <c r="F3" s="72"/>
-      <c r="G3" s="100" t="s">
+      <c r="G3" s="110" t="s">
         <v>14</v>
       </c>
-      <c r="H3" s="101"/>
-      <c r="I3" s="101"/>
-      <c r="J3" s="101"/>
-      <c r="K3" s="101"/>
-      <c r="L3" s="101"/>
+      <c r="H3" s="111"/>
+      <c r="I3" s="111"/>
+      <c r="J3" s="111"/>
+      <c r="K3" s="111"/>
+      <c r="L3" s="111"/>
       <c r="M3" s="72"/>
       <c r="N3" s="73"/>
-      <c r="O3" s="100" t="s">
+      <c r="O3" s="110" t="s">
         <v>15</v>
       </c>
-      <c r="P3" s="101"/>
-      <c r="Q3" s="100" t="s">
+      <c r="P3" s="111"/>
+      <c r="Q3" s="110" t="s">
         <v>16</v>
       </c>
-      <c r="R3" s="101"/>
-      <c r="S3" s="101"/>
-      <c r="T3" s="108"/>
-      <c r="U3" s="104"/>
-      <c r="V3" s="104"/>
-      <c r="W3" s="106"/>
-      <c r="X3" s="99"/>
-      <c r="Y3" s="99"/>
-      <c r="Z3" s="99"/>
-      <c r="AA3" s="99"/>
-      <c r="AB3" s="99"/>
-      <c r="AC3" s="99"/>
-      <c r="AD3" s="93"/>
-      <c r="AE3" s="93"/>
-      <c r="AF3" s="93"/>
+      <c r="R3" s="111"/>
+      <c r="S3" s="111"/>
+      <c r="T3" s="118"/>
+      <c r="U3" s="114"/>
+      <c r="V3" s="114"/>
+      <c r="W3" s="116"/>
+      <c r="X3" s="105"/>
+      <c r="Y3" s="105"/>
+      <c r="Z3" s="105"/>
+      <c r="AA3" s="105"/>
+      <c r="AB3" s="105"/>
+      <c r="AC3" s="105"/>
+      <c r="AD3" s="103"/>
+      <c r="AE3" s="103"/>
+      <c r="AF3" s="103"/>
     </row>
     <row r="4" spans="1:32" s="80" customFormat="1" ht="57.75" customHeight="1" thickBot="1">
       <c r="B4" s="81" t="s">
@@ -2451,16 +2451,16 @@
       <c r="V4" s="83" t="s">
         <v>35</v>
       </c>
-      <c r="W4" s="107"/>
-      <c r="X4" s="99"/>
-      <c r="Y4" s="99"/>
-      <c r="Z4" s="99"/>
-      <c r="AA4" s="99"/>
-      <c r="AB4" s="99"/>
-      <c r="AC4" s="99"/>
-      <c r="AD4" s="93"/>
-      <c r="AE4" s="93"/>
-      <c r="AF4" s="94"/>
+      <c r="W4" s="117"/>
+      <c r="X4" s="105"/>
+      <c r="Y4" s="105"/>
+      <c r="Z4" s="105"/>
+      <c r="AA4" s="105"/>
+      <c r="AB4" s="105"/>
+      <c r="AC4" s="105"/>
+      <c r="AD4" s="103"/>
+      <c r="AE4" s="103"/>
+      <c r="AF4" s="106"/>
     </row>
     <row r="5" spans="1:32" s="80" customFormat="1" ht="10.15" customHeight="1" thickBot="1">
       <c r="B5" s="87"/>
@@ -2581,10 +2581,10 @@
       </c>
     </row>
     <row r="7" spans="1:32" s="1" customFormat="1" ht="18" customHeight="1">
-      <c r="A7" s="95" t="s">
+      <c r="A7" s="107" t="s">
         <v>49</v>
       </c>
-      <c r="B7" s="116" t="s">
+      <c r="B7" s="98" t="s">
         <v>50</v>
       </c>
       <c r="C7" s="11" t="s">
@@ -2641,8 +2641,8 @@
       <c r="AF7" s="76"/>
     </row>
     <row r="8" spans="1:32" s="1" customFormat="1" ht="18" customHeight="1">
-      <c r="A8" s="96"/>
-      <c r="B8" s="114"/>
+      <c r="A8" s="108"/>
+      <c r="B8" s="96"/>
       <c r="C8" s="11" t="s">
         <v>58</v>
       </c>
@@ -2705,8 +2705,8 @@
       <c r="AF8" s="76"/>
     </row>
     <row r="9" spans="1:32" s="1" customFormat="1" ht="18" customHeight="1">
-      <c r="A9" s="96"/>
-      <c r="B9" s="114"/>
+      <c r="A9" s="108"/>
+      <c r="B9" s="96"/>
       <c r="C9" s="11"/>
       <c r="D9" s="11"/>
       <c r="E9" s="11"/>
@@ -2753,8 +2753,8 @@
       <c r="AF9" s="76"/>
     </row>
     <row r="10" spans="1:32" s="1" customFormat="1" ht="18" customHeight="1">
-      <c r="A10" s="96"/>
-      <c r="B10" s="114"/>
+      <c r="A10" s="108"/>
+      <c r="B10" s="96"/>
       <c r="C10" s="11"/>
       <c r="D10" s="11"/>
       <c r="E10" s="11"/>
@@ -2793,8 +2793,8 @@
       <c r="AF10" s="76"/>
     </row>
     <row r="11" spans="1:32" s="1" customFormat="1" ht="18" customHeight="1">
-      <c r="A11" s="96"/>
-      <c r="B11" s="115"/>
+      <c r="A11" s="108"/>
+      <c r="B11" s="97"/>
       <c r="C11" s="52"/>
       <c r="D11" s="52"/>
       <c r="E11" s="52"/>
@@ -2835,8 +2835,8 @@
       <c r="AF11" s="76"/>
     </row>
     <row r="12" spans="1:32" ht="18" customHeight="1">
-      <c r="A12" s="96"/>
-      <c r="B12" s="113" t="s">
+      <c r="A12" s="108"/>
+      <c r="B12" s="95" t="s">
         <v>75</v>
       </c>
       <c r="C12" s="61" t="s">
@@ -2925,8 +2925,8 @@
       <c r="AF12" s="75"/>
     </row>
     <row r="13" spans="1:32" ht="18" customHeight="1">
-      <c r="A13" s="96"/>
-      <c r="B13" s="114"/>
+      <c r="A13" s="108"/>
+      <c r="B13" s="96"/>
       <c r="C13" s="11" t="s">
         <v>91</v>
       </c>
@@ -2997,8 +2997,8 @@
       <c r="AF13" s="40"/>
     </row>
     <row r="14" spans="1:32" ht="18" customHeight="1">
-      <c r="A14" s="96"/>
-      <c r="B14" s="114"/>
+      <c r="A14" s="108"/>
+      <c r="B14" s="96"/>
       <c r="C14" s="11" t="s">
         <v>102</v>
       </c>
@@ -3062,8 +3062,8 @@
       <c r="AF14" s="40"/>
     </row>
     <row r="15" spans="1:32" ht="18" customHeight="1">
-      <c r="A15" s="96"/>
-      <c r="B15" s="114"/>
+      <c r="A15" s="108"/>
+      <c r="B15" s="96"/>
       <c r="C15" s="11" t="s">
         <v>110</v>
       </c>
@@ -3122,8 +3122,8 @@
       <c r="AF15" s="40"/>
     </row>
     <row r="16" spans="1:32" ht="18" customHeight="1">
-      <c r="A16" s="96"/>
-      <c r="B16" s="114"/>
+      <c r="A16" s="108"/>
+      <c r="B16" s="96"/>
       <c r="C16" s="11" t="s">
         <v>116</v>
       </c>
@@ -3178,8 +3178,8 @@
       <c r="AF16" s="40"/>
     </row>
     <row r="17" spans="1:155" ht="18" customHeight="1">
-      <c r="A17" s="96"/>
-      <c r="B17" s="114"/>
+      <c r="A17" s="108"/>
+      <c r="B17" s="96"/>
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
@@ -3226,8 +3226,8 @@
       <c r="AF17" s="40"/>
     </row>
     <row r="18" spans="1:155" ht="18" customHeight="1">
-      <c r="A18" s="97"/>
-      <c r="B18" s="115"/>
+      <c r="A18" s="109"/>
+      <c r="B18" s="97"/>
       <c r="C18" s="32"/>
       <c r="D18" s="32"/>
       <c r="E18" s="32"/>
@@ -3349,7 +3349,7 @@
     </row>
     <row r="20" spans="1:155" s="1" customFormat="1" ht="36" customHeight="1">
       <c r="A20" s="21"/>
-      <c r="B20" s="110" t="s">
+      <c r="B20" s="92" t="s">
         <v>146</v>
       </c>
       <c r="C20" s="22" t="s">
@@ -3445,7 +3445,7 @@
     </row>
     <row r="21" spans="1:155" ht="18" customHeight="1">
       <c r="A21" s="24"/>
-      <c r="B21" s="111"/>
+      <c r="B21" s="93"/>
       <c r="C21" s="25" t="s">
         <v>168</v>
       </c>
@@ -3517,7 +3517,7 @@
     </row>
     <row r="22" spans="1:155" ht="18" customHeight="1">
       <c r="A22" s="24"/>
-      <c r="B22" s="111"/>
+      <c r="B22" s="93"/>
       <c r="C22" s="25" t="s">
         <v>186</v>
       </c>
@@ -3583,7 +3583,7 @@
     </row>
     <row r="23" spans="1:155" ht="18" customHeight="1">
       <c r="A23" s="24"/>
-      <c r="B23" s="111"/>
+      <c r="B23" s="93"/>
       <c r="C23" s="25" t="s">
         <v>200</v>
       </c>
@@ -3645,7 +3645,7 @@
     </row>
     <row r="24" spans="1:155" ht="18" customHeight="1">
       <c r="A24" s="24"/>
-      <c r="B24" s="111"/>
+      <c r="B24" s="93"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
       <c r="E24" s="4"/>
@@ -3701,7 +3701,7 @@
     </row>
     <row r="25" spans="1:155" ht="18" customHeight="1">
       <c r="A25" s="24"/>
-      <c r="B25" s="111"/>
+      <c r="B25" s="93"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
       <c r="E25" s="4"/>
@@ -3753,7 +3753,7 @@
     </row>
     <row r="26" spans="1:155" ht="18" customHeight="1">
       <c r="A26" s="28"/>
-      <c r="B26" s="111"/>
+      <c r="B26" s="93"/>
       <c r="C26" s="6"/>
       <c r="D26" s="6"/>
       <c r="E26" s="6"/>
@@ -3801,7 +3801,7 @@
     </row>
     <row r="27" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1">
       <c r="A27" s="30"/>
-      <c r="B27" s="112"/>
+      <c r="B27" s="94"/>
       <c r="C27" s="32"/>
       <c r="D27" s="32"/>
       <c r="E27" s="32"/>
@@ -3962,7 +3962,7 @@
     </row>
     <row r="28" spans="1:155" s="10" customFormat="1" ht="36" customHeight="1">
       <c r="A28" s="21"/>
-      <c r="B28" s="117" t="s">
+      <c r="B28" s="99" t="s">
         <v>222</v>
       </c>
       <c r="C28" s="36" t="s">
@@ -4161,7 +4161,7 @@
     </row>
     <row r="29" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1">
       <c r="A29" s="24"/>
-      <c r="B29" s="118"/>
+      <c r="B29" s="100"/>
       <c r="C29" s="13" t="s">
         <v>239</v>
       </c>
@@ -4348,7 +4348,7 @@
     </row>
     <row r="30" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1">
       <c r="A30" s="24"/>
-      <c r="B30" s="118"/>
+      <c r="B30" s="100"/>
       <c r="C30" s="13" t="s">
         <v>251</v>
       </c>
@@ -4529,7 +4529,7 @@
     </row>
     <row r="31" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1">
       <c r="A31" s="24"/>
-      <c r="B31" s="118"/>
+      <c r="B31" s="100"/>
       <c r="C31" s="13" t="s">
         <v>260</v>
       </c>
@@ -4698,7 +4698,7 @@
     </row>
     <row r="32" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1">
       <c r="A32" s="24"/>
-      <c r="B32" s="118"/>
+      <c r="B32" s="100"/>
       <c r="C32" s="13" t="s">
         <v>263</v>
       </c>
@@ -4867,7 +4867,7 @@
     </row>
     <row r="33" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1">
       <c r="A33" s="30"/>
-      <c r="B33" s="119"/>
+      <c r="B33" s="101"/>
       <c r="C33" s="33" t="s">
         <v>266</v>
       </c>
@@ -5675,12 +5675,6 @@
     <filterColumn colId="20" showButton="0"/>
   </autoFilter>
   <mergeCells count="22">
-    <mergeCell ref="B20:B27"/>
-    <mergeCell ref="B12:B18"/>
-    <mergeCell ref="B7:B11"/>
-    <mergeCell ref="B28:B33"/>
-    <mergeCell ref="AD2:AD4"/>
-    <mergeCell ref="Z2:Z4"/>
     <mergeCell ref="AE2:AE4"/>
     <mergeCell ref="AF2:AF4"/>
     <mergeCell ref="A7:A18"/>
@@ -5697,6 +5691,12 @@
     <mergeCell ref="O2:T2"/>
     <mergeCell ref="O3:P3"/>
     <mergeCell ref="Y2:Y4"/>
+    <mergeCell ref="B20:B27"/>
+    <mergeCell ref="B12:B18"/>
+    <mergeCell ref="B7:B11"/>
+    <mergeCell ref="B28:B33"/>
+    <mergeCell ref="AD2:AD4"/>
+    <mergeCell ref="Z2:Z4"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C21" r:id="rId1" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/sp?tab=models" xr:uid="{FE987DC0-578A-4A81-AB17-6E49D6983782}"/>
@@ -5846,31 +5846,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <FileHash xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
-    <nombre xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
-    <CloudMigratorVersion xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <CloudMigratorOriginId xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
-    <TaxCatchAll xmlns="c4b3ccb6-1a3d-47c8-9c28-87cc19c94359" xsi:nil="true"/>
-    <UniqueSourceRef xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101004976F38B5FA2A5428FEEC343358A0CB6" ma:contentTypeVersion="19" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="d78edfbf191a497d28ab4f4b405a2c3f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xmlns:ns3="c4b3ccb6-1a3d-47c8-9c28-87cc19c94359" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="79eaa508d83d12f280b303d7506ce0b5" ns2:_="" ns3:_="">
     <xsd:import namespace="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5"/>
@@ -6121,8 +6096,33 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <FileHash xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
+    <nombre xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
+    <CloudMigratorVersion xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <CloudMigratorOriginId xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
+    <TaxCatchAll xmlns="c4b3ccb6-1a3d-47c8-9c28-87cc19c94359" xsi:nil="true"/>
+    <UniqueSourceRef xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DFA46023-FA4E-40CC-AE09-8D10AF59D952}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2B67381A-06A2-445B-9B84-A17F50FAEFF2}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6130,11 +6130,11 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2B67381A-06A2-445B-9B84-A17F50FAEFF2}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DFA46023-FA4E-40CC-AE09-8D10AF59D952}"/>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{7d7ef55b-d006-4101-afe3-f2bbfa26e84b}" enabled="0" method="" siteId="{7d7ef55b-d006-4101-afe3-f2bbfa26e84b}" removed="1"/>
+  <clbl:label id="{3e7a5884-aef9-4d53-85a1-19dae5fd11e1}" enabled="1" method="Standard" siteId="{7d7ef55b-d006-4101-afe3-f2bbfa26e84b}" removed="0"/>
 </clbl:labelList>
 </file>
</xml_diff>

<commit_message>
Mise à jour depuis Excel — 2026-09-21T12:11:45.619Z
</commit_message>
<xml_diff>
--- a/comparatif.xlsx
+++ b/comparatif.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nge1.sharepoint.com/sites/FR_SADE_DAM/Documents partages/01 - Achats/Achats Production/Pompes &amp; Instrum/Pompes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{94D0A4EA-9542-40D9-B97B-C7BBE4822744}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8F617838-BBAD-44C6-8A48-80F8B68FD725}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="7716" yWindow="12852" windowWidth="23256" windowHeight="12456" xr2:uid="{723C6001-552E-447F-BEBB-92F546F7738F}"/>
   </bookViews>
@@ -87,7 +87,7 @@
     <t>Pompes immergées</t>
   </si>
   <si>
-    <t>Surface 2</t>
+    <t>Surface 3</t>
   </si>
   <si>
     <t>Immergées</t>

</xml_diff>

<commit_message>
Mise à jour depuis Excel — 2026-09-22T13:06:46.553Z
</commit_message>
<xml_diff>
--- a/comparatif.xlsx
+++ b/comparatif.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nge1.sharepoint.com/sites/FR_SADE_DAM/Documents partages/01 - Achats/Achats Production/Pompes &amp; Instrum/Pompes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8F617838-BBAD-44C6-8A48-80F8B68FD725}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3AF0930F-4E2D-4EA3-92AF-769AB043B375}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="7716" yWindow="12852" windowWidth="23256" windowHeight="12456" xr2:uid="{723C6001-552E-447F-BEBB-92F546F7738F}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Feuil2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Feuil1!$A$2:$AF$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Feuil1!$A$2:$AF$34</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="288">
   <si>
     <t>Eau potable et irrigation</t>
   </si>
@@ -87,13 +87,19 @@
     <t>Pompes immergées</t>
   </si>
   <si>
-    <t>Surface 3</t>
+    <t>Surface 4 4</t>
   </si>
   <si>
     <t>Immergées</t>
   </si>
   <si>
     <t>De surface</t>
+  </si>
+  <si>
+    <t>essai</t>
+  </si>
+  <si>
+    <t>&amp;</t>
   </si>
   <si>
     <t>Types</t>
@@ -1092,7 +1098,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="38">
+  <borders count="39">
     <border>
       <left/>
       <right/>
@@ -1579,13 +1585,22 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="120">
+  <cellXfs count="124">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1920,6 +1935,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2267,7 +2294,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:EY60"/>
+  <dimension ref="A1:EY61"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="7.140625" style="1" customWidth="1"/>
@@ -2345,7 +2372,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:32" s="70" customFormat="1" ht="23.25" customHeight="1" thickBot="1">
+    <row r="3" spans="1:32" s="70" customFormat="1" ht="23.25" customHeight="1">
       <c r="A3" s="68"/>
       <c r="B3" s="71"/>
       <c r="C3" s="110" t="s">
@@ -2387,70 +2414,41 @@
       <c r="AE3" s="103"/>
       <c r="AF3" s="103"/>
     </row>
-    <row r="4" spans="1:32" s="80" customFormat="1" ht="57.75" customHeight="1" thickBot="1">
-      <c r="B4" s="81" t="s">
+    <row r="4" spans="1:32" s="70" customFormat="1" ht="23.25" customHeight="1">
+      <c r="A4" s="68"/>
+      <c r="B4" s="71" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="82" t="s">
+      <c r="C4" s="120" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="82" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" s="82" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" s="82" t="s">
-        <v>21</v>
-      </c>
-      <c r="G4" s="82" t="s">
-        <v>22</v>
-      </c>
-      <c r="H4" s="82" t="s">
-        <v>23</v>
-      </c>
-      <c r="I4" s="82" t="s">
-        <v>24</v>
-      </c>
-      <c r="J4" s="82" t="s">
-        <v>25</v>
-      </c>
-      <c r="K4" s="82" t="s">
-        <v>26</v>
-      </c>
-      <c r="L4" s="82" t="s">
-        <v>27</v>
-      </c>
-      <c r="M4" s="82" t="s">
-        <v>28</v>
-      </c>
-      <c r="N4" s="82" t="s">
-        <v>28</v>
-      </c>
-      <c r="O4" s="82" t="s">
-        <v>29</v>
-      </c>
-      <c r="P4" s="82" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q4" s="82" t="s">
-        <v>31</v>
-      </c>
-      <c r="R4" s="82" t="s">
-        <v>32</v>
-      </c>
-      <c r="S4" s="82" t="s">
-        <v>33</v>
-      </c>
-      <c r="T4" s="82" t="s">
-        <v>34</v>
-      </c>
-      <c r="U4" s="83" t="s">
-        <v>15</v>
-      </c>
-      <c r="V4" s="83" t="s">
-        <v>35</v>
-      </c>
+      <c r="D4" s="121">
+        <v>2</v>
+      </c>
+      <c r="E4" s="121">
+        <v>3</v>
+      </c>
+      <c r="F4" s="121"/>
+      <c r="G4" s="120">
+        <v>4</v>
+      </c>
+      <c r="H4" s="121">
+        <v>9</v>
+      </c>
+      <c r="I4" s="121"/>
+      <c r="J4" s="121"/>
+      <c r="K4" s="121"/>
+      <c r="L4" s="121"/>
+      <c r="M4" s="121"/>
+      <c r="N4" s="122"/>
+      <c r="O4" s="120"/>
+      <c r="P4" s="121"/>
+      <c r="Q4" s="120"/>
+      <c r="R4" s="121"/>
+      <c r="S4" s="121"/>
+      <c r="T4" s="122"/>
+      <c r="U4" s="123"/>
+      <c r="V4" s="123"/>
       <c r="W4" s="117"/>
       <c r="X4" s="105"/>
       <c r="Y4" s="105"/>
@@ -2462,235 +2460,246 @@
       <c r="AE4" s="103"/>
       <c r="AF4" s="106"/>
     </row>
-    <row r="5" spans="1:32" s="80" customFormat="1" ht="10.15" customHeight="1" thickBot="1">
-      <c r="B5" s="87"/>
-      <c r="C5" s="88"/>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="88"/>
-      <c r="K5" s="88"/>
-      <c r="L5" s="88"/>
-      <c r="M5" s="88"/>
-      <c r="N5" s="88"/>
-      <c r="O5" s="88"/>
-      <c r="P5" s="88"/>
-      <c r="Q5" s="88"/>
-      <c r="R5" s="88"/>
-      <c r="S5" s="88"/>
-      <c r="T5" s="88"/>
-      <c r="U5" s="89"/>
-      <c r="V5" s="89"/>
-      <c r="W5" s="86"/>
-      <c r="X5" s="86"/>
-      <c r="Y5" s="86"/>
-      <c r="Z5" s="86"/>
-      <c r="AA5" s="86"/>
-      <c r="AB5" s="86"/>
-      <c r="AC5" s="90"/>
-      <c r="AD5" s="91"/>
-      <c r="AE5" s="91"/>
-      <c r="AF5" s="91"/>
+    <row r="5" spans="1:32" s="80" customFormat="1" ht="57.75" customHeight="1">
+      <c r="B5" s="81" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="82" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="82" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" s="82" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" s="82" t="s">
+        <v>23</v>
+      </c>
+      <c r="G5" s="82" t="s">
+        <v>24</v>
+      </c>
+      <c r="H5" s="82" t="s">
+        <v>25</v>
+      </c>
+      <c r="I5" s="82" t="s">
+        <v>26</v>
+      </c>
+      <c r="J5" s="82" t="s">
+        <v>27</v>
+      </c>
+      <c r="K5" s="82" t="s">
+        <v>28</v>
+      </c>
+      <c r="L5" s="82" t="s">
+        <v>29</v>
+      </c>
+      <c r="M5" s="82" t="s">
+        <v>30</v>
+      </c>
+      <c r="N5" s="82" t="s">
+        <v>30</v>
+      </c>
+      <c r="O5" s="82" t="s">
+        <v>31</v>
+      </c>
+      <c r="P5" s="82" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q5" s="82" t="s">
+        <v>33</v>
+      </c>
+      <c r="R5" s="82" t="s">
+        <v>34</v>
+      </c>
+      <c r="S5" s="82" t="s">
+        <v>35</v>
+      </c>
+      <c r="T5" s="82" t="s">
+        <v>36</v>
+      </c>
+      <c r="U5" s="83" t="s">
+        <v>15</v>
+      </c>
+      <c r="V5" s="83" t="s">
+        <v>37</v>
+      </c>
+      <c r="W5" s="117"/>
+      <c r="X5" s="105"/>
+      <c r="Y5" s="105"/>
+      <c r="Z5" s="105"/>
+      <c r="AA5" s="105"/>
+      <c r="AB5" s="105"/>
+      <c r="AC5" s="105"/>
+      <c r="AD5" s="103"/>
+      <c r="AE5" s="103"/>
+      <c r="AF5" s="106"/>
     </row>
-    <row r="6" spans="1:32" s="74" customFormat="1" ht="52.9" customHeight="1">
-      <c r="B6" s="84" t="s">
-        <v>36</v>
-      </c>
-      <c r="C6" s="77" t="s">
-        <v>37</v>
-      </c>
-      <c r="D6" s="77" t="s">
+    <row r="6" spans="1:32" s="80" customFormat="1" ht="10.15" customHeight="1" thickBot="1">
+      <c r="B6" s="87"/>
+      <c r="C6" s="88"/>
+      <c r="D6" s="88"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="88"/>
+      <c r="G6" s="88"/>
+      <c r="H6" s="88"/>
+      <c r="I6" s="88"/>
+      <c r="J6" s="88"/>
+      <c r="K6" s="88"/>
+      <c r="L6" s="88"/>
+      <c r="M6" s="88"/>
+      <c r="N6" s="88"/>
+      <c r="O6" s="88"/>
+      <c r="P6" s="88"/>
+      <c r="Q6" s="88"/>
+      <c r="R6" s="88"/>
+      <c r="S6" s="88"/>
+      <c r="T6" s="88"/>
+      <c r="U6" s="89"/>
+      <c r="V6" s="89"/>
+      <c r="W6" s="86"/>
+      <c r="X6" s="86"/>
+      <c r="Y6" s="86"/>
+      <c r="Z6" s="86"/>
+      <c r="AA6" s="86"/>
+      <c r="AB6" s="86"/>
+      <c r="AC6" s="90"/>
+      <c r="AD6" s="91"/>
+      <c r="AE6" s="91"/>
+      <c r="AF6" s="91"/>
+    </row>
+    <row r="7" spans="1:32" s="74" customFormat="1" ht="52.9" customHeight="1">
+      <c r="B7" s="84" t="s">
         <v>38</v>
       </c>
-      <c r="E6" s="77" t="s">
+      <c r="C7" s="77" t="s">
         <v>39</v>
       </c>
-      <c r="F6" s="77" t="s">
-        <v>38</v>
-      </c>
-      <c r="G6" s="77" t="s">
+      <c r="D7" s="77" t="s">
         <v>40</v>
       </c>
-      <c r="H6" s="77" t="s">
-        <v>38</v>
-      </c>
-      <c r="I6" s="77" t="s">
+      <c r="E7" s="77" t="s">
         <v>41</v>
       </c>
-      <c r="J6" s="77" t="s">
-        <v>38</v>
-      </c>
-      <c r="K6" s="77" t="s">
-        <v>38</v>
-      </c>
-      <c r="L6" s="77" t="s">
-        <v>37</v>
-      </c>
-      <c r="M6" s="77" t="s">
-        <v>38</v>
-      </c>
-      <c r="N6" s="77" t="s">
+      <c r="F7" s="77" t="s">
+        <v>40</v>
+      </c>
+      <c r="G7" s="77" t="s">
         <v>42</v>
       </c>
-      <c r="O6" s="77" t="s">
+      <c r="H7" s="77" t="s">
+        <v>40</v>
+      </c>
+      <c r="I7" s="77" t="s">
         <v>43</v>
       </c>
-      <c r="P6" s="77" t="s">
-        <v>43</v>
-      </c>
-      <c r="Q6" s="77" t="s">
-        <v>43</v>
-      </c>
-      <c r="R6" s="77" t="s">
-        <v>43</v>
-      </c>
-      <c r="S6" s="77" t="s">
-        <v>43</v>
-      </c>
-      <c r="T6" s="77" t="s">
-        <v>43</v>
-      </c>
-      <c r="U6" s="77" t="s">
-        <v>43</v>
-      </c>
-      <c r="V6" s="77" t="s">
-        <v>43</v>
-      </c>
-      <c r="W6" s="77"/>
-      <c r="X6" s="77" t="s">
+      <c r="J7" s="77" t="s">
+        <v>40</v>
+      </c>
+      <c r="K7" s="77" t="s">
+        <v>40</v>
+      </c>
+      <c r="L7" s="77" t="s">
+        <v>39</v>
+      </c>
+      <c r="M7" s="77" t="s">
+        <v>40</v>
+      </c>
+      <c r="N7" s="77" t="s">
         <v>44</v>
       </c>
-      <c r="Y6" s="77" t="s">
+      <c r="O7" s="77" t="s">
         <v>45</v>
       </c>
-      <c r="Z6" s="77"/>
-      <c r="AA6" s="77"/>
-      <c r="AB6" s="77"/>
-      <c r="AC6" s="78"/>
-      <c r="AD6" s="79" t="s">
+      <c r="P7" s="77" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q7" s="77" t="s">
+        <v>45</v>
+      </c>
+      <c r="R7" s="77" t="s">
+        <v>45</v>
+      </c>
+      <c r="S7" s="77" t="s">
+        <v>45</v>
+      </c>
+      <c r="T7" s="77" t="s">
+        <v>45</v>
+      </c>
+      <c r="U7" s="77" t="s">
+        <v>45</v>
+      </c>
+      <c r="V7" s="77" t="s">
+        <v>45</v>
+      </c>
+      <c r="W7" s="77"/>
+      <c r="X7" s="77" t="s">
         <v>46</v>
       </c>
-      <c r="AE6" s="79" t="s">
+      <c r="Y7" s="77" t="s">
         <v>47</v>
       </c>
-      <c r="AF6" s="76" t="s">
+      <c r="Z7" s="77"/>
+      <c r="AA7" s="77"/>
+      <c r="AB7" s="77"/>
+      <c r="AC7" s="78"/>
+      <c r="AD7" s="79" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="7" spans="1:32" s="1" customFormat="1" ht="18" customHeight="1">
-      <c r="A7" s="107" t="s">
+      <c r="AE7" s="79" t="s">
         <v>49</v>
       </c>
-      <c r="B7" s="98" t="s">
+      <c r="AF7" s="76" t="s">
         <v>50</v>
       </c>
-      <c r="C7" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="I7" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="J7" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="K7" s="11"/>
-      <c r="L7" s="11"/>
-      <c r="M7" s="11"/>
-      <c r="N7" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="O7" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="P7" s="11"/>
-      <c r="Q7" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="R7" s="11"/>
-      <c r="S7" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="T7" s="11"/>
-      <c r="U7" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="V7" s="11"/>
-      <c r="W7" s="11"/>
-      <c r="X7" s="11"/>
-      <c r="Y7" s="11"/>
-      <c r="Z7" s="11"/>
-      <c r="AA7" s="11"/>
-      <c r="AB7" s="5"/>
-      <c r="AC7" s="54"/>
-      <c r="AD7" s="76"/>
-      <c r="AE7" s="76"/>
-      <c r="AF7" s="76"/>
     </row>
     <row r="8" spans="1:32" s="1" customFormat="1" ht="18" customHeight="1">
-      <c r="A8" s="108"/>
-      <c r="B8" s="96"/>
+      <c r="A8" s="107" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" s="98" t="s">
+        <v>52</v>
+      </c>
       <c r="C8" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="E8" s="11"/>
+      <c r="F8" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="G8" s="11"/>
+      <c r="H8" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="I8" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="J8" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="K8" s="11"/>
+      <c r="L8" s="11"/>
+      <c r="M8" s="11"/>
+      <c r="N8" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="O8" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="E8" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="F8" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="G8" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="H8" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="I8" s="11"/>
-      <c r="J8" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="K8" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="L8" s="11"/>
-      <c r="M8" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="N8" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="O8" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="P8" s="11" t="s">
-        <v>65</v>
-      </c>
+      <c r="P8" s="11"/>
       <c r="Q8" s="11" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="R8" s="11"/>
       <c r="S8" s="11" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="T8" s="11"/>
       <c r="U8" s="11" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="V8" s="11"/>
       <c r="W8" s="11"/>
@@ -2707,39 +2716,55 @@
     <row r="9" spans="1:32" s="1" customFormat="1" ht="18" customHeight="1">
       <c r="A9" s="108"/>
       <c r="B9" s="96"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
+      <c r="C9" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="G9" s="11" t="s">
+        <v>62</v>
+      </c>
       <c r="H9" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="I9" s="11"/>
+      <c r="J9" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="K9" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="L9" s="11"/>
+      <c r="M9" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="N9" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="O9" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="I9" s="11"/>
-      <c r="J9" s="11"/>
-      <c r="K9" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="L9" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="M9" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="N9" s="11" t="s">
+      <c r="P9" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q9" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="O9" s="11" t="s">
-        <v>69</v>
-      </c>
-      <c r="P9" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="Q9" s="11"/>
       <c r="R9" s="11"/>
-      <c r="S9" s="11"/>
+      <c r="S9" s="11" t="s">
+        <v>68</v>
+      </c>
       <c r="T9" s="11"/>
-      <c r="U9" s="11"/>
+      <c r="U9" s="11" t="s">
+        <v>67</v>
+      </c>
       <c r="V9" s="11"/>
       <c r="W9" s="11"/>
       <c r="X9" s="11"/>
@@ -2761,20 +2786,28 @@
       <c r="F10" s="11"/>
       <c r="G10" s="11"/>
       <c r="H10" s="11" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I10" s="11"/>
       <c r="J10" s="11"/>
-      <c r="K10" s="11"/>
+      <c r="K10" s="11" t="s">
+        <v>54</v>
+      </c>
       <c r="L10" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="M10" s="11"/>
-      <c r="N10" s="11"/>
+        <v>66</v>
+      </c>
+      <c r="M10" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="N10" s="11" t="s">
+        <v>70</v>
+      </c>
       <c r="O10" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="P10" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="P10" s="11"/>
       <c r="Q10" s="11"/>
       <c r="R10" s="11"/>
       <c r="S10" s="11"/>
@@ -2794,268 +2827,243 @@
     </row>
     <row r="11" spans="1:32" s="1" customFormat="1" ht="18" customHeight="1">
       <c r="A11" s="108"/>
-      <c r="B11" s="97"/>
-      <c r="C11" s="52"/>
-      <c r="D11" s="52"/>
-      <c r="E11" s="52"/>
-      <c r="F11" s="52"/>
-      <c r="G11" s="52"/>
-      <c r="H11" s="52"/>
-      <c r="I11" s="52"/>
-      <c r="J11" s="52"/>
-      <c r="K11" s="52"/>
-      <c r="L11" s="52" t="s">
-        <v>63</v>
-      </c>
-      <c r="M11" s="52"/>
-      <c r="N11" s="52" t="s">
+      <c r="B11" s="96"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="O11" s="52"/>
-      <c r="P11" s="52"/>
-      <c r="Q11" s="52" t="s">
+      <c r="I11" s="11"/>
+      <c r="J11" s="11"/>
+      <c r="K11" s="11"/>
+      <c r="L11" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="M11" s="11"/>
+      <c r="N11" s="11"/>
+      <c r="O11" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="R11" s="52"/>
-      <c r="S11" s="52" t="s">
-        <v>74</v>
-      </c>
-      <c r="T11" s="52"/>
-      <c r="U11" s="52"/>
-      <c r="V11" s="52"/>
-      <c r="W11" s="52"/>
-      <c r="X11" s="52"/>
-      <c r="Y11" s="52"/>
-      <c r="Z11" s="52"/>
-      <c r="AA11" s="52"/>
-      <c r="AB11" s="53"/>
-      <c r="AC11" s="55"/>
+      <c r="P11" s="11"/>
+      <c r="Q11" s="11"/>
+      <c r="R11" s="11"/>
+      <c r="S11" s="11"/>
+      <c r="T11" s="11"/>
+      <c r="U11" s="11"/>
+      <c r="V11" s="11"/>
+      <c r="W11" s="11"/>
+      <c r="X11" s="11"/>
+      <c r="Y11" s="11"/>
+      <c r="Z11" s="11"/>
+      <c r="AA11" s="11"/>
+      <c r="AB11" s="5"/>
+      <c r="AC11" s="54"/>
       <c r="AD11" s="76"/>
       <c r="AE11" s="76"/>
       <c r="AF11" s="76"/>
     </row>
-    <row r="12" spans="1:32" ht="18" customHeight="1">
+    <row r="12" spans="1:32" s="1" customFormat="1" ht="18" customHeight="1">
       <c r="A12" s="108"/>
-      <c r="B12" s="95" t="s">
+      <c r="B12" s="97"/>
+      <c r="C12" s="52"/>
+      <c r="D12" s="52"/>
+      <c r="E12" s="52"/>
+      <c r="F12" s="52"/>
+      <c r="G12" s="52"/>
+      <c r="H12" s="52"/>
+      <c r="I12" s="52"/>
+      <c r="J12" s="52"/>
+      <c r="K12" s="52"/>
+      <c r="L12" s="52" t="s">
+        <v>65</v>
+      </c>
+      <c r="M12" s="52"/>
+      <c r="N12" s="52" t="s">
         <v>75</v>
       </c>
-      <c r="C12" s="61" t="s">
+      <c r="O12" s="52"/>
+      <c r="P12" s="52"/>
+      <c r="Q12" s="52" t="s">
         <v>76</v>
       </c>
-      <c r="D12" s="62" t="s">
-        <v>77</v>
-      </c>
-      <c r="E12" s="63" t="s">
-        <v>78</v>
-      </c>
-      <c r="F12" s="62" t="s">
-        <v>77</v>
-      </c>
-      <c r="G12" s="62" t="s">
-        <v>77</v>
-      </c>
-      <c r="H12" s="62" t="s">
-        <v>77</v>
-      </c>
-      <c r="I12" s="61" t="s">
-        <v>79</v>
-      </c>
-      <c r="J12" s="61" t="s">
-        <v>80</v>
-      </c>
-      <c r="K12" s="37" t="s">
-        <v>81</v>
-      </c>
-      <c r="L12" s="61" t="s">
-        <v>82</v>
-      </c>
-      <c r="M12" s="62" t="s">
-        <v>77</v>
-      </c>
-      <c r="N12" s="61" t="s">
-        <v>83</v>
-      </c>
-      <c r="O12" s="61" t="s">
-        <v>84</v>
-      </c>
-      <c r="P12" s="37" t="s">
-        <v>85</v>
-      </c>
-      <c r="Q12" s="61" t="s">
-        <v>85</v>
-      </c>
-      <c r="R12" s="37" t="s">
-        <v>86</v>
-      </c>
-      <c r="S12" s="61" t="s">
-        <v>85</v>
-      </c>
-      <c r="T12" s="61" t="s">
-        <v>85</v>
-      </c>
-      <c r="U12" s="61" t="s">
-        <v>85</v>
-      </c>
-      <c r="V12" s="62" t="s">
-        <v>77</v>
-      </c>
-      <c r="W12" s="61" t="s">
-        <v>87</v>
-      </c>
-      <c r="X12" s="62" t="s">
-        <v>77</v>
-      </c>
-      <c r="Y12" s="61" t="s">
-        <v>88</v>
-      </c>
-      <c r="Z12" s="61" t="s">
-        <v>87</v>
-      </c>
-      <c r="AA12" s="61" t="s">
-        <v>85</v>
-      </c>
-      <c r="AB12" s="37" t="s">
-        <v>89</v>
-      </c>
-      <c r="AC12" s="61" t="s">
-        <v>90</v>
-      </c>
-      <c r="AD12" s="20"/>
-      <c r="AE12" s="20"/>
-      <c r="AF12" s="75"/>
+      <c r="R12" s="52"/>
+      <c r="S12" s="52" t="s">
+        <v>76</v>
+      </c>
+      <c r="T12" s="52"/>
+      <c r="U12" s="52"/>
+      <c r="V12" s="52"/>
+      <c r="W12" s="52"/>
+      <c r="X12" s="52"/>
+      <c r="Y12" s="52"/>
+      <c r="Z12" s="52"/>
+      <c r="AA12" s="52"/>
+      <c r="AB12" s="53"/>
+      <c r="AC12" s="55"/>
+      <c r="AD12" s="76"/>
+      <c r="AE12" s="76"/>
+      <c r="AF12" s="76"/>
     </row>
     <row r="13" spans="1:32" ht="18" customHeight="1">
       <c r="A13" s="108"/>
-      <c r="B13" s="96"/>
-      <c r="C13" s="11" t="s">
+      <c r="B13" s="95" t="s">
+        <v>77</v>
+      </c>
+      <c r="C13" s="61" t="s">
+        <v>78</v>
+      </c>
+      <c r="D13" s="62" t="s">
+        <v>79</v>
+      </c>
+      <c r="E13" s="63" t="s">
+        <v>80</v>
+      </c>
+      <c r="F13" s="62" t="s">
+        <v>79</v>
+      </c>
+      <c r="G13" s="62" t="s">
+        <v>79</v>
+      </c>
+      <c r="H13" s="62" t="s">
+        <v>79</v>
+      </c>
+      <c r="I13" s="61" t="s">
+        <v>81</v>
+      </c>
+      <c r="J13" s="61" t="s">
+        <v>82</v>
+      </c>
+      <c r="K13" s="37" t="s">
+        <v>83</v>
+      </c>
+      <c r="L13" s="61" t="s">
+        <v>84</v>
+      </c>
+      <c r="M13" s="62" t="s">
+        <v>79</v>
+      </c>
+      <c r="N13" s="61" t="s">
+        <v>85</v>
+      </c>
+      <c r="O13" s="61" t="s">
+        <v>86</v>
+      </c>
+      <c r="P13" s="37" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q13" s="61" t="s">
+        <v>87</v>
+      </c>
+      <c r="R13" s="37" t="s">
+        <v>88</v>
+      </c>
+      <c r="S13" s="61" t="s">
+        <v>87</v>
+      </c>
+      <c r="T13" s="61" t="s">
+        <v>87</v>
+      </c>
+      <c r="U13" s="61" t="s">
+        <v>87</v>
+      </c>
+      <c r="V13" s="62" t="s">
+        <v>79</v>
+      </c>
+      <c r="W13" s="61" t="s">
+        <v>89</v>
+      </c>
+      <c r="X13" s="62" t="s">
+        <v>79</v>
+      </c>
+      <c r="Y13" s="61" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z13" s="61" t="s">
+        <v>89</v>
+      </c>
+      <c r="AA13" s="61" t="s">
+        <v>87</v>
+      </c>
+      <c r="AB13" s="37" t="s">
         <v>91</v>
       </c>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4" t="s">
+      <c r="AC13" s="61" t="s">
         <v>92</v>
       </c>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-      <c r="I13" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="J13" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="K13" s="11" t="s">
-        <v>94</v>
-      </c>
-      <c r="L13" s="11" t="s">
-        <v>95</v>
-      </c>
-      <c r="M13" s="4"/>
-      <c r="N13" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="O13" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="P13" s="4"/>
-      <c r="Q13" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="R13" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="S13" s="11" t="s">
-        <v>97</v>
-      </c>
-      <c r="T13" s="11" t="s">
-        <v>97</v>
-      </c>
-      <c r="U13" s="12" t="s">
-        <v>89</v>
-      </c>
-      <c r="V13" s="4"/>
-      <c r="W13" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="X13" s="4"/>
-      <c r="Y13" s="12" t="s">
-        <v>99</v>
-      </c>
-      <c r="Z13" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="AA13" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="AB13" s="12" t="s">
-        <v>100</v>
-      </c>
-      <c r="AC13" s="11" t="s">
-        <v>101</v>
-      </c>
-      <c r="AD13" s="10"/>
-      <c r="AE13" s="10"/>
-      <c r="AF13" s="40"/>
+      <c r="AD13" s="20"/>
+      <c r="AE13" s="20"/>
+      <c r="AF13" s="75"/>
     </row>
     <row r="14" spans="1:32" ht="18" customHeight="1">
       <c r="A14" s="108"/>
       <c r="B14" s="96"/>
       <c r="C14" s="11" t="s">
-        <v>102</v>
+        <v>93</v>
       </c>
       <c r="D14" s="4"/>
       <c r="E14" s="4" t="s">
-        <v>103</v>
+        <v>94</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
-      <c r="I14" s="4" t="s">
-        <v>92</v>
+      <c r="I14" s="11" t="s">
+        <v>80</v>
       </c>
       <c r="J14" s="11" t="s">
-        <v>104</v>
+        <v>95</v>
       </c>
       <c r="K14" s="11" t="s">
-        <v>105</v>
+        <v>96</v>
       </c>
       <c r="L14" s="11" t="s">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="M14" s="4"/>
       <c r="N14" s="11" t="s">
-        <v>107</v>
+        <v>98</v>
       </c>
       <c r="O14" s="11" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="P14" s="4"/>
-      <c r="Q14" s="12" t="s">
+      <c r="Q14" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="R14" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="S14" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="R14" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="S14" s="4"/>
       <c r="T14" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="U14" s="11" t="s">
-        <v>98</v>
+        <v>99</v>
+      </c>
+      <c r="U14" s="12" t="s">
+        <v>91</v>
       </c>
       <c r="V14" s="4"/>
       <c r="W14" s="11" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="X14" s="4"/>
-      <c r="Y14" s="4"/>
+      <c r="Y14" s="12" t="s">
+        <v>101</v>
+      </c>
       <c r="Z14" s="11" t="s">
-        <v>108</v>
-      </c>
-      <c r="AA14" s="12" t="s">
         <v>100</v>
       </c>
+      <c r="AA14" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="AB14" s="12" t="s">
+        <v>102</v>
+      </c>
       <c r="AC14" s="11" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="AD14" s="10"/>
       <c r="AE14" s="10"/>
@@ -3065,57 +3073,62 @@
       <c r="A15" s="108"/>
       <c r="B15" s="96"/>
       <c r="C15" s="11" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="D15" s="4"/>
       <c r="E15" s="4" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
       <c r="I15" s="4" t="s">
-        <v>103</v>
+        <v>94</v>
       </c>
       <c r="J15" s="11" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="K15" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="L15" s="4"/>
+        <v>107</v>
+      </c>
+      <c r="L15" s="11" t="s">
+        <v>108</v>
+      </c>
       <c r="M15" s="4"/>
-      <c r="N15" s="4"/>
+      <c r="N15" s="11" t="s">
+        <v>109</v>
+      </c>
       <c r="O15" s="11" t="s">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="P15" s="4"/>
-      <c r="Q15" s="4" t="s">
-        <v>113</v>
+      <c r="Q15" s="12" t="s">
+        <v>101</v>
       </c>
       <c r="R15" s="11" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="S15" s="4"/>
-      <c r="T15" s="4"/>
+      <c r="T15" s="11" t="s">
+        <v>88</v>
+      </c>
       <c r="U15" s="11" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="V15" s="4"/>
       <c r="W15" s="11" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="X15" s="4"/>
       <c r="Y15" s="4"/>
       <c r="Z15" s="11" t="s">
-        <v>114</v>
-      </c>
-      <c r="AA15" s="11" t="s">
-        <v>97</v>
-      </c>
-      <c r="AB15" s="11"/>
+        <v>110</v>
+      </c>
+      <c r="AA15" s="12" t="s">
+        <v>102</v>
+      </c>
       <c r="AC15" s="11" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="AD15" s="10"/>
       <c r="AE15" s="10"/>
@@ -3125,53 +3138,57 @@
       <c r="A16" s="108"/>
       <c r="B16" s="96"/>
       <c r="C16" s="11" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
+      <c r="E16" s="4" t="s">
+        <v>113</v>
+      </c>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
       <c r="I16" s="4" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="J16" s="11" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="K16" s="11" t="s">
-        <v>118</v>
+        <v>84</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4"/>
       <c r="N16" s="4"/>
       <c r="O16" s="11" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="P16" s="4"/>
-      <c r="Q16" s="4"/>
+      <c r="Q16" s="4" t="s">
+        <v>115</v>
+      </c>
       <c r="R16" s="11" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="S16" s="4"/>
       <c r="T16" s="4"/>
       <c r="U16" s="11" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="V16" s="4"/>
       <c r="W16" s="11" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="X16" s="4"/>
       <c r="Y16" s="4"/>
       <c r="Z16" s="11" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="AA16" s="11" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="AB16" s="11"/>
       <c r="AC16" s="11" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="AD16" s="10"/>
       <c r="AE16" s="10"/>
@@ -3180,42 +3197,50 @@
     <row r="17" spans="1:155" ht="18" customHeight="1">
       <c r="A17" s="108"/>
       <c r="B17" s="96"/>
-      <c r="C17" s="4"/>
+      <c r="C17" s="11" t="s">
+        <v>118</v>
+      </c>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
-      <c r="I17" s="4"/>
+      <c r="I17" s="4" t="s">
+        <v>113</v>
+      </c>
       <c r="J17" s="11" t="s">
-        <v>121</v>
-      </c>
-      <c r="K17" s="4"/>
+        <v>119</v>
+      </c>
+      <c r="K17" s="11" t="s">
+        <v>120</v>
+      </c>
       <c r="L17" s="4"/>
       <c r="M17" s="4"/>
       <c r="N17" s="4"/>
       <c r="O17" s="11" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="P17" s="4"/>
       <c r="Q17" s="4"/>
       <c r="R17" s="11" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="S17" s="4"/>
       <c r="T17" s="4"/>
       <c r="U17" s="11" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="V17" s="4"/>
-      <c r="W17" s="12" t="s">
-        <v>99</v>
+      <c r="W17" s="11" t="s">
+        <v>121</v>
       </c>
       <c r="X17" s="4"/>
       <c r="Y17" s="4"/>
-      <c r="Z17" s="4"/>
+      <c r="Z17" s="11" t="s">
+        <v>121</v>
+      </c>
       <c r="AA17" s="11" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="AB17" s="11"/>
       <c r="AC17" s="11" t="s">
@@ -3226,478 +3251,470 @@
       <c r="AF17" s="40"/>
     </row>
     <row r="18" spans="1:155" ht="18" customHeight="1">
-      <c r="A18" s="109"/>
-      <c r="B18" s="97"/>
-      <c r="C18" s="32"/>
-      <c r="D18" s="32"/>
-      <c r="E18" s="32"/>
-      <c r="F18" s="32"/>
-      <c r="G18" s="32"/>
-      <c r="H18" s="32"/>
-      <c r="I18" s="32"/>
-      <c r="J18" s="52" t="s">
+      <c r="A18" s="108"/>
+      <c r="B18" s="96"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="4"/>
+      <c r="H18" s="4"/>
+      <c r="I18" s="4"/>
+      <c r="J18" s="11" t="s">
         <v>123</v>
       </c>
-      <c r="K18" s="32"/>
-      <c r="L18" s="32"/>
-      <c r="M18" s="32"/>
-      <c r="N18" s="32"/>
-      <c r="O18" s="52" t="s">
-        <v>108</v>
-      </c>
-      <c r="P18" s="32"/>
-      <c r="Q18" s="32"/>
-      <c r="R18" s="64" t="s">
-        <v>99</v>
-      </c>
-      <c r="S18" s="32"/>
-      <c r="T18" s="32"/>
-      <c r="U18" s="52" t="s">
-        <v>88</v>
-      </c>
-      <c r="V18" s="32"/>
-      <c r="W18" s="64" t="s">
+      <c r="K18" s="4"/>
+      <c r="L18" s="4"/>
+      <c r="M18" s="4"/>
+      <c r="N18" s="4"/>
+      <c r="O18" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="P18" s="4"/>
+      <c r="Q18" s="4"/>
+      <c r="R18" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="S18" s="4"/>
+      <c r="T18" s="4"/>
+      <c r="U18" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="V18" s="4"/>
+      <c r="W18" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="X18" s="4"/>
+      <c r="Y18" s="4"/>
+      <c r="Z18" s="4"/>
+      <c r="AA18" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="AB18" s="11"/>
+      <c r="AC18" s="11" t="s">
         <v>124</v>
       </c>
-      <c r="X18" s="32"/>
-      <c r="Y18" s="32"/>
-      <c r="Z18" s="32"/>
-      <c r="AA18" s="52" t="s">
-        <v>108</v>
-      </c>
-      <c r="AB18" s="52"/>
-      <c r="AC18" s="52"/>
-      <c r="AD18" s="31"/>
-      <c r="AE18" s="31"/>
-      <c r="AF18" s="41"/>
+      <c r="AD18" s="10"/>
+      <c r="AE18" s="10"/>
+      <c r="AF18" s="40"/>
     </row>
-    <row r="19" spans="1:155" s="3" customFormat="1" ht="89.45" customHeight="1">
-      <c r="A19" s="56" t="s">
+    <row r="19" spans="1:155" ht="18" customHeight="1">
+      <c r="A19" s="109"/>
+      <c r="B19" s="97"/>
+      <c r="C19" s="32"/>
+      <c r="D19" s="32"/>
+      <c r="E19" s="32"/>
+      <c r="F19" s="32"/>
+      <c r="G19" s="32"/>
+      <c r="H19" s="32"/>
+      <c r="I19" s="32"/>
+      <c r="J19" s="52" t="s">
         <v>125</v>
       </c>
-      <c r="B19" s="85" t="s">
+      <c r="K19" s="32"/>
+      <c r="L19" s="32"/>
+      <c r="M19" s="32"/>
+      <c r="N19" s="32"/>
+      <c r="O19" s="52" t="s">
+        <v>110</v>
+      </c>
+      <c r="P19" s="32"/>
+      <c r="Q19" s="32"/>
+      <c r="R19" s="64" t="s">
+        <v>101</v>
+      </c>
+      <c r="S19" s="32"/>
+      <c r="T19" s="32"/>
+      <c r="U19" s="52" t="s">
+        <v>90</v>
+      </c>
+      <c r="V19" s="32"/>
+      <c r="W19" s="64" t="s">
         <v>126</v>
       </c>
-      <c r="C19" s="43"/>
-      <c r="D19" s="43"/>
-      <c r="E19" s="44" t="s">
+      <c r="X19" s="32"/>
+      <c r="Y19" s="32"/>
+      <c r="Z19" s="32"/>
+      <c r="AA19" s="52" t="s">
+        <v>110</v>
+      </c>
+      <c r="AB19" s="52"/>
+      <c r="AC19" s="52"/>
+      <c r="AD19" s="31"/>
+      <c r="AE19" s="31"/>
+      <c r="AF19" s="41"/>
+    </row>
+    <row r="20" spans="1:155" s="3" customFormat="1" ht="89.45" customHeight="1">
+      <c r="A20" s="56" t="s">
         <v>127</v>
       </c>
-      <c r="F19" s="44" t="s">
+      <c r="B20" s="85" t="s">
         <v>128</v>
       </c>
-      <c r="G19" s="44" t="s">
+      <c r="C20" s="43"/>
+      <c r="D20" s="43"/>
+      <c r="E20" s="44" t="s">
         <v>129</v>
       </c>
-      <c r="H19" s="43"/>
-      <c r="I19" s="44" t="s">
+      <c r="F20" s="44" t="s">
         <v>130</v>
       </c>
-      <c r="J19" s="43" t="s">
+      <c r="G20" s="44" t="s">
         <v>131</v>
       </c>
-      <c r="K19" s="43" t="s">
+      <c r="H20" s="43"/>
+      <c r="I20" s="44" t="s">
         <v>132</v>
       </c>
-      <c r="L19" s="43" t="s">
+      <c r="J20" s="43" t="s">
         <v>133</v>
       </c>
-      <c r="M19" s="43" t="s">
+      <c r="K20" s="43" t="s">
         <v>134</v>
       </c>
-      <c r="N19" s="43"/>
-      <c r="O19" s="44" t="s">
+      <c r="L20" s="43" t="s">
         <v>135</v>
       </c>
-      <c r="P19" s="44" t="s">
+      <c r="M20" s="43" t="s">
         <v>136</v>
       </c>
-      <c r="Q19" s="44" t="s">
+      <c r="N20" s="43"/>
+      <c r="O20" s="44" t="s">
         <v>137</v>
       </c>
-      <c r="R19" s="57" t="s">
+      <c r="P20" s="44" t="s">
         <v>138</v>
       </c>
-      <c r="S19" s="58" t="s">
+      <c r="Q20" s="44" t="s">
         <v>139</v>
       </c>
-      <c r="T19" s="57"/>
-      <c r="U19" s="58" t="s">
+      <c r="R20" s="57" t="s">
         <v>140</v>
       </c>
-      <c r="V19" s="57"/>
-      <c r="W19" s="59" t="s">
+      <c r="S20" s="58" t="s">
         <v>141</v>
       </c>
-      <c r="X19" s="57"/>
-      <c r="Y19" s="58" t="s">
+      <c r="T20" s="57"/>
+      <c r="U20" s="58" t="s">
         <v>142</v>
       </c>
-      <c r="Z19" s="57"/>
-      <c r="AA19" s="58" t="s">
+      <c r="V20" s="57"/>
+      <c r="W20" s="59" t="s">
         <v>143</v>
       </c>
-      <c r="AB19" s="58" t="s">
+      <c r="X20" s="57"/>
+      <c r="Y20" s="58" t="s">
         <v>144</v>
       </c>
-      <c r="AC19" s="58" t="s">
+      <c r="Z20" s="57"/>
+      <c r="AA20" s="58" t="s">
         <v>145</v>
       </c>
-      <c r="AD19" s="57"/>
-      <c r="AE19" s="57"/>
-      <c r="AF19" s="60"/>
+      <c r="AB20" s="58" t="s">
+        <v>146</v>
+      </c>
+      <c r="AC20" s="58" t="s">
+        <v>147</v>
+      </c>
+      <c r="AD20" s="57"/>
+      <c r="AE20" s="57"/>
+      <c r="AF20" s="60"/>
     </row>
-    <row r="20" spans="1:155" s="1" customFormat="1" ht="36" customHeight="1">
-      <c r="A20" s="21"/>
-      <c r="B20" s="92" t="s">
-        <v>146</v>
-      </c>
-      <c r="C20" s="22" t="s">
-        <v>147</v>
-      </c>
-      <c r="D20" s="22" t="s">
+    <row r="21" spans="1:155" s="1" customFormat="1" ht="36" customHeight="1">
+      <c r="A21" s="21"/>
+      <c r="B21" s="92" t="s">
         <v>148</v>
       </c>
-      <c r="E20" s="22" t="s">
+      <c r="C21" s="22" t="s">
         <v>149</v>
       </c>
-      <c r="F20" s="22" t="s">
+      <c r="D21" s="22" t="s">
         <v>150</v>
       </c>
-      <c r="G20" s="22" t="s">
+      <c r="E21" s="22" t="s">
         <v>151</v>
       </c>
-      <c r="H20" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="I20" s="22" t="s">
+      <c r="F21" s="22" t="s">
         <v>152</v>
       </c>
-      <c r="J20" s="22" t="s">
+      <c r="G21" s="22" t="s">
         <v>153</v>
       </c>
-      <c r="K20" s="22" t="s">
+      <c r="H21" s="22" t="s">
+        <v>153</v>
+      </c>
+      <c r="I21" s="22" t="s">
         <v>154</v>
       </c>
-      <c r="L20" s="22" t="s">
+      <c r="J21" s="22" t="s">
         <v>155</v>
       </c>
-      <c r="M20" s="22" t="s">
+      <c r="K21" s="22" t="s">
         <v>156</v>
       </c>
-      <c r="N20" s="22" t="s">
+      <c r="L21" s="22" t="s">
         <v>157</v>
       </c>
-      <c r="O20" s="22" t="s">
+      <c r="M21" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="P20" s="22" t="s">
+      <c r="N21" s="22" t="s">
         <v>159</v>
       </c>
-      <c r="Q20" s="22" t="s">
+      <c r="O21" s="22" t="s">
         <v>160</v>
       </c>
-      <c r="R20" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="S20" s="22" t="s">
+      <c r="P21" s="22" t="s">
         <v>161</v>
       </c>
-      <c r="T20" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="U20" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="V20" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="W20" s="22" t="s">
+      <c r="Q21" s="22" t="s">
         <v>162</v>
       </c>
-      <c r="X20" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="Y20" s="22" t="s">
+      <c r="R21" s="22" t="s">
+        <v>153</v>
+      </c>
+      <c r="S21" s="22" t="s">
         <v>163</v>
       </c>
-      <c r="Z20" s="22" t="s">
+      <c r="T21" s="22" t="s">
+        <v>153</v>
+      </c>
+      <c r="U21" s="22" t="s">
+        <v>153</v>
+      </c>
+      <c r="V21" s="22" t="s">
+        <v>153</v>
+      </c>
+      <c r="W21" s="22" t="s">
         <v>164</v>
       </c>
-      <c r="AA20" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="AB20" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="AC20" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="AD20" s="22" t="s">
+      <c r="X21" s="22" t="s">
+        <v>153</v>
+      </c>
+      <c r="Y21" s="22" t="s">
         <v>165</v>
       </c>
-      <c r="AE20" s="22" t="s">
+      <c r="Z21" s="22" t="s">
         <v>166</v>
       </c>
-      <c r="AF20" s="23" t="s">
+      <c r="AA21" s="22" t="s">
+        <v>153</v>
+      </c>
+      <c r="AB21" s="22" t="s">
+        <v>153</v>
+      </c>
+      <c r="AC21" s="22" t="s">
+        <v>153</v>
+      </c>
+      <c r="AD21" s="22" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="21" spans="1:155" ht="18" customHeight="1">
-      <c r="A21" s="24"/>
-      <c r="B21" s="93"/>
-      <c r="C21" s="25" t="s">
+      <c r="AE21" s="22" t="s">
         <v>168</v>
       </c>
-      <c r="D21" s="25" t="s">
+      <c r="AF21" s="23" t="s">
         <v>169</v>
-      </c>
-      <c r="E21" s="25" t="s">
-        <v>170</v>
-      </c>
-      <c r="F21" s="25" t="s">
-        <v>171</v>
-      </c>
-      <c r="G21" s="4"/>
-      <c r="H21" s="4"/>
-      <c r="I21" s="13" t="s">
-        <v>172</v>
-      </c>
-      <c r="J21" s="13" t="s">
-        <v>173</v>
-      </c>
-      <c r="K21" s="13" t="s">
-        <v>174</v>
-      </c>
-      <c r="L21" s="14"/>
-      <c r="M21" s="13" t="s">
-        <v>175</v>
-      </c>
-      <c r="N21" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="O21" s="13" t="s">
-        <v>177</v>
-      </c>
-      <c r="P21" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q21" s="13" t="s">
-        <v>179</v>
-      </c>
-      <c r="R21" s="14"/>
-      <c r="S21" s="13" t="s">
-        <v>179</v>
-      </c>
-      <c r="T21" s="14"/>
-      <c r="U21" s="4"/>
-      <c r="V21" s="4"/>
-      <c r="W21" s="13" t="s">
-        <v>180</v>
-      </c>
-      <c r="X21" s="4"/>
-      <c r="Y21" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="Z21" s="13" t="s">
-        <v>182</v>
-      </c>
-      <c r="AA21" s="4"/>
-      <c r="AB21" s="4"/>
-      <c r="AC21" s="4"/>
-      <c r="AD21" s="13" t="s">
-        <v>183</v>
-      </c>
-      <c r="AE21" s="13" t="s">
-        <v>184</v>
-      </c>
-      <c r="AF21" s="26" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="22" spans="1:155" ht="18" customHeight="1">
       <c r="A22" s="24"/>
       <c r="B22" s="93"/>
       <c r="C22" s="25" t="s">
-        <v>186</v>
+        <v>170</v>
       </c>
       <c r="D22" s="25" t="s">
-        <v>187</v>
+        <v>171</v>
       </c>
       <c r="E22" s="25" t="s">
-        <v>188</v>
-      </c>
-      <c r="F22" s="4"/>
+        <v>172</v>
+      </c>
+      <c r="F22" s="25" t="s">
+        <v>173</v>
+      </c>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
-      <c r="I22" s="14"/>
+      <c r="I22" s="13" t="s">
+        <v>174</v>
+      </c>
       <c r="J22" s="13" t="s">
-        <v>189</v>
-      </c>
-      <c r="K22" s="14"/>
-      <c r="L22" s="13" t="s">
-        <v>190</v>
-      </c>
+        <v>175</v>
+      </c>
+      <c r="K22" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="L22" s="14"/>
       <c r="M22" s="13" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="N22" s="13" t="s">
-        <v>191</v>
+        <v>178</v>
       </c>
       <c r="O22" s="13" t="s">
-        <v>192</v>
+        <v>179</v>
       </c>
       <c r="P22" s="13" t="s">
-        <v>193</v>
+        <v>180</v>
       </c>
       <c r="Q22" s="13" t="s">
-        <v>194</v>
+        <v>181</v>
       </c>
       <c r="R22" s="14"/>
       <c r="S22" s="13" t="s">
-        <v>194</v>
+        <v>181</v>
       </c>
       <c r="T22" s="14"/>
       <c r="U22" s="4"/>
       <c r="V22" s="4"/>
       <c r="W22" s="13" t="s">
-        <v>195</v>
+        <v>182</v>
       </c>
       <c r="X22" s="4"/>
       <c r="Y22" s="13" t="s">
-        <v>196</v>
-      </c>
-      <c r="Z22" s="13"/>
+        <v>183</v>
+      </c>
+      <c r="Z22" s="13" t="s">
+        <v>184</v>
+      </c>
       <c r="AA22" s="4"/>
       <c r="AB22" s="4"/>
       <c r="AC22" s="4"/>
       <c r="AD22" s="13" t="s">
-        <v>197</v>
+        <v>185</v>
       </c>
       <c r="AE22" s="13" t="s">
-        <v>198</v>
+        <v>186</v>
       </c>
       <c r="AF22" s="26" t="s">
-        <v>199</v>
+        <v>187</v>
       </c>
     </row>
     <row r="23" spans="1:155" ht="18" customHeight="1">
       <c r="A23" s="24"/>
       <c r="B23" s="93"/>
       <c r="C23" s="25" t="s">
-        <v>200</v>
+        <v>188</v>
       </c>
       <c r="D23" s="25" t="s">
-        <v>201</v>
-      </c>
-      <c r="E23" s="4"/>
+        <v>189</v>
+      </c>
+      <c r="E23" s="25" t="s">
+        <v>190</v>
+      </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
       <c r="I23" s="14"/>
       <c r="J23" s="13" t="s">
-        <v>176</v>
+        <v>191</v>
       </c>
       <c r="K23" s="14"/>
       <c r="L23" s="13" t="s">
-        <v>202</v>
+        <v>192</v>
       </c>
       <c r="M23" s="13" t="s">
-        <v>191</v>
+        <v>178</v>
       </c>
       <c r="N23" s="13" t="s">
-        <v>203</v>
+        <v>193</v>
       </c>
       <c r="O23" s="13" t="s">
-        <v>204</v>
-      </c>
-      <c r="P23" s="14"/>
+        <v>194</v>
+      </c>
+      <c r="P23" s="13" t="s">
+        <v>195</v>
+      </c>
       <c r="Q23" s="13" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="R23" s="14"/>
       <c r="S23" s="13" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="T23" s="14"/>
       <c r="U23" s="4"/>
       <c r="V23" s="4"/>
       <c r="W23" s="13" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="X23" s="4"/>
       <c r="Y23" s="13" t="s">
-        <v>189</v>
-      </c>
-      <c r="Z23" s="14"/>
+        <v>198</v>
+      </c>
+      <c r="Z23" s="13"/>
       <c r="AA23" s="4"/>
       <c r="AB23" s="4"/>
       <c r="AC23" s="4"/>
       <c r="AD23" s="13" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="AE23" s="13" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="AF23" s="26" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
     </row>
     <row r="24" spans="1:155" ht="18" customHeight="1">
       <c r="A24" s="24"/>
       <c r="B24" s="93"/>
-      <c r="C24" s="4"/>
-      <c r="D24" s="4"/>
+      <c r="C24" s="25" t="s">
+        <v>202</v>
+      </c>
+      <c r="D24" s="25" t="s">
+        <v>203</v>
+      </c>
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
       <c r="I24" s="14"/>
       <c r="J24" s="13" t="s">
-        <v>191</v>
+        <v>178</v>
       </c>
       <c r="K24" s="14"/>
       <c r="L24" s="13" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="M24" s="13" t="s">
-        <v>210</v>
+        <v>193</v>
       </c>
       <c r="N24" s="13" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="O24" s="13" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="P24" s="14"/>
       <c r="Q24" s="13" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="R24" s="14"/>
       <c r="S24" s="13" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="T24" s="14"/>
       <c r="U24" s="4"/>
       <c r="V24" s="4"/>
       <c r="W24" s="13" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="X24" s="4"/>
       <c r="Y24" s="13" t="s">
-        <v>176</v>
+        <v>191</v>
       </c>
       <c r="Z24" s="14"/>
       <c r="AA24" s="4"/>
       <c r="AB24" s="4"/>
       <c r="AC24" s="4"/>
       <c r="AD24" s="13" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="AE24" s="13" t="s">
-        <v>214</v>
-      </c>
-      <c r="AF24" s="27"/>
+        <v>209</v>
+      </c>
+      <c r="AF24" s="26" t="s">
+        <v>210</v>
+      </c>
     </row>
     <row r="25" spans="1:155" ht="18" customHeight="1">
       <c r="A25" s="24"/>
@@ -3710,331 +3727,188 @@
       <c r="H25" s="4"/>
       <c r="I25" s="14"/>
       <c r="J25" s="13" t="s">
-        <v>210</v>
+        <v>193</v>
       </c>
       <c r="K25" s="14"/>
       <c r="L25" s="13" t="s">
-        <v>215</v>
-      </c>
-      <c r="M25" s="14"/>
-      <c r="N25" s="14"/>
+        <v>211</v>
+      </c>
+      <c r="M25" s="13" t="s">
+        <v>212</v>
+      </c>
+      <c r="N25" s="13" t="s">
+        <v>212</v>
+      </c>
       <c r="O25" s="13" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="P25" s="14"/>
       <c r="Q25" s="13" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="R25" s="14"/>
       <c r="S25" s="13" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="T25" s="14"/>
       <c r="U25" s="4"/>
       <c r="V25" s="4"/>
       <c r="W25" s="13" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="X25" s="4"/>
       <c r="Y25" s="13" t="s">
-        <v>191</v>
+        <v>178</v>
       </c>
       <c r="Z25" s="14"/>
       <c r="AA25" s="4"/>
       <c r="AB25" s="4"/>
       <c r="AC25" s="4"/>
       <c r="AD25" s="13" t="s">
-        <v>168</v>
+        <v>215</v>
       </c>
       <c r="AE25" s="13" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="AF25" s="27"/>
     </row>
     <row r="26" spans="1:155" ht="18" customHeight="1">
-      <c r="A26" s="28"/>
+      <c r="A26" s="24"/>
       <c r="B26" s="93"/>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
-      <c r="E26" s="6"/>
-      <c r="F26" s="6"/>
-      <c r="G26" s="6"/>
-      <c r="H26" s="6"/>
-      <c r="I26" s="17"/>
-      <c r="J26" s="18" t="s">
-        <v>203</v>
-      </c>
-      <c r="K26" s="17"/>
-      <c r="L26" s="18" t="s">
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4"/>
+      <c r="F26" s="4"/>
+      <c r="G26" s="4"/>
+      <c r="H26" s="4"/>
+      <c r="I26" s="14"/>
+      <c r="J26" s="13" t="s">
+        <v>212</v>
+      </c>
+      <c r="K26" s="14"/>
+      <c r="L26" s="13" t="s">
+        <v>217</v>
+      </c>
+      <c r="M26" s="14"/>
+      <c r="N26" s="14"/>
+      <c r="O26" s="13" t="s">
+        <v>218</v>
+      </c>
+      <c r="P26" s="14"/>
+      <c r="Q26" s="13" t="s">
+        <v>218</v>
+      </c>
+      <c r="R26" s="14"/>
+      <c r="S26" s="13" t="s">
+        <v>218</v>
+      </c>
+      <c r="T26" s="14"/>
+      <c r="U26" s="4"/>
+      <c r="V26" s="4"/>
+      <c r="W26" s="13" t="s">
         <v>219</v>
       </c>
-      <c r="M26" s="17"/>
-      <c r="N26" s="17"/>
-      <c r="O26" s="18" t="s">
+      <c r="X26" s="4"/>
+      <c r="Y26" s="13" t="s">
+        <v>193</v>
+      </c>
+      <c r="Z26" s="14"/>
+      <c r="AA26" s="4"/>
+      <c r="AB26" s="4"/>
+      <c r="AC26" s="4"/>
+      <c r="AD26" s="13" t="s">
+        <v>170</v>
+      </c>
+      <c r="AE26" s="13" t="s">
         <v>220</v>
       </c>
-      <c r="P26" s="17"/>
-      <c r="Q26" s="18" t="s">
+      <c r="AF26" s="27"/>
+    </row>
+    <row r="27" spans="1:155" ht="18" customHeight="1">
+      <c r="A27" s="28"/>
+      <c r="B27" s="93"/>
+      <c r="C27" s="6"/>
+      <c r="D27" s="6"/>
+      <c r="E27" s="6"/>
+      <c r="F27" s="6"/>
+      <c r="G27" s="6"/>
+      <c r="H27" s="6"/>
+      <c r="I27" s="17"/>
+      <c r="J27" s="18" t="s">
+        <v>205</v>
+      </c>
+      <c r="K27" s="17"/>
+      <c r="L27" s="18" t="s">
         <v>221</v>
       </c>
-      <c r="R26" s="17"/>
-      <c r="S26" s="18" t="s">
-        <v>221</v>
-      </c>
-      <c r="T26" s="17"/>
-      <c r="U26" s="6"/>
-      <c r="V26" s="6"/>
-      <c r="W26" s="6"/>
-      <c r="X26" s="6"/>
-      <c r="Y26" s="18" t="s">
-        <v>203</v>
-      </c>
-      <c r="Z26" s="17"/>
-      <c r="AA26" s="6"/>
-      <c r="AB26" s="6"/>
-      <c r="AC26" s="6"/>
-      <c r="AD26" s="18" t="s">
-        <v>186</v>
-      </c>
-      <c r="AE26" s="17"/>
-      <c r="AF26" s="29"/>
+      <c r="M27" s="17"/>
+      <c r="N27" s="17"/>
+      <c r="O27" s="18" t="s">
+        <v>222</v>
+      </c>
+      <c r="P27" s="17"/>
+      <c r="Q27" s="18" t="s">
+        <v>223</v>
+      </c>
+      <c r="R27" s="17"/>
+      <c r="S27" s="18" t="s">
+        <v>223</v>
+      </c>
+      <c r="T27" s="17"/>
+      <c r="U27" s="6"/>
+      <c r="V27" s="6"/>
+      <c r="W27" s="6"/>
+      <c r="X27" s="6"/>
+      <c r="Y27" s="18" t="s">
+        <v>205</v>
+      </c>
+      <c r="Z27" s="17"/>
+      <c r="AA27" s="6"/>
+      <c r="AB27" s="6"/>
+      <c r="AC27" s="6"/>
+      <c r="AD27" s="18" t="s">
+        <v>188</v>
+      </c>
+      <c r="AE27" s="17"/>
+      <c r="AF27" s="29"/>
     </row>
-    <row r="27" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1">
-      <c r="A27" s="30"/>
-      <c r="B27" s="94"/>
-      <c r="C27" s="32"/>
-      <c r="D27" s="32"/>
-      <c r="E27" s="32"/>
-      <c r="F27" s="32"/>
-      <c r="G27" s="32"/>
-      <c r="H27" s="32"/>
-      <c r="I27" s="32"/>
-      <c r="J27" s="32"/>
-      <c r="K27" s="32"/>
-      <c r="L27" s="32"/>
-      <c r="M27" s="32"/>
-      <c r="N27" s="32"/>
-      <c r="O27" s="32"/>
-      <c r="P27" s="32"/>
-      <c r="Q27" s="32"/>
-      <c r="R27" s="32"/>
-      <c r="S27" s="32"/>
-      <c r="T27" s="32"/>
-      <c r="U27" s="32"/>
-      <c r="V27" s="32"/>
-      <c r="W27" s="32"/>
-      <c r="X27" s="32"/>
-      <c r="Y27" s="33" t="s">
-        <v>174</v>
-      </c>
-      <c r="Z27" s="34"/>
-      <c r="AA27" s="32"/>
-      <c r="AB27" s="32"/>
-      <c r="AC27" s="32"/>
-      <c r="AD27" s="33" t="s">
-        <v>174</v>
-      </c>
-      <c r="AE27" s="34"/>
-      <c r="AF27" s="35"/>
-      <c r="AG27" s="2"/>
-      <c r="AH27" s="2"/>
-      <c r="AI27" s="2"/>
-      <c r="AJ27" s="2"/>
-      <c r="AK27" s="2"/>
-      <c r="AL27" s="2"/>
-      <c r="AM27" s="2"/>
-      <c r="AN27" s="2"/>
-      <c r="AO27" s="2"/>
-      <c r="AP27" s="2"/>
-      <c r="AQ27" s="2"/>
-      <c r="AR27" s="2"/>
-      <c r="AS27" s="2"/>
-      <c r="AT27" s="2"/>
-      <c r="AU27" s="2"/>
-      <c r="AV27" s="2"/>
-      <c r="AW27" s="2"/>
-      <c r="AX27" s="2"/>
-      <c r="AY27" s="2"/>
-      <c r="AZ27" s="2"/>
-      <c r="BA27" s="2"/>
-      <c r="BB27" s="2"/>
-      <c r="BC27" s="2"/>
-      <c r="BD27" s="2"/>
-      <c r="BE27" s="2"/>
-      <c r="BF27" s="2"/>
-      <c r="BG27" s="2"/>
-      <c r="BH27" s="2"/>
-      <c r="BI27" s="2"/>
-      <c r="BJ27" s="2"/>
-      <c r="BK27" s="2"/>
-      <c r="BL27" s="2"/>
-      <c r="BM27" s="2"/>
-      <c r="BN27" s="2"/>
-      <c r="BO27" s="2"/>
-      <c r="BP27" s="2"/>
-      <c r="BQ27" s="2"/>
-      <c r="BR27" s="2"/>
-      <c r="BS27" s="2"/>
-      <c r="BT27" s="2"/>
-      <c r="BU27" s="2"/>
-      <c r="BV27" s="2"/>
-      <c r="BW27" s="2"/>
-      <c r="BX27" s="2"/>
-      <c r="BY27" s="2"/>
-      <c r="BZ27" s="2"/>
-      <c r="CA27" s="2"/>
-      <c r="CB27" s="2"/>
-      <c r="CC27" s="2"/>
-      <c r="CD27" s="2"/>
-      <c r="CE27" s="2"/>
-      <c r="CF27" s="2"/>
-      <c r="CG27" s="2"/>
-      <c r="CH27" s="2"/>
-      <c r="CI27" s="2"/>
-      <c r="CJ27" s="2"/>
-      <c r="CK27" s="2"/>
-      <c r="CL27" s="2"/>
-      <c r="CM27" s="2"/>
-      <c r="CN27" s="2"/>
-      <c r="CO27" s="2"/>
-      <c r="CP27" s="2"/>
-      <c r="CQ27" s="2"/>
-      <c r="CR27" s="2"/>
-      <c r="CS27" s="2"/>
-      <c r="CT27" s="2"/>
-      <c r="CU27" s="2"/>
-      <c r="CV27" s="2"/>
-      <c r="CW27" s="2"/>
-      <c r="CX27" s="2"/>
-      <c r="CY27" s="2"/>
-      <c r="CZ27" s="2"/>
-      <c r="DA27" s="2"/>
-      <c r="DB27" s="2"/>
-      <c r="DC27" s="2"/>
-      <c r="DD27" s="2"/>
-      <c r="DE27" s="2"/>
-      <c r="DF27" s="2"/>
-      <c r="DG27" s="2"/>
-      <c r="DH27" s="2"/>
-      <c r="DI27" s="2"/>
-      <c r="DJ27" s="2"/>
-      <c r="DK27" s="2"/>
-      <c r="DL27" s="2"/>
-      <c r="DM27" s="2"/>
-      <c r="DN27" s="2"/>
-      <c r="DO27" s="2"/>
-      <c r="DP27" s="2"/>
-      <c r="DQ27" s="2"/>
-      <c r="DR27" s="2"/>
-      <c r="DS27" s="2"/>
-      <c r="DT27" s="2"/>
-      <c r="DU27" s="2"/>
-      <c r="DV27" s="2"/>
-      <c r="DW27" s="2"/>
-      <c r="DX27" s="2"/>
-      <c r="DY27" s="2"/>
-      <c r="DZ27" s="2"/>
-      <c r="EA27" s="2"/>
-      <c r="EB27" s="2"/>
-      <c r="EC27" s="2"/>
-      <c r="ED27" s="2"/>
-      <c r="EE27" s="2"/>
-      <c r="EF27" s="2"/>
-      <c r="EG27" s="2"/>
-      <c r="EH27" s="2"/>
-      <c r="EI27" s="2"/>
-      <c r="EJ27" s="2"/>
-      <c r="EK27" s="2"/>
-      <c r="EL27" s="2"/>
-      <c r="EM27" s="2"/>
-      <c r="EN27" s="2"/>
-      <c r="EO27" s="2"/>
-      <c r="EP27" s="2"/>
-      <c r="EQ27" s="2"/>
-      <c r="ER27" s="2"/>
-      <c r="ES27" s="2"/>
-      <c r="ET27" s="2"/>
-      <c r="EU27" s="2"/>
-      <c r="EV27" s="2"/>
-      <c r="EW27" s="2"/>
-      <c r="EX27" s="2"/>
-      <c r="EY27" s="2"/>
-    </row>
-    <row r="28" spans="1:155" s="10" customFormat="1" ht="36" customHeight="1">
-      <c r="A28" s="21"/>
-      <c r="B28" s="99" t="s">
-        <v>222</v>
-      </c>
-      <c r="C28" s="36" t="s">
-        <v>223</v>
-      </c>
-      <c r="D28" s="36" t="s">
-        <v>223</v>
-      </c>
-      <c r="E28" s="36" t="s">
-        <v>224</v>
-      </c>
-      <c r="F28" s="36" t="s">
-        <v>225</v>
-      </c>
-      <c r="G28" s="36" t="s">
-        <v>226</v>
-      </c>
-      <c r="H28" s="37"/>
-      <c r="I28" s="36" t="s">
-        <v>227</v>
-      </c>
-      <c r="J28" s="36" t="s">
-        <v>228</v>
-      </c>
-      <c r="K28" s="36" t="s">
-        <v>229</v>
-      </c>
-      <c r="L28" s="36" t="s">
-        <v>230</v>
-      </c>
-      <c r="M28" s="36" t="s">
-        <v>231</v>
-      </c>
-      <c r="N28" s="36" t="s">
-        <v>232</v>
-      </c>
-      <c r="O28" s="36" t="s">
-        <v>233</v>
-      </c>
-      <c r="P28" s="36" t="s">
-        <v>234</v>
-      </c>
-      <c r="Q28" s="36" t="s">
-        <v>235</v>
-      </c>
-      <c r="R28" s="36" t="s">
-        <v>227</v>
-      </c>
-      <c r="S28" s="36" t="s">
-        <v>233</v>
-      </c>
-      <c r="T28" s="37"/>
-      <c r="U28" s="36" t="s">
-        <v>233</v>
-      </c>
-      <c r="V28" s="37"/>
-      <c r="W28" s="36" t="s">
-        <v>236</v>
-      </c>
-      <c r="X28" s="37"/>
-      <c r="Y28" s="37"/>
-      <c r="Z28" s="36" t="s">
-        <v>237</v>
-      </c>
-      <c r="AA28" s="37" t="s">
-        <v>238</v>
-      </c>
-      <c r="AB28" s="37"/>
-      <c r="AC28" s="37"/>
-      <c r="AD28" s="38"/>
-      <c r="AE28" s="38"/>
-      <c r="AF28" s="39"/>
+    <row r="28" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1">
+      <c r="A28" s="30"/>
+      <c r="B28" s="94"/>
+      <c r="C28" s="32"/>
+      <c r="D28" s="32"/>
+      <c r="E28" s="32"/>
+      <c r="F28" s="32"/>
+      <c r="G28" s="32"/>
+      <c r="H28" s="32"/>
+      <c r="I28" s="32"/>
+      <c r="J28" s="32"/>
+      <c r="K28" s="32"/>
+      <c r="L28" s="32"/>
+      <c r="M28" s="32"/>
+      <c r="N28" s="32"/>
+      <c r="O28" s="32"/>
+      <c r="P28" s="32"/>
+      <c r="Q28" s="32"/>
+      <c r="R28" s="32"/>
+      <c r="S28" s="32"/>
+      <c r="T28" s="32"/>
+      <c r="U28" s="32"/>
+      <c r="V28" s="32"/>
+      <c r="W28" s="32"/>
+      <c r="X28" s="32"/>
+      <c r="Y28" s="33" t="s">
+        <v>176</v>
+      </c>
+      <c r="Z28" s="34"/>
+      <c r="AA28" s="32"/>
+      <c r="AB28" s="32"/>
+      <c r="AC28" s="32"/>
+      <c r="AD28" s="33" t="s">
+        <v>176</v>
+      </c>
+      <c r="AE28" s="34"/>
+      <c r="AF28" s="35"/>
       <c r="AG28" s="2"/>
       <c r="AH28" s="2"/>
       <c r="AI28" s="2"/>
@@ -4159,69 +4033,81 @@
       <c r="EX28" s="2"/>
       <c r="EY28" s="2"/>
     </row>
-    <row r="29" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1">
-      <c r="A29" s="24"/>
-      <c r="B29" s="100"/>
-      <c r="C29" s="13" t="s">
+    <row r="29" spans="1:155" s="10" customFormat="1" ht="36" customHeight="1">
+      <c r="A29" s="21"/>
+      <c r="B29" s="99" t="s">
+        <v>224</v>
+      </c>
+      <c r="C29" s="36" t="s">
+        <v>225</v>
+      </c>
+      <c r="D29" s="36" t="s">
+        <v>225</v>
+      </c>
+      <c r="E29" s="36" t="s">
+        <v>226</v>
+      </c>
+      <c r="F29" s="36" t="s">
+        <v>227</v>
+      </c>
+      <c r="G29" s="36" t="s">
+        <v>228</v>
+      </c>
+      <c r="H29" s="37"/>
+      <c r="I29" s="36" t="s">
+        <v>229</v>
+      </c>
+      <c r="J29" s="36" t="s">
+        <v>230</v>
+      </c>
+      <c r="K29" s="36" t="s">
+        <v>231</v>
+      </c>
+      <c r="L29" s="36" t="s">
+        <v>232</v>
+      </c>
+      <c r="M29" s="36" t="s">
+        <v>233</v>
+      </c>
+      <c r="N29" s="36" t="s">
+        <v>234</v>
+      </c>
+      <c r="O29" s="36" t="s">
+        <v>235</v>
+      </c>
+      <c r="P29" s="36" t="s">
+        <v>236</v>
+      </c>
+      <c r="Q29" s="36" t="s">
+        <v>237</v>
+      </c>
+      <c r="R29" s="36" t="s">
+        <v>229</v>
+      </c>
+      <c r="S29" s="36" t="s">
+        <v>235</v>
+      </c>
+      <c r="T29" s="37"/>
+      <c r="U29" s="36" t="s">
+        <v>235</v>
+      </c>
+      <c r="V29" s="37"/>
+      <c r="W29" s="36" t="s">
+        <v>238</v>
+      </c>
+      <c r="X29" s="37"/>
+      <c r="Y29" s="37"/>
+      <c r="Z29" s="36" t="s">
         <v>239</v>
       </c>
-      <c r="D29" s="13" t="s">
-        <v>239</v>
-      </c>
-      <c r="E29" s="4"/>
-      <c r="F29" s="13" t="s">
+      <c r="AA29" s="37" t="s">
         <v>240</v>
       </c>
-      <c r="G29" s="13" t="s">
-        <v>239</v>
-      </c>
-      <c r="H29" s="4"/>
-      <c r="I29" s="4"/>
-      <c r="J29" s="13" t="s">
-        <v>241</v>
-      </c>
-      <c r="K29" s="13" t="s">
-        <v>242</v>
-      </c>
-      <c r="L29" s="13" t="s">
-        <v>243</v>
-      </c>
-      <c r="M29" s="13" t="s">
-        <v>244</v>
-      </c>
-      <c r="N29" s="13" t="s">
-        <v>245</v>
-      </c>
-      <c r="O29" s="13" t="s">
-        <v>246</v>
-      </c>
-      <c r="P29" s="13" t="s">
-        <v>247</v>
-      </c>
-      <c r="Q29" s="13" t="s">
-        <v>248</v>
-      </c>
-      <c r="R29" s="14"/>
-      <c r="S29" s="13" t="s">
-        <v>246</v>
-      </c>
-      <c r="T29" s="4"/>
-      <c r="U29" s="13" t="s">
-        <v>246</v>
-      </c>
-      <c r="V29" s="4"/>
-      <c r="W29" s="13" t="s">
-        <v>249</v>
-      </c>
-      <c r="X29" s="4"/>
-      <c r="Y29" s="4"/>
-      <c r="Z29" s="13" t="s">
-        <v>250</v>
-      </c>
-      <c r="AA29" s="4"/>
-      <c r="AB29" s="4"/>
-      <c r="AC29" s="4"/>
-      <c r="AF29" s="40"/>
+      <c r="AB29" s="37"/>
+      <c r="AC29" s="37"/>
+      <c r="AD29" s="38"/>
+      <c r="AE29" s="38"/>
+      <c r="AF29" s="39"/>
       <c r="AG29" s="2"/>
       <c r="AH29" s="2"/>
       <c r="AI29" s="2"/>
@@ -4350,55 +4236,61 @@
       <c r="A30" s="24"/>
       <c r="B30" s="100"/>
       <c r="C30" s="13" t="s">
-        <v>251</v>
+        <v>241</v>
       </c>
       <c r="D30" s="13" t="s">
-        <v>251</v>
+        <v>241</v>
       </c>
       <c r="E30" s="4"/>
       <c r="F30" s="13" t="s">
-        <v>252</v>
+        <v>242</v>
       </c>
       <c r="G30" s="13" t="s">
-        <v>251</v>
+        <v>241</v>
       </c>
       <c r="H30" s="4"/>
       <c r="I30" s="4"/>
       <c r="J30" s="13" t="s">
-        <v>253</v>
+        <v>243</v>
       </c>
       <c r="K30" s="13" t="s">
-        <v>254</v>
+        <v>244</v>
       </c>
       <c r="L30" s="13" t="s">
-        <v>255</v>
-      </c>
-      <c r="M30" s="14"/>
+        <v>245</v>
+      </c>
+      <c r="M30" s="13" t="s">
+        <v>246</v>
+      </c>
       <c r="N30" s="13" t="s">
-        <v>256</v>
+        <v>247</v>
       </c>
       <c r="O30" s="13" t="s">
-        <v>257</v>
-      </c>
-      <c r="P30" s="14"/>
+        <v>248</v>
+      </c>
+      <c r="P30" s="13" t="s">
+        <v>249</v>
+      </c>
       <c r="Q30" s="13" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="R30" s="14"/>
       <c r="S30" s="13" t="s">
-        <v>257</v>
+        <v>248</v>
       </c>
       <c r="T30" s="4"/>
       <c r="U30" s="13" t="s">
-        <v>257</v>
+        <v>248</v>
       </c>
       <c r="V30" s="4"/>
       <c r="W30" s="13" t="s">
-        <v>259</v>
+        <v>251</v>
       </c>
       <c r="X30" s="4"/>
       <c r="Y30" s="4"/>
-      <c r="Z30" s="14"/>
+      <c r="Z30" s="13" t="s">
+        <v>252</v>
+      </c>
       <c r="AA30" s="4"/>
       <c r="AB30" s="4"/>
       <c r="AC30" s="4"/>
@@ -4531,43 +4423,55 @@
       <c r="A31" s="24"/>
       <c r="B31" s="100"/>
       <c r="C31" s="13" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="D31" s="13" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="E31" s="4"/>
-      <c r="F31" s="4"/>
+      <c r="F31" s="13" t="s">
+        <v>254</v>
+      </c>
       <c r="G31" s="13" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="H31" s="4"/>
       <c r="I31" s="4"/>
-      <c r="J31" s="14"/>
-      <c r="K31" s="14"/>
-      <c r="L31" s="14"/>
+      <c r="J31" s="13" t="s">
+        <v>255</v>
+      </c>
+      <c r="K31" s="13" t="s">
+        <v>256</v>
+      </c>
+      <c r="L31" s="13" t="s">
+        <v>257</v>
+      </c>
       <c r="M31" s="14"/>
-      <c r="N31" s="14"/>
+      <c r="N31" s="13" t="s">
+        <v>258</v>
+      </c>
       <c r="O31" s="13" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="P31" s="14"/>
-      <c r="Q31" s="14"/>
+      <c r="Q31" s="13" t="s">
+        <v>260</v>
+      </c>
       <c r="R31" s="14"/>
       <c r="S31" s="13" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="T31" s="4"/>
       <c r="U31" s="13" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="V31" s="4"/>
       <c r="W31" s="13" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="X31" s="4"/>
       <c r="Y31" s="4"/>
-      <c r="Z31" s="4"/>
+      <c r="Z31" s="14"/>
       <c r="AA31" s="4"/>
       <c r="AB31" s="4"/>
       <c r="AC31" s="4"/>
@@ -4700,15 +4604,15 @@
       <c r="A32" s="24"/>
       <c r="B32" s="100"/>
       <c r="C32" s="13" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D32" s="13" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E32" s="4"/>
       <c r="F32" s="4"/>
       <c r="G32" s="13" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="H32" s="4"/>
       <c r="I32" s="4"/>
@@ -4718,21 +4622,21 @@
       <c r="M32" s="14"/>
       <c r="N32" s="14"/>
       <c r="O32" s="13" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="P32" s="14"/>
       <c r="Q32" s="14"/>
       <c r="R32" s="14"/>
       <c r="S32" s="13" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="T32" s="4"/>
       <c r="U32" s="13" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="V32" s="4"/>
       <c r="W32" s="13" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="X32" s="4"/>
       <c r="Y32" s="4"/>
@@ -4866,44 +4770,50 @@
       <c r="EY32" s="2"/>
     </row>
     <row r="33" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1">
-      <c r="A33" s="30"/>
-      <c r="B33" s="101"/>
-      <c r="C33" s="33" t="s">
+      <c r="A33" s="24"/>
+      <c r="B33" s="100"/>
+      <c r="C33" s="13" t="s">
+        <v>265</v>
+      </c>
+      <c r="D33" s="13" t="s">
+        <v>265</v>
+      </c>
+      <c r="E33" s="4"/>
+      <c r="F33" s="4"/>
+      <c r="G33" s="13" t="s">
+        <v>265</v>
+      </c>
+      <c r="H33" s="4"/>
+      <c r="I33" s="4"/>
+      <c r="J33" s="14"/>
+      <c r="K33" s="14"/>
+      <c r="L33" s="14"/>
+      <c r="M33" s="14"/>
+      <c r="N33" s="14"/>
+      <c r="O33" s="13" t="s">
         <v>266</v>
       </c>
-      <c r="D33" s="33" t="s">
+      <c r="P33" s="14"/>
+      <c r="Q33" s="14"/>
+      <c r="R33" s="14"/>
+      <c r="S33" s="13" t="s">
         <v>266</v>
       </c>
-      <c r="E33" s="32"/>
-      <c r="F33" s="32"/>
-      <c r="G33" s="33" t="s">
+      <c r="T33" s="4"/>
+      <c r="U33" s="13" t="s">
         <v>266</v>
       </c>
-      <c r="H33" s="32"/>
-      <c r="I33" s="32"/>
-      <c r="J33" s="34"/>
-      <c r="K33" s="34"/>
-      <c r="L33" s="34"/>
-      <c r="M33" s="34"/>
-      <c r="N33" s="34"/>
-      <c r="O33" s="34"/>
-      <c r="P33" s="34"/>
-      <c r="Q33" s="34"/>
-      <c r="R33" s="34"/>
-      <c r="S33" s="34"/>
-      <c r="T33" s="32"/>
-      <c r="U33" s="34"/>
-      <c r="V33" s="32"/>
-      <c r="W33" s="34"/>
-      <c r="X33" s="32"/>
-      <c r="Y33" s="32"/>
-      <c r="Z33" s="32"/>
-      <c r="AA33" s="32"/>
-      <c r="AB33" s="32"/>
-      <c r="AC33" s="32"/>
-      <c r="AD33" s="31"/>
-      <c r="AE33" s="31"/>
-      <c r="AF33" s="41"/>
+      <c r="V33" s="4"/>
+      <c r="W33" s="13" t="s">
+        <v>267</v>
+      </c>
+      <c r="X33" s="4"/>
+      <c r="Y33" s="4"/>
+      <c r="Z33" s="4"/>
+      <c r="AA33" s="4"/>
+      <c r="AB33" s="4"/>
+      <c r="AC33" s="4"/>
+      <c r="AF33" s="40"/>
       <c r="AG33" s="2"/>
       <c r="AH33" s="2"/>
       <c r="AI33" s="2"/>
@@ -5028,280 +4938,395 @@
       <c r="EX33" s="2"/>
       <c r="EY33" s="2"/>
     </row>
-    <row r="34" spans="1:155" ht="18" customHeight="1">
-      <c r="A34" s="42"/>
-      <c r="B34" s="66" t="s">
-        <v>267</v>
-      </c>
-      <c r="C34" s="43"/>
-      <c r="D34" s="43"/>
-      <c r="E34" s="43"/>
-      <c r="F34" s="43"/>
-      <c r="G34" s="43"/>
-      <c r="H34" s="43"/>
-      <c r="I34" s="43"/>
-      <c r="J34" s="43"/>
-      <c r="K34" s="43"/>
-      <c r="L34" s="43"/>
-      <c r="M34" s="43"/>
-      <c r="N34" s="43"/>
-      <c r="O34" s="43"/>
-      <c r="P34" s="43"/>
-      <c r="Q34" s="43"/>
-      <c r="R34" s="43"/>
-      <c r="S34" s="43"/>
-      <c r="T34" s="43"/>
-      <c r="U34" s="43"/>
-      <c r="V34" s="43"/>
-      <c r="W34" s="43"/>
-      <c r="X34" s="44" t="s">
+    <row r="34" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1">
+      <c r="A34" s="30"/>
+      <c r="B34" s="101"/>
+      <c r="C34" s="33" t="s">
         <v>268</v>
       </c>
-      <c r="Y34" s="44" t="s">
-        <v>269</v>
-      </c>
-      <c r="Z34" s="43"/>
-      <c r="AA34" s="43"/>
-      <c r="AB34" s="43"/>
-      <c r="AC34" s="45"/>
-      <c r="AD34" s="46"/>
-      <c r="AE34" s="46"/>
-      <c r="AF34" s="47"/>
+      <c r="D34" s="33" t="s">
+        <v>268</v>
+      </c>
+      <c r="E34" s="32"/>
+      <c r="F34" s="32"/>
+      <c r="G34" s="33" t="s">
+        <v>268</v>
+      </c>
+      <c r="H34" s="32"/>
+      <c r="I34" s="32"/>
+      <c r="J34" s="34"/>
+      <c r="K34" s="34"/>
+      <c r="L34" s="34"/>
+      <c r="M34" s="34"/>
+      <c r="N34" s="34"/>
+      <c r="O34" s="34"/>
+      <c r="P34" s="34"/>
+      <c r="Q34" s="34"/>
+      <c r="R34" s="34"/>
+      <c r="S34" s="34"/>
+      <c r="T34" s="32"/>
+      <c r="U34" s="34"/>
+      <c r="V34" s="32"/>
+      <c r="W34" s="34"/>
+      <c r="X34" s="32"/>
+      <c r="Y34" s="32"/>
+      <c r="Z34" s="32"/>
+      <c r="AA34" s="32"/>
+      <c r="AB34" s="32"/>
+      <c r="AC34" s="32"/>
+      <c r="AD34" s="31"/>
+      <c r="AE34" s="31"/>
+      <c r="AF34" s="41"/>
+      <c r="AG34" s="2"/>
+      <c r="AH34" s="2"/>
+      <c r="AI34" s="2"/>
+      <c r="AJ34" s="2"/>
+      <c r="AK34" s="2"/>
+      <c r="AL34" s="2"/>
+      <c r="AM34" s="2"/>
+      <c r="AN34" s="2"/>
+      <c r="AO34" s="2"/>
+      <c r="AP34" s="2"/>
+      <c r="AQ34" s="2"/>
+      <c r="AR34" s="2"/>
+      <c r="AS34" s="2"/>
+      <c r="AT34" s="2"/>
+      <c r="AU34" s="2"/>
+      <c r="AV34" s="2"/>
+      <c r="AW34" s="2"/>
+      <c r="AX34" s="2"/>
+      <c r="AY34" s="2"/>
+      <c r="AZ34" s="2"/>
+      <c r="BA34" s="2"/>
+      <c r="BB34" s="2"/>
+      <c r="BC34" s="2"/>
+      <c r="BD34" s="2"/>
+      <c r="BE34" s="2"/>
+      <c r="BF34" s="2"/>
+      <c r="BG34" s="2"/>
+      <c r="BH34" s="2"/>
+      <c r="BI34" s="2"/>
+      <c r="BJ34" s="2"/>
+      <c r="BK34" s="2"/>
+      <c r="BL34" s="2"/>
+      <c r="BM34" s="2"/>
+      <c r="BN34" s="2"/>
+      <c r="BO34" s="2"/>
+      <c r="BP34" s="2"/>
+      <c r="BQ34" s="2"/>
+      <c r="BR34" s="2"/>
+      <c r="BS34" s="2"/>
+      <c r="BT34" s="2"/>
+      <c r="BU34" s="2"/>
+      <c r="BV34" s="2"/>
+      <c r="BW34" s="2"/>
+      <c r="BX34" s="2"/>
+      <c r="BY34" s="2"/>
+      <c r="BZ34" s="2"/>
+      <c r="CA34" s="2"/>
+      <c r="CB34" s="2"/>
+      <c r="CC34" s="2"/>
+      <c r="CD34" s="2"/>
+      <c r="CE34" s="2"/>
+      <c r="CF34" s="2"/>
+      <c r="CG34" s="2"/>
+      <c r="CH34" s="2"/>
+      <c r="CI34" s="2"/>
+      <c r="CJ34" s="2"/>
+      <c r="CK34" s="2"/>
+      <c r="CL34" s="2"/>
+      <c r="CM34" s="2"/>
+      <c r="CN34" s="2"/>
+      <c r="CO34" s="2"/>
+      <c r="CP34" s="2"/>
+      <c r="CQ34" s="2"/>
+      <c r="CR34" s="2"/>
+      <c r="CS34" s="2"/>
+      <c r="CT34" s="2"/>
+      <c r="CU34" s="2"/>
+      <c r="CV34" s="2"/>
+      <c r="CW34" s="2"/>
+      <c r="CX34" s="2"/>
+      <c r="CY34" s="2"/>
+      <c r="CZ34" s="2"/>
+      <c r="DA34" s="2"/>
+      <c r="DB34" s="2"/>
+      <c r="DC34" s="2"/>
+      <c r="DD34" s="2"/>
+      <c r="DE34" s="2"/>
+      <c r="DF34" s="2"/>
+      <c r="DG34" s="2"/>
+      <c r="DH34" s="2"/>
+      <c r="DI34" s="2"/>
+      <c r="DJ34" s="2"/>
+      <c r="DK34" s="2"/>
+      <c r="DL34" s="2"/>
+      <c r="DM34" s="2"/>
+      <c r="DN34" s="2"/>
+      <c r="DO34" s="2"/>
+      <c r="DP34" s="2"/>
+      <c r="DQ34" s="2"/>
+      <c r="DR34" s="2"/>
+      <c r="DS34" s="2"/>
+      <c r="DT34" s="2"/>
+      <c r="DU34" s="2"/>
+      <c r="DV34" s="2"/>
+      <c r="DW34" s="2"/>
+      <c r="DX34" s="2"/>
+      <c r="DY34" s="2"/>
+      <c r="DZ34" s="2"/>
+      <c r="EA34" s="2"/>
+      <c r="EB34" s="2"/>
+      <c r="EC34" s="2"/>
+      <c r="ED34" s="2"/>
+      <c r="EE34" s="2"/>
+      <c r="EF34" s="2"/>
+      <c r="EG34" s="2"/>
+      <c r="EH34" s="2"/>
+      <c r="EI34" s="2"/>
+      <c r="EJ34" s="2"/>
+      <c r="EK34" s="2"/>
+      <c r="EL34" s="2"/>
+      <c r="EM34" s="2"/>
+      <c r="EN34" s="2"/>
+      <c r="EO34" s="2"/>
+      <c r="EP34" s="2"/>
+      <c r="EQ34" s="2"/>
+      <c r="ER34" s="2"/>
+      <c r="ES34" s="2"/>
+      <c r="ET34" s="2"/>
+      <c r="EU34" s="2"/>
+      <c r="EV34" s="2"/>
+      <c r="EW34" s="2"/>
+      <c r="EX34" s="2"/>
+      <c r="EY34" s="2"/>
     </row>
     <row r="35" spans="1:155" ht="18" customHeight="1">
-      <c r="A35" s="19"/>
-      <c r="B35" s="51" t="s">
+      <c r="A35" s="42"/>
+      <c r="B35" s="66" t="s">
+        <v>269</v>
+      </c>
+      <c r="C35" s="43"/>
+      <c r="D35" s="43"/>
+      <c r="E35" s="43"/>
+      <c r="F35" s="43"/>
+      <c r="G35" s="43"/>
+      <c r="H35" s="43"/>
+      <c r="I35" s="43"/>
+      <c r="J35" s="43"/>
+      <c r="K35" s="43"/>
+      <c r="L35" s="43"/>
+      <c r="M35" s="43"/>
+      <c r="N35" s="43"/>
+      <c r="O35" s="43"/>
+      <c r="P35" s="43"/>
+      <c r="Q35" s="43"/>
+      <c r="R35" s="43"/>
+      <c r="S35" s="43"/>
+      <c r="T35" s="43"/>
+      <c r="U35" s="43"/>
+      <c r="V35" s="43"/>
+      <c r="W35" s="43"/>
+      <c r="X35" s="44" t="s">
         <v>270</v>
       </c>
-      <c r="C35" s="8"/>
-      <c r="D35" s="8"/>
-      <c r="E35" s="8"/>
-      <c r="F35" s="8"/>
-      <c r="G35" s="8"/>
-      <c r="H35" s="8"/>
-      <c r="I35" s="8"/>
-      <c r="J35" s="8"/>
-      <c r="K35" s="8"/>
-      <c r="L35" s="8"/>
-      <c r="M35" s="8"/>
-      <c r="N35" s="8"/>
-      <c r="O35" s="8"/>
-      <c r="P35" s="8"/>
-      <c r="Q35" s="8"/>
-      <c r="R35" s="8"/>
-      <c r="S35" s="8"/>
-      <c r="T35" s="8"/>
-      <c r="U35" s="8"/>
-      <c r="V35" s="8" t="s">
-        <v>238</v>
-      </c>
-      <c r="W35" s="8"/>
-      <c r="X35" s="8" t="s">
-        <v>238</v>
-      </c>
-      <c r="Y35" s="8" t="s">
-        <v>238</v>
-      </c>
-      <c r="Z35" s="8"/>
-      <c r="AA35" s="8"/>
-      <c r="AB35" s="8"/>
-      <c r="AC35" s="7"/>
-      <c r="AD35" s="20"/>
-      <c r="AE35" s="20"/>
-      <c r="AF35" s="20"/>
+      <c r="Y35" s="44" t="s">
+        <v>271</v>
+      </c>
+      <c r="Z35" s="43"/>
+      <c r="AA35" s="43"/>
+      <c r="AB35" s="43"/>
+      <c r="AC35" s="45"/>
+      <c r="AD35" s="46"/>
+      <c r="AE35" s="46"/>
+      <c r="AF35" s="47"/>
     </row>
     <row r="36" spans="1:155" ht="18" customHeight="1">
-      <c r="A36" s="15"/>
-      <c r="B36" s="67" t="s">
-        <v>271</v>
-      </c>
-      <c r="C36" s="6"/>
-      <c r="D36" s="6"/>
-      <c r="E36" s="6"/>
-      <c r="F36" s="6"/>
-      <c r="G36" s="6"/>
-      <c r="H36" s="6"/>
-      <c r="I36" s="6"/>
-      <c r="J36" s="6"/>
-      <c r="K36" s="6"/>
-      <c r="L36" s="6"/>
-      <c r="M36" s="6"/>
-      <c r="N36" s="6"/>
-      <c r="O36" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="P36" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="Q36" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="R36" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="S36" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="T36" s="6"/>
-      <c r="U36" s="6"/>
-      <c r="V36" s="6"/>
-      <c r="W36" s="6"/>
-      <c r="X36" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="Y36" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="Z36" s="6"/>
-      <c r="AA36" s="6"/>
-      <c r="AB36" s="6"/>
-      <c r="AC36" s="48"/>
-      <c r="AD36" s="16"/>
-      <c r="AE36" s="16"/>
-      <c r="AF36" s="16"/>
+      <c r="A36" s="19"/>
+      <c r="B36" s="51" t="s">
+        <v>272</v>
+      </c>
+      <c r="C36" s="8"/>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="8"/>
+      <c r="G36" s="8"/>
+      <c r="H36" s="8"/>
+      <c r="I36" s="8"/>
+      <c r="J36" s="8"/>
+      <c r="K36" s="8"/>
+      <c r="L36" s="8"/>
+      <c r="M36" s="8"/>
+      <c r="N36" s="8"/>
+      <c r="O36" s="8"/>
+      <c r="P36" s="8"/>
+      <c r="Q36" s="8"/>
+      <c r="R36" s="8"/>
+      <c r="S36" s="8"/>
+      <c r="T36" s="8"/>
+      <c r="U36" s="8"/>
+      <c r="V36" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="W36" s="8"/>
+      <c r="X36" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="Y36" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="Z36" s="8"/>
+      <c r="AA36" s="8"/>
+      <c r="AB36" s="8"/>
+      <c r="AC36" s="7"/>
+      <c r="AD36" s="20"/>
+      <c r="AE36" s="20"/>
+      <c r="AF36" s="20"/>
     </row>
     <row r="37" spans="1:155" ht="18" customHeight="1">
-      <c r="A37" s="42"/>
-      <c r="B37" s="66" t="s">
-        <v>272</v>
-      </c>
-      <c r="C37" s="43"/>
-      <c r="D37" s="43"/>
-      <c r="E37" s="43"/>
-      <c r="F37" s="43"/>
-      <c r="G37" s="43"/>
-      <c r="H37" s="43"/>
-      <c r="I37" s="43"/>
-      <c r="J37" s="43"/>
-      <c r="K37" s="43"/>
-      <c r="L37" s="43"/>
-      <c r="M37" s="43"/>
-      <c r="N37" s="43"/>
-      <c r="O37" s="43"/>
-      <c r="P37" s="43"/>
-      <c r="Q37" s="43"/>
-      <c r="R37" s="43"/>
-      <c r="S37" s="43"/>
-      <c r="T37" s="43"/>
-      <c r="U37" s="43"/>
-      <c r="V37" s="43"/>
-      <c r="W37" s="43"/>
-      <c r="X37" s="49" t="s">
+      <c r="A37" s="15"/>
+      <c r="B37" s="67" t="s">
         <v>273</v>
       </c>
-      <c r="Y37" s="43"/>
-      <c r="Z37" s="43"/>
-      <c r="AA37" s="43"/>
-      <c r="AB37" s="43"/>
-      <c r="AC37" s="43"/>
-      <c r="AD37" s="46"/>
-      <c r="AE37" s="44" t="s">
-        <v>274</v>
-      </c>
-      <c r="AF37" s="50" t="s">
-        <v>275</v>
-      </c>
+      <c r="C37" s="6"/>
+      <c r="D37" s="6"/>
+      <c r="E37" s="6"/>
+      <c r="F37" s="6"/>
+      <c r="G37" s="6"/>
+      <c r="H37" s="6"/>
+      <c r="I37" s="6"/>
+      <c r="J37" s="6"/>
+      <c r="K37" s="6"/>
+      <c r="L37" s="6"/>
+      <c r="M37" s="6"/>
+      <c r="N37" s="6"/>
+      <c r="O37" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="P37" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="Q37" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="R37" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="S37" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="T37" s="6"/>
+      <c r="U37" s="6"/>
+      <c r="V37" s="6"/>
+      <c r="W37" s="6"/>
+      <c r="X37" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="Y37" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="Z37" s="6"/>
+      <c r="AA37" s="6"/>
+      <c r="AB37" s="6"/>
+      <c r="AC37" s="48"/>
+      <c r="AD37" s="16"/>
+      <c r="AE37" s="16"/>
+      <c r="AF37" s="16"/>
     </row>
     <row r="38" spans="1:155" ht="18" customHeight="1">
-      <c r="A38" s="19"/>
-      <c r="B38" s="51" t="s">
+      <c r="A38" s="42"/>
+      <c r="B38" s="66" t="s">
+        <v>274</v>
+      </c>
+      <c r="C38" s="43"/>
+      <c r="D38" s="43"/>
+      <c r="E38" s="43"/>
+      <c r="F38" s="43"/>
+      <c r="G38" s="43"/>
+      <c r="H38" s="43"/>
+      <c r="I38" s="43"/>
+      <c r="J38" s="43"/>
+      <c r="K38" s="43"/>
+      <c r="L38" s="43"/>
+      <c r="M38" s="43"/>
+      <c r="N38" s="43"/>
+      <c r="O38" s="43"/>
+      <c r="P38" s="43"/>
+      <c r="Q38" s="43"/>
+      <c r="R38" s="43"/>
+      <c r="S38" s="43"/>
+      <c r="T38" s="43"/>
+      <c r="U38" s="43"/>
+      <c r="V38" s="43"/>
+      <c r="W38" s="43"/>
+      <c r="X38" s="49" t="s">
+        <v>275</v>
+      </c>
+      <c r="Y38" s="43"/>
+      <c r="Z38" s="43"/>
+      <c r="AA38" s="43"/>
+      <c r="AB38" s="43"/>
+      <c r="AC38" s="43"/>
+      <c r="AD38" s="46"/>
+      <c r="AE38" s="44" t="s">
         <v>276</v>
       </c>
-      <c r="C38" s="8" t="s">
-        <v>238</v>
-      </c>
-      <c r="D38" s="8" t="s">
-        <v>238</v>
-      </c>
-      <c r="E38" s="8"/>
-      <c r="F38" s="8"/>
-      <c r="G38" s="8" t="s">
-        <v>238</v>
-      </c>
-      <c r="H38" s="8"/>
-      <c r="I38" s="8"/>
-      <c r="J38" s="8" t="s">
-        <v>238</v>
-      </c>
-      <c r="K38" s="8" t="s">
-        <v>238</v>
-      </c>
-      <c r="L38" s="8"/>
-      <c r="M38" s="8"/>
-      <c r="N38" s="8"/>
-      <c r="O38" s="8"/>
-      <c r="P38" s="8"/>
-      <c r="Q38" s="8"/>
-      <c r="R38" s="8"/>
-      <c r="S38" s="8"/>
-      <c r="T38" s="8"/>
-      <c r="U38" s="8"/>
-      <c r="V38" s="8"/>
-      <c r="W38" s="8"/>
-      <c r="X38" s="8"/>
-      <c r="Y38" s="8" t="s">
-        <v>238</v>
-      </c>
-      <c r="Z38" s="8"/>
-      <c r="AA38" s="8"/>
-      <c r="AB38" s="8"/>
-      <c r="AC38" s="8"/>
-      <c r="AD38" s="20"/>
-      <c r="AE38" s="20"/>
-      <c r="AF38" s="20"/>
+      <c r="AF38" s="50" t="s">
+        <v>277</v>
+      </c>
     </row>
     <row r="39" spans="1:155" ht="18" customHeight="1">
-      <c r="A39" s="9"/>
-      <c r="B39" s="12" t="s">
-        <v>277</v>
-      </c>
-      <c r="C39" s="4"/>
-      <c r="D39" s="4"/>
-      <c r="E39" s="4"/>
-      <c r="F39" s="4"/>
-      <c r="G39" s="4"/>
-      <c r="H39" s="4"/>
-      <c r="I39" s="4"/>
-      <c r="J39" s="4"/>
-      <c r="K39" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="L39" s="4"/>
-      <c r="M39" s="4"/>
-      <c r="N39" s="4"/>
-      <c r="O39" s="4"/>
-      <c r="P39" s="4"/>
-      <c r="Q39" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="R39" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="S39" s="4"/>
-      <c r="T39" s="4"/>
-      <c r="U39" s="4"/>
-      <c r="V39" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="W39" s="4"/>
-      <c r="X39" s="4"/>
-      <c r="Y39" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="Z39" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="AA39" s="4"/>
-      <c r="AB39" s="4"/>
-      <c r="AC39" s="4"/>
-      <c r="AD39" s="10"/>
-      <c r="AE39" s="10"/>
-      <c r="AF39" s="10"/>
+      <c r="A39" s="19"/>
+      <c r="B39" s="51" t="s">
+        <v>278</v>
+      </c>
+      <c r="C39" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="D39" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="E39" s="8"/>
+      <c r="F39" s="8"/>
+      <c r="G39" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="H39" s="8"/>
+      <c r="I39" s="8"/>
+      <c r="J39" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="K39" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="L39" s="8"/>
+      <c r="M39" s="8"/>
+      <c r="N39" s="8"/>
+      <c r="O39" s="8"/>
+      <c r="P39" s="8"/>
+      <c r="Q39" s="8"/>
+      <c r="R39" s="8"/>
+      <c r="S39" s="8"/>
+      <c r="T39" s="8"/>
+      <c r="U39" s="8"/>
+      <c r="V39" s="8"/>
+      <c r="W39" s="8"/>
+      <c r="X39" s="8"/>
+      <c r="Y39" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="Z39" s="8"/>
+      <c r="AA39" s="8"/>
+      <c r="AB39" s="8"/>
+      <c r="AC39" s="8"/>
+      <c r="AD39" s="20"/>
+      <c r="AE39" s="20"/>
+      <c r="AF39" s="20"/>
     </row>
     <row r="40" spans="1:155" ht="18" customHeight="1">
       <c r="A40" s="9"/>
       <c r="B40" s="12" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C40" s="4"/>
       <c r="D40" s="4"/>
@@ -5311,27 +5336,35 @@
       <c r="H40" s="4"/>
       <c r="I40" s="4"/>
       <c r="J40" s="4"/>
-      <c r="K40" s="4"/>
+      <c r="K40" s="4" t="s">
+        <v>240</v>
+      </c>
       <c r="L40" s="4"/>
       <c r="M40" s="4"/>
       <c r="N40" s="4"/>
       <c r="O40" s="4"/>
       <c r="P40" s="4"/>
-      <c r="Q40" s="4"/>
-      <c r="R40" s="4"/>
+      <c r="Q40" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="R40" s="4" t="s">
+        <v>240</v>
+      </c>
       <c r="S40" s="4"/>
       <c r="T40" s="4"/>
       <c r="U40" s="4"/>
-      <c r="V40" s="4"/>
+      <c r="V40" s="4" t="s">
+        <v>240</v>
+      </c>
       <c r="W40" s="4"/>
       <c r="X40" s="4"/>
       <c r="Y40" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="Z40" s="4"/>
-      <c r="AA40" s="4" t="s">
-        <v>238</v>
-      </c>
+        <v>240</v>
+      </c>
+      <c r="Z40" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="AA40" s="4"/>
       <c r="AB40" s="4"/>
       <c r="AC40" s="4"/>
       <c r="AD40" s="10"/>
@@ -5341,7 +5374,7 @@
     <row r="41" spans="1:155" ht="18" customHeight="1">
       <c r="A41" s="9"/>
       <c r="B41" s="12" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C41" s="4"/>
       <c r="D41" s="4"/>
@@ -5365,9 +5398,13 @@
       <c r="V41" s="4"/>
       <c r="W41" s="4"/>
       <c r="X41" s="4"/>
-      <c r="Y41" s="4"/>
+      <c r="Y41" s="4" t="s">
+        <v>240</v>
+      </c>
       <c r="Z41" s="4"/>
-      <c r="AA41" s="4"/>
+      <c r="AA41" s="4" t="s">
+        <v>240</v>
+      </c>
       <c r="AB41" s="4"/>
       <c r="AC41" s="4"/>
       <c r="AD41" s="10"/>
@@ -5377,15 +5414,13 @@
     <row r="42" spans="1:155" ht="18" customHeight="1">
       <c r="A42" s="9"/>
       <c r="B42" s="12" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C42" s="4"/>
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>
       <c r="F42" s="4"/>
-      <c r="G42" s="4" t="s">
-        <v>238</v>
-      </c>
+      <c r="G42" s="4"/>
       <c r="H42" s="4"/>
       <c r="I42" s="4"/>
       <c r="J42" s="4"/>
@@ -5415,13 +5450,15 @@
     <row r="43" spans="1:155" ht="18" customHeight="1">
       <c r="A43" s="9"/>
       <c r="B43" s="12" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C43" s="4"/>
       <c r="D43" s="4"/>
       <c r="E43" s="4"/>
       <c r="F43" s="4"/>
-      <c r="G43" s="4"/>
+      <c r="G43" s="4" t="s">
+        <v>240</v>
+      </c>
       <c r="H43" s="4"/>
       <c r="I43" s="4"/>
       <c r="J43" s="4"/>
@@ -5438,21 +5475,20 @@
       <c r="U43" s="4"/>
       <c r="V43" s="4"/>
       <c r="W43" s="4"/>
-      <c r="X43" s="10"/>
-      <c r="Y43" s="10"/>
-      <c r="Z43" s="10"/>
-      <c r="AA43" s="10"/>
-      <c r="AB43" s="10" t="s">
-        <v>238</v>
-      </c>
-      <c r="AC43" s="10"/>
+      <c r="X43" s="4"/>
+      <c r="Y43" s="4"/>
+      <c r="Z43" s="4"/>
+      <c r="AA43" s="4"/>
+      <c r="AB43" s="4"/>
+      <c r="AC43" s="4"/>
       <c r="AD43" s="10"/>
       <c r="AE43" s="10"/>
+      <c r="AF43" s="10"/>
     </row>
     <row r="44" spans="1:155" ht="18" customHeight="1">
       <c r="A44" s="9"/>
       <c r="B44" s="12" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C44" s="4"/>
       <c r="D44" s="4"/>
@@ -5479,7 +5515,9 @@
       <c r="Y44" s="10"/>
       <c r="Z44" s="10"/>
       <c r="AA44" s="10"/>
-      <c r="AB44" s="10"/>
+      <c r="AB44" s="10" t="s">
+        <v>240</v>
+      </c>
       <c r="AC44" s="10"/>
       <c r="AD44" s="10"/>
       <c r="AE44" s="10"/>
@@ -5487,7 +5525,7 @@
     <row r="45" spans="1:155" ht="18" customHeight="1">
       <c r="A45" s="9"/>
       <c r="B45" s="12" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C45" s="4"/>
       <c r="D45" s="4"/>
@@ -5522,7 +5560,7 @@
     <row r="46" spans="1:155" ht="18" customHeight="1">
       <c r="A46" s="9"/>
       <c r="B46" s="12" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C46" s="4"/>
       <c r="D46" s="4"/>
@@ -5557,7 +5595,7 @@
     <row r="47" spans="1:155" ht="18" customHeight="1">
       <c r="A47" s="9"/>
       <c r="B47" s="12" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C47" s="4"/>
       <c r="D47" s="4"/>
@@ -5589,10 +5627,40 @@
       <c r="AD47" s="10"/>
       <c r="AE47" s="10"/>
     </row>
-    <row r="48" spans="1:155">
-      <c r="X48" s="2"/>
-      <c r="Y48" s="2"/>
-      <c r="Z48" s="2"/>
+    <row r="48" spans="1:155" ht="18" customHeight="1">
+      <c r="A48" s="9"/>
+      <c r="B48" s="12" t="s">
+        <v>287</v>
+      </c>
+      <c r="C48" s="4"/>
+      <c r="D48" s="4"/>
+      <c r="E48" s="4"/>
+      <c r="F48" s="4"/>
+      <c r="G48" s="4"/>
+      <c r="H48" s="4"/>
+      <c r="I48" s="4"/>
+      <c r="J48" s="4"/>
+      <c r="K48" s="4"/>
+      <c r="L48" s="4"/>
+      <c r="M48" s="4"/>
+      <c r="N48" s="4"/>
+      <c r="O48" s="4"/>
+      <c r="P48" s="4"/>
+      <c r="Q48" s="4"/>
+      <c r="R48" s="4"/>
+      <c r="S48" s="4"/>
+      <c r="T48" s="4"/>
+      <c r="U48" s="4"/>
+      <c r="V48" s="4"/>
+      <c r="W48" s="4"/>
+      <c r="X48" s="10"/>
+      <c r="Y48" s="10"/>
+      <c r="Z48" s="10"/>
+      <c r="AA48" s="10"/>
+      <c r="AB48" s="10"/>
+      <c r="AC48" s="10"/>
+      <c r="AD48" s="10"/>
+      <c r="AE48" s="10"/>
     </row>
     <row r="49" spans="24:26">
       <c r="X49" s="2"/>
@@ -5654,8 +5722,13 @@
       <c r="Y60" s="2"/>
       <c r="Z60" s="2"/>
     </row>
+    <row r="61" spans="24:26">
+      <c r="X61" s="2"/>
+      <c r="Y61" s="2"/>
+      <c r="Z61" s="2"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:AF33" xr:uid="{D8B0CA4D-B55F-4AFA-903E-3D529FFFD0A1}">
+  <autoFilter ref="A2:AF34" xr:uid="{D8B0CA4D-B55F-4AFA-903E-3D529FFFD0A1}">
     <filterColumn colId="2" showButton="0"/>
     <filterColumn colId="3" showButton="0"/>
     <filterColumn colId="4" showButton="0"/>
@@ -5675,154 +5748,154 @@
     <filterColumn colId="20" showButton="0"/>
   </autoFilter>
   <mergeCells count="22">
-    <mergeCell ref="AE2:AE4"/>
-    <mergeCell ref="AF2:AF4"/>
-    <mergeCell ref="A7:A18"/>
-    <mergeCell ref="AB2:AB4"/>
-    <mergeCell ref="AC2:AC4"/>
+    <mergeCell ref="AE2:AE5"/>
+    <mergeCell ref="AF2:AF5"/>
+    <mergeCell ref="A8:A19"/>
+    <mergeCell ref="AB2:AB5"/>
+    <mergeCell ref="AC2:AC5"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="G3:L3"/>
     <mergeCell ref="C2:N2"/>
-    <mergeCell ref="X2:X4"/>
-    <mergeCell ref="AA2:AA4"/>
+    <mergeCell ref="X2:X5"/>
+    <mergeCell ref="AA2:AA5"/>
     <mergeCell ref="U2:V3"/>
-    <mergeCell ref="W2:W4"/>
+    <mergeCell ref="W2:W5"/>
     <mergeCell ref="Q3:T3"/>
     <mergeCell ref="O2:T2"/>
     <mergeCell ref="O3:P3"/>
-    <mergeCell ref="Y2:Y4"/>
-    <mergeCell ref="B20:B27"/>
-    <mergeCell ref="B12:B18"/>
-    <mergeCell ref="B7:B11"/>
-    <mergeCell ref="B28:B33"/>
-    <mergeCell ref="AD2:AD4"/>
-    <mergeCell ref="Z2:Z4"/>
+    <mergeCell ref="Y2:Y5"/>
+    <mergeCell ref="B21:B28"/>
+    <mergeCell ref="B13:B19"/>
+    <mergeCell ref="B8:B12"/>
+    <mergeCell ref="B29:B34"/>
+    <mergeCell ref="AD2:AD5"/>
+    <mergeCell ref="Z2:Z5"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="C21" r:id="rId1" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/sp?tab=models" xr:uid="{FE987DC0-578A-4A81-AB17-6E49D6983782}"/>
-    <hyperlink ref="C22" r:id="rId2" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/spe?tab=models" xr:uid="{E414E66B-6D50-4BC0-93B6-EEDD71D1D349}"/>
-    <hyperlink ref="C23" r:id="rId3" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/sp-ne?tab=models" xr:uid="{79A82224-5E75-416A-BD5C-1C442DB4F9E7}"/>
-    <hyperlink ref="D21" r:id="rId4" display="https://product-selection.grundfos.com/fr/products/bm?tab=products" xr:uid="{39935FC4-BF60-4ADA-99B8-6280D11B4087}"/>
-    <hyperlink ref="D22" r:id="rId5" display="https://product-selection.grundfos.com/fr/products/bms?tab=products" xr:uid="{201298BF-F5B7-4DD8-896A-A6CFDF20A155}"/>
-    <hyperlink ref="D23" r:id="rId6" display="https://product-selection.grundfos.com/fr/products/bm-hp?tab=products" xr:uid="{0AA34BB7-1783-4351-AB39-2E3E2C9E6D24}"/>
-    <hyperlink ref="E21" r:id="rId7" display="https://product-selection.grundfos.com/fr/products/kpl?tab=models" xr:uid="{02FD05D5-211D-4185-A911-F718E163AF22}"/>
-    <hyperlink ref="E22" r:id="rId8" display="https://product-selection.grundfos.com/fr/products/kwm?tab=documentation" xr:uid="{F11B5E61-F53C-4DA1-93C5-A57D0408930C}"/>
-    <hyperlink ref="F21" r:id="rId9" display="https://product-selection.grundfos.com/fr/products/ls?tab=products" xr:uid="{070C34E9-9C05-4522-9AD2-8E6D82261A9B}"/>
-    <hyperlink ref="J21" r:id="rId10" display="https://product-selection.grundfos.com/fr/products/cm-cme?tab=products" xr:uid="{E79A5B97-E6E0-4649-B070-9A1CF47F88B2}"/>
-    <hyperlink ref="I21" r:id="rId11" display="https://product-selection.grundfos.com/fr/products/cm-cme/cm-self-priming?tab=models" xr:uid="{CFEF6DD3-2F90-4195-BA05-DEE28F55BD3E}"/>
-    <hyperlink ref="J22" r:id="rId12" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nb?tab=documentation" xr:uid="{ABC208A8-FE5B-4CC4-B585-6A3873FA7294}"/>
-    <hyperlink ref="J23" r:id="rId13" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nbe?tab=models" xr:uid="{1D4EF590-19C1-44EB-8B92-46AD5F28F62F}"/>
-    <hyperlink ref="J24" r:id="rId14" display="https://product-selection.grundfos.com/fr/products/nk-nke-nke-series-2000-nk-bare-shaft?tab=products" xr:uid="{76D3161D-F2DD-4CCA-AC1D-AD2E393D8694}"/>
-    <hyperlink ref="J25" r:id="rId15" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft?tab=products" xr:uid="{9CA4757F-439C-4161-8B60-7C14A9EDCA69}"/>
-    <hyperlink ref="J26" r:id="rId16" display="https://product-selection.grundfos.com/fr/products/tp-tpe?tab=products" xr:uid="{0C9A1473-1926-417A-947F-8561754B7D76}"/>
-    <hyperlink ref="N23" r:id="rId17" display="https://product-selection.grundfos.com/fr/products/tp-tpe?tab=products" xr:uid="{7D2D046F-1C95-42DD-8F35-90280675B9EA}"/>
-    <hyperlink ref="N21" r:id="rId18" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nbe?tab=models" xr:uid="{303D01A6-AC7B-42EE-AE09-2A10FBED3940}"/>
-    <hyperlink ref="N22" r:id="rId19" display="https://product-selection.grundfos.com/fr/products/nk-nke-nke-series-2000-nk-bare-shaft?tab=products" xr:uid="{A1442A3E-E286-4D87-BF5A-B52C00F11931}"/>
-    <hyperlink ref="N24" r:id="rId20" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft?tab=products" xr:uid="{91C811C0-E7C2-45CC-8C4A-41851188982F}"/>
-    <hyperlink ref="K21" r:id="rId21" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte?tab=products" xr:uid="{168A97AE-925F-4CB8-99FA-4D28B053F7CB}"/>
-    <hyperlink ref="L22" r:id="rId22" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte/cre?tab=models" xr:uid="{43E68B92-4EB3-4ECE-A299-C7DDCAFB1889}"/>
-    <hyperlink ref="L23" r:id="rId23" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte/crne?tab=models" xr:uid="{9DD9406E-F477-49F6-BA29-841ED00CE74B}"/>
-    <hyperlink ref="M21" r:id="rId24" display="https://product-selection.grundfos.com/fr/products/cm-cme/cme?tab=models" xr:uid="{CB210458-379C-4663-B0FD-73E843090C67}"/>
-    <hyperlink ref="M22" r:id="rId25" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nbe?tab=models" xr:uid="{3776F606-4CBE-49B1-912C-5B2BC9586206}"/>
-    <hyperlink ref="M23" r:id="rId26" display="https://product-selection.grundfos.com/fr/products/nk-nke-nke-series-2000-nk-bare-shaft?tab=products" xr:uid="{8731A9E7-9B51-450F-BCB5-013214A2B33F}"/>
-    <hyperlink ref="M24" r:id="rId27" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft?tab=products" xr:uid="{EDB8C821-F675-4CE1-B7B0-0FAF39DCEFD4}"/>
-    <hyperlink ref="L25" r:id="rId28" display="https://product-selection.grundfos.com/fr/products/hydro-multi-e?tab=models" xr:uid="{5995DFA3-65AE-4378-BD2E-CDA4F6FA5ED7}"/>
-    <hyperlink ref="L26" r:id="rId29" display="https://product-selection.grundfos.com/fr/products/hydro-mpc?tab=products" xr:uid="{2E37CE89-9B22-43AA-B967-C6F20A25613F}"/>
-    <hyperlink ref="L24" r:id="rId30" display="https://product-selection.grundfos.com/fr/products/hydro-solo-e?tab=models" xr:uid="{5A1F2584-1AA0-4C8B-A55D-39C825C8A3F8}"/>
-    <hyperlink ref="O21" r:id="rId31" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/sl1?tab=models" xr:uid="{9C7E88DB-59BA-4B5C-8769-45D64CC97D40}"/>
-    <hyperlink ref="O22" r:id="rId32" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/slv?tab=models" xr:uid="{00039B9D-B404-44A8-B557-BBF172D7CD31}"/>
-    <hyperlink ref="O23" r:id="rId33" display="https://product-selection.grundfos.com/fr/products/sesl-9-30-kw?tab=models" xr:uid="{C90FBAD5-7C9C-4429-9BAC-9BE027B562FD}"/>
-    <hyperlink ref="O25" r:id="rId34" display="https://product-selection.grundfos.com/fr/products/s?tab=products" xr:uid="{6F267867-1729-460E-9939-DEBA10D95429}"/>
-    <hyperlink ref="O24" r:id="rId35" display="https://product-selection.grundfos.com/fr/products/sesl-frame-size-56?tab=models" xr:uid="{541D6F69-2D4F-412B-91C7-A0B79C20C0CA}"/>
-    <hyperlink ref="P22" r:id="rId36" display="https://product-selection.grundfos.com/fr/products/unilift-ap/unilift-apg?tab=models" xr:uid="{CF6542DD-C411-4584-A2A2-ADD9BD336104}"/>
-    <hyperlink ref="P21" r:id="rId37" display="https://product-selection.grundfos.com/fr/products/seg?tab=models" xr:uid="{AF847B64-9B08-45DD-8487-57C6900B0D5F}"/>
-    <hyperlink ref="Q21" r:id="rId38" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/se1?tab=models" xr:uid="{D2271F27-967E-46DC-8195-E2EAFD3339EB}"/>
-    <hyperlink ref="Q22" r:id="rId39" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/sev?tab=models" xr:uid="{6D042873-5F32-4A50-8803-93F40528C6A1}"/>
-    <hyperlink ref="Q23" r:id="rId40" display="https://product-selection.grundfos.com/fr/products/sesl-9-30-kw?tab=models" xr:uid="{A344F5B5-8A97-456F-87D5-4C6EFCA52D3A}"/>
-    <hyperlink ref="Q24" r:id="rId41" display="https://product-selection.grundfos.com/fr/products/sesl-frame-size-56?tab=models" xr:uid="{BB0B40A3-A20A-44BC-9FC9-E9EE00FC9F45}"/>
-    <hyperlink ref="Q25" r:id="rId42" display="https://product-selection.grundfos.com/fr/products/s?tab=products" xr:uid="{2E26D22E-3FD7-4718-9B39-661D30AF938C}"/>
-    <hyperlink ref="Q26" r:id="rId43" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft/nkg-supervortex-impeller?tab=explore" xr:uid="{FA539854-B47D-4B47-9F9A-7CE595B28025}"/>
-    <hyperlink ref="S21" r:id="rId44" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/se1?tab=models" xr:uid="{66C50FE8-D6EA-4602-866A-7B3258A9261C}"/>
-    <hyperlink ref="S22" r:id="rId45" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/sev?tab=models" xr:uid="{DEFE3A48-5152-4917-935D-8BAB7D40CDD7}"/>
-    <hyperlink ref="S23" r:id="rId46" display="https://product-selection.grundfos.com/fr/products/sesl-9-30-kw?tab=models" xr:uid="{62BA715F-3850-4F49-A593-7645C6C0C3CC}"/>
-    <hyperlink ref="S24" r:id="rId47" display="https://product-selection.grundfos.com/fr/products/sesl-frame-size-56?tab=models" xr:uid="{F0AA29DC-4DA5-4CA6-94B3-C22351F6904E}"/>
-    <hyperlink ref="S25" r:id="rId48" display="https://product-selection.grundfos.com/fr/products/s?tab=products" xr:uid="{96671AB9-9AEA-4A5F-B84F-E78888F9B311}"/>
-    <hyperlink ref="S26" r:id="rId49" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft/nkg-supervortex-impeller?tab=explore" xr:uid="{8A1CF826-08F5-4AF2-B984-9AA020480952}"/>
-    <hyperlink ref="O26" r:id="rId50" display="https://product-selection.grundfos.com/fr/products/unilift-ap/unilift-ap50b?tab=models" xr:uid="{14E21A07-FF5F-4129-AE6E-260A1AA5098C}"/>
-    <hyperlink ref="W21" r:id="rId51" display="https://product-selection.grundfos.com/fr/products/unilift-ap?tab=products" xr:uid="{FF1F3D5A-16C1-4C5A-8F69-37BEB2C51657}"/>
-    <hyperlink ref="W22" r:id="rId52" display="https://product-selection.grundfos.com/fr/products/unilift-kp?tab=models" xr:uid="{D8B15CDE-A46F-4955-8CE5-B1F2491BDDEE}"/>
-    <hyperlink ref="W23" r:id="rId53" display="https://product-selection.grundfos.com/fr/products/unilift-cc?tab=models" xr:uid="{5DA16314-BD6C-4DB3-8EC0-A99C56D3006D}"/>
-    <hyperlink ref="W24" r:id="rId54" display="https://product-selection.grundfos.com/fr/products/dp?tab=models" xr:uid="{4D82ED98-3DD6-4697-9C9C-A060C7E06489}"/>
-    <hyperlink ref="W25" r:id="rId55" display="https://product-selection.grundfos.com/fr/products/ef?tab=models" xr:uid="{ABDE8970-72CB-4EB8-979F-99183A9FD9D3}"/>
-    <hyperlink ref="Y21" r:id="rId56" display="https://product-selection.grundfos.com/fr/products/mt-tank-mounted-pumps/mtr?tab=models" xr:uid="{D5799B15-EF87-41DF-88D8-05F25935D793}"/>
-    <hyperlink ref="Y22" r:id="rId57" display="https://product-selection.grundfos.com/fr/products/mt-tank-mounted-pumps/mtre?tab=models" xr:uid="{7E2DAAB5-3884-49DD-BF25-FA92C2CE9951}"/>
-    <hyperlink ref="Y23" r:id="rId58" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nb?tab=documentation" xr:uid="{92C19ACB-7462-4938-A66E-478979299908}"/>
-    <hyperlink ref="Y24" r:id="rId59" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nbe?tab=models" xr:uid="{D2CCE95F-A5DF-4715-B3CA-DB297F6DF5C8}"/>
-    <hyperlink ref="Y25" r:id="rId60" display="https://product-selection.grundfos.com/fr/products/nk-nke-nke-series-2000-nk-bare-shaft?tab=products" xr:uid="{EA080A36-FCEB-4D04-B389-F8ABE5514300}"/>
-    <hyperlink ref="Y26" r:id="rId61" display="https://product-selection.grundfos.com/fr/products/tp-tpe?tab=products" xr:uid="{2A2A6B6D-2CAA-4110-9FED-BCA8DC5F1709}"/>
-    <hyperlink ref="Y27" r:id="rId62" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte?tab=products" xr:uid="{D902984C-2BC5-48A4-BF49-DCE4C7E629F6}"/>
-    <hyperlink ref="Z21" r:id="rId63" display="https://product-selection.grundfos.com/fr/products/hydro-en?tab=models" xr:uid="{69CECDCF-71ED-40D6-A274-30663F73D3A6}"/>
-    <hyperlink ref="AD21" r:id="rId64" display="https://product-selection.grundfos.com/fr/products/poweradapt?tab=models" xr:uid="{CBB79406-3EE4-4CC7-BCD3-398882D58A96}"/>
-    <hyperlink ref="AD22" r:id="rId65" display="https://product-selection.grundfos.com/fr/products/rsi?tab=models" xr:uid="{2ECDD4BA-B757-4A11-9F78-EB235920F462}"/>
-    <hyperlink ref="AD23" r:id="rId66" display="https://product-selection.grundfos.com/fr/products/crflex?tab=models" xr:uid="{F1835770-C21F-4E8A-9EBF-7C701B0E9CF4}"/>
-    <hyperlink ref="AD24" r:id="rId67" display="https://product-selection.grundfos.com/fr/products/sqflex?tab=models" xr:uid="{2932EAA4-553E-42B6-AD4B-37D91C9B845C}"/>
-    <hyperlink ref="AD25" r:id="rId68" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/sp?tab=models" xr:uid="{25A70C6E-05E1-4E40-956B-50B78B088135}"/>
-    <hyperlink ref="AD26" r:id="rId69" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/spe?tab=models" xr:uid="{7C346AF6-2EEB-4DFC-A819-DAE2C3B09113}"/>
-    <hyperlink ref="AD27" r:id="rId70" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte?tab=products" xr:uid="{9F4AE584-6CDD-45BE-ABC9-5087AAD766B9}"/>
-    <hyperlink ref="AE21" r:id="rId71" display="https://product-selection.grundfos.com/fr/products/dosing-pumps-digital/dda?tab=models" xr:uid="{68600FE5-FDB0-4237-8B8A-45786462FE8A}"/>
-    <hyperlink ref="AE22" r:id="rId72" display="https://product-selection.grundfos.com/fr/products/dosing-pumps-digital/dme?tab=models" xr:uid="{41502941-2297-46B7-A840-2EF7A24064D7}"/>
-    <hyperlink ref="AE23" r:id="rId73" display="https://product-selection.grundfos.com/fr/products/dosing-pumps-mechanical/dmx?tab=models" xr:uid="{A892A826-C3E1-4B26-9529-8174E76C068D}"/>
-    <hyperlink ref="AE24" r:id="rId74" display="https://product-selection.grundfos.com/fr/products/dosing-pumps-mechanical/dmh?tab=models" xr:uid="{60926621-C7DA-4892-9ACA-4145E303C37B}"/>
-    <hyperlink ref="AE25" r:id="rId75" xr:uid="{EB339B7E-AAB0-4720-A5DC-B7E47BEFE888}"/>
-    <hyperlink ref="AF23" r:id="rId76" display="https://product-selection.grundfos.com/fr/products/disinfection-systems/oxiperm?tab=models" xr:uid="{D1CFBDC1-076A-4661-B343-B5087946D2BF}"/>
-    <hyperlink ref="AF21" r:id="rId77" display="https://product-selection.grundfos.com/fr/products/disinfection-systems/vaccuperm?tab=models" xr:uid="{0E5CA30E-D80E-4BC1-BE8D-5757C0E703F9}"/>
-    <hyperlink ref="AF22" r:id="rId78" display="https://product-selection.grundfos.com/fr/products/disinfection-systems/selcoperm?tab=models" xr:uid="{3FE337C4-03C2-4326-92F3-2ADF14429172}"/>
-    <hyperlink ref="C29" r:id="rId79" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-4" xr:uid="{7CECB146-2C6E-4D8C-8362-B574F0A0B1CD}"/>
-    <hyperlink ref="C30" r:id="rId80" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-6" xr:uid="{77066640-D437-4393-AE04-9291CA2EA2E2}"/>
-    <hyperlink ref="C31" r:id="rId81" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-8" xr:uid="{440D559C-9B55-46F7-B47D-809066594D8E}"/>
-    <hyperlink ref="C32" r:id="rId82" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-actun-zetos" xr:uid="{6B88B868-32F8-4635-8067-C4F8AA30A87A}"/>
-    <hyperlink ref="C33" r:id="rId83" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-14-24" xr:uid="{6AAEB27D-0CD4-409C-9175-B5DC81BA5B91}"/>
-    <hyperlink ref="D29" r:id="rId84" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-4" xr:uid="{70B5668C-6DE4-4721-BD0D-15695ACCFD10}"/>
-    <hyperlink ref="D30" r:id="rId85" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-6" xr:uid="{AB0F5528-0721-49E7-9EB4-443A836A5BE6}"/>
-    <hyperlink ref="D31" r:id="rId86" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-8" xr:uid="{CE5D4CF5-B9AD-4786-AF2A-5CBA0FB4461E}"/>
-    <hyperlink ref="D32" r:id="rId87" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-actun-zetos" xr:uid="{F3302311-60D3-4257-BE0E-8ADCE8FD3F26}"/>
-    <hyperlink ref="D33" r:id="rId88" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-14-24" xr:uid="{C714C692-05B2-43B9-83CE-06CDCF547DAA}"/>
-    <hyperlink ref="F29" r:id="rId89" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-scp" xr:uid="{7BEBF8BE-E457-43DD-A078-9A05C9712ED1}"/>
-    <hyperlink ref="F30" r:id="rId90" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-atmos-tera-sch" xr:uid="{8AC9B5FF-3554-4A3F-9A49-254FDDC1D679}"/>
-    <hyperlink ref="G29" r:id="rId91" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-4" xr:uid="{A6F45EEC-DFC1-4F41-A737-7D50D323F858}"/>
-    <hyperlink ref="G30" r:id="rId92" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-6" xr:uid="{E8092E13-22EC-4AA4-A0E2-CB8C894814DA}"/>
-    <hyperlink ref="G31" r:id="rId93" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-8" xr:uid="{06C47C82-BB6B-4167-9AFC-F87F629A6D2D}"/>
-    <hyperlink ref="G32" r:id="rId94" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-actun-zetos" xr:uid="{7F484481-A382-4AA7-BC6F-9F9E8E881F13}"/>
-    <hyperlink ref="G33" r:id="rId95" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-14-24" xr:uid="{145E082E-ACF5-4C03-95AA-D5FF287B68E9}"/>
-    <hyperlink ref="J29" r:id="rId96" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-medana-ch1-l" xr:uid="{CB6CAFF8-329E-47DC-8F46-39C8BB5E04DD}"/>
-    <hyperlink ref="J30" r:id="rId97" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-zeox-first-h" xr:uid="{2D403080-ECF0-434D-8570-2DCE4384BDB3}"/>
-    <hyperlink ref="K29" r:id="rId98" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-helix-v" xr:uid="{24EB14FB-8853-4DD9-BFF7-D08622F6269E}"/>
-    <hyperlink ref="K30" r:id="rId99" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-helix-first-v" xr:uid="{292648A6-CEF7-4F6A-B9E8-2C2D1935D493}"/>
-    <hyperlink ref="L29" r:id="rId100" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-helix-ve" xr:uid="{CB04A41A-2CE9-45EC-90FB-F63D1D7003E0}"/>
-    <hyperlink ref="L30" r:id="rId101" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-helix2-0-ve" xr:uid="{0D95BEE0-BF20-4117-86C3-9423999074AC}"/>
-    <hyperlink ref="M29" r:id="rId102" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-medana-ch3-le" xr:uid="{E61CDC21-E587-41FD-8720-AA95E8F2BCB8}"/>
-    <hyperlink ref="N29" r:id="rId103" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-isar-modh1-e-2-3" xr:uid="{2D23D0CC-B7DF-4FF1-ABE9-A9C38B0D675F}"/>
-    <hyperlink ref="N30" r:id="rId104" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-siboost2-0-smart-helix-ve" xr:uid="{FFEEE275-2C73-4EC4-B193-CB85762B0142}"/>
-    <hyperlink ref="O29" r:id="rId105" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-pro" xr:uid="{40187CA6-E027-4F57-B695-B124E41E9781}"/>
-    <hyperlink ref="O30" r:id="rId106" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-supra" xr:uid="{6510CD0A-CFE7-486C-91AF-7C7A655B4AFB}"/>
-    <hyperlink ref="O31" r:id="rId107" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-solid" xr:uid="{BDC567B5-AC65-4996-9A0B-1AF09DF2041A}"/>
-    <hyperlink ref="Q29" r:id="rId108" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-bloc" xr:uid="{3980AF89-63D6-4F8A-AA62-E67520B41458}"/>
-    <hyperlink ref="Q30" r:id="rId109" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-norm" xr:uid="{713EE9E0-CE07-4B5A-8098-8828FD7A2BE1}"/>
-    <hyperlink ref="P29" r:id="rId110" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-pro-s" xr:uid="{7EA67BA6-0CB9-4BC2-8D2F-2187D3E3EC87}"/>
-    <hyperlink ref="O32" r:id="rId111" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-fa-configure" xr:uid="{F271E929-C189-489C-95BA-44C8F95B9706}"/>
-    <hyperlink ref="S29" r:id="rId112" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-pro" xr:uid="{4E520461-D8CA-4714-95A3-4A07D979003B}"/>
-    <hyperlink ref="S30" r:id="rId113" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-supra" xr:uid="{7E747CBF-258D-4F97-AE71-AF52B950EDDE}"/>
-    <hyperlink ref="S31" r:id="rId114" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-solid" xr:uid="{90F21445-AD91-480E-9E60-99DEEB471A24}"/>
-    <hyperlink ref="S32" r:id="rId115" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-fa-configure" xr:uid="{CAC9CBDD-5033-4067-92F5-E1A89E7A10BF}"/>
-    <hyperlink ref="U29" r:id="rId116" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-pro" xr:uid="{DED143CB-BC81-4CC1-99AF-6D9EFDCA04A2}"/>
-    <hyperlink ref="U30" r:id="rId117" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-supra" xr:uid="{AD0F4A4E-82E3-443D-B5CE-BB1383456F96}"/>
-    <hyperlink ref="U31" r:id="rId118" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-solid" xr:uid="{F30C0BD2-ACC1-498E-B06C-26D556B514B6}"/>
-    <hyperlink ref="U32" r:id="rId119" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-fa-configure" xr:uid="{FC92FF04-817E-49C9-B9E1-3FED19E3DBAA}"/>
-    <hyperlink ref="W29" r:id="rId120" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-drain-tm-tmw-tmr-32" xr:uid="{0F177732-3552-46D9-B2A1-0858315CC611}"/>
-    <hyperlink ref="W30" r:id="rId121" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-padus-uni" xr:uid="{31C21B43-5DBE-431A-A886-4FBC3A6BE491}"/>
-    <hyperlink ref="W31" r:id="rId122" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-padus-mini3" xr:uid="{D91894CF-CB16-4C43-980E-41E743666848}"/>
-    <hyperlink ref="W32" r:id="rId123" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-padus-pro" xr:uid="{79DE7E3B-A7A2-4098-B5DF-694F7F93640D}"/>
-    <hyperlink ref="Z29" r:id="rId124" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-cof-helix" xr:uid="{2E5216D3-37DA-48CB-ABA0-7C21064BB2D3}"/>
+    <hyperlink ref="C22" r:id="rId1" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/sp?tab=models" xr:uid="{FE987DC0-578A-4A81-AB17-6E49D6983782}"/>
+    <hyperlink ref="C23" r:id="rId2" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/spe?tab=models" xr:uid="{E414E66B-6D50-4BC0-93B6-EEDD71D1D349}"/>
+    <hyperlink ref="C24" r:id="rId3" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/sp-ne?tab=models" xr:uid="{79A82224-5E75-416A-BD5C-1C442DB4F9E7}"/>
+    <hyperlink ref="D22" r:id="rId4" display="https://product-selection.grundfos.com/fr/products/bm?tab=products" xr:uid="{39935FC4-BF60-4ADA-99B8-6280D11B4087}"/>
+    <hyperlink ref="D23" r:id="rId5" display="https://product-selection.grundfos.com/fr/products/bms?tab=products" xr:uid="{201298BF-F5B7-4DD8-896A-A6CFDF20A155}"/>
+    <hyperlink ref="D24" r:id="rId6" display="https://product-selection.grundfos.com/fr/products/bm-hp?tab=products" xr:uid="{0AA34BB7-1783-4351-AB39-2E3E2C9E6D24}"/>
+    <hyperlink ref="E22" r:id="rId7" display="https://product-selection.grundfos.com/fr/products/kpl?tab=models" xr:uid="{02FD05D5-211D-4185-A911-F718E163AF22}"/>
+    <hyperlink ref="E23" r:id="rId8" display="https://product-selection.grundfos.com/fr/products/kwm?tab=documentation" xr:uid="{F11B5E61-F53C-4DA1-93C5-A57D0408930C}"/>
+    <hyperlink ref="F22" r:id="rId9" display="https://product-selection.grundfos.com/fr/products/ls?tab=products" xr:uid="{070C34E9-9C05-4522-9AD2-8E6D82261A9B}"/>
+    <hyperlink ref="J22" r:id="rId10" display="https://product-selection.grundfos.com/fr/products/cm-cme?tab=products" xr:uid="{E79A5B97-E6E0-4649-B070-9A1CF47F88B2}"/>
+    <hyperlink ref="I22" r:id="rId11" display="https://product-selection.grundfos.com/fr/products/cm-cme/cm-self-priming?tab=models" xr:uid="{CFEF6DD3-2F90-4195-BA05-DEE28F55BD3E}"/>
+    <hyperlink ref="J23" r:id="rId12" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nb?tab=documentation" xr:uid="{ABC208A8-FE5B-4CC4-B585-6A3873FA7294}"/>
+    <hyperlink ref="J24" r:id="rId13" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nbe?tab=models" xr:uid="{1D4EF590-19C1-44EB-8B92-46AD5F28F62F}"/>
+    <hyperlink ref="J25" r:id="rId14" display="https://product-selection.grundfos.com/fr/products/nk-nke-nke-series-2000-nk-bare-shaft?tab=products" xr:uid="{76D3161D-F2DD-4CCA-AC1D-AD2E393D8694}"/>
+    <hyperlink ref="J26" r:id="rId15" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft?tab=products" xr:uid="{9CA4757F-439C-4161-8B60-7C14A9EDCA69}"/>
+    <hyperlink ref="J27" r:id="rId16" display="https://product-selection.grundfos.com/fr/products/tp-tpe?tab=products" xr:uid="{0C9A1473-1926-417A-947F-8561754B7D76}"/>
+    <hyperlink ref="N24" r:id="rId17" display="https://product-selection.grundfos.com/fr/products/tp-tpe?tab=products" xr:uid="{7D2D046F-1C95-42DD-8F35-90280675B9EA}"/>
+    <hyperlink ref="N22" r:id="rId18" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nbe?tab=models" xr:uid="{303D01A6-AC7B-42EE-AE09-2A10FBED3940}"/>
+    <hyperlink ref="N23" r:id="rId19" display="https://product-selection.grundfos.com/fr/products/nk-nke-nke-series-2000-nk-bare-shaft?tab=products" xr:uid="{A1442A3E-E286-4D87-BF5A-B52C00F11931}"/>
+    <hyperlink ref="N25" r:id="rId20" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft?tab=products" xr:uid="{91C811C0-E7C2-45CC-8C4A-41851188982F}"/>
+    <hyperlink ref="K22" r:id="rId21" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte?tab=products" xr:uid="{168A97AE-925F-4CB8-99FA-4D28B053F7CB}"/>
+    <hyperlink ref="L23" r:id="rId22" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte/cre?tab=models" xr:uid="{43E68B92-4EB3-4ECE-A299-C7DDCAFB1889}"/>
+    <hyperlink ref="L24" r:id="rId23" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte/crne?tab=models" xr:uid="{9DD9406E-F477-49F6-BA29-841ED00CE74B}"/>
+    <hyperlink ref="M22" r:id="rId24" display="https://product-selection.grundfos.com/fr/products/cm-cme/cme?tab=models" xr:uid="{CB210458-379C-4663-B0FD-73E843090C67}"/>
+    <hyperlink ref="M23" r:id="rId25" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nbe?tab=models" xr:uid="{3776F606-4CBE-49B1-912C-5B2BC9586206}"/>
+    <hyperlink ref="M24" r:id="rId26" display="https://product-selection.grundfos.com/fr/products/nk-nke-nke-series-2000-nk-bare-shaft?tab=products" xr:uid="{8731A9E7-9B51-450F-BCB5-013214A2B33F}"/>
+    <hyperlink ref="M25" r:id="rId27" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft?tab=products" xr:uid="{EDB8C821-F675-4CE1-B7B0-0FAF39DCEFD4}"/>
+    <hyperlink ref="L26" r:id="rId28" display="https://product-selection.grundfos.com/fr/products/hydro-multi-e?tab=models" xr:uid="{5995DFA3-65AE-4378-BD2E-CDA4F6FA5ED7}"/>
+    <hyperlink ref="L27" r:id="rId29" display="https://product-selection.grundfos.com/fr/products/hydro-mpc?tab=products" xr:uid="{2E37CE89-9B22-43AA-B967-C6F20A25613F}"/>
+    <hyperlink ref="L25" r:id="rId30" display="https://product-selection.grundfos.com/fr/products/hydro-solo-e?tab=models" xr:uid="{5A1F2584-1AA0-4C8B-A55D-39C825C8A3F8}"/>
+    <hyperlink ref="O22" r:id="rId31" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/sl1?tab=models" xr:uid="{9C7E88DB-59BA-4B5C-8769-45D64CC97D40}"/>
+    <hyperlink ref="O23" r:id="rId32" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/slv?tab=models" xr:uid="{00039B9D-B404-44A8-B557-BBF172D7CD31}"/>
+    <hyperlink ref="O24" r:id="rId33" display="https://product-selection.grundfos.com/fr/products/sesl-9-30-kw?tab=models" xr:uid="{C90FBAD5-7C9C-4429-9BAC-9BE027B562FD}"/>
+    <hyperlink ref="O26" r:id="rId34" display="https://product-selection.grundfos.com/fr/products/s?tab=products" xr:uid="{6F267867-1729-460E-9939-DEBA10D95429}"/>
+    <hyperlink ref="O25" r:id="rId35" display="https://product-selection.grundfos.com/fr/products/sesl-frame-size-56?tab=models" xr:uid="{541D6F69-2D4F-412B-91C7-A0B79C20C0CA}"/>
+    <hyperlink ref="P23" r:id="rId36" display="https://product-selection.grundfos.com/fr/products/unilift-ap/unilift-apg?tab=models" xr:uid="{CF6542DD-C411-4584-A2A2-ADD9BD336104}"/>
+    <hyperlink ref="P22" r:id="rId37" display="https://product-selection.grundfos.com/fr/products/seg?tab=models" xr:uid="{AF847B64-9B08-45DD-8487-57C6900B0D5F}"/>
+    <hyperlink ref="Q22" r:id="rId38" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/se1?tab=models" xr:uid="{D2271F27-967E-46DC-8195-E2EAFD3339EB}"/>
+    <hyperlink ref="Q23" r:id="rId39" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/sev?tab=models" xr:uid="{6D042873-5F32-4A50-8803-93F40528C6A1}"/>
+    <hyperlink ref="Q24" r:id="rId40" display="https://product-selection.grundfos.com/fr/products/sesl-9-30-kw?tab=models" xr:uid="{A344F5B5-8A97-456F-87D5-4C6EFCA52D3A}"/>
+    <hyperlink ref="Q25" r:id="rId41" display="https://product-selection.grundfos.com/fr/products/sesl-frame-size-56?tab=models" xr:uid="{BB0B40A3-A20A-44BC-9FC9-E9EE00FC9F45}"/>
+    <hyperlink ref="Q26" r:id="rId42" display="https://product-selection.grundfos.com/fr/products/s?tab=products" xr:uid="{2E26D22E-3FD7-4718-9B39-661D30AF938C}"/>
+    <hyperlink ref="Q27" r:id="rId43" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft/nkg-supervortex-impeller?tab=explore" xr:uid="{FA539854-B47D-4B47-9F9A-7CE595B28025}"/>
+    <hyperlink ref="S22" r:id="rId44" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/se1?tab=models" xr:uid="{66C50FE8-D6EA-4602-866A-7B3258A9261C}"/>
+    <hyperlink ref="S23" r:id="rId45" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/sev?tab=models" xr:uid="{DEFE3A48-5152-4917-935D-8BAB7D40CDD7}"/>
+    <hyperlink ref="S24" r:id="rId46" display="https://product-selection.grundfos.com/fr/products/sesl-9-30-kw?tab=models" xr:uid="{62BA715F-3850-4F49-A593-7645C6C0C3CC}"/>
+    <hyperlink ref="S25" r:id="rId47" display="https://product-selection.grundfos.com/fr/products/sesl-frame-size-56?tab=models" xr:uid="{F0AA29DC-4DA5-4CA6-94B3-C22351F6904E}"/>
+    <hyperlink ref="S26" r:id="rId48" display="https://product-selection.grundfos.com/fr/products/s?tab=products" xr:uid="{96671AB9-9AEA-4A5F-B84F-E78888F9B311}"/>
+    <hyperlink ref="S27" r:id="rId49" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft/nkg-supervortex-impeller?tab=explore" xr:uid="{8A1CF826-08F5-4AF2-B984-9AA020480952}"/>
+    <hyperlink ref="O27" r:id="rId50" display="https://product-selection.grundfos.com/fr/products/unilift-ap/unilift-ap50b?tab=models" xr:uid="{14E21A07-FF5F-4129-AE6E-260A1AA5098C}"/>
+    <hyperlink ref="W22" r:id="rId51" display="https://product-selection.grundfos.com/fr/products/unilift-ap?tab=products" xr:uid="{FF1F3D5A-16C1-4C5A-8F69-37BEB2C51657}"/>
+    <hyperlink ref="W23" r:id="rId52" display="https://product-selection.grundfos.com/fr/products/unilift-kp?tab=models" xr:uid="{D8B15CDE-A46F-4955-8CE5-B1F2491BDDEE}"/>
+    <hyperlink ref="W24" r:id="rId53" display="https://product-selection.grundfos.com/fr/products/unilift-cc?tab=models" xr:uid="{5DA16314-BD6C-4DB3-8EC0-A99C56D3006D}"/>
+    <hyperlink ref="W25" r:id="rId54" display="https://product-selection.grundfos.com/fr/products/dp?tab=models" xr:uid="{4D82ED98-3DD6-4697-9C9C-A060C7E06489}"/>
+    <hyperlink ref="W26" r:id="rId55" display="https://product-selection.grundfos.com/fr/products/ef?tab=models" xr:uid="{ABDE8970-72CB-4EB8-979F-99183A9FD9D3}"/>
+    <hyperlink ref="Y22" r:id="rId56" display="https://product-selection.grundfos.com/fr/products/mt-tank-mounted-pumps/mtr?tab=models" xr:uid="{D5799B15-EF87-41DF-88D8-05F25935D793}"/>
+    <hyperlink ref="Y23" r:id="rId57" display="https://product-selection.grundfos.com/fr/products/mt-tank-mounted-pumps/mtre?tab=models" xr:uid="{7E2DAAB5-3884-49DD-BF25-FA92C2CE9951}"/>
+    <hyperlink ref="Y24" r:id="rId58" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nb?tab=documentation" xr:uid="{92C19ACB-7462-4938-A66E-478979299908}"/>
+    <hyperlink ref="Y25" r:id="rId59" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nbe?tab=models" xr:uid="{D2CCE95F-A5DF-4715-B3CA-DB297F6DF5C8}"/>
+    <hyperlink ref="Y26" r:id="rId60" display="https://product-selection.grundfos.com/fr/products/nk-nke-nke-series-2000-nk-bare-shaft?tab=products" xr:uid="{EA080A36-FCEB-4D04-B389-F8ABE5514300}"/>
+    <hyperlink ref="Y27" r:id="rId61" display="https://product-selection.grundfos.com/fr/products/tp-tpe?tab=products" xr:uid="{2A2A6B6D-2CAA-4110-9FED-BCA8DC5F1709}"/>
+    <hyperlink ref="Y28" r:id="rId62" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte?tab=products" xr:uid="{D902984C-2BC5-48A4-BF49-DCE4C7E629F6}"/>
+    <hyperlink ref="Z22" r:id="rId63" display="https://product-selection.grundfos.com/fr/products/hydro-en?tab=models" xr:uid="{69CECDCF-71ED-40D6-A274-30663F73D3A6}"/>
+    <hyperlink ref="AD22" r:id="rId64" display="https://product-selection.grundfos.com/fr/products/poweradapt?tab=models" xr:uid="{CBB79406-3EE4-4CC7-BCD3-398882D58A96}"/>
+    <hyperlink ref="AD23" r:id="rId65" display="https://product-selection.grundfos.com/fr/products/rsi?tab=models" xr:uid="{2ECDD4BA-B757-4A11-9F78-EB235920F462}"/>
+    <hyperlink ref="AD24" r:id="rId66" display="https://product-selection.grundfos.com/fr/products/crflex?tab=models" xr:uid="{F1835770-C21F-4E8A-9EBF-7C701B0E9CF4}"/>
+    <hyperlink ref="AD25" r:id="rId67" display="https://product-selection.grundfos.com/fr/products/sqflex?tab=models" xr:uid="{2932EAA4-553E-42B6-AD4B-37D91C9B845C}"/>
+    <hyperlink ref="AD26" r:id="rId68" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/sp?tab=models" xr:uid="{25A70C6E-05E1-4E40-956B-50B78B088135}"/>
+    <hyperlink ref="AD27" r:id="rId69" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/spe?tab=models" xr:uid="{7C346AF6-2EEB-4DFC-A819-DAE2C3B09113}"/>
+    <hyperlink ref="AD28" r:id="rId70" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte?tab=products" xr:uid="{9F4AE584-6CDD-45BE-ABC9-5087AAD766B9}"/>
+    <hyperlink ref="AE22" r:id="rId71" display="https://product-selection.grundfos.com/fr/products/dosing-pumps-digital/dda?tab=models" xr:uid="{68600FE5-FDB0-4237-8B8A-45786462FE8A}"/>
+    <hyperlink ref="AE23" r:id="rId72" display="https://product-selection.grundfos.com/fr/products/dosing-pumps-digital/dme?tab=models" xr:uid="{41502941-2297-46B7-A840-2EF7A24064D7}"/>
+    <hyperlink ref="AE24" r:id="rId73" display="https://product-selection.grundfos.com/fr/products/dosing-pumps-mechanical/dmx?tab=models" xr:uid="{A892A826-C3E1-4B26-9529-8174E76C068D}"/>
+    <hyperlink ref="AE25" r:id="rId74" display="https://product-selection.grundfos.com/fr/products/dosing-pumps-mechanical/dmh?tab=models" xr:uid="{60926621-C7DA-4892-9ACA-4145E303C37B}"/>
+    <hyperlink ref="AE26" r:id="rId75" xr:uid="{EB339B7E-AAB0-4720-A5DC-B7E47BEFE888}"/>
+    <hyperlink ref="AF24" r:id="rId76" display="https://product-selection.grundfos.com/fr/products/disinfection-systems/oxiperm?tab=models" xr:uid="{D1CFBDC1-076A-4661-B343-B5087946D2BF}"/>
+    <hyperlink ref="AF22" r:id="rId77" display="https://product-selection.grundfos.com/fr/products/disinfection-systems/vaccuperm?tab=models" xr:uid="{0E5CA30E-D80E-4BC1-BE8D-5757C0E703F9}"/>
+    <hyperlink ref="AF23" r:id="rId78" display="https://product-selection.grundfos.com/fr/products/disinfection-systems/selcoperm?tab=models" xr:uid="{3FE337C4-03C2-4326-92F3-2ADF14429172}"/>
+    <hyperlink ref="C30" r:id="rId79" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-4" xr:uid="{7CECB146-2C6E-4D8C-8362-B574F0A0B1CD}"/>
+    <hyperlink ref="C31" r:id="rId80" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-6" xr:uid="{77066640-D437-4393-AE04-9291CA2EA2E2}"/>
+    <hyperlink ref="C32" r:id="rId81" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-8" xr:uid="{440D559C-9B55-46F7-B47D-809066594D8E}"/>
+    <hyperlink ref="C33" r:id="rId82" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-actun-zetos" xr:uid="{6B88B868-32F8-4635-8067-C4F8AA30A87A}"/>
+    <hyperlink ref="C34" r:id="rId83" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-14-24" xr:uid="{6AAEB27D-0CD4-409C-9175-B5DC81BA5B91}"/>
+    <hyperlink ref="D30" r:id="rId84" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-4" xr:uid="{70B5668C-6DE4-4721-BD0D-15695ACCFD10}"/>
+    <hyperlink ref="D31" r:id="rId85" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-6" xr:uid="{AB0F5528-0721-49E7-9EB4-443A836A5BE6}"/>
+    <hyperlink ref="D32" r:id="rId86" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-8" xr:uid="{CE5D4CF5-B9AD-4786-AF2A-5CBA0FB4461E}"/>
+    <hyperlink ref="D33" r:id="rId87" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-actun-zetos" xr:uid="{F3302311-60D3-4257-BE0E-8ADCE8FD3F26}"/>
+    <hyperlink ref="D34" r:id="rId88" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-14-24" xr:uid="{C714C692-05B2-43B9-83CE-06CDCF547DAA}"/>
+    <hyperlink ref="F30" r:id="rId89" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-scp" xr:uid="{7BEBF8BE-E457-43DD-A078-9A05C9712ED1}"/>
+    <hyperlink ref="F31" r:id="rId90" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-atmos-tera-sch" xr:uid="{8AC9B5FF-3554-4A3F-9A49-254FDDC1D679}"/>
+    <hyperlink ref="G30" r:id="rId91" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-4" xr:uid="{A6F45EEC-DFC1-4F41-A737-7D50D323F858}"/>
+    <hyperlink ref="G31" r:id="rId92" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-6" xr:uid="{E8092E13-22EC-4AA4-A0E2-CB8C894814DA}"/>
+    <hyperlink ref="G32" r:id="rId93" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-8" xr:uid="{06C47C82-BB6B-4167-9AFC-F87F629A6D2D}"/>
+    <hyperlink ref="G33" r:id="rId94" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-actun-zetos" xr:uid="{7F484481-A382-4AA7-BC6F-9F9E8E881F13}"/>
+    <hyperlink ref="G34" r:id="rId95" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-14-24" xr:uid="{145E082E-ACF5-4C03-95AA-D5FF287B68E9}"/>
+    <hyperlink ref="J30" r:id="rId96" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-medana-ch1-l" xr:uid="{CB6CAFF8-329E-47DC-8F46-39C8BB5E04DD}"/>
+    <hyperlink ref="J31" r:id="rId97" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-zeox-first-h" xr:uid="{2D403080-ECF0-434D-8570-2DCE4384BDB3}"/>
+    <hyperlink ref="K30" r:id="rId98" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-helix-v" xr:uid="{24EB14FB-8853-4DD9-BFF7-D08622F6269E}"/>
+    <hyperlink ref="K31" r:id="rId99" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-helix-first-v" xr:uid="{292648A6-CEF7-4F6A-B9E8-2C2D1935D493}"/>
+    <hyperlink ref="L30" r:id="rId100" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-helix-ve" xr:uid="{CB04A41A-2CE9-45EC-90FB-F63D1D7003E0}"/>
+    <hyperlink ref="L31" r:id="rId101" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-helix2-0-ve" xr:uid="{0D95BEE0-BF20-4117-86C3-9423999074AC}"/>
+    <hyperlink ref="M30" r:id="rId102" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-medana-ch3-le" xr:uid="{E61CDC21-E587-41FD-8720-AA95E8F2BCB8}"/>
+    <hyperlink ref="N30" r:id="rId103" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-isar-modh1-e-2-3" xr:uid="{2D23D0CC-B7DF-4FF1-ABE9-A9C38B0D675F}"/>
+    <hyperlink ref="N31" r:id="rId104" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-siboost2-0-smart-helix-ve" xr:uid="{FFEEE275-2C73-4EC4-B193-CB85762B0142}"/>
+    <hyperlink ref="O30" r:id="rId105" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-pro" xr:uid="{40187CA6-E027-4F57-B695-B124E41E9781}"/>
+    <hyperlink ref="O31" r:id="rId106" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-supra" xr:uid="{6510CD0A-CFE7-486C-91AF-7C7A655B4AFB}"/>
+    <hyperlink ref="O32" r:id="rId107" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-solid" xr:uid="{BDC567B5-AC65-4996-9A0B-1AF09DF2041A}"/>
+    <hyperlink ref="Q30" r:id="rId108" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-bloc" xr:uid="{3980AF89-63D6-4F8A-AA62-E67520B41458}"/>
+    <hyperlink ref="Q31" r:id="rId109" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-norm" xr:uid="{713EE9E0-CE07-4B5A-8098-8828FD7A2BE1}"/>
+    <hyperlink ref="P30" r:id="rId110" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-pro-s" xr:uid="{7EA67BA6-0CB9-4BC2-8D2F-2187D3E3EC87}"/>
+    <hyperlink ref="O33" r:id="rId111" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-fa-configure" xr:uid="{F271E929-C189-489C-95BA-44C8F95B9706}"/>
+    <hyperlink ref="S30" r:id="rId112" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-pro" xr:uid="{4E520461-D8CA-4714-95A3-4A07D979003B}"/>
+    <hyperlink ref="S31" r:id="rId113" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-supra" xr:uid="{7E747CBF-258D-4F97-AE71-AF52B950EDDE}"/>
+    <hyperlink ref="S32" r:id="rId114" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-solid" xr:uid="{90F21445-AD91-480E-9E60-99DEEB471A24}"/>
+    <hyperlink ref="S33" r:id="rId115" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-fa-configure" xr:uid="{CAC9CBDD-5033-4067-92F5-E1A89E7A10BF}"/>
+    <hyperlink ref="U30" r:id="rId116" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-pro" xr:uid="{DED143CB-BC81-4CC1-99AF-6D9EFDCA04A2}"/>
+    <hyperlink ref="U31" r:id="rId117" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-supra" xr:uid="{AD0F4A4E-82E3-443D-B5CE-BB1383456F96}"/>
+    <hyperlink ref="U32" r:id="rId118" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-solid" xr:uid="{F30C0BD2-ACC1-498E-B06C-26D556B514B6}"/>
+    <hyperlink ref="U33" r:id="rId119" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-fa-configure" xr:uid="{FC92FF04-817E-49C9-B9E1-3FED19E3DBAA}"/>
+    <hyperlink ref="W30" r:id="rId120" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-drain-tm-tmw-tmr-32" xr:uid="{0F177732-3552-46D9-B2A1-0858315CC611}"/>
+    <hyperlink ref="W31" r:id="rId121" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-padus-uni" xr:uid="{31C21B43-5DBE-431A-A886-4FBC3A6BE491}"/>
+    <hyperlink ref="W32" r:id="rId122" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-padus-mini3" xr:uid="{D91894CF-CB16-4C43-980E-41E743666848}"/>
+    <hyperlink ref="W33" r:id="rId123" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-padus-pro" xr:uid="{79DE7E3B-A7A2-4098-B5DF-694F7F93640D}"/>
+    <hyperlink ref="Z30" r:id="rId124" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-cof-helix" xr:uid="{2E5216D3-37DA-48CB-ABA0-7C21064BB2D3}"/>
   </hyperlinks>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="8" scale="83" orientation="landscape" r:id="rId125"/>

</xml_diff>

<commit_message>
Mise à jour depuis Excel — 2026-10-05T17:33:21.715Z
</commit_message>
<xml_diff>
--- a/comparatif.xlsx
+++ b/comparatif.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30516"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30601"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nge1.sharepoint.com/sites/FR_SADE_DAM/Documents partages/01 - Achats/Achats Production/Pompes &amp; Instrum/Pompes/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nge1.sharepoint.com/sites/FR_SADE_DAM/Documents partages/01 - Achats/Achats Production/Pompes &amp; Instrum/Pompes/ABAQUE POMPES/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3AF0930F-4E2D-4EA3-92AF-769AB043B375}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7827D0F7-18B5-442C-A64F-98E374DE428A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7716" yWindow="12852" windowWidth="23256" windowHeight="12456" xr2:uid="{723C6001-552E-447F-BEBB-92F546F7738F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{723C6001-552E-447F-BEBB-92F546F7738F}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
     <sheet name="Feuil2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Feuil1!$A$2:$AF$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Feuil1!$A$2:$AF$33</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="286">
   <si>
     <t>Eau potable et irrigation</t>
   </si>
@@ -87,19 +87,13 @@
     <t>Pompes immergées</t>
   </si>
   <si>
-    <t>Surface 4 4</t>
+    <t>Surface</t>
   </si>
   <si>
     <t>Immergées</t>
   </si>
   <si>
     <t>De surface</t>
-  </si>
-  <si>
-    <t>essai</t>
-  </si>
-  <si>
-    <t>&amp;</t>
   </si>
   <si>
     <t>Types</t>
@@ -1098,7 +1092,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="39">
+  <borders count="38">
     <border>
       <left/>
       <right/>
@@ -1585,22 +1579,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="124">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1935,18 +1920,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2294,7 +2267,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:EY61"/>
+  <dimension ref="A1:EY60"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="7.140625" style="1" customWidth="1"/>
@@ -2311,7 +2284,7 @@
     <col min="33" max="16384" width="11.42578125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" ht="12.75" thickBot="1"/>
+    <row r="1" spans="1:32" ht="12.6" thickBot="1"/>
     <row r="2" spans="1:32" s="70" customFormat="1" ht="23.25" customHeight="1" thickBot="1">
       <c r="A2" s="68"/>
       <c r="B2" s="69"/>
@@ -2414,41 +2387,70 @@
       <c r="AE3" s="103"/>
       <c r="AF3" s="103"/>
     </row>
-    <row r="4" spans="1:32" s="70" customFormat="1" ht="23.25" customHeight="1">
-      <c r="A4" s="68"/>
-      <c r="B4" s="71" t="s">
+    <row r="4" spans="1:32" s="80" customFormat="1" ht="57.75" customHeight="1">
+      <c r="B4" s="81" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="120" t="s">
+      <c r="C4" s="82" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="121">
-        <v>2</v>
-      </c>
-      <c r="E4" s="121">
-        <v>3</v>
-      </c>
-      <c r="F4" s="121"/>
-      <c r="G4" s="120">
-        <v>4</v>
-      </c>
-      <c r="H4" s="121">
-        <v>9</v>
-      </c>
-      <c r="I4" s="121"/>
-      <c r="J4" s="121"/>
-      <c r="K4" s="121"/>
-      <c r="L4" s="121"/>
-      <c r="M4" s="121"/>
-      <c r="N4" s="122"/>
-      <c r="O4" s="120"/>
-      <c r="P4" s="121"/>
-      <c r="Q4" s="120"/>
-      <c r="R4" s="121"/>
-      <c r="S4" s="121"/>
-      <c r="T4" s="122"/>
-      <c r="U4" s="123"/>
-      <c r="V4" s="123"/>
+      <c r="D4" s="82" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="82" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="82" t="s">
+        <v>21</v>
+      </c>
+      <c r="G4" s="82" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="82" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" s="82" t="s">
+        <v>24</v>
+      </c>
+      <c r="J4" s="82" t="s">
+        <v>25</v>
+      </c>
+      <c r="K4" s="82" t="s">
+        <v>26</v>
+      </c>
+      <c r="L4" s="82" t="s">
+        <v>27</v>
+      </c>
+      <c r="M4" s="82" t="s">
+        <v>28</v>
+      </c>
+      <c r="N4" s="82" t="s">
+        <v>28</v>
+      </c>
+      <c r="O4" s="82" t="s">
+        <v>29</v>
+      </c>
+      <c r="P4" s="82" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q4" s="82" t="s">
+        <v>31</v>
+      </c>
+      <c r="R4" s="82" t="s">
+        <v>32</v>
+      </c>
+      <c r="S4" s="82" t="s">
+        <v>33</v>
+      </c>
+      <c r="T4" s="82" t="s">
+        <v>34</v>
+      </c>
+      <c r="U4" s="83" t="s">
+        <v>15</v>
+      </c>
+      <c r="V4" s="83" t="s">
+        <v>35</v>
+      </c>
       <c r="W4" s="117"/>
       <c r="X4" s="105"/>
       <c r="Y4" s="105"/>
@@ -2460,246 +2462,235 @@
       <c r="AE4" s="103"/>
       <c r="AF4" s="106"/>
     </row>
-    <row r="5" spans="1:32" s="80" customFormat="1" ht="57.75" customHeight="1">
-      <c r="B5" s="81" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" s="82" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5" s="82" t="s">
-        <v>21</v>
-      </c>
-      <c r="E5" s="82" t="s">
-        <v>22</v>
-      </c>
-      <c r="F5" s="82" t="s">
-        <v>23</v>
-      </c>
-      <c r="G5" s="82" t="s">
-        <v>24</v>
-      </c>
-      <c r="H5" s="82" t="s">
-        <v>25</v>
-      </c>
-      <c r="I5" s="82" t="s">
-        <v>26</v>
-      </c>
-      <c r="J5" s="82" t="s">
-        <v>27</v>
-      </c>
-      <c r="K5" s="82" t="s">
-        <v>28</v>
-      </c>
-      <c r="L5" s="82" t="s">
-        <v>29</v>
-      </c>
-      <c r="M5" s="82" t="s">
-        <v>30</v>
-      </c>
-      <c r="N5" s="82" t="s">
-        <v>30</v>
-      </c>
-      <c r="O5" s="82" t="s">
-        <v>31</v>
-      </c>
-      <c r="P5" s="82" t="s">
-        <v>32</v>
-      </c>
-      <c r="Q5" s="82" t="s">
-        <v>33</v>
-      </c>
-      <c r="R5" s="82" t="s">
-        <v>34</v>
-      </c>
-      <c r="S5" s="82" t="s">
-        <v>35</v>
-      </c>
-      <c r="T5" s="82" t="s">
+    <row r="5" spans="1:32" s="80" customFormat="1" ht="10.15" customHeight="1" thickBot="1">
+      <c r="B5" s="87"/>
+      <c r="C5" s="88"/>
+      <c r="D5" s="88"/>
+      <c r="E5" s="88"/>
+      <c r="F5" s="88"/>
+      <c r="G5" s="88"/>
+      <c r="H5" s="88"/>
+      <c r="I5" s="88"/>
+      <c r="J5" s="88"/>
+      <c r="K5" s="88"/>
+      <c r="L5" s="88"/>
+      <c r="M5" s="88"/>
+      <c r="N5" s="88"/>
+      <c r="O5" s="88"/>
+      <c r="P5" s="88"/>
+      <c r="Q5" s="88"/>
+      <c r="R5" s="88"/>
+      <c r="S5" s="88"/>
+      <c r="T5" s="88"/>
+      <c r="U5" s="89"/>
+      <c r="V5" s="89"/>
+      <c r="W5" s="86"/>
+      <c r="X5" s="86"/>
+      <c r="Y5" s="86"/>
+      <c r="Z5" s="86"/>
+      <c r="AA5" s="86"/>
+      <c r="AB5" s="86"/>
+      <c r="AC5" s="90"/>
+      <c r="AD5" s="91"/>
+      <c r="AE5" s="91"/>
+      <c r="AF5" s="91"/>
+    </row>
+    <row r="6" spans="1:32" s="74" customFormat="1" ht="52.9" customHeight="1">
+      <c r="B6" s="84" t="s">
         <v>36</v>
       </c>
-      <c r="U5" s="83" t="s">
-        <v>15</v>
-      </c>
-      <c r="V5" s="83" t="s">
+      <c r="C6" s="77" t="s">
         <v>37</v>
       </c>
-      <c r="W5" s="117"/>
-      <c r="X5" s="105"/>
-      <c r="Y5" s="105"/>
-      <c r="Z5" s="105"/>
-      <c r="AA5" s="105"/>
-      <c r="AB5" s="105"/>
-      <c r="AC5" s="105"/>
-      <c r="AD5" s="103"/>
-      <c r="AE5" s="103"/>
-      <c r="AF5" s="106"/>
+      <c r="D6" s="77" t="s">
+        <v>38</v>
+      </c>
+      <c r="E6" s="77" t="s">
+        <v>39</v>
+      </c>
+      <c r="F6" s="77" t="s">
+        <v>38</v>
+      </c>
+      <c r="G6" s="77" t="s">
+        <v>40</v>
+      </c>
+      <c r="H6" s="77" t="s">
+        <v>38</v>
+      </c>
+      <c r="I6" s="77" t="s">
+        <v>41</v>
+      </c>
+      <c r="J6" s="77" t="s">
+        <v>38</v>
+      </c>
+      <c r="K6" s="77" t="s">
+        <v>38</v>
+      </c>
+      <c r="L6" s="77" t="s">
+        <v>37</v>
+      </c>
+      <c r="M6" s="77" t="s">
+        <v>38</v>
+      </c>
+      <c r="N6" s="77" t="s">
+        <v>42</v>
+      </c>
+      <c r="O6" s="77" t="s">
+        <v>43</v>
+      </c>
+      <c r="P6" s="77" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q6" s="77" t="s">
+        <v>43</v>
+      </c>
+      <c r="R6" s="77" t="s">
+        <v>43</v>
+      </c>
+      <c r="S6" s="77" t="s">
+        <v>43</v>
+      </c>
+      <c r="T6" s="77" t="s">
+        <v>43</v>
+      </c>
+      <c r="U6" s="77" t="s">
+        <v>43</v>
+      </c>
+      <c r="V6" s="77" t="s">
+        <v>43</v>
+      </c>
+      <c r="W6" s="77"/>
+      <c r="X6" s="77" t="s">
+        <v>44</v>
+      </c>
+      <c r="Y6" s="77" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z6" s="77"/>
+      <c r="AA6" s="77"/>
+      <c r="AB6" s="77"/>
+      <c r="AC6" s="78"/>
+      <c r="AD6" s="79" t="s">
+        <v>46</v>
+      </c>
+      <c r="AE6" s="79" t="s">
+        <v>47</v>
+      </c>
+      <c r="AF6" s="76" t="s">
+        <v>48</v>
+      </c>
     </row>
-    <row r="6" spans="1:32" s="80" customFormat="1" ht="10.15" customHeight="1" thickBot="1">
-      <c r="B6" s="87"/>
-      <c r="C6" s="88"/>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="88"/>
-      <c r="K6" s="88"/>
-      <c r="L6" s="88"/>
-      <c r="M6" s="88"/>
-      <c r="N6" s="88"/>
-      <c r="O6" s="88"/>
-      <c r="P6" s="88"/>
-      <c r="Q6" s="88"/>
-      <c r="R6" s="88"/>
-      <c r="S6" s="88"/>
-      <c r="T6" s="88"/>
-      <c r="U6" s="89"/>
-      <c r="V6" s="89"/>
-      <c r="W6" s="86"/>
-      <c r="X6" s="86"/>
-      <c r="Y6" s="86"/>
-      <c r="Z6" s="86"/>
-      <c r="AA6" s="86"/>
-      <c r="AB6" s="86"/>
-      <c r="AC6" s="90"/>
-      <c r="AD6" s="91"/>
-      <c r="AE6" s="91"/>
-      <c r="AF6" s="91"/>
-    </row>
-    <row r="7" spans="1:32" s="74" customFormat="1" ht="52.9" customHeight="1">
-      <c r="B7" s="84" t="s">
-        <v>38</v>
-      </c>
-      <c r="C7" s="77" t="s">
-        <v>39</v>
-      </c>
-      <c r="D7" s="77" t="s">
-        <v>40</v>
-      </c>
-      <c r="E7" s="77" t="s">
-        <v>41</v>
-      </c>
-      <c r="F7" s="77" t="s">
-        <v>40</v>
-      </c>
-      <c r="G7" s="77" t="s">
-        <v>42</v>
-      </c>
-      <c r="H7" s="77" t="s">
-        <v>40</v>
-      </c>
-      <c r="I7" s="77" t="s">
-        <v>43</v>
-      </c>
-      <c r="J7" s="77" t="s">
-        <v>40</v>
-      </c>
-      <c r="K7" s="77" t="s">
-        <v>40</v>
-      </c>
-      <c r="L7" s="77" t="s">
-        <v>39</v>
-      </c>
-      <c r="M7" s="77" t="s">
-        <v>40</v>
-      </c>
-      <c r="N7" s="77" t="s">
-        <v>44</v>
-      </c>
-      <c r="O7" s="77" t="s">
-        <v>45</v>
-      </c>
-      <c r="P7" s="77" t="s">
-        <v>45</v>
-      </c>
-      <c r="Q7" s="77" t="s">
-        <v>45</v>
-      </c>
-      <c r="R7" s="77" t="s">
-        <v>45</v>
-      </c>
-      <c r="S7" s="77" t="s">
-        <v>45</v>
-      </c>
-      <c r="T7" s="77" t="s">
-        <v>45</v>
-      </c>
-      <c r="U7" s="77" t="s">
-        <v>45</v>
-      </c>
-      <c r="V7" s="77" t="s">
-        <v>45</v>
-      </c>
-      <c r="W7" s="77"/>
-      <c r="X7" s="77" t="s">
-        <v>46</v>
-      </c>
-      <c r="Y7" s="77" t="s">
-        <v>47</v>
-      </c>
-      <c r="Z7" s="77"/>
-      <c r="AA7" s="77"/>
-      <c r="AB7" s="77"/>
-      <c r="AC7" s="78"/>
-      <c r="AD7" s="79" t="s">
-        <v>48</v>
-      </c>
-      <c r="AE7" s="79" t="s">
+    <row r="7" spans="1:32" s="1" customFormat="1" ht="18" customHeight="1">
+      <c r="A7" s="107" t="s">
         <v>49</v>
       </c>
-      <c r="AF7" s="76" t="s">
+      <c r="B7" s="98" t="s">
         <v>50</v>
       </c>
+      <c r="C7" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="E7" s="11"/>
+      <c r="F7" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="I7" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="J7" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="K7" s="11"/>
+      <c r="L7" s="11"/>
+      <c r="M7" s="11"/>
+      <c r="N7" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="O7" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="P7" s="11"/>
+      <c r="Q7" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="R7" s="11"/>
+      <c r="S7" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="T7" s="11"/>
+      <c r="U7" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="V7" s="11"/>
+      <c r="W7" s="11"/>
+      <c r="X7" s="11"/>
+      <c r="Y7" s="11"/>
+      <c r="Z7" s="11"/>
+      <c r="AA7" s="11"/>
+      <c r="AB7" s="5"/>
+      <c r="AC7" s="54"/>
+      <c r="AD7" s="76"/>
+      <c r="AE7" s="76"/>
+      <c r="AF7" s="76"/>
     </row>
     <row r="8" spans="1:32" s="1" customFormat="1" ht="18" customHeight="1">
-      <c r="A8" s="107" t="s">
-        <v>51</v>
-      </c>
-      <c r="B8" s="98" t="s">
-        <v>52</v>
-      </c>
+      <c r="A8" s="108"/>
+      <c r="B8" s="96"/>
       <c r="C8" s="11" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="E8" s="11"/>
+        <v>59</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>60</v>
+      </c>
       <c r="F8" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="G8" s="11"/>
+        <v>61</v>
+      </c>
+      <c r="G8" s="11" t="s">
+        <v>60</v>
+      </c>
       <c r="H8" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="I8" s="11" t="s">
-        <v>57</v>
-      </c>
+        <v>62</v>
+      </c>
+      <c r="I8" s="11"/>
       <c r="J8" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="K8" s="11"/>
+        <v>59</v>
+      </c>
+      <c r="K8" s="11" t="s">
+        <v>63</v>
+      </c>
       <c r="L8" s="11"/>
-      <c r="M8" s="11"/>
+      <c r="M8" s="11" t="s">
+        <v>64</v>
+      </c>
       <c r="N8" s="11" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="O8" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="P8" s="11"/>
+        <v>65</v>
+      </c>
+      <c r="P8" s="11" t="s">
+        <v>65</v>
+      </c>
       <c r="Q8" s="11" t="s">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="R8" s="11"/>
       <c r="S8" s="11" t="s">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="T8" s="11"/>
       <c r="U8" s="11" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="V8" s="11"/>
       <c r="W8" s="11"/>
@@ -2716,55 +2707,39 @@
     <row r="9" spans="1:32" s="1" customFormat="1" ht="18" customHeight="1">
       <c r="A9" s="108"/>
       <c r="B9" s="96"/>
-      <c r="C9" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="E9" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="F9" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="G9" s="11" t="s">
-        <v>62</v>
-      </c>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
       <c r="H9" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="I9" s="11"/>
+      <c r="J9" s="11"/>
+      <c r="K9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="L9" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="I9" s="11"/>
-      <c r="J9" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="K9" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="L9" s="11"/>
       <c r="M9" s="11" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="N9" s="11" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="O9" s="11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="P9" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="Q9" s="11" t="s">
-        <v>68</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="Q9" s="11"/>
       <c r="R9" s="11"/>
-      <c r="S9" s="11" t="s">
-        <v>68</v>
-      </c>
+      <c r="S9" s="11"/>
       <c r="T9" s="11"/>
-      <c r="U9" s="11" t="s">
-        <v>67</v>
-      </c>
+      <c r="U9" s="11"/>
       <c r="V9" s="11"/>
       <c r="W9" s="11"/>
       <c r="X9" s="11"/>
@@ -2786,28 +2761,20 @@
       <c r="F10" s="11"/>
       <c r="G10" s="11"/>
       <c r="H10" s="11" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I10" s="11"/>
       <c r="J10" s="11"/>
-      <c r="K10" s="11" t="s">
-        <v>54</v>
-      </c>
+      <c r="K10" s="11"/>
       <c r="L10" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="M10" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="N10" s="11" t="s">
-        <v>70</v>
-      </c>
+        <v>59</v>
+      </c>
+      <c r="M10" s="11"/>
+      <c r="N10" s="11"/>
       <c r="O10" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="P10" s="11" t="s">
         <v>72</v>
       </c>
+      <c r="P10" s="11"/>
       <c r="Q10" s="11"/>
       <c r="R10" s="11"/>
       <c r="S10" s="11"/>
@@ -2827,243 +2794,268 @@
     </row>
     <row r="11" spans="1:32" s="1" customFormat="1" ht="18" customHeight="1">
       <c r="A11" s="108"/>
-      <c r="B11" s="96"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="11" t="s">
+      <c r="B11" s="97"/>
+      <c r="C11" s="52"/>
+      <c r="D11" s="52"/>
+      <c r="E11" s="52"/>
+      <c r="F11" s="52"/>
+      <c r="G11" s="52"/>
+      <c r="H11" s="52"/>
+      <c r="I11" s="52"/>
+      <c r="J11" s="52"/>
+      <c r="K11" s="52"/>
+      <c r="L11" s="52" t="s">
+        <v>63</v>
+      </c>
+      <c r="M11" s="52"/>
+      <c r="N11" s="52" t="s">
         <v>73</v>
       </c>
-      <c r="I11" s="11"/>
-      <c r="J11" s="11"/>
-      <c r="K11" s="11"/>
-      <c r="L11" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="M11" s="11"/>
-      <c r="N11" s="11"/>
-      <c r="O11" s="11" t="s">
+      <c r="O11" s="52"/>
+      <c r="P11" s="52"/>
+      <c r="Q11" s="52" t="s">
         <v>74</v>
       </c>
-      <c r="P11" s="11"/>
-      <c r="Q11" s="11"/>
-      <c r="R11" s="11"/>
-      <c r="S11" s="11"/>
-      <c r="T11" s="11"/>
-      <c r="U11" s="11"/>
-      <c r="V11" s="11"/>
-      <c r="W11" s="11"/>
-      <c r="X11" s="11"/>
-      <c r="Y11" s="11"/>
-      <c r="Z11" s="11"/>
-      <c r="AA11" s="11"/>
-      <c r="AB11" s="5"/>
-      <c r="AC11" s="54"/>
+      <c r="R11" s="52"/>
+      <c r="S11" s="52" t="s">
+        <v>74</v>
+      </c>
+      <c r="T11" s="52"/>
+      <c r="U11" s="52"/>
+      <c r="V11" s="52"/>
+      <c r="W11" s="52"/>
+      <c r="X11" s="52"/>
+      <c r="Y11" s="52"/>
+      <c r="Z11" s="52"/>
+      <c r="AA11" s="52"/>
+      <c r="AB11" s="53"/>
+      <c r="AC11" s="55"/>
       <c r="AD11" s="76"/>
       <c r="AE11" s="76"/>
       <c r="AF11" s="76"/>
     </row>
-    <row r="12" spans="1:32" s="1" customFormat="1" ht="18" customHeight="1">
+    <row r="12" spans="1:32" ht="18" customHeight="1">
       <c r="A12" s="108"/>
-      <c r="B12" s="97"/>
-      <c r="C12" s="52"/>
-      <c r="D12" s="52"/>
-      <c r="E12" s="52"/>
-      <c r="F12" s="52"/>
-      <c r="G12" s="52"/>
-      <c r="H12" s="52"/>
-      <c r="I12" s="52"/>
-      <c r="J12" s="52"/>
-      <c r="K12" s="52"/>
-      <c r="L12" s="52" t="s">
-        <v>65</v>
-      </c>
-      <c r="M12" s="52"/>
-      <c r="N12" s="52" t="s">
+      <c r="B12" s="95" t="s">
         <v>75</v>
       </c>
-      <c r="O12" s="52"/>
-      <c r="P12" s="52"/>
-      <c r="Q12" s="52" t="s">
+      <c r="C12" s="61" t="s">
         <v>76</v>
       </c>
-      <c r="R12" s="52"/>
-      <c r="S12" s="52" t="s">
-        <v>76</v>
-      </c>
-      <c r="T12" s="52"/>
-      <c r="U12" s="52"/>
-      <c r="V12" s="52"/>
-      <c r="W12" s="52"/>
-      <c r="X12" s="52"/>
-      <c r="Y12" s="52"/>
-      <c r="Z12" s="52"/>
-      <c r="AA12" s="52"/>
-      <c r="AB12" s="53"/>
-      <c r="AC12" s="55"/>
-      <c r="AD12" s="76"/>
-      <c r="AE12" s="76"/>
-      <c r="AF12" s="76"/>
+      <c r="D12" s="62" t="s">
+        <v>77</v>
+      </c>
+      <c r="E12" s="63" t="s">
+        <v>78</v>
+      </c>
+      <c r="F12" s="62" t="s">
+        <v>77</v>
+      </c>
+      <c r="G12" s="62" t="s">
+        <v>77</v>
+      </c>
+      <c r="H12" s="62" t="s">
+        <v>77</v>
+      </c>
+      <c r="I12" s="61" t="s">
+        <v>79</v>
+      </c>
+      <c r="J12" s="61" t="s">
+        <v>80</v>
+      </c>
+      <c r="K12" s="37" t="s">
+        <v>81</v>
+      </c>
+      <c r="L12" s="61" t="s">
+        <v>82</v>
+      </c>
+      <c r="M12" s="62" t="s">
+        <v>77</v>
+      </c>
+      <c r="N12" s="61" t="s">
+        <v>83</v>
+      </c>
+      <c r="O12" s="61" t="s">
+        <v>84</v>
+      </c>
+      <c r="P12" s="37" t="s">
+        <v>85</v>
+      </c>
+      <c r="Q12" s="61" t="s">
+        <v>85</v>
+      </c>
+      <c r="R12" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="S12" s="61" t="s">
+        <v>85</v>
+      </c>
+      <c r="T12" s="61" t="s">
+        <v>85</v>
+      </c>
+      <c r="U12" s="61" t="s">
+        <v>85</v>
+      </c>
+      <c r="V12" s="62" t="s">
+        <v>77</v>
+      </c>
+      <c r="W12" s="61" t="s">
+        <v>87</v>
+      </c>
+      <c r="X12" s="62" t="s">
+        <v>77</v>
+      </c>
+      <c r="Y12" s="61" t="s">
+        <v>88</v>
+      </c>
+      <c r="Z12" s="61" t="s">
+        <v>87</v>
+      </c>
+      <c r="AA12" s="61" t="s">
+        <v>85</v>
+      </c>
+      <c r="AB12" s="37" t="s">
+        <v>89</v>
+      </c>
+      <c r="AC12" s="61" t="s">
+        <v>90</v>
+      </c>
+      <c r="AD12" s="20"/>
+      <c r="AE12" s="20"/>
+      <c r="AF12" s="75"/>
     </row>
     <row r="13" spans="1:32" ht="18" customHeight="1">
       <c r="A13" s="108"/>
-      <c r="B13" s="95" t="s">
-        <v>77</v>
-      </c>
-      <c r="C13" s="61" t="s">
+      <c r="B13" s="96"/>
+      <c r="C13" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
+      <c r="I13" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="D13" s="62" t="s">
-        <v>79</v>
-      </c>
-      <c r="E13" s="63" t="s">
-        <v>80</v>
-      </c>
-      <c r="F13" s="62" t="s">
-        <v>79</v>
-      </c>
-      <c r="G13" s="62" t="s">
-        <v>79</v>
-      </c>
-      <c r="H13" s="62" t="s">
-        <v>79</v>
-      </c>
-      <c r="I13" s="61" t="s">
-        <v>81</v>
-      </c>
-      <c r="J13" s="61" t="s">
-        <v>82</v>
-      </c>
-      <c r="K13" s="37" t="s">
-        <v>83</v>
-      </c>
-      <c r="L13" s="61" t="s">
-        <v>84</v>
-      </c>
-      <c r="M13" s="62" t="s">
-        <v>79</v>
-      </c>
-      <c r="N13" s="61" t="s">
+      <c r="J13" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="K13" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="L13" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="M13" s="4"/>
+      <c r="N13" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="O13" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="O13" s="61" t="s">
+      <c r="P13" s="4"/>
+      <c r="Q13" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="P13" s="37" t="s">
+      <c r="R13" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="Q13" s="61" t="s">
-        <v>87</v>
-      </c>
-      <c r="R13" s="37" t="s">
-        <v>88</v>
-      </c>
-      <c r="S13" s="61" t="s">
-        <v>87</v>
-      </c>
-      <c r="T13" s="61" t="s">
-        <v>87</v>
-      </c>
-      <c r="U13" s="61" t="s">
-        <v>87</v>
-      </c>
-      <c r="V13" s="62" t="s">
-        <v>79</v>
-      </c>
-      <c r="W13" s="61" t="s">
+      <c r="S13" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="T13" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="U13" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="X13" s="62" t="s">
-        <v>79</v>
-      </c>
-      <c r="Y13" s="61" t="s">
-        <v>90</v>
-      </c>
-      <c r="Z13" s="61" t="s">
+      <c r="V13" s="4"/>
+      <c r="W13" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="X13" s="4"/>
+      <c r="Y13" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="Z13" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="AA13" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="AA13" s="61" t="s">
-        <v>87</v>
-      </c>
-      <c r="AB13" s="37" t="s">
-        <v>91</v>
-      </c>
-      <c r="AC13" s="61" t="s">
-        <v>92</v>
-      </c>
-      <c r="AD13" s="20"/>
-      <c r="AE13" s="20"/>
-      <c r="AF13" s="75"/>
+      <c r="AB13" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="AC13" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="AD13" s="10"/>
+      <c r="AE13" s="10"/>
+      <c r="AF13" s="40"/>
     </row>
     <row r="14" spans="1:32" ht="18" customHeight="1">
       <c r="A14" s="108"/>
       <c r="B14" s="96"/>
       <c r="C14" s="11" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="D14" s="4"/>
       <c r="E14" s="4" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
-      <c r="I14" s="11" t="s">
-        <v>80</v>
+      <c r="I14" s="4" t="s">
+        <v>92</v>
       </c>
       <c r="J14" s="11" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="K14" s="11" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="L14" s="11" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="M14" s="4"/>
       <c r="N14" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="O14" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="P14" s="4"/>
+      <c r="Q14" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="R14" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="O14" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="P14" s="4"/>
-      <c r="Q14" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="R14" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="S14" s="11" t="s">
-        <v>99</v>
-      </c>
+      <c r="S14" s="4"/>
       <c r="T14" s="11" t="s">
-        <v>99</v>
-      </c>
-      <c r="U14" s="12" t="s">
-        <v>91</v>
+        <v>86</v>
+      </c>
+      <c r="U14" s="11" t="s">
+        <v>98</v>
       </c>
       <c r="V14" s="4"/>
       <c r="W14" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="X14" s="4"/>
+      <c r="Y14" s="4"/>
+      <c r="Z14" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="AA14" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="X14" s="4"/>
-      <c r="Y14" s="12" t="s">
-        <v>101</v>
-      </c>
-      <c r="Z14" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="AA14" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="AB14" s="12" t="s">
-        <v>102</v>
-      </c>
       <c r="AC14" s="11" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="AD14" s="10"/>
       <c r="AE14" s="10"/>
@@ -3073,62 +3065,57 @@
       <c r="A15" s="108"/>
       <c r="B15" s="96"/>
       <c r="C15" s="11" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="D15" s="4"/>
       <c r="E15" s="4" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
       <c r="I15" s="4" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="J15" s="11" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="K15" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="L15" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="L15" s="4"/>
+      <c r="M15" s="4"/>
+      <c r="N15" s="4"/>
+      <c r="O15" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="P15" s="4"/>
+      <c r="Q15" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="R15" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="M15" s="4"/>
-      <c r="N15" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="O15" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="P15" s="4"/>
-      <c r="Q15" s="12" t="s">
-        <v>101</v>
-      </c>
-      <c r="R15" s="11" t="s">
-        <v>100</v>
-      </c>
       <c r="S15" s="4"/>
-      <c r="T15" s="11" t="s">
-        <v>88</v>
-      </c>
+      <c r="T15" s="4"/>
       <c r="U15" s="11" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="V15" s="4"/>
       <c r="W15" s="11" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="X15" s="4"/>
       <c r="Y15" s="4"/>
       <c r="Z15" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA15" s="12" t="s">
-        <v>102</v>
-      </c>
+        <v>114</v>
+      </c>
+      <c r="AA15" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="AB15" s="11"/>
       <c r="AC15" s="11" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="AD15" s="10"/>
       <c r="AE15" s="10"/>
@@ -3138,57 +3125,53 @@
       <c r="A16" s="108"/>
       <c r="B16" s="96"/>
       <c r="C16" s="11" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="D16" s="4"/>
-      <c r="E16" s="4" t="s">
-        <v>113</v>
-      </c>
+      <c r="E16" s="4"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
       <c r="I16" s="4" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="J16" s="11" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="K16" s="11" t="s">
-        <v>84</v>
+        <v>118</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4"/>
       <c r="N16" s="4"/>
       <c r="O16" s="11" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="P16" s="4"/>
-      <c r="Q16" s="4" t="s">
-        <v>115</v>
-      </c>
+      <c r="Q16" s="4"/>
       <c r="R16" s="11" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="S16" s="4"/>
       <c r="T16" s="4"/>
       <c r="U16" s="11" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="V16" s="4"/>
       <c r="W16" s="11" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="X16" s="4"/>
       <c r="Y16" s="4"/>
       <c r="Z16" s="11" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="AA16" s="11" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="AB16" s="11"/>
       <c r="AC16" s="11" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="AD16" s="10"/>
       <c r="AE16" s="10"/>
@@ -3197,50 +3180,42 @@
     <row r="17" spans="1:155" ht="18" customHeight="1">
       <c r="A17" s="108"/>
       <c r="B17" s="96"/>
-      <c r="C17" s="11" t="s">
-        <v>118</v>
-      </c>
+      <c r="C17" s="4"/>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
-      <c r="I17" s="4" t="s">
-        <v>113</v>
-      </c>
+      <c r="I17" s="4"/>
       <c r="J17" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="K17" s="11" t="s">
-        <v>120</v>
-      </c>
+        <v>121</v>
+      </c>
+      <c r="K17" s="4"/>
       <c r="L17" s="4"/>
       <c r="M17" s="4"/>
       <c r="N17" s="4"/>
       <c r="O17" s="11" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="P17" s="4"/>
       <c r="Q17" s="4"/>
       <c r="R17" s="11" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="S17" s="4"/>
       <c r="T17" s="4"/>
       <c r="U17" s="11" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="V17" s="4"/>
-      <c r="W17" s="11" t="s">
-        <v>121</v>
+      <c r="W17" s="12" t="s">
+        <v>99</v>
       </c>
       <c r="X17" s="4"/>
       <c r="Y17" s="4"/>
-      <c r="Z17" s="11" t="s">
-        <v>121</v>
-      </c>
+      <c r="Z17" s="4"/>
       <c r="AA17" s="11" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="AB17" s="11"/>
       <c r="AC17" s="11" t="s">
@@ -3251,470 +3226,478 @@
       <c r="AF17" s="40"/>
     </row>
     <row r="18" spans="1:155" ht="18" customHeight="1">
-      <c r="A18" s="108"/>
-      <c r="B18" s="96"/>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
-      <c r="H18" s="4"/>
-      <c r="I18" s="4"/>
-      <c r="J18" s="11" t="s">
+      <c r="A18" s="109"/>
+      <c r="B18" s="97"/>
+      <c r="C18" s="32"/>
+      <c r="D18" s="32"/>
+      <c r="E18" s="32"/>
+      <c r="F18" s="32"/>
+      <c r="G18" s="32"/>
+      <c r="H18" s="32"/>
+      <c r="I18" s="32"/>
+      <c r="J18" s="52" t="s">
         <v>123</v>
       </c>
-      <c r="K18" s="4"/>
-      <c r="L18" s="4"/>
-      <c r="M18" s="4"/>
-      <c r="N18" s="4"/>
-      <c r="O18" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="P18" s="4"/>
-      <c r="Q18" s="4"/>
-      <c r="R18" s="11" t="s">
-        <v>121</v>
-      </c>
-      <c r="S18" s="4"/>
-      <c r="T18" s="4"/>
-      <c r="U18" s="11" t="s">
-        <v>121</v>
-      </c>
-      <c r="V18" s="4"/>
-      <c r="W18" s="12" t="s">
-        <v>101</v>
-      </c>
-      <c r="X18" s="4"/>
-      <c r="Y18" s="4"/>
-      <c r="Z18" s="4"/>
-      <c r="AA18" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="AB18" s="11"/>
-      <c r="AC18" s="11" t="s">
+      <c r="K18" s="32"/>
+      <c r="L18" s="32"/>
+      <c r="M18" s="32"/>
+      <c r="N18" s="32"/>
+      <c r="O18" s="52" t="s">
+        <v>108</v>
+      </c>
+      <c r="P18" s="32"/>
+      <c r="Q18" s="32"/>
+      <c r="R18" s="64" t="s">
+        <v>99</v>
+      </c>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="52" t="s">
+        <v>88</v>
+      </c>
+      <c r="V18" s="32"/>
+      <c r="W18" s="64" t="s">
         <v>124</v>
       </c>
-      <c r="AD18" s="10"/>
-      <c r="AE18" s="10"/>
-      <c r="AF18" s="40"/>
+      <c r="X18" s="32"/>
+      <c r="Y18" s="32"/>
+      <c r="Z18" s="32"/>
+      <c r="AA18" s="52" t="s">
+        <v>108</v>
+      </c>
+      <c r="AB18" s="52"/>
+      <c r="AC18" s="52"/>
+      <c r="AD18" s="31"/>
+      <c r="AE18" s="31"/>
+      <c r="AF18" s="41"/>
     </row>
-    <row r="19" spans="1:155" ht="18" customHeight="1">
-      <c r="A19" s="109"/>
-      <c r="B19" s="97"/>
-      <c r="C19" s="32"/>
-      <c r="D19" s="32"/>
-      <c r="E19" s="32"/>
-      <c r="F19" s="32"/>
-      <c r="G19" s="32"/>
-      <c r="H19" s="32"/>
-      <c r="I19" s="32"/>
-      <c r="J19" s="52" t="s">
+    <row r="19" spans="1:155" s="3" customFormat="1" ht="89.45" customHeight="1">
+      <c r="A19" s="56" t="s">
         <v>125</v>
       </c>
-      <c r="K19" s="32"/>
-      <c r="L19" s="32"/>
-      <c r="M19" s="32"/>
-      <c r="N19" s="32"/>
-      <c r="O19" s="52" t="s">
-        <v>110</v>
-      </c>
-      <c r="P19" s="32"/>
-      <c r="Q19" s="32"/>
-      <c r="R19" s="64" t="s">
-        <v>101</v>
-      </c>
-      <c r="S19" s="32"/>
-      <c r="T19" s="32"/>
-      <c r="U19" s="52" t="s">
-        <v>90</v>
-      </c>
-      <c r="V19" s="32"/>
-      <c r="W19" s="64" t="s">
+      <c r="B19" s="85" t="s">
         <v>126</v>
       </c>
-      <c r="X19" s="32"/>
-      <c r="Y19" s="32"/>
-      <c r="Z19" s="32"/>
-      <c r="AA19" s="52" t="s">
-        <v>110</v>
-      </c>
-      <c r="AB19" s="52"/>
-      <c r="AC19" s="52"/>
-      <c r="AD19" s="31"/>
-      <c r="AE19" s="31"/>
-      <c r="AF19" s="41"/>
+      <c r="C19" s="43"/>
+      <c r="D19" s="43"/>
+      <c r="E19" s="44" t="s">
+        <v>127</v>
+      </c>
+      <c r="F19" s="44" t="s">
+        <v>128</v>
+      </c>
+      <c r="G19" s="44" t="s">
+        <v>129</v>
+      </c>
+      <c r="H19" s="43"/>
+      <c r="I19" s="44" t="s">
+        <v>130</v>
+      </c>
+      <c r="J19" s="43" t="s">
+        <v>131</v>
+      </c>
+      <c r="K19" s="43" t="s">
+        <v>132</v>
+      </c>
+      <c r="L19" s="43" t="s">
+        <v>133</v>
+      </c>
+      <c r="M19" s="43" t="s">
+        <v>134</v>
+      </c>
+      <c r="N19" s="43"/>
+      <c r="O19" s="44" t="s">
+        <v>135</v>
+      </c>
+      <c r="P19" s="44" t="s">
+        <v>136</v>
+      </c>
+      <c r="Q19" s="44" t="s">
+        <v>137</v>
+      </c>
+      <c r="R19" s="57" t="s">
+        <v>138</v>
+      </c>
+      <c r="S19" s="58" t="s">
+        <v>139</v>
+      </c>
+      <c r="T19" s="57"/>
+      <c r="U19" s="58" t="s">
+        <v>140</v>
+      </c>
+      <c r="V19" s="57"/>
+      <c r="W19" s="59" t="s">
+        <v>141</v>
+      </c>
+      <c r="X19" s="57"/>
+      <c r="Y19" s="58" t="s">
+        <v>142</v>
+      </c>
+      <c r="Z19" s="57"/>
+      <c r="AA19" s="58" t="s">
+        <v>143</v>
+      </c>
+      <c r="AB19" s="58" t="s">
+        <v>144</v>
+      </c>
+      <c r="AC19" s="58" t="s">
+        <v>145</v>
+      </c>
+      <c r="AD19" s="57"/>
+      <c r="AE19" s="57"/>
+      <c r="AF19" s="60"/>
     </row>
-    <row r="20" spans="1:155" s="3" customFormat="1" ht="89.45" customHeight="1">
-      <c r="A20" s="56" t="s">
-        <v>127</v>
-      </c>
-      <c r="B20" s="85" t="s">
-        <v>128</v>
-      </c>
-      <c r="C20" s="43"/>
-      <c r="D20" s="43"/>
-      <c r="E20" s="44" t="s">
-        <v>129</v>
-      </c>
-      <c r="F20" s="44" t="s">
-        <v>130</v>
-      </c>
-      <c r="G20" s="44" t="s">
-        <v>131</v>
-      </c>
-      <c r="H20" s="43"/>
-      <c r="I20" s="44" t="s">
-        <v>132</v>
-      </c>
-      <c r="J20" s="43" t="s">
-        <v>133</v>
-      </c>
-      <c r="K20" s="43" t="s">
-        <v>134</v>
-      </c>
-      <c r="L20" s="43" t="s">
-        <v>135</v>
-      </c>
-      <c r="M20" s="43" t="s">
-        <v>136</v>
-      </c>
-      <c r="N20" s="43"/>
-      <c r="O20" s="44" t="s">
-        <v>137</v>
-      </c>
-      <c r="P20" s="44" t="s">
-        <v>138</v>
-      </c>
-      <c r="Q20" s="44" t="s">
-        <v>139</v>
-      </c>
-      <c r="R20" s="57" t="s">
-        <v>140</v>
-      </c>
-      <c r="S20" s="58" t="s">
-        <v>141</v>
-      </c>
-      <c r="T20" s="57"/>
-      <c r="U20" s="58" t="s">
-        <v>142</v>
-      </c>
-      <c r="V20" s="57"/>
-      <c r="W20" s="59" t="s">
-        <v>143</v>
-      </c>
-      <c r="X20" s="57"/>
-      <c r="Y20" s="58" t="s">
-        <v>144</v>
-      </c>
-      <c r="Z20" s="57"/>
-      <c r="AA20" s="58" t="s">
-        <v>145</v>
-      </c>
-      <c r="AB20" s="58" t="s">
+    <row r="20" spans="1:155" s="1" customFormat="1" ht="36" customHeight="1">
+      <c r="A20" s="21"/>
+      <c r="B20" s="92" t="s">
         <v>146</v>
       </c>
-      <c r="AC20" s="58" t="s">
+      <c r="C20" s="22" t="s">
         <v>147</v>
       </c>
-      <c r="AD20" s="57"/>
-      <c r="AE20" s="57"/>
-      <c r="AF20" s="60"/>
+      <c r="D20" s="22" t="s">
+        <v>148</v>
+      </c>
+      <c r="E20" s="22" t="s">
+        <v>149</v>
+      </c>
+      <c r="F20" s="22" t="s">
+        <v>150</v>
+      </c>
+      <c r="G20" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="H20" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="I20" s="22" t="s">
+        <v>152</v>
+      </c>
+      <c r="J20" s="22" t="s">
+        <v>153</v>
+      </c>
+      <c r="K20" s="22" t="s">
+        <v>154</v>
+      </c>
+      <c r="L20" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="M20" s="22" t="s">
+        <v>156</v>
+      </c>
+      <c r="N20" s="22" t="s">
+        <v>157</v>
+      </c>
+      <c r="O20" s="22" t="s">
+        <v>158</v>
+      </c>
+      <c r="P20" s="22" t="s">
+        <v>159</v>
+      </c>
+      <c r="Q20" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="R20" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="S20" s="22" t="s">
+        <v>161</v>
+      </c>
+      <c r="T20" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="U20" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="V20" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="W20" s="22" t="s">
+        <v>162</v>
+      </c>
+      <c r="X20" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="Y20" s="22" t="s">
+        <v>163</v>
+      </c>
+      <c r="Z20" s="22" t="s">
+        <v>164</v>
+      </c>
+      <c r="AA20" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="AB20" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="AC20" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="AD20" s="22" t="s">
+        <v>165</v>
+      </c>
+      <c r="AE20" s="22" t="s">
+        <v>166</v>
+      </c>
+      <c r="AF20" s="23" t="s">
+        <v>167</v>
+      </c>
     </row>
-    <row r="21" spans="1:155" s="1" customFormat="1" ht="36" customHeight="1">
-      <c r="A21" s="21"/>
-      <c r="B21" s="92" t="s">
-        <v>148</v>
-      </c>
-      <c r="C21" s="22" t="s">
-        <v>149</v>
-      </c>
-      <c r="D21" s="22" t="s">
-        <v>150</v>
-      </c>
-      <c r="E21" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="F21" s="22" t="s">
-        <v>152</v>
-      </c>
-      <c r="G21" s="22" t="s">
-        <v>153</v>
-      </c>
-      <c r="H21" s="22" t="s">
-        <v>153</v>
-      </c>
-      <c r="I21" s="22" t="s">
-        <v>154</v>
-      </c>
-      <c r="J21" s="22" t="s">
-        <v>155</v>
-      </c>
-      <c r="K21" s="22" t="s">
-        <v>156</v>
-      </c>
-      <c r="L21" s="22" t="s">
-        <v>157</v>
-      </c>
-      <c r="M21" s="22" t="s">
-        <v>158</v>
-      </c>
-      <c r="N21" s="22" t="s">
-        <v>159</v>
-      </c>
-      <c r="O21" s="22" t="s">
-        <v>160</v>
-      </c>
-      <c r="P21" s="22" t="s">
-        <v>161</v>
-      </c>
-      <c r="Q21" s="22" t="s">
-        <v>162</v>
-      </c>
-      <c r="R21" s="22" t="s">
-        <v>153</v>
-      </c>
-      <c r="S21" s="22" t="s">
-        <v>163</v>
-      </c>
-      <c r="T21" s="22" t="s">
-        <v>153</v>
-      </c>
-      <c r="U21" s="22" t="s">
-        <v>153</v>
-      </c>
-      <c r="V21" s="22" t="s">
-        <v>153</v>
-      </c>
-      <c r="W21" s="22" t="s">
-        <v>164</v>
-      </c>
-      <c r="X21" s="22" t="s">
-        <v>153</v>
-      </c>
-      <c r="Y21" s="22" t="s">
-        <v>165</v>
-      </c>
-      <c r="Z21" s="22" t="s">
-        <v>166</v>
-      </c>
-      <c r="AA21" s="22" t="s">
-        <v>153</v>
-      </c>
-      <c r="AB21" s="22" t="s">
-        <v>153</v>
-      </c>
-      <c r="AC21" s="22" t="s">
-        <v>153</v>
-      </c>
-      <c r="AD21" s="22" t="s">
-        <v>167</v>
-      </c>
-      <c r="AE21" s="22" t="s">
+    <row r="21" spans="1:155" ht="18" customHeight="1">
+      <c r="A21" s="24"/>
+      <c r="B21" s="93"/>
+      <c r="C21" s="25" t="s">
         <v>168</v>
       </c>
-      <c r="AF21" s="23" t="s">
+      <c r="D21" s="25" t="s">
         <v>169</v>
+      </c>
+      <c r="E21" s="25" t="s">
+        <v>170</v>
+      </c>
+      <c r="F21" s="25" t="s">
+        <v>171</v>
+      </c>
+      <c r="G21" s="4"/>
+      <c r="H21" s="4"/>
+      <c r="I21" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="J21" s="13" t="s">
+        <v>173</v>
+      </c>
+      <c r="K21" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="L21" s="14"/>
+      <c r="M21" s="13" t="s">
+        <v>175</v>
+      </c>
+      <c r="N21" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="O21" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="P21" s="13" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q21" s="13" t="s">
+        <v>179</v>
+      </c>
+      <c r="R21" s="14"/>
+      <c r="S21" s="13" t="s">
+        <v>179</v>
+      </c>
+      <c r="T21" s="14"/>
+      <c r="U21" s="4"/>
+      <c r="V21" s="4"/>
+      <c r="W21" s="13" t="s">
+        <v>180</v>
+      </c>
+      <c r="X21" s="4"/>
+      <c r="Y21" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="Z21" s="13" t="s">
+        <v>182</v>
+      </c>
+      <c r="AA21" s="4"/>
+      <c r="AB21" s="4"/>
+      <c r="AC21" s="4"/>
+      <c r="AD21" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="AE21" s="13" t="s">
+        <v>184</v>
+      </c>
+      <c r="AF21" s="26" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="22" spans="1:155" ht="18" customHeight="1">
       <c r="A22" s="24"/>
       <c r="B22" s="93"/>
       <c r="C22" s="25" t="s">
-        <v>170</v>
+        <v>186</v>
       </c>
       <c r="D22" s="25" t="s">
-        <v>171</v>
+        <v>187</v>
       </c>
       <c r="E22" s="25" t="s">
-        <v>172</v>
-      </c>
-      <c r="F22" s="25" t="s">
-        <v>173</v>
-      </c>
+        <v>188</v>
+      </c>
+      <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
-      <c r="I22" s="13" t="s">
-        <v>174</v>
-      </c>
+      <c r="I22" s="14"/>
       <c r="J22" s="13" t="s">
-        <v>175</v>
-      </c>
-      <c r="K22" s="13" t="s">
+        <v>189</v>
+      </c>
+      <c r="K22" s="14"/>
+      <c r="L22" s="13" t="s">
+        <v>190</v>
+      </c>
+      <c r="M22" s="13" t="s">
         <v>176</v>
       </c>
-      <c r="L22" s="14"/>
-      <c r="M22" s="13" t="s">
-        <v>177</v>
-      </c>
       <c r="N22" s="13" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
       <c r="O22" s="13" t="s">
-        <v>179</v>
+        <v>192</v>
       </c>
       <c r="P22" s="13" t="s">
-        <v>180</v>
+        <v>193</v>
       </c>
       <c r="Q22" s="13" t="s">
-        <v>181</v>
+        <v>194</v>
       </c>
       <c r="R22" s="14"/>
       <c r="S22" s="13" t="s">
-        <v>181</v>
+        <v>194</v>
       </c>
       <c r="T22" s="14"/>
       <c r="U22" s="4"/>
       <c r="V22" s="4"/>
       <c r="W22" s="13" t="s">
-        <v>182</v>
+        <v>195</v>
       </c>
       <c r="X22" s="4"/>
       <c r="Y22" s="13" t="s">
-        <v>183</v>
-      </c>
-      <c r="Z22" s="13" t="s">
-        <v>184</v>
-      </c>
+        <v>196</v>
+      </c>
+      <c r="Z22" s="13"/>
       <c r="AA22" s="4"/>
       <c r="AB22" s="4"/>
       <c r="AC22" s="4"/>
       <c r="AD22" s="13" t="s">
-        <v>185</v>
+        <v>197</v>
       </c>
       <c r="AE22" s="13" t="s">
-        <v>186</v>
+        <v>198</v>
       </c>
       <c r="AF22" s="26" t="s">
-        <v>187</v>
+        <v>199</v>
       </c>
     </row>
     <row r="23" spans="1:155" ht="18" customHeight="1">
       <c r="A23" s="24"/>
       <c r="B23" s="93"/>
       <c r="C23" s="25" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
       <c r="D23" s="25" t="s">
-        <v>189</v>
-      </c>
-      <c r="E23" s="25" t="s">
-        <v>190</v>
-      </c>
+        <v>201</v>
+      </c>
+      <c r="E23" s="4"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
       <c r="I23" s="14"/>
       <c r="J23" s="13" t="s">
-        <v>191</v>
+        <v>176</v>
       </c>
       <c r="K23" s="14"/>
       <c r="L23" s="13" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="M23" s="13" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
       <c r="N23" s="13" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="O23" s="13" t="s">
-        <v>194</v>
-      </c>
-      <c r="P23" s="13" t="s">
-        <v>195</v>
-      </c>
+        <v>204</v>
+      </c>
+      <c r="P23" s="14"/>
       <c r="Q23" s="13" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="R23" s="14"/>
       <c r="S23" s="13" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="T23" s="14"/>
       <c r="U23" s="4"/>
       <c r="V23" s="4"/>
       <c r="W23" s="13" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="X23" s="4"/>
       <c r="Y23" s="13" t="s">
-        <v>198</v>
-      </c>
-      <c r="Z23" s="13"/>
+        <v>189</v>
+      </c>
+      <c r="Z23" s="14"/>
       <c r="AA23" s="4"/>
       <c r="AB23" s="4"/>
       <c r="AC23" s="4"/>
       <c r="AD23" s="13" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="AE23" s="13" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="AF23" s="26" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
     </row>
     <row r="24" spans="1:155" ht="18" customHeight="1">
       <c r="A24" s="24"/>
       <c r="B24" s="93"/>
-      <c r="C24" s="25" t="s">
-        <v>202</v>
-      </c>
-      <c r="D24" s="25" t="s">
-        <v>203</v>
-      </c>
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
       <c r="I24" s="14"/>
       <c r="J24" s="13" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
       <c r="K24" s="14"/>
       <c r="L24" s="13" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="M24" s="13" t="s">
-        <v>193</v>
+        <v>210</v>
       </c>
       <c r="N24" s="13" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="O24" s="13" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="P24" s="14"/>
       <c r="Q24" s="13" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="R24" s="14"/>
       <c r="S24" s="13" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="T24" s="14"/>
       <c r="U24" s="4"/>
       <c r="V24" s="4"/>
       <c r="W24" s="13" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="X24" s="4"/>
       <c r="Y24" s="13" t="s">
-        <v>191</v>
+        <v>176</v>
       </c>
       <c r="Z24" s="14"/>
       <c r="AA24" s="4"/>
       <c r="AB24" s="4"/>
       <c r="AC24" s="4"/>
       <c r="AD24" s="13" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="AE24" s="13" t="s">
-        <v>209</v>
-      </c>
-      <c r="AF24" s="26" t="s">
-        <v>210</v>
-      </c>
+        <v>214</v>
+      </c>
+      <c r="AF24" s="27"/>
     </row>
     <row r="25" spans="1:155" ht="18" customHeight="1">
       <c r="A25" s="24"/>
@@ -3727,188 +3710,331 @@
       <c r="H25" s="4"/>
       <c r="I25" s="14"/>
       <c r="J25" s="13" t="s">
-        <v>193</v>
+        <v>210</v>
       </c>
       <c r="K25" s="14"/>
       <c r="L25" s="13" t="s">
-        <v>211</v>
-      </c>
-      <c r="M25" s="13" t="s">
-        <v>212</v>
-      </c>
-      <c r="N25" s="13" t="s">
-        <v>212</v>
-      </c>
+        <v>215</v>
+      </c>
+      <c r="M25" s="14"/>
+      <c r="N25" s="14"/>
       <c r="O25" s="13" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="P25" s="14"/>
       <c r="Q25" s="13" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="R25" s="14"/>
       <c r="S25" s="13" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="T25" s="14"/>
       <c r="U25" s="4"/>
       <c r="V25" s="4"/>
       <c r="W25" s="13" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="X25" s="4"/>
       <c r="Y25" s="13" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
       <c r="Z25" s="14"/>
       <c r="AA25" s="4"/>
       <c r="AB25" s="4"/>
       <c r="AC25" s="4"/>
       <c r="AD25" s="13" t="s">
-        <v>215</v>
+        <v>168</v>
       </c>
       <c r="AE25" s="13" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="AF25" s="27"/>
     </row>
     <row r="26" spans="1:155" ht="18" customHeight="1">
-      <c r="A26" s="24"/>
+      <c r="A26" s="28"/>
       <c r="B26" s="93"/>
-      <c r="C26" s="4"/>
-      <c r="D26" s="4"/>
-      <c r="E26" s="4"/>
-      <c r="F26" s="4"/>
-      <c r="G26" s="4"/>
-      <c r="H26" s="4"/>
-      <c r="I26" s="14"/>
-      <c r="J26" s="13" t="s">
-        <v>212</v>
-      </c>
-      <c r="K26" s="14"/>
-      <c r="L26" s="13" t="s">
-        <v>217</v>
-      </c>
-      <c r="M26" s="14"/>
-      <c r="N26" s="14"/>
-      <c r="O26" s="13" t="s">
-        <v>218</v>
-      </c>
-      <c r="P26" s="14"/>
-      <c r="Q26" s="13" t="s">
-        <v>218</v>
-      </c>
-      <c r="R26" s="14"/>
-      <c r="S26" s="13" t="s">
-        <v>218</v>
-      </c>
-      <c r="T26" s="14"/>
-      <c r="U26" s="4"/>
-      <c r="V26" s="4"/>
-      <c r="W26" s="13" t="s">
+      <c r="C26" s="6"/>
+      <c r="D26" s="6"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="6"/>
+      <c r="G26" s="6"/>
+      <c r="H26" s="6"/>
+      <c r="I26" s="17"/>
+      <c r="J26" s="18" t="s">
+        <v>203</v>
+      </c>
+      <c r="K26" s="17"/>
+      <c r="L26" s="18" t="s">
         <v>219</v>
       </c>
-      <c r="X26" s="4"/>
-      <c r="Y26" s="13" t="s">
-        <v>193</v>
-      </c>
-      <c r="Z26" s="14"/>
-      <c r="AA26" s="4"/>
-      <c r="AB26" s="4"/>
-      <c r="AC26" s="4"/>
-      <c r="AD26" s="13" t="s">
-        <v>170</v>
-      </c>
-      <c r="AE26" s="13" t="s">
+      <c r="M26" s="17"/>
+      <c r="N26" s="17"/>
+      <c r="O26" s="18" t="s">
         <v>220</v>
       </c>
-      <c r="AF26" s="27"/>
+      <c r="P26" s="17"/>
+      <c r="Q26" s="18" t="s">
+        <v>221</v>
+      </c>
+      <c r="R26" s="17"/>
+      <c r="S26" s="18" t="s">
+        <v>221</v>
+      </c>
+      <c r="T26" s="17"/>
+      <c r="U26" s="6"/>
+      <c r="V26" s="6"/>
+      <c r="W26" s="6"/>
+      <c r="X26" s="6"/>
+      <c r="Y26" s="18" t="s">
+        <v>203</v>
+      </c>
+      <c r="Z26" s="17"/>
+      <c r="AA26" s="6"/>
+      <c r="AB26" s="6"/>
+      <c r="AC26" s="6"/>
+      <c r="AD26" s="18" t="s">
+        <v>186</v>
+      </c>
+      <c r="AE26" s="17"/>
+      <c r="AF26" s="29"/>
     </row>
-    <row r="27" spans="1:155" ht="18" customHeight="1">
-      <c r="A27" s="28"/>
-      <c r="B27" s="93"/>
-      <c r="C27" s="6"/>
-      <c r="D27" s="6"/>
-      <c r="E27" s="6"/>
-      <c r="F27" s="6"/>
-      <c r="G27" s="6"/>
-      <c r="H27" s="6"/>
-      <c r="I27" s="17"/>
-      <c r="J27" s="18" t="s">
-        <v>205</v>
-      </c>
-      <c r="K27" s="17"/>
-      <c r="L27" s="18" t="s">
-        <v>221</v>
-      </c>
-      <c r="M27" s="17"/>
-      <c r="N27" s="17"/>
-      <c r="O27" s="18" t="s">
+    <row r="27" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1">
+      <c r="A27" s="30"/>
+      <c r="B27" s="94"/>
+      <c r="C27" s="32"/>
+      <c r="D27" s="32"/>
+      <c r="E27" s="32"/>
+      <c r="F27" s="32"/>
+      <c r="G27" s="32"/>
+      <c r="H27" s="32"/>
+      <c r="I27" s="32"/>
+      <c r="J27" s="32"/>
+      <c r="K27" s="32"/>
+      <c r="L27" s="32"/>
+      <c r="M27" s="32"/>
+      <c r="N27" s="32"/>
+      <c r="O27" s="32"/>
+      <c r="P27" s="32"/>
+      <c r="Q27" s="32"/>
+      <c r="R27" s="32"/>
+      <c r="S27" s="32"/>
+      <c r="T27" s="32"/>
+      <c r="U27" s="32"/>
+      <c r="V27" s="32"/>
+      <c r="W27" s="32"/>
+      <c r="X27" s="32"/>
+      <c r="Y27" s="33" t="s">
+        <v>174</v>
+      </c>
+      <c r="Z27" s="34"/>
+      <c r="AA27" s="32"/>
+      <c r="AB27" s="32"/>
+      <c r="AC27" s="32"/>
+      <c r="AD27" s="33" t="s">
+        <v>174</v>
+      </c>
+      <c r="AE27" s="34"/>
+      <c r="AF27" s="35"/>
+      <c r="AG27" s="2"/>
+      <c r="AH27" s="2"/>
+      <c r="AI27" s="2"/>
+      <c r="AJ27" s="2"/>
+      <c r="AK27" s="2"/>
+      <c r="AL27" s="2"/>
+      <c r="AM27" s="2"/>
+      <c r="AN27" s="2"/>
+      <c r="AO27" s="2"/>
+      <c r="AP27" s="2"/>
+      <c r="AQ27" s="2"/>
+      <c r="AR27" s="2"/>
+      <c r="AS27" s="2"/>
+      <c r="AT27" s="2"/>
+      <c r="AU27" s="2"/>
+      <c r="AV27" s="2"/>
+      <c r="AW27" s="2"/>
+      <c r="AX27" s="2"/>
+      <c r="AY27" s="2"/>
+      <c r="AZ27" s="2"/>
+      <c r="BA27" s="2"/>
+      <c r="BB27" s="2"/>
+      <c r="BC27" s="2"/>
+      <c r="BD27" s="2"/>
+      <c r="BE27" s="2"/>
+      <c r="BF27" s="2"/>
+      <c r="BG27" s="2"/>
+      <c r="BH27" s="2"/>
+      <c r="BI27" s="2"/>
+      <c r="BJ27" s="2"/>
+      <c r="BK27" s="2"/>
+      <c r="BL27" s="2"/>
+      <c r="BM27" s="2"/>
+      <c r="BN27" s="2"/>
+      <c r="BO27" s="2"/>
+      <c r="BP27" s="2"/>
+      <c r="BQ27" s="2"/>
+      <c r="BR27" s="2"/>
+      <c r="BS27" s="2"/>
+      <c r="BT27" s="2"/>
+      <c r="BU27" s="2"/>
+      <c r="BV27" s="2"/>
+      <c r="BW27" s="2"/>
+      <c r="BX27" s="2"/>
+      <c r="BY27" s="2"/>
+      <c r="BZ27" s="2"/>
+      <c r="CA27" s="2"/>
+      <c r="CB27" s="2"/>
+      <c r="CC27" s="2"/>
+      <c r="CD27" s="2"/>
+      <c r="CE27" s="2"/>
+      <c r="CF27" s="2"/>
+      <c r="CG27" s="2"/>
+      <c r="CH27" s="2"/>
+      <c r="CI27" s="2"/>
+      <c r="CJ27" s="2"/>
+      <c r="CK27" s="2"/>
+      <c r="CL27" s="2"/>
+      <c r="CM27" s="2"/>
+      <c r="CN27" s="2"/>
+      <c r="CO27" s="2"/>
+      <c r="CP27" s="2"/>
+      <c r="CQ27" s="2"/>
+      <c r="CR27" s="2"/>
+      <c r="CS27" s="2"/>
+      <c r="CT27" s="2"/>
+      <c r="CU27" s="2"/>
+      <c r="CV27" s="2"/>
+      <c r="CW27" s="2"/>
+      <c r="CX27" s="2"/>
+      <c r="CY27" s="2"/>
+      <c r="CZ27" s="2"/>
+      <c r="DA27" s="2"/>
+      <c r="DB27" s="2"/>
+      <c r="DC27" s="2"/>
+      <c r="DD27" s="2"/>
+      <c r="DE27" s="2"/>
+      <c r="DF27" s="2"/>
+      <c r="DG27" s="2"/>
+      <c r="DH27" s="2"/>
+      <c r="DI27" s="2"/>
+      <c r="DJ27" s="2"/>
+      <c r="DK27" s="2"/>
+      <c r="DL27" s="2"/>
+      <c r="DM27" s="2"/>
+      <c r="DN27" s="2"/>
+      <c r="DO27" s="2"/>
+      <c r="DP27" s="2"/>
+      <c r="DQ27" s="2"/>
+      <c r="DR27" s="2"/>
+      <c r="DS27" s="2"/>
+      <c r="DT27" s="2"/>
+      <c r="DU27" s="2"/>
+      <c r="DV27" s="2"/>
+      <c r="DW27" s="2"/>
+      <c r="DX27" s="2"/>
+      <c r="DY27" s="2"/>
+      <c r="DZ27" s="2"/>
+      <c r="EA27" s="2"/>
+      <c r="EB27" s="2"/>
+      <c r="EC27" s="2"/>
+      <c r="ED27" s="2"/>
+      <c r="EE27" s="2"/>
+      <c r="EF27" s="2"/>
+      <c r="EG27" s="2"/>
+      <c r="EH27" s="2"/>
+      <c r="EI27" s="2"/>
+      <c r="EJ27" s="2"/>
+      <c r="EK27" s="2"/>
+      <c r="EL27" s="2"/>
+      <c r="EM27" s="2"/>
+      <c r="EN27" s="2"/>
+      <c r="EO27" s="2"/>
+      <c r="EP27" s="2"/>
+      <c r="EQ27" s="2"/>
+      <c r="ER27" s="2"/>
+      <c r="ES27" s="2"/>
+      <c r="ET27" s="2"/>
+      <c r="EU27" s="2"/>
+      <c r="EV27" s="2"/>
+      <c r="EW27" s="2"/>
+      <c r="EX27" s="2"/>
+      <c r="EY27" s="2"/>
+    </row>
+    <row r="28" spans="1:155" s="10" customFormat="1" ht="36" customHeight="1">
+      <c r="A28" s="21"/>
+      <c r="B28" s="99" t="s">
         <v>222</v>
       </c>
-      <c r="P27" s="17"/>
-      <c r="Q27" s="18" t="s">
+      <c r="C28" s="36" t="s">
         <v>223</v>
       </c>
-      <c r="R27" s="17"/>
-      <c r="S27" s="18" t="s">
+      <c r="D28" s="36" t="s">
         <v>223</v>
       </c>
-      <c r="T27" s="17"/>
-      <c r="U27" s="6"/>
-      <c r="V27" s="6"/>
-      <c r="W27" s="6"/>
-      <c r="X27" s="6"/>
-      <c r="Y27" s="18" t="s">
-        <v>205</v>
-      </c>
-      <c r="Z27" s="17"/>
-      <c r="AA27" s="6"/>
-      <c r="AB27" s="6"/>
-      <c r="AC27" s="6"/>
-      <c r="AD27" s="18" t="s">
-        <v>188</v>
-      </c>
-      <c r="AE27" s="17"/>
-      <c r="AF27" s="29"/>
-    </row>
-    <row r="28" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1">
-      <c r="A28" s="30"/>
-      <c r="B28" s="94"/>
-      <c r="C28" s="32"/>
-      <c r="D28" s="32"/>
-      <c r="E28" s="32"/>
-      <c r="F28" s="32"/>
-      <c r="G28" s="32"/>
-      <c r="H28" s="32"/>
-      <c r="I28" s="32"/>
-      <c r="J28" s="32"/>
-      <c r="K28" s="32"/>
-      <c r="L28" s="32"/>
-      <c r="M28" s="32"/>
-      <c r="N28" s="32"/>
-      <c r="O28" s="32"/>
-      <c r="P28" s="32"/>
-      <c r="Q28" s="32"/>
-      <c r="R28" s="32"/>
-      <c r="S28" s="32"/>
-      <c r="T28" s="32"/>
-      <c r="U28" s="32"/>
-      <c r="V28" s="32"/>
-      <c r="W28" s="32"/>
-      <c r="X28" s="32"/>
-      <c r="Y28" s="33" t="s">
-        <v>176</v>
-      </c>
-      <c r="Z28" s="34"/>
-      <c r="AA28" s="32"/>
-      <c r="AB28" s="32"/>
-      <c r="AC28" s="32"/>
-      <c r="AD28" s="33" t="s">
-        <v>176</v>
-      </c>
-      <c r="AE28" s="34"/>
-      <c r="AF28" s="35"/>
+      <c r="E28" s="36" t="s">
+        <v>224</v>
+      </c>
+      <c r="F28" s="36" t="s">
+        <v>225</v>
+      </c>
+      <c r="G28" s="36" t="s">
+        <v>226</v>
+      </c>
+      <c r="H28" s="37"/>
+      <c r="I28" s="36" t="s">
+        <v>227</v>
+      </c>
+      <c r="J28" s="36" t="s">
+        <v>228</v>
+      </c>
+      <c r="K28" s="36" t="s">
+        <v>229</v>
+      </c>
+      <c r="L28" s="36" t="s">
+        <v>230</v>
+      </c>
+      <c r="M28" s="36" t="s">
+        <v>231</v>
+      </c>
+      <c r="N28" s="36" t="s">
+        <v>232</v>
+      </c>
+      <c r="O28" s="36" t="s">
+        <v>233</v>
+      </c>
+      <c r="P28" s="36" t="s">
+        <v>234</v>
+      </c>
+      <c r="Q28" s="36" t="s">
+        <v>235</v>
+      </c>
+      <c r="R28" s="36" t="s">
+        <v>227</v>
+      </c>
+      <c r="S28" s="36" t="s">
+        <v>233</v>
+      </c>
+      <c r="T28" s="37"/>
+      <c r="U28" s="36" t="s">
+        <v>233</v>
+      </c>
+      <c r="V28" s="37"/>
+      <c r="W28" s="36" t="s">
+        <v>236</v>
+      </c>
+      <c r="X28" s="37"/>
+      <c r="Y28" s="37"/>
+      <c r="Z28" s="36" t="s">
+        <v>237</v>
+      </c>
+      <c r="AA28" s="37" t="s">
+        <v>238</v>
+      </c>
+      <c r="AB28" s="37"/>
+      <c r="AC28" s="37"/>
+      <c r="AD28" s="38"/>
+      <c r="AE28" s="38"/>
+      <c r="AF28" s="39"/>
       <c r="AG28" s="2"/>
       <c r="AH28" s="2"/>
       <c r="AI28" s="2"/>
@@ -4033,81 +4159,69 @@
       <c r="EX28" s="2"/>
       <c r="EY28" s="2"/>
     </row>
-    <row r="29" spans="1:155" s="10" customFormat="1" ht="36" customHeight="1">
-      <c r="A29" s="21"/>
-      <c r="B29" s="99" t="s">
-        <v>224</v>
-      </c>
-      <c r="C29" s="36" t="s">
-        <v>225</v>
-      </c>
-      <c r="D29" s="36" t="s">
-        <v>225</v>
-      </c>
-      <c r="E29" s="36" t="s">
-        <v>226</v>
-      </c>
-      <c r="F29" s="36" t="s">
-        <v>227</v>
-      </c>
-      <c r="G29" s="36" t="s">
-        <v>228</v>
-      </c>
-      <c r="H29" s="37"/>
-      <c r="I29" s="36" t="s">
-        <v>229</v>
-      </c>
-      <c r="J29" s="36" t="s">
-        <v>230</v>
-      </c>
-      <c r="K29" s="36" t="s">
-        <v>231</v>
-      </c>
-      <c r="L29" s="36" t="s">
-        <v>232</v>
-      </c>
-      <c r="M29" s="36" t="s">
-        <v>233</v>
-      </c>
-      <c r="N29" s="36" t="s">
-        <v>234</v>
-      </c>
-      <c r="O29" s="36" t="s">
-        <v>235</v>
-      </c>
-      <c r="P29" s="36" t="s">
-        <v>236</v>
-      </c>
-      <c r="Q29" s="36" t="s">
-        <v>237</v>
-      </c>
-      <c r="R29" s="36" t="s">
-        <v>229</v>
-      </c>
-      <c r="S29" s="36" t="s">
-        <v>235</v>
-      </c>
-      <c r="T29" s="37"/>
-      <c r="U29" s="36" t="s">
-        <v>235</v>
-      </c>
-      <c r="V29" s="37"/>
-      <c r="W29" s="36" t="s">
-        <v>238</v>
-      </c>
-      <c r="X29" s="37"/>
-      <c r="Y29" s="37"/>
-      <c r="Z29" s="36" t="s">
+    <row r="29" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1">
+      <c r="A29" s="24"/>
+      <c r="B29" s="100"/>
+      <c r="C29" s="13" t="s">
         <v>239</v>
       </c>
-      <c r="AA29" s="37" t="s">
+      <c r="D29" s="13" t="s">
+        <v>239</v>
+      </c>
+      <c r="E29" s="4"/>
+      <c r="F29" s="13" t="s">
         <v>240</v>
       </c>
-      <c r="AB29" s="37"/>
-      <c r="AC29" s="37"/>
-      <c r="AD29" s="38"/>
-      <c r="AE29" s="38"/>
-      <c r="AF29" s="39"/>
+      <c r="G29" s="13" t="s">
+        <v>239</v>
+      </c>
+      <c r="H29" s="4"/>
+      <c r="I29" s="4"/>
+      <c r="J29" s="13" t="s">
+        <v>241</v>
+      </c>
+      <c r="K29" s="13" t="s">
+        <v>242</v>
+      </c>
+      <c r="L29" s="13" t="s">
+        <v>243</v>
+      </c>
+      <c r="M29" s="13" t="s">
+        <v>244</v>
+      </c>
+      <c r="N29" s="13" t="s">
+        <v>245</v>
+      </c>
+      <c r="O29" s="13" t="s">
+        <v>246</v>
+      </c>
+      <c r="P29" s="13" t="s">
+        <v>247</v>
+      </c>
+      <c r="Q29" s="13" t="s">
+        <v>248</v>
+      </c>
+      <c r="R29" s="14"/>
+      <c r="S29" s="13" t="s">
+        <v>246</v>
+      </c>
+      <c r="T29" s="4"/>
+      <c r="U29" s="13" t="s">
+        <v>246</v>
+      </c>
+      <c r="V29" s="4"/>
+      <c r="W29" s="13" t="s">
+        <v>249</v>
+      </c>
+      <c r="X29" s="4"/>
+      <c r="Y29" s="4"/>
+      <c r="Z29" s="13" t="s">
+        <v>250</v>
+      </c>
+      <c r="AA29" s="4"/>
+      <c r="AB29" s="4"/>
+      <c r="AC29" s="4"/>
+      <c r="AF29" s="40"/>
       <c r="AG29" s="2"/>
       <c r="AH29" s="2"/>
       <c r="AI29" s="2"/>
@@ -4236,61 +4350,55 @@
       <c r="A30" s="24"/>
       <c r="B30" s="100"/>
       <c r="C30" s="13" t="s">
-        <v>241</v>
+        <v>251</v>
       </c>
       <c r="D30" s="13" t="s">
-        <v>241</v>
+        <v>251</v>
       </c>
       <c r="E30" s="4"/>
       <c r="F30" s="13" t="s">
-        <v>242</v>
+        <v>252</v>
       </c>
       <c r="G30" s="13" t="s">
-        <v>241</v>
+        <v>251</v>
       </c>
       <c r="H30" s="4"/>
       <c r="I30" s="4"/>
       <c r="J30" s="13" t="s">
-        <v>243</v>
+        <v>253</v>
       </c>
       <c r="K30" s="13" t="s">
-        <v>244</v>
+        <v>254</v>
       </c>
       <c r="L30" s="13" t="s">
-        <v>245</v>
-      </c>
-      <c r="M30" s="13" t="s">
-        <v>246</v>
-      </c>
+        <v>255</v>
+      </c>
+      <c r="M30" s="14"/>
       <c r="N30" s="13" t="s">
-        <v>247</v>
+        <v>256</v>
       </c>
       <c r="O30" s="13" t="s">
-        <v>248</v>
-      </c>
-      <c r="P30" s="13" t="s">
-        <v>249</v>
-      </c>
+        <v>257</v>
+      </c>
+      <c r="P30" s="14"/>
       <c r="Q30" s="13" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="R30" s="14"/>
       <c r="S30" s="13" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
       <c r="T30" s="4"/>
       <c r="U30" s="13" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
       <c r="V30" s="4"/>
       <c r="W30" s="13" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="X30" s="4"/>
       <c r="Y30" s="4"/>
-      <c r="Z30" s="13" t="s">
-        <v>252</v>
-      </c>
+      <c r="Z30" s="14"/>
       <c r="AA30" s="4"/>
       <c r="AB30" s="4"/>
       <c r="AC30" s="4"/>
@@ -4423,55 +4531,43 @@
       <c r="A31" s="24"/>
       <c r="B31" s="100"/>
       <c r="C31" s="13" t="s">
-        <v>253</v>
+        <v>260</v>
       </c>
       <c r="D31" s="13" t="s">
-        <v>253</v>
+        <v>260</v>
       </c>
       <c r="E31" s="4"/>
-      <c r="F31" s="13" t="s">
-        <v>254</v>
-      </c>
+      <c r="F31" s="4"/>
       <c r="G31" s="13" t="s">
-        <v>253</v>
+        <v>260</v>
       </c>
       <c r="H31" s="4"/>
       <c r="I31" s="4"/>
-      <c r="J31" s="13" t="s">
-        <v>255</v>
-      </c>
-      <c r="K31" s="13" t="s">
-        <v>256</v>
-      </c>
-      <c r="L31" s="13" t="s">
-        <v>257</v>
-      </c>
+      <c r="J31" s="14"/>
+      <c r="K31" s="14"/>
+      <c r="L31" s="14"/>
       <c r="M31" s="14"/>
-      <c r="N31" s="13" t="s">
-        <v>258</v>
-      </c>
+      <c r="N31" s="14"/>
       <c r="O31" s="13" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="P31" s="14"/>
-      <c r="Q31" s="13" t="s">
-        <v>260</v>
-      </c>
+      <c r="Q31" s="14"/>
       <c r="R31" s="14"/>
       <c r="S31" s="13" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="T31" s="4"/>
       <c r="U31" s="13" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="V31" s="4"/>
       <c r="W31" s="13" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="X31" s="4"/>
       <c r="Y31" s="4"/>
-      <c r="Z31" s="14"/>
+      <c r="Z31" s="4"/>
       <c r="AA31" s="4"/>
       <c r="AB31" s="4"/>
       <c r="AC31" s="4"/>
@@ -4604,15 +4700,15 @@
       <c r="A32" s="24"/>
       <c r="B32" s="100"/>
       <c r="C32" s="13" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D32" s="13" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E32" s="4"/>
       <c r="F32" s="4"/>
       <c r="G32" s="13" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="H32" s="4"/>
       <c r="I32" s="4"/>
@@ -4622,21 +4718,21 @@
       <c r="M32" s="14"/>
       <c r="N32" s="14"/>
       <c r="O32" s="13" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="P32" s="14"/>
       <c r="Q32" s="14"/>
       <c r="R32" s="14"/>
       <c r="S32" s="13" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="T32" s="4"/>
       <c r="U32" s="13" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="V32" s="4"/>
       <c r="W32" s="13" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="X32" s="4"/>
       <c r="Y32" s="4"/>
@@ -4770,50 +4866,44 @@
       <c r="EY32" s="2"/>
     </row>
     <row r="33" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1">
-      <c r="A33" s="24"/>
-      <c r="B33" s="100"/>
-      <c r="C33" s="13" t="s">
-        <v>265</v>
-      </c>
-      <c r="D33" s="13" t="s">
-        <v>265</v>
-      </c>
-      <c r="E33" s="4"/>
-      <c r="F33" s="4"/>
-      <c r="G33" s="13" t="s">
-        <v>265</v>
-      </c>
-      <c r="H33" s="4"/>
-      <c r="I33" s="4"/>
-      <c r="J33" s="14"/>
-      <c r="K33" s="14"/>
-      <c r="L33" s="14"/>
-      <c r="M33" s="14"/>
-      <c r="N33" s="14"/>
-      <c r="O33" s="13" t="s">
+      <c r="A33" s="30"/>
+      <c r="B33" s="101"/>
+      <c r="C33" s="33" t="s">
         <v>266</v>
       </c>
-      <c r="P33" s="14"/>
-      <c r="Q33" s="14"/>
-      <c r="R33" s="14"/>
-      <c r="S33" s="13" t="s">
+      <c r="D33" s="33" t="s">
         <v>266</v>
       </c>
-      <c r="T33" s="4"/>
-      <c r="U33" s="13" t="s">
+      <c r="E33" s="32"/>
+      <c r="F33" s="32"/>
+      <c r="G33" s="33" t="s">
         <v>266</v>
       </c>
-      <c r="V33" s="4"/>
-      <c r="W33" s="13" t="s">
-        <v>267</v>
-      </c>
-      <c r="X33" s="4"/>
-      <c r="Y33" s="4"/>
-      <c r="Z33" s="4"/>
-      <c r="AA33" s="4"/>
-      <c r="AB33" s="4"/>
-      <c r="AC33" s="4"/>
-      <c r="AF33" s="40"/>
+      <c r="H33" s="32"/>
+      <c r="I33" s="32"/>
+      <c r="J33" s="34"/>
+      <c r="K33" s="34"/>
+      <c r="L33" s="34"/>
+      <c r="M33" s="34"/>
+      <c r="N33" s="34"/>
+      <c r="O33" s="34"/>
+      <c r="P33" s="34"/>
+      <c r="Q33" s="34"/>
+      <c r="R33" s="34"/>
+      <c r="S33" s="34"/>
+      <c r="T33" s="32"/>
+      <c r="U33" s="34"/>
+      <c r="V33" s="32"/>
+      <c r="W33" s="34"/>
+      <c r="X33" s="32"/>
+      <c r="Y33" s="32"/>
+      <c r="Z33" s="32"/>
+      <c r="AA33" s="32"/>
+      <c r="AB33" s="32"/>
+      <c r="AC33" s="32"/>
+      <c r="AD33" s="31"/>
+      <c r="AE33" s="31"/>
+      <c r="AF33" s="41"/>
       <c r="AG33" s="2"/>
       <c r="AH33" s="2"/>
       <c r="AI33" s="2"/>
@@ -4938,395 +5028,280 @@
       <c r="EX33" s="2"/>
       <c r="EY33" s="2"/>
     </row>
-    <row r="34" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1">
-      <c r="A34" s="30"/>
-      <c r="B34" s="101"/>
-      <c r="C34" s="33" t="s">
+    <row r="34" spans="1:155" ht="18" customHeight="1">
+      <c r="A34" s="42"/>
+      <c r="B34" s="66" t="s">
+        <v>267</v>
+      </c>
+      <c r="C34" s="43"/>
+      <c r="D34" s="43"/>
+      <c r="E34" s="43"/>
+      <c r="F34" s="43"/>
+      <c r="G34" s="43"/>
+      <c r="H34" s="43"/>
+      <c r="I34" s="43"/>
+      <c r="J34" s="43"/>
+      <c r="K34" s="43"/>
+      <c r="L34" s="43"/>
+      <c r="M34" s="43"/>
+      <c r="N34" s="43"/>
+      <c r="O34" s="43"/>
+      <c r="P34" s="43"/>
+      <c r="Q34" s="43"/>
+      <c r="R34" s="43"/>
+      <c r="S34" s="43"/>
+      <c r="T34" s="43"/>
+      <c r="U34" s="43"/>
+      <c r="V34" s="43"/>
+      <c r="W34" s="43"/>
+      <c r="X34" s="44" t="s">
         <v>268</v>
       </c>
-      <c r="D34" s="33" t="s">
-        <v>268</v>
-      </c>
-      <c r="E34" s="32"/>
-      <c r="F34" s="32"/>
-      <c r="G34" s="33" t="s">
-        <v>268</v>
-      </c>
-      <c r="H34" s="32"/>
-      <c r="I34" s="32"/>
-      <c r="J34" s="34"/>
-      <c r="K34" s="34"/>
-      <c r="L34" s="34"/>
-      <c r="M34" s="34"/>
-      <c r="N34" s="34"/>
-      <c r="O34" s="34"/>
-      <c r="P34" s="34"/>
-      <c r="Q34" s="34"/>
-      <c r="R34" s="34"/>
-      <c r="S34" s="34"/>
-      <c r="T34" s="32"/>
-      <c r="U34" s="34"/>
-      <c r="V34" s="32"/>
-      <c r="W34" s="34"/>
-      <c r="X34" s="32"/>
-      <c r="Y34" s="32"/>
-      <c r="Z34" s="32"/>
-      <c r="AA34" s="32"/>
-      <c r="AB34" s="32"/>
-      <c r="AC34" s="32"/>
-      <c r="AD34" s="31"/>
-      <c r="AE34" s="31"/>
-      <c r="AF34" s="41"/>
-      <c r="AG34" s="2"/>
-      <c r="AH34" s="2"/>
-      <c r="AI34" s="2"/>
-      <c r="AJ34" s="2"/>
-      <c r="AK34" s="2"/>
-      <c r="AL34" s="2"/>
-      <c r="AM34" s="2"/>
-      <c r="AN34" s="2"/>
-      <c r="AO34" s="2"/>
-      <c r="AP34" s="2"/>
-      <c r="AQ34" s="2"/>
-      <c r="AR34" s="2"/>
-      <c r="AS34" s="2"/>
-      <c r="AT34" s="2"/>
-      <c r="AU34" s="2"/>
-      <c r="AV34" s="2"/>
-      <c r="AW34" s="2"/>
-      <c r="AX34" s="2"/>
-      <c r="AY34" s="2"/>
-      <c r="AZ34" s="2"/>
-      <c r="BA34" s="2"/>
-      <c r="BB34" s="2"/>
-      <c r="BC34" s="2"/>
-      <c r="BD34" s="2"/>
-      <c r="BE34" s="2"/>
-      <c r="BF34" s="2"/>
-      <c r="BG34" s="2"/>
-      <c r="BH34" s="2"/>
-      <c r="BI34" s="2"/>
-      <c r="BJ34" s="2"/>
-      <c r="BK34" s="2"/>
-      <c r="BL34" s="2"/>
-      <c r="BM34" s="2"/>
-      <c r="BN34" s="2"/>
-      <c r="BO34" s="2"/>
-      <c r="BP34" s="2"/>
-      <c r="BQ34" s="2"/>
-      <c r="BR34" s="2"/>
-      <c r="BS34" s="2"/>
-      <c r="BT34" s="2"/>
-      <c r="BU34" s="2"/>
-      <c r="BV34" s="2"/>
-      <c r="BW34" s="2"/>
-      <c r="BX34" s="2"/>
-      <c r="BY34" s="2"/>
-      <c r="BZ34" s="2"/>
-      <c r="CA34" s="2"/>
-      <c r="CB34" s="2"/>
-      <c r="CC34" s="2"/>
-      <c r="CD34" s="2"/>
-      <c r="CE34" s="2"/>
-      <c r="CF34" s="2"/>
-      <c r="CG34" s="2"/>
-      <c r="CH34" s="2"/>
-      <c r="CI34" s="2"/>
-      <c r="CJ34" s="2"/>
-      <c r="CK34" s="2"/>
-      <c r="CL34" s="2"/>
-      <c r="CM34" s="2"/>
-      <c r="CN34" s="2"/>
-      <c r="CO34" s="2"/>
-      <c r="CP34" s="2"/>
-      <c r="CQ34" s="2"/>
-      <c r="CR34" s="2"/>
-      <c r="CS34" s="2"/>
-      <c r="CT34" s="2"/>
-      <c r="CU34" s="2"/>
-      <c r="CV34" s="2"/>
-      <c r="CW34" s="2"/>
-      <c r="CX34" s="2"/>
-      <c r="CY34" s="2"/>
-      <c r="CZ34" s="2"/>
-      <c r="DA34" s="2"/>
-      <c r="DB34" s="2"/>
-      <c r="DC34" s="2"/>
-      <c r="DD34" s="2"/>
-      <c r="DE34" s="2"/>
-      <c r="DF34" s="2"/>
-      <c r="DG34" s="2"/>
-      <c r="DH34" s="2"/>
-      <c r="DI34" s="2"/>
-      <c r="DJ34" s="2"/>
-      <c r="DK34" s="2"/>
-      <c r="DL34" s="2"/>
-      <c r="DM34" s="2"/>
-      <c r="DN34" s="2"/>
-      <c r="DO34" s="2"/>
-      <c r="DP34" s="2"/>
-      <c r="DQ34" s="2"/>
-      <c r="DR34" s="2"/>
-      <c r="DS34" s="2"/>
-      <c r="DT34" s="2"/>
-      <c r="DU34" s="2"/>
-      <c r="DV34" s="2"/>
-      <c r="DW34" s="2"/>
-      <c r="DX34" s="2"/>
-      <c r="DY34" s="2"/>
-      <c r="DZ34" s="2"/>
-      <c r="EA34" s="2"/>
-      <c r="EB34" s="2"/>
-      <c r="EC34" s="2"/>
-      <c r="ED34" s="2"/>
-      <c r="EE34" s="2"/>
-      <c r="EF34" s="2"/>
-      <c r="EG34" s="2"/>
-      <c r="EH34" s="2"/>
-      <c r="EI34" s="2"/>
-      <c r="EJ34" s="2"/>
-      <c r="EK34" s="2"/>
-      <c r="EL34" s="2"/>
-      <c r="EM34" s="2"/>
-      <c r="EN34" s="2"/>
-      <c r="EO34" s="2"/>
-      <c r="EP34" s="2"/>
-      <c r="EQ34" s="2"/>
-      <c r="ER34" s="2"/>
-      <c r="ES34" s="2"/>
-      <c r="ET34" s="2"/>
-      <c r="EU34" s="2"/>
-      <c r="EV34" s="2"/>
-      <c r="EW34" s="2"/>
-      <c r="EX34" s="2"/>
-      <c r="EY34" s="2"/>
+      <c r="Y34" s="44" t="s">
+        <v>269</v>
+      </c>
+      <c r="Z34" s="43"/>
+      <c r="AA34" s="43"/>
+      <c r="AB34" s="43"/>
+      <c r="AC34" s="45"/>
+      <c r="AD34" s="46"/>
+      <c r="AE34" s="46"/>
+      <c r="AF34" s="47"/>
     </row>
     <row r="35" spans="1:155" ht="18" customHeight="1">
-      <c r="A35" s="42"/>
-      <c r="B35" s="66" t="s">
-        <v>269</v>
-      </c>
-      <c r="C35" s="43"/>
-      <c r="D35" s="43"/>
-      <c r="E35" s="43"/>
-      <c r="F35" s="43"/>
-      <c r="G35" s="43"/>
-      <c r="H35" s="43"/>
-      <c r="I35" s="43"/>
-      <c r="J35" s="43"/>
-      <c r="K35" s="43"/>
-      <c r="L35" s="43"/>
-      <c r="M35" s="43"/>
-      <c r="N35" s="43"/>
-      <c r="O35" s="43"/>
-      <c r="P35" s="43"/>
-      <c r="Q35" s="43"/>
-      <c r="R35" s="43"/>
-      <c r="S35" s="43"/>
-      <c r="T35" s="43"/>
-      <c r="U35" s="43"/>
-      <c r="V35" s="43"/>
-      <c r="W35" s="43"/>
-      <c r="X35" s="44" t="s">
+      <c r="A35" s="19"/>
+      <c r="B35" s="51" t="s">
         <v>270</v>
       </c>
-      <c r="Y35" s="44" t="s">
-        <v>271</v>
-      </c>
-      <c r="Z35" s="43"/>
-      <c r="AA35" s="43"/>
-      <c r="AB35" s="43"/>
-      <c r="AC35" s="45"/>
-      <c r="AD35" s="46"/>
-      <c r="AE35" s="46"/>
-      <c r="AF35" s="47"/>
+      <c r="C35" s="8"/>
+      <c r="D35" s="8"/>
+      <c r="E35" s="8"/>
+      <c r="F35" s="8"/>
+      <c r="G35" s="8"/>
+      <c r="H35" s="8"/>
+      <c r="I35" s="8"/>
+      <c r="J35" s="8"/>
+      <c r="K35" s="8"/>
+      <c r="L35" s="8"/>
+      <c r="M35" s="8"/>
+      <c r="N35" s="8"/>
+      <c r="O35" s="8"/>
+      <c r="P35" s="8"/>
+      <c r="Q35" s="8"/>
+      <c r="R35" s="8"/>
+      <c r="S35" s="8"/>
+      <c r="T35" s="8"/>
+      <c r="U35" s="8"/>
+      <c r="V35" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="W35" s="8"/>
+      <c r="X35" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="Y35" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="Z35" s="8"/>
+      <c r="AA35" s="8"/>
+      <c r="AB35" s="8"/>
+      <c r="AC35" s="7"/>
+      <c r="AD35" s="20"/>
+      <c r="AE35" s="20"/>
+      <c r="AF35" s="20"/>
     </row>
     <row r="36" spans="1:155" ht="18" customHeight="1">
-      <c r="A36" s="19"/>
-      <c r="B36" s="51" t="s">
-        <v>272</v>
-      </c>
-      <c r="C36" s="8"/>
-      <c r="D36" s="8"/>
-      <c r="E36" s="8"/>
-      <c r="F36" s="8"/>
-      <c r="G36" s="8"/>
-      <c r="H36" s="8"/>
-      <c r="I36" s="8"/>
-      <c r="J36" s="8"/>
-      <c r="K36" s="8"/>
-      <c r="L36" s="8"/>
-      <c r="M36" s="8"/>
-      <c r="N36" s="8"/>
-      <c r="O36" s="8"/>
-      <c r="P36" s="8"/>
-      <c r="Q36" s="8"/>
-      <c r="R36" s="8"/>
-      <c r="S36" s="8"/>
-      <c r="T36" s="8"/>
-      <c r="U36" s="8"/>
-      <c r="V36" s="8" t="s">
-        <v>240</v>
-      </c>
-      <c r="W36" s="8"/>
-      <c r="X36" s="8" t="s">
-        <v>240</v>
-      </c>
-      <c r="Y36" s="8" t="s">
-        <v>240</v>
-      </c>
-      <c r="Z36" s="8"/>
-      <c r="AA36" s="8"/>
-      <c r="AB36" s="8"/>
-      <c r="AC36" s="7"/>
-      <c r="AD36" s="20"/>
-      <c r="AE36" s="20"/>
-      <c r="AF36" s="20"/>
+      <c r="A36" s="15"/>
+      <c r="B36" s="67" t="s">
+        <v>271</v>
+      </c>
+      <c r="C36" s="6"/>
+      <c r="D36" s="6"/>
+      <c r="E36" s="6"/>
+      <c r="F36" s="6"/>
+      <c r="G36" s="6"/>
+      <c r="H36" s="6"/>
+      <c r="I36" s="6"/>
+      <c r="J36" s="6"/>
+      <c r="K36" s="6"/>
+      <c r="L36" s="6"/>
+      <c r="M36" s="6"/>
+      <c r="N36" s="6"/>
+      <c r="O36" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="P36" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="Q36" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="R36" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="S36" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="T36" s="6"/>
+      <c r="U36" s="6"/>
+      <c r="V36" s="6"/>
+      <c r="W36" s="6"/>
+      <c r="X36" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="Y36" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="Z36" s="6"/>
+      <c r="AA36" s="6"/>
+      <c r="AB36" s="6"/>
+      <c r="AC36" s="48"/>
+      <c r="AD36" s="16"/>
+      <c r="AE36" s="16"/>
+      <c r="AF36" s="16"/>
     </row>
     <row r="37" spans="1:155" ht="18" customHeight="1">
-      <c r="A37" s="15"/>
-      <c r="B37" s="67" t="s">
+      <c r="A37" s="42"/>
+      <c r="B37" s="66" t="s">
+        <v>272</v>
+      </c>
+      <c r="C37" s="43"/>
+      <c r="D37" s="43"/>
+      <c r="E37" s="43"/>
+      <c r="F37" s="43"/>
+      <c r="G37" s="43"/>
+      <c r="H37" s="43"/>
+      <c r="I37" s="43"/>
+      <c r="J37" s="43"/>
+      <c r="K37" s="43"/>
+      <c r="L37" s="43"/>
+      <c r="M37" s="43"/>
+      <c r="N37" s="43"/>
+      <c r="O37" s="43"/>
+      <c r="P37" s="43"/>
+      <c r="Q37" s="43"/>
+      <c r="R37" s="43"/>
+      <c r="S37" s="43"/>
+      <c r="T37" s="43"/>
+      <c r="U37" s="43"/>
+      <c r="V37" s="43"/>
+      <c r="W37" s="43"/>
+      <c r="X37" s="49" t="s">
         <v>273</v>
       </c>
-      <c r="C37" s="6"/>
-      <c r="D37" s="6"/>
-      <c r="E37" s="6"/>
-      <c r="F37" s="6"/>
-      <c r="G37" s="6"/>
-      <c r="H37" s="6"/>
-      <c r="I37" s="6"/>
-      <c r="J37" s="6"/>
-      <c r="K37" s="6"/>
-      <c r="L37" s="6"/>
-      <c r="M37" s="6"/>
-      <c r="N37" s="6"/>
-      <c r="O37" s="6" t="s">
-        <v>240</v>
-      </c>
-      <c r="P37" s="6" t="s">
-        <v>240</v>
-      </c>
-      <c r="Q37" s="6" t="s">
-        <v>240</v>
-      </c>
-      <c r="R37" s="6" t="s">
-        <v>240</v>
-      </c>
-      <c r="S37" s="6" t="s">
-        <v>240</v>
-      </c>
-      <c r="T37" s="6"/>
-      <c r="U37" s="6"/>
-      <c r="V37" s="6"/>
-      <c r="W37" s="6"/>
-      <c r="X37" s="6" t="s">
-        <v>240</v>
-      </c>
-      <c r="Y37" s="6" t="s">
-        <v>240</v>
-      </c>
-      <c r="Z37" s="6"/>
-      <c r="AA37" s="6"/>
-      <c r="AB37" s="6"/>
-      <c r="AC37" s="48"/>
-      <c r="AD37" s="16"/>
-      <c r="AE37" s="16"/>
-      <c r="AF37" s="16"/>
+      <c r="Y37" s="43"/>
+      <c r="Z37" s="43"/>
+      <c r="AA37" s="43"/>
+      <c r="AB37" s="43"/>
+      <c r="AC37" s="43"/>
+      <c r="AD37" s="46"/>
+      <c r="AE37" s="44" t="s">
+        <v>274</v>
+      </c>
+      <c r="AF37" s="50" t="s">
+        <v>275</v>
+      </c>
     </row>
     <row r="38" spans="1:155" ht="18" customHeight="1">
-      <c r="A38" s="42"/>
-      <c r="B38" s="66" t="s">
-        <v>274</v>
-      </c>
-      <c r="C38" s="43"/>
-      <c r="D38" s="43"/>
-      <c r="E38" s="43"/>
-      <c r="F38" s="43"/>
-      <c r="G38" s="43"/>
-      <c r="H38" s="43"/>
-      <c r="I38" s="43"/>
-      <c r="J38" s="43"/>
-      <c r="K38" s="43"/>
-      <c r="L38" s="43"/>
-      <c r="M38" s="43"/>
-      <c r="N38" s="43"/>
-      <c r="O38" s="43"/>
-      <c r="P38" s="43"/>
-      <c r="Q38" s="43"/>
-      <c r="R38" s="43"/>
-      <c r="S38" s="43"/>
-      <c r="T38" s="43"/>
-      <c r="U38" s="43"/>
-      <c r="V38" s="43"/>
-      <c r="W38" s="43"/>
-      <c r="X38" s="49" t="s">
-        <v>275</v>
-      </c>
-      <c r="Y38" s="43"/>
-      <c r="Z38" s="43"/>
-      <c r="AA38" s="43"/>
-      <c r="AB38" s="43"/>
-      <c r="AC38" s="43"/>
-      <c r="AD38" s="46"/>
-      <c r="AE38" s="44" t="s">
+      <c r="A38" s="19"/>
+      <c r="B38" s="51" t="s">
         <v>276</v>
       </c>
-      <c r="AF38" s="50" t="s">
-        <v>277</v>
-      </c>
+      <c r="C38" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="D38" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="E38" s="8"/>
+      <c r="F38" s="8"/>
+      <c r="G38" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="H38" s="8"/>
+      <c r="I38" s="8"/>
+      <c r="J38" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="K38" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="L38" s="8"/>
+      <c r="M38" s="8"/>
+      <c r="N38" s="8"/>
+      <c r="O38" s="8"/>
+      <c r="P38" s="8"/>
+      <c r="Q38" s="8"/>
+      <c r="R38" s="8"/>
+      <c r="S38" s="8"/>
+      <c r="T38" s="8"/>
+      <c r="U38" s="8"/>
+      <c r="V38" s="8"/>
+      <c r="W38" s="8"/>
+      <c r="X38" s="8"/>
+      <c r="Y38" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="Z38" s="8"/>
+      <c r="AA38" s="8"/>
+      <c r="AB38" s="8"/>
+      <c r="AC38" s="8"/>
+      <c r="AD38" s="20"/>
+      <c r="AE38" s="20"/>
+      <c r="AF38" s="20"/>
     </row>
     <row r="39" spans="1:155" ht="18" customHeight="1">
-      <c r="A39" s="19"/>
-      <c r="B39" s="51" t="s">
-        <v>278</v>
-      </c>
-      <c r="C39" s="8" t="s">
-        <v>240</v>
-      </c>
-      <c r="D39" s="8" t="s">
-        <v>240</v>
-      </c>
-      <c r="E39" s="8"/>
-      <c r="F39" s="8"/>
-      <c r="G39" s="8" t="s">
-        <v>240</v>
-      </c>
-      <c r="H39" s="8"/>
-      <c r="I39" s="8"/>
-      <c r="J39" s="8" t="s">
-        <v>240</v>
-      </c>
-      <c r="K39" s="8" t="s">
-        <v>240</v>
-      </c>
-      <c r="L39" s="8"/>
-      <c r="M39" s="8"/>
-      <c r="N39" s="8"/>
-      <c r="O39" s="8"/>
-      <c r="P39" s="8"/>
-      <c r="Q39" s="8"/>
-      <c r="R39" s="8"/>
-      <c r="S39" s="8"/>
-      <c r="T39" s="8"/>
-      <c r="U39" s="8"/>
-      <c r="V39" s="8"/>
-      <c r="W39" s="8"/>
-      <c r="X39" s="8"/>
-      <c r="Y39" s="8" t="s">
-        <v>240</v>
-      </c>
-      <c r="Z39" s="8"/>
-      <c r="AA39" s="8"/>
-      <c r="AB39" s="8"/>
-      <c r="AC39" s="8"/>
-      <c r="AD39" s="20"/>
-      <c r="AE39" s="20"/>
-      <c r="AF39" s="20"/>
+      <c r="A39" s="9"/>
+      <c r="B39" s="12" t="s">
+        <v>277</v>
+      </c>
+      <c r="C39" s="4"/>
+      <c r="D39" s="4"/>
+      <c r="E39" s="4"/>
+      <c r="F39" s="4"/>
+      <c r="G39" s="4"/>
+      <c r="H39" s="4"/>
+      <c r="I39" s="4"/>
+      <c r="J39" s="4"/>
+      <c r="K39" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="L39" s="4"/>
+      <c r="M39" s="4"/>
+      <c r="N39" s="4"/>
+      <c r="O39" s="4"/>
+      <c r="P39" s="4"/>
+      <c r="Q39" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="R39" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="S39" s="4"/>
+      <c r="T39" s="4"/>
+      <c r="U39" s="4"/>
+      <c r="V39" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="W39" s="4"/>
+      <c r="X39" s="4"/>
+      <c r="Y39" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="Z39" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="AA39" s="4"/>
+      <c r="AB39" s="4"/>
+      <c r="AC39" s="4"/>
+      <c r="AD39" s="10"/>
+      <c r="AE39" s="10"/>
+      <c r="AF39" s="10"/>
     </row>
     <row r="40" spans="1:155" ht="18" customHeight="1">
       <c r="A40" s="9"/>
       <c r="B40" s="12" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C40" s="4"/>
       <c r="D40" s="4"/>
@@ -5336,35 +5311,27 @@
       <c r="H40" s="4"/>
       <c r="I40" s="4"/>
       <c r="J40" s="4"/>
-      <c r="K40" s="4" t="s">
-        <v>240</v>
-      </c>
+      <c r="K40" s="4"/>
       <c r="L40" s="4"/>
       <c r="M40" s="4"/>
       <c r="N40" s="4"/>
       <c r="O40" s="4"/>
       <c r="P40" s="4"/>
-      <c r="Q40" s="4" t="s">
-        <v>240</v>
-      </c>
-      <c r="R40" s="4" t="s">
-        <v>240</v>
-      </c>
+      <c r="Q40" s="4"/>
+      <c r="R40" s="4"/>
       <c r="S40" s="4"/>
       <c r="T40" s="4"/>
       <c r="U40" s="4"/>
-      <c r="V40" s="4" t="s">
-        <v>240</v>
-      </c>
+      <c r="V40" s="4"/>
       <c r="W40" s="4"/>
       <c r="X40" s="4"/>
       <c r="Y40" s="4" t="s">
-        <v>240</v>
-      </c>
-      <c r="Z40" s="4" t="s">
-        <v>240</v>
-      </c>
-      <c r="AA40" s="4"/>
+        <v>238</v>
+      </c>
+      <c r="Z40" s="4"/>
+      <c r="AA40" s="4" t="s">
+        <v>238</v>
+      </c>
       <c r="AB40" s="4"/>
       <c r="AC40" s="4"/>
       <c r="AD40" s="10"/>
@@ -5374,7 +5341,7 @@
     <row r="41" spans="1:155" ht="18" customHeight="1">
       <c r="A41" s="9"/>
       <c r="B41" s="12" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C41" s="4"/>
       <c r="D41" s="4"/>
@@ -5398,13 +5365,9 @@
       <c r="V41" s="4"/>
       <c r="W41" s="4"/>
       <c r="X41" s="4"/>
-      <c r="Y41" s="4" t="s">
-        <v>240</v>
-      </c>
+      <c r="Y41" s="4"/>
       <c r="Z41" s="4"/>
-      <c r="AA41" s="4" t="s">
-        <v>240</v>
-      </c>
+      <c r="AA41" s="4"/>
       <c r="AB41" s="4"/>
       <c r="AC41" s="4"/>
       <c r="AD41" s="10"/>
@@ -5414,13 +5377,15 @@
     <row r="42" spans="1:155" ht="18" customHeight="1">
       <c r="A42" s="9"/>
       <c r="B42" s="12" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C42" s="4"/>
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>
       <c r="F42" s="4"/>
-      <c r="G42" s="4"/>
+      <c r="G42" s="4" t="s">
+        <v>238</v>
+      </c>
       <c r="H42" s="4"/>
       <c r="I42" s="4"/>
       <c r="J42" s="4"/>
@@ -5450,15 +5415,13 @@
     <row r="43" spans="1:155" ht="18" customHeight="1">
       <c r="A43" s="9"/>
       <c r="B43" s="12" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C43" s="4"/>
       <c r="D43" s="4"/>
       <c r="E43" s="4"/>
       <c r="F43" s="4"/>
-      <c r="G43" s="4" t="s">
-        <v>240</v>
-      </c>
+      <c r="G43" s="4"/>
       <c r="H43" s="4"/>
       <c r="I43" s="4"/>
       <c r="J43" s="4"/>
@@ -5475,20 +5438,21 @@
       <c r="U43" s="4"/>
       <c r="V43" s="4"/>
       <c r="W43" s="4"/>
-      <c r="X43" s="4"/>
-      <c r="Y43" s="4"/>
-      <c r="Z43" s="4"/>
-      <c r="AA43" s="4"/>
-      <c r="AB43" s="4"/>
-      <c r="AC43" s="4"/>
+      <c r="X43" s="10"/>
+      <c r="Y43" s="10"/>
+      <c r="Z43" s="10"/>
+      <c r="AA43" s="10"/>
+      <c r="AB43" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="AC43" s="10"/>
       <c r="AD43" s="10"/>
       <c r="AE43" s="10"/>
-      <c r="AF43" s="10"/>
     </row>
     <row r="44" spans="1:155" ht="18" customHeight="1">
       <c r="A44" s="9"/>
       <c r="B44" s="12" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C44" s="4"/>
       <c r="D44" s="4"/>
@@ -5515,9 +5479,7 @@
       <c r="Y44" s="10"/>
       <c r="Z44" s="10"/>
       <c r="AA44" s="10"/>
-      <c r="AB44" s="10" t="s">
-        <v>240</v>
-      </c>
+      <c r="AB44" s="10"/>
       <c r="AC44" s="10"/>
       <c r="AD44" s="10"/>
       <c r="AE44" s="10"/>
@@ -5525,7 +5487,7 @@
     <row r="45" spans="1:155" ht="18" customHeight="1">
       <c r="A45" s="9"/>
       <c r="B45" s="12" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C45" s="4"/>
       <c r="D45" s="4"/>
@@ -5560,7 +5522,7 @@
     <row r="46" spans="1:155" ht="18" customHeight="1">
       <c r="A46" s="9"/>
       <c r="B46" s="12" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C46" s="4"/>
       <c r="D46" s="4"/>
@@ -5595,7 +5557,7 @@
     <row r="47" spans="1:155" ht="18" customHeight="1">
       <c r="A47" s="9"/>
       <c r="B47" s="12" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C47" s="4"/>
       <c r="D47" s="4"/>
@@ -5627,40 +5589,10 @@
       <c r="AD47" s="10"/>
       <c r="AE47" s="10"/>
     </row>
-    <row r="48" spans="1:155" ht="18" customHeight="1">
-      <c r="A48" s="9"/>
-      <c r="B48" s="12" t="s">
-        <v>287</v>
-      </c>
-      <c r="C48" s="4"/>
-      <c r="D48" s="4"/>
-      <c r="E48" s="4"/>
-      <c r="F48" s="4"/>
-      <c r="G48" s="4"/>
-      <c r="H48" s="4"/>
-      <c r="I48" s="4"/>
-      <c r="J48" s="4"/>
-      <c r="K48" s="4"/>
-      <c r="L48" s="4"/>
-      <c r="M48" s="4"/>
-      <c r="N48" s="4"/>
-      <c r="O48" s="4"/>
-      <c r="P48" s="4"/>
-      <c r="Q48" s="4"/>
-      <c r="R48" s="4"/>
-      <c r="S48" s="4"/>
-      <c r="T48" s="4"/>
-      <c r="U48" s="4"/>
-      <c r="V48" s="4"/>
-      <c r="W48" s="4"/>
-      <c r="X48" s="10"/>
-      <c r="Y48" s="10"/>
-      <c r="Z48" s="10"/>
-      <c r="AA48" s="10"/>
-      <c r="AB48" s="10"/>
-      <c r="AC48" s="10"/>
-      <c r="AD48" s="10"/>
-      <c r="AE48" s="10"/>
+    <row r="48" spans="1:155">
+      <c r="X48" s="2"/>
+      <c r="Y48" s="2"/>
+      <c r="Z48" s="2"/>
     </row>
     <row r="49" spans="24:26">
       <c r="X49" s="2"/>
@@ -5722,13 +5654,8 @@
       <c r="Y60" s="2"/>
       <c r="Z60" s="2"/>
     </row>
-    <row r="61" spans="24:26">
-      <c r="X61" s="2"/>
-      <c r="Y61" s="2"/>
-      <c r="Z61" s="2"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A2:AF34" xr:uid="{D8B0CA4D-B55F-4AFA-903E-3D529FFFD0A1}">
+  <autoFilter ref="A2:AF33" xr:uid="{D8B0CA4D-B55F-4AFA-903E-3D529FFFD0A1}">
     <filterColumn colId="2" showButton="0"/>
     <filterColumn colId="3" showButton="0"/>
     <filterColumn colId="4" showButton="0"/>
@@ -5748,154 +5675,154 @@
     <filterColumn colId="20" showButton="0"/>
   </autoFilter>
   <mergeCells count="22">
-    <mergeCell ref="AE2:AE5"/>
-    <mergeCell ref="AF2:AF5"/>
-    <mergeCell ref="A8:A19"/>
-    <mergeCell ref="AB2:AB5"/>
-    <mergeCell ref="AC2:AC5"/>
+    <mergeCell ref="AE2:AE4"/>
+    <mergeCell ref="AF2:AF4"/>
+    <mergeCell ref="A7:A18"/>
+    <mergeCell ref="AB2:AB4"/>
+    <mergeCell ref="AC2:AC4"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="G3:L3"/>
     <mergeCell ref="C2:N2"/>
-    <mergeCell ref="X2:X5"/>
-    <mergeCell ref="AA2:AA5"/>
+    <mergeCell ref="X2:X4"/>
+    <mergeCell ref="AA2:AA4"/>
     <mergeCell ref="U2:V3"/>
-    <mergeCell ref="W2:W5"/>
+    <mergeCell ref="W2:W4"/>
     <mergeCell ref="Q3:T3"/>
     <mergeCell ref="O2:T2"/>
     <mergeCell ref="O3:P3"/>
-    <mergeCell ref="Y2:Y5"/>
-    <mergeCell ref="B21:B28"/>
-    <mergeCell ref="B13:B19"/>
-    <mergeCell ref="B8:B12"/>
-    <mergeCell ref="B29:B34"/>
-    <mergeCell ref="AD2:AD5"/>
-    <mergeCell ref="Z2:Z5"/>
+    <mergeCell ref="Y2:Y4"/>
+    <mergeCell ref="B20:B27"/>
+    <mergeCell ref="B12:B18"/>
+    <mergeCell ref="B7:B11"/>
+    <mergeCell ref="B28:B33"/>
+    <mergeCell ref="AD2:AD4"/>
+    <mergeCell ref="Z2:Z4"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="C22" r:id="rId1" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/sp?tab=models" xr:uid="{FE987DC0-578A-4A81-AB17-6E49D6983782}"/>
-    <hyperlink ref="C23" r:id="rId2" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/spe?tab=models" xr:uid="{E414E66B-6D50-4BC0-93B6-EEDD71D1D349}"/>
-    <hyperlink ref="C24" r:id="rId3" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/sp-ne?tab=models" xr:uid="{79A82224-5E75-416A-BD5C-1C442DB4F9E7}"/>
-    <hyperlink ref="D22" r:id="rId4" display="https://product-selection.grundfos.com/fr/products/bm?tab=products" xr:uid="{39935FC4-BF60-4ADA-99B8-6280D11B4087}"/>
-    <hyperlink ref="D23" r:id="rId5" display="https://product-selection.grundfos.com/fr/products/bms?tab=products" xr:uid="{201298BF-F5B7-4DD8-896A-A6CFDF20A155}"/>
-    <hyperlink ref="D24" r:id="rId6" display="https://product-selection.grundfos.com/fr/products/bm-hp?tab=products" xr:uid="{0AA34BB7-1783-4351-AB39-2E3E2C9E6D24}"/>
-    <hyperlink ref="E22" r:id="rId7" display="https://product-selection.grundfos.com/fr/products/kpl?tab=models" xr:uid="{02FD05D5-211D-4185-A911-F718E163AF22}"/>
-    <hyperlink ref="E23" r:id="rId8" display="https://product-selection.grundfos.com/fr/products/kwm?tab=documentation" xr:uid="{F11B5E61-F53C-4DA1-93C5-A57D0408930C}"/>
-    <hyperlink ref="F22" r:id="rId9" display="https://product-selection.grundfos.com/fr/products/ls?tab=products" xr:uid="{070C34E9-9C05-4522-9AD2-8E6D82261A9B}"/>
-    <hyperlink ref="J22" r:id="rId10" display="https://product-selection.grundfos.com/fr/products/cm-cme?tab=products" xr:uid="{E79A5B97-E6E0-4649-B070-9A1CF47F88B2}"/>
-    <hyperlink ref="I22" r:id="rId11" display="https://product-selection.grundfos.com/fr/products/cm-cme/cm-self-priming?tab=models" xr:uid="{CFEF6DD3-2F90-4195-BA05-DEE28F55BD3E}"/>
-    <hyperlink ref="J23" r:id="rId12" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nb?tab=documentation" xr:uid="{ABC208A8-FE5B-4CC4-B585-6A3873FA7294}"/>
-    <hyperlink ref="J24" r:id="rId13" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nbe?tab=models" xr:uid="{1D4EF590-19C1-44EB-8B92-46AD5F28F62F}"/>
-    <hyperlink ref="J25" r:id="rId14" display="https://product-selection.grundfos.com/fr/products/nk-nke-nke-series-2000-nk-bare-shaft?tab=products" xr:uid="{76D3161D-F2DD-4CCA-AC1D-AD2E393D8694}"/>
-    <hyperlink ref="J26" r:id="rId15" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft?tab=products" xr:uid="{9CA4757F-439C-4161-8B60-7C14A9EDCA69}"/>
-    <hyperlink ref="J27" r:id="rId16" display="https://product-selection.grundfos.com/fr/products/tp-tpe?tab=products" xr:uid="{0C9A1473-1926-417A-947F-8561754B7D76}"/>
-    <hyperlink ref="N24" r:id="rId17" display="https://product-selection.grundfos.com/fr/products/tp-tpe?tab=products" xr:uid="{7D2D046F-1C95-42DD-8F35-90280675B9EA}"/>
-    <hyperlink ref="N22" r:id="rId18" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nbe?tab=models" xr:uid="{303D01A6-AC7B-42EE-AE09-2A10FBED3940}"/>
-    <hyperlink ref="N23" r:id="rId19" display="https://product-selection.grundfos.com/fr/products/nk-nke-nke-series-2000-nk-bare-shaft?tab=products" xr:uid="{A1442A3E-E286-4D87-BF5A-B52C00F11931}"/>
-    <hyperlink ref="N25" r:id="rId20" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft?tab=products" xr:uid="{91C811C0-E7C2-45CC-8C4A-41851188982F}"/>
-    <hyperlink ref="K22" r:id="rId21" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte?tab=products" xr:uid="{168A97AE-925F-4CB8-99FA-4D28B053F7CB}"/>
-    <hyperlink ref="L23" r:id="rId22" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte/cre?tab=models" xr:uid="{43E68B92-4EB3-4ECE-A299-C7DDCAFB1889}"/>
-    <hyperlink ref="L24" r:id="rId23" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte/crne?tab=models" xr:uid="{9DD9406E-F477-49F6-BA29-841ED00CE74B}"/>
-    <hyperlink ref="M22" r:id="rId24" display="https://product-selection.grundfos.com/fr/products/cm-cme/cme?tab=models" xr:uid="{CB210458-379C-4663-B0FD-73E843090C67}"/>
-    <hyperlink ref="M23" r:id="rId25" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nbe?tab=models" xr:uid="{3776F606-4CBE-49B1-912C-5B2BC9586206}"/>
-    <hyperlink ref="M24" r:id="rId26" display="https://product-selection.grundfos.com/fr/products/nk-nke-nke-series-2000-nk-bare-shaft?tab=products" xr:uid="{8731A9E7-9B51-450F-BCB5-013214A2B33F}"/>
-    <hyperlink ref="M25" r:id="rId27" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft?tab=products" xr:uid="{EDB8C821-F675-4CE1-B7B0-0FAF39DCEFD4}"/>
-    <hyperlink ref="L26" r:id="rId28" display="https://product-selection.grundfos.com/fr/products/hydro-multi-e?tab=models" xr:uid="{5995DFA3-65AE-4378-BD2E-CDA4F6FA5ED7}"/>
-    <hyperlink ref="L27" r:id="rId29" display="https://product-selection.grundfos.com/fr/products/hydro-mpc?tab=products" xr:uid="{2E37CE89-9B22-43AA-B967-C6F20A25613F}"/>
-    <hyperlink ref="L25" r:id="rId30" display="https://product-selection.grundfos.com/fr/products/hydro-solo-e?tab=models" xr:uid="{5A1F2584-1AA0-4C8B-A55D-39C825C8A3F8}"/>
-    <hyperlink ref="O22" r:id="rId31" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/sl1?tab=models" xr:uid="{9C7E88DB-59BA-4B5C-8769-45D64CC97D40}"/>
-    <hyperlink ref="O23" r:id="rId32" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/slv?tab=models" xr:uid="{00039B9D-B404-44A8-B557-BBF172D7CD31}"/>
-    <hyperlink ref="O24" r:id="rId33" display="https://product-selection.grundfos.com/fr/products/sesl-9-30-kw?tab=models" xr:uid="{C90FBAD5-7C9C-4429-9BAC-9BE027B562FD}"/>
-    <hyperlink ref="O26" r:id="rId34" display="https://product-selection.grundfos.com/fr/products/s?tab=products" xr:uid="{6F267867-1729-460E-9939-DEBA10D95429}"/>
-    <hyperlink ref="O25" r:id="rId35" display="https://product-selection.grundfos.com/fr/products/sesl-frame-size-56?tab=models" xr:uid="{541D6F69-2D4F-412B-91C7-A0B79C20C0CA}"/>
-    <hyperlink ref="P23" r:id="rId36" display="https://product-selection.grundfos.com/fr/products/unilift-ap/unilift-apg?tab=models" xr:uid="{CF6542DD-C411-4584-A2A2-ADD9BD336104}"/>
-    <hyperlink ref="P22" r:id="rId37" display="https://product-selection.grundfos.com/fr/products/seg?tab=models" xr:uid="{AF847B64-9B08-45DD-8487-57C6900B0D5F}"/>
-    <hyperlink ref="Q22" r:id="rId38" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/se1?tab=models" xr:uid="{D2271F27-967E-46DC-8195-E2EAFD3339EB}"/>
-    <hyperlink ref="Q23" r:id="rId39" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/sev?tab=models" xr:uid="{6D042873-5F32-4A50-8803-93F40528C6A1}"/>
-    <hyperlink ref="Q24" r:id="rId40" display="https://product-selection.grundfos.com/fr/products/sesl-9-30-kw?tab=models" xr:uid="{A344F5B5-8A97-456F-87D5-4C6EFCA52D3A}"/>
-    <hyperlink ref="Q25" r:id="rId41" display="https://product-selection.grundfos.com/fr/products/sesl-frame-size-56?tab=models" xr:uid="{BB0B40A3-A20A-44BC-9FC9-E9EE00FC9F45}"/>
-    <hyperlink ref="Q26" r:id="rId42" display="https://product-selection.grundfos.com/fr/products/s?tab=products" xr:uid="{2E26D22E-3FD7-4718-9B39-661D30AF938C}"/>
-    <hyperlink ref="Q27" r:id="rId43" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft/nkg-supervortex-impeller?tab=explore" xr:uid="{FA539854-B47D-4B47-9F9A-7CE595B28025}"/>
-    <hyperlink ref="S22" r:id="rId44" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/se1?tab=models" xr:uid="{66C50FE8-D6EA-4602-866A-7B3258A9261C}"/>
-    <hyperlink ref="S23" r:id="rId45" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/sev?tab=models" xr:uid="{DEFE3A48-5152-4917-935D-8BAB7D40CDD7}"/>
-    <hyperlink ref="S24" r:id="rId46" display="https://product-selection.grundfos.com/fr/products/sesl-9-30-kw?tab=models" xr:uid="{62BA715F-3850-4F49-A593-7645C6C0C3CC}"/>
-    <hyperlink ref="S25" r:id="rId47" display="https://product-selection.grundfos.com/fr/products/sesl-frame-size-56?tab=models" xr:uid="{F0AA29DC-4DA5-4CA6-94B3-C22351F6904E}"/>
-    <hyperlink ref="S26" r:id="rId48" display="https://product-selection.grundfos.com/fr/products/s?tab=products" xr:uid="{96671AB9-9AEA-4A5F-B84F-E78888F9B311}"/>
-    <hyperlink ref="S27" r:id="rId49" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft/nkg-supervortex-impeller?tab=explore" xr:uid="{8A1CF826-08F5-4AF2-B984-9AA020480952}"/>
-    <hyperlink ref="O27" r:id="rId50" display="https://product-selection.grundfos.com/fr/products/unilift-ap/unilift-ap50b?tab=models" xr:uid="{14E21A07-FF5F-4129-AE6E-260A1AA5098C}"/>
-    <hyperlink ref="W22" r:id="rId51" display="https://product-selection.grundfos.com/fr/products/unilift-ap?tab=products" xr:uid="{FF1F3D5A-16C1-4C5A-8F69-37BEB2C51657}"/>
-    <hyperlink ref="W23" r:id="rId52" display="https://product-selection.grundfos.com/fr/products/unilift-kp?tab=models" xr:uid="{D8B15CDE-A46F-4955-8CE5-B1F2491BDDEE}"/>
-    <hyperlink ref="W24" r:id="rId53" display="https://product-selection.grundfos.com/fr/products/unilift-cc?tab=models" xr:uid="{5DA16314-BD6C-4DB3-8EC0-A99C56D3006D}"/>
-    <hyperlink ref="W25" r:id="rId54" display="https://product-selection.grundfos.com/fr/products/dp?tab=models" xr:uid="{4D82ED98-3DD6-4697-9C9C-A060C7E06489}"/>
-    <hyperlink ref="W26" r:id="rId55" display="https://product-selection.grundfos.com/fr/products/ef?tab=models" xr:uid="{ABDE8970-72CB-4EB8-979F-99183A9FD9D3}"/>
-    <hyperlink ref="Y22" r:id="rId56" display="https://product-selection.grundfos.com/fr/products/mt-tank-mounted-pumps/mtr?tab=models" xr:uid="{D5799B15-EF87-41DF-88D8-05F25935D793}"/>
-    <hyperlink ref="Y23" r:id="rId57" display="https://product-selection.grundfos.com/fr/products/mt-tank-mounted-pumps/mtre?tab=models" xr:uid="{7E2DAAB5-3884-49DD-BF25-FA92C2CE9951}"/>
-    <hyperlink ref="Y24" r:id="rId58" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nb?tab=documentation" xr:uid="{92C19ACB-7462-4938-A66E-478979299908}"/>
-    <hyperlink ref="Y25" r:id="rId59" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nbe?tab=models" xr:uid="{D2CCE95F-A5DF-4715-B3CA-DB297F6DF5C8}"/>
-    <hyperlink ref="Y26" r:id="rId60" display="https://product-selection.grundfos.com/fr/products/nk-nke-nke-series-2000-nk-bare-shaft?tab=products" xr:uid="{EA080A36-FCEB-4D04-B389-F8ABE5514300}"/>
-    <hyperlink ref="Y27" r:id="rId61" display="https://product-selection.grundfos.com/fr/products/tp-tpe?tab=products" xr:uid="{2A2A6B6D-2CAA-4110-9FED-BCA8DC5F1709}"/>
-    <hyperlink ref="Y28" r:id="rId62" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte?tab=products" xr:uid="{D902984C-2BC5-48A4-BF49-DCE4C7E629F6}"/>
-    <hyperlink ref="Z22" r:id="rId63" display="https://product-selection.grundfos.com/fr/products/hydro-en?tab=models" xr:uid="{69CECDCF-71ED-40D6-A274-30663F73D3A6}"/>
-    <hyperlink ref="AD22" r:id="rId64" display="https://product-selection.grundfos.com/fr/products/poweradapt?tab=models" xr:uid="{CBB79406-3EE4-4CC7-BCD3-398882D58A96}"/>
-    <hyperlink ref="AD23" r:id="rId65" display="https://product-selection.grundfos.com/fr/products/rsi?tab=models" xr:uid="{2ECDD4BA-B757-4A11-9F78-EB235920F462}"/>
-    <hyperlink ref="AD24" r:id="rId66" display="https://product-selection.grundfos.com/fr/products/crflex?tab=models" xr:uid="{F1835770-C21F-4E8A-9EBF-7C701B0E9CF4}"/>
-    <hyperlink ref="AD25" r:id="rId67" display="https://product-selection.grundfos.com/fr/products/sqflex?tab=models" xr:uid="{2932EAA4-553E-42B6-AD4B-37D91C9B845C}"/>
-    <hyperlink ref="AD26" r:id="rId68" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/sp?tab=models" xr:uid="{25A70C6E-05E1-4E40-956B-50B78B088135}"/>
-    <hyperlink ref="AD27" r:id="rId69" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/spe?tab=models" xr:uid="{7C346AF6-2EEB-4DFC-A819-DAE2C3B09113}"/>
-    <hyperlink ref="AD28" r:id="rId70" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte?tab=products" xr:uid="{9F4AE584-6CDD-45BE-ABC9-5087AAD766B9}"/>
-    <hyperlink ref="AE22" r:id="rId71" display="https://product-selection.grundfos.com/fr/products/dosing-pumps-digital/dda?tab=models" xr:uid="{68600FE5-FDB0-4237-8B8A-45786462FE8A}"/>
-    <hyperlink ref="AE23" r:id="rId72" display="https://product-selection.grundfos.com/fr/products/dosing-pumps-digital/dme?tab=models" xr:uid="{41502941-2297-46B7-A840-2EF7A24064D7}"/>
-    <hyperlink ref="AE24" r:id="rId73" display="https://product-selection.grundfos.com/fr/products/dosing-pumps-mechanical/dmx?tab=models" xr:uid="{A892A826-C3E1-4B26-9529-8174E76C068D}"/>
-    <hyperlink ref="AE25" r:id="rId74" display="https://product-selection.grundfos.com/fr/products/dosing-pumps-mechanical/dmh?tab=models" xr:uid="{60926621-C7DA-4892-9ACA-4145E303C37B}"/>
-    <hyperlink ref="AE26" r:id="rId75" xr:uid="{EB339B7E-AAB0-4720-A5DC-B7E47BEFE888}"/>
-    <hyperlink ref="AF24" r:id="rId76" display="https://product-selection.grundfos.com/fr/products/disinfection-systems/oxiperm?tab=models" xr:uid="{D1CFBDC1-076A-4661-B343-B5087946D2BF}"/>
-    <hyperlink ref="AF22" r:id="rId77" display="https://product-selection.grundfos.com/fr/products/disinfection-systems/vaccuperm?tab=models" xr:uid="{0E5CA30E-D80E-4BC1-BE8D-5757C0E703F9}"/>
-    <hyperlink ref="AF23" r:id="rId78" display="https://product-selection.grundfos.com/fr/products/disinfection-systems/selcoperm?tab=models" xr:uid="{3FE337C4-03C2-4326-92F3-2ADF14429172}"/>
-    <hyperlink ref="C30" r:id="rId79" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-4" xr:uid="{7CECB146-2C6E-4D8C-8362-B574F0A0B1CD}"/>
-    <hyperlink ref="C31" r:id="rId80" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-6" xr:uid="{77066640-D437-4393-AE04-9291CA2EA2E2}"/>
-    <hyperlink ref="C32" r:id="rId81" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-8" xr:uid="{440D559C-9B55-46F7-B47D-809066594D8E}"/>
-    <hyperlink ref="C33" r:id="rId82" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-actun-zetos" xr:uid="{6B88B868-32F8-4635-8067-C4F8AA30A87A}"/>
-    <hyperlink ref="C34" r:id="rId83" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-14-24" xr:uid="{6AAEB27D-0CD4-409C-9175-B5DC81BA5B91}"/>
-    <hyperlink ref="D30" r:id="rId84" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-4" xr:uid="{70B5668C-6DE4-4721-BD0D-15695ACCFD10}"/>
-    <hyperlink ref="D31" r:id="rId85" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-6" xr:uid="{AB0F5528-0721-49E7-9EB4-443A836A5BE6}"/>
-    <hyperlink ref="D32" r:id="rId86" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-8" xr:uid="{CE5D4CF5-B9AD-4786-AF2A-5CBA0FB4461E}"/>
-    <hyperlink ref="D33" r:id="rId87" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-actun-zetos" xr:uid="{F3302311-60D3-4257-BE0E-8ADCE8FD3F26}"/>
-    <hyperlink ref="D34" r:id="rId88" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-14-24" xr:uid="{C714C692-05B2-43B9-83CE-06CDCF547DAA}"/>
-    <hyperlink ref="F30" r:id="rId89" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-scp" xr:uid="{7BEBF8BE-E457-43DD-A078-9A05C9712ED1}"/>
-    <hyperlink ref="F31" r:id="rId90" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-atmos-tera-sch" xr:uid="{8AC9B5FF-3554-4A3F-9A49-254FDDC1D679}"/>
-    <hyperlink ref="G30" r:id="rId91" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-4" xr:uid="{A6F45EEC-DFC1-4F41-A737-7D50D323F858}"/>
-    <hyperlink ref="G31" r:id="rId92" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-6" xr:uid="{E8092E13-22EC-4AA4-A0E2-CB8C894814DA}"/>
-    <hyperlink ref="G32" r:id="rId93" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-8" xr:uid="{06C47C82-BB6B-4167-9AFC-F87F629A6D2D}"/>
-    <hyperlink ref="G33" r:id="rId94" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-actun-zetos" xr:uid="{7F484481-A382-4AA7-BC6F-9F9E8E881F13}"/>
-    <hyperlink ref="G34" r:id="rId95" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-14-24" xr:uid="{145E082E-ACF5-4C03-95AA-D5FF287B68E9}"/>
-    <hyperlink ref="J30" r:id="rId96" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-medana-ch1-l" xr:uid="{CB6CAFF8-329E-47DC-8F46-39C8BB5E04DD}"/>
-    <hyperlink ref="J31" r:id="rId97" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-zeox-first-h" xr:uid="{2D403080-ECF0-434D-8570-2DCE4384BDB3}"/>
-    <hyperlink ref="K30" r:id="rId98" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-helix-v" xr:uid="{24EB14FB-8853-4DD9-BFF7-D08622F6269E}"/>
-    <hyperlink ref="K31" r:id="rId99" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-helix-first-v" xr:uid="{292648A6-CEF7-4F6A-B9E8-2C2D1935D493}"/>
-    <hyperlink ref="L30" r:id="rId100" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-helix-ve" xr:uid="{CB04A41A-2CE9-45EC-90FB-F63D1D7003E0}"/>
-    <hyperlink ref="L31" r:id="rId101" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-helix2-0-ve" xr:uid="{0D95BEE0-BF20-4117-86C3-9423999074AC}"/>
-    <hyperlink ref="M30" r:id="rId102" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-medana-ch3-le" xr:uid="{E61CDC21-E587-41FD-8720-AA95E8F2BCB8}"/>
-    <hyperlink ref="N30" r:id="rId103" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-isar-modh1-e-2-3" xr:uid="{2D23D0CC-B7DF-4FF1-ABE9-A9C38B0D675F}"/>
-    <hyperlink ref="N31" r:id="rId104" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-siboost2-0-smart-helix-ve" xr:uid="{FFEEE275-2C73-4EC4-B193-CB85762B0142}"/>
-    <hyperlink ref="O30" r:id="rId105" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-pro" xr:uid="{40187CA6-E027-4F57-B695-B124E41E9781}"/>
-    <hyperlink ref="O31" r:id="rId106" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-supra" xr:uid="{6510CD0A-CFE7-486C-91AF-7C7A655B4AFB}"/>
-    <hyperlink ref="O32" r:id="rId107" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-solid" xr:uid="{BDC567B5-AC65-4996-9A0B-1AF09DF2041A}"/>
-    <hyperlink ref="Q30" r:id="rId108" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-bloc" xr:uid="{3980AF89-63D6-4F8A-AA62-E67520B41458}"/>
-    <hyperlink ref="Q31" r:id="rId109" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-norm" xr:uid="{713EE9E0-CE07-4B5A-8098-8828FD7A2BE1}"/>
-    <hyperlink ref="P30" r:id="rId110" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-pro-s" xr:uid="{7EA67BA6-0CB9-4BC2-8D2F-2187D3E3EC87}"/>
-    <hyperlink ref="O33" r:id="rId111" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-fa-configure" xr:uid="{F271E929-C189-489C-95BA-44C8F95B9706}"/>
-    <hyperlink ref="S30" r:id="rId112" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-pro" xr:uid="{4E520461-D8CA-4714-95A3-4A07D979003B}"/>
-    <hyperlink ref="S31" r:id="rId113" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-supra" xr:uid="{7E747CBF-258D-4F97-AE71-AF52B950EDDE}"/>
-    <hyperlink ref="S32" r:id="rId114" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-solid" xr:uid="{90F21445-AD91-480E-9E60-99DEEB471A24}"/>
-    <hyperlink ref="S33" r:id="rId115" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-fa-configure" xr:uid="{CAC9CBDD-5033-4067-92F5-E1A89E7A10BF}"/>
-    <hyperlink ref="U30" r:id="rId116" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-pro" xr:uid="{DED143CB-BC81-4CC1-99AF-6D9EFDCA04A2}"/>
-    <hyperlink ref="U31" r:id="rId117" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-supra" xr:uid="{AD0F4A4E-82E3-443D-B5CE-BB1383456F96}"/>
-    <hyperlink ref="U32" r:id="rId118" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-solid" xr:uid="{F30C0BD2-ACC1-498E-B06C-26D556B514B6}"/>
-    <hyperlink ref="U33" r:id="rId119" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-fa-configure" xr:uid="{FC92FF04-817E-49C9-B9E1-3FED19E3DBAA}"/>
-    <hyperlink ref="W30" r:id="rId120" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-drain-tm-tmw-tmr-32" xr:uid="{0F177732-3552-46D9-B2A1-0858315CC611}"/>
-    <hyperlink ref="W31" r:id="rId121" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-padus-uni" xr:uid="{31C21B43-5DBE-431A-A886-4FBC3A6BE491}"/>
-    <hyperlink ref="W32" r:id="rId122" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-padus-mini3" xr:uid="{D91894CF-CB16-4C43-980E-41E743666848}"/>
-    <hyperlink ref="W33" r:id="rId123" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-padus-pro" xr:uid="{79DE7E3B-A7A2-4098-B5DF-694F7F93640D}"/>
-    <hyperlink ref="Z30" r:id="rId124" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-cof-helix" xr:uid="{2E5216D3-37DA-48CB-ABA0-7C21064BB2D3}"/>
+    <hyperlink ref="C21" r:id="rId1" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/sp?tab=models" xr:uid="{FE987DC0-578A-4A81-AB17-6E49D6983782}"/>
+    <hyperlink ref="C22" r:id="rId2" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/spe?tab=models" xr:uid="{E414E66B-6D50-4BC0-93B6-EEDD71D1D349}"/>
+    <hyperlink ref="C23" r:id="rId3" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/sp-ne?tab=models" xr:uid="{79A82224-5E75-416A-BD5C-1C442DB4F9E7}"/>
+    <hyperlink ref="D21" r:id="rId4" display="https://product-selection.grundfos.com/fr/products/bm?tab=products" xr:uid="{39935FC4-BF60-4ADA-99B8-6280D11B4087}"/>
+    <hyperlink ref="D22" r:id="rId5" display="https://product-selection.grundfos.com/fr/products/bms?tab=products" xr:uid="{201298BF-F5B7-4DD8-896A-A6CFDF20A155}"/>
+    <hyperlink ref="D23" r:id="rId6" display="https://product-selection.grundfos.com/fr/products/bm-hp?tab=products" xr:uid="{0AA34BB7-1783-4351-AB39-2E3E2C9E6D24}"/>
+    <hyperlink ref="E21" r:id="rId7" display="https://product-selection.grundfos.com/fr/products/kpl?tab=models" xr:uid="{02FD05D5-211D-4185-A911-F718E163AF22}"/>
+    <hyperlink ref="E22" r:id="rId8" display="https://product-selection.grundfos.com/fr/products/kwm?tab=documentation" xr:uid="{F11B5E61-F53C-4DA1-93C5-A57D0408930C}"/>
+    <hyperlink ref="F21" r:id="rId9" display="https://product-selection.grundfos.com/fr/products/ls?tab=products" xr:uid="{070C34E9-9C05-4522-9AD2-8E6D82261A9B}"/>
+    <hyperlink ref="J21" r:id="rId10" display="https://product-selection.grundfos.com/fr/products/cm-cme?tab=products" xr:uid="{E79A5B97-E6E0-4649-B070-9A1CF47F88B2}"/>
+    <hyperlink ref="I21" r:id="rId11" display="https://product-selection.grundfos.com/fr/products/cm-cme/cm-self-priming?tab=models" xr:uid="{CFEF6DD3-2F90-4195-BA05-DEE28F55BD3E}"/>
+    <hyperlink ref="J22" r:id="rId12" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nb?tab=documentation" xr:uid="{ABC208A8-FE5B-4CC4-B585-6A3873FA7294}"/>
+    <hyperlink ref="J23" r:id="rId13" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nbe?tab=models" xr:uid="{1D4EF590-19C1-44EB-8B92-46AD5F28F62F}"/>
+    <hyperlink ref="J24" r:id="rId14" display="https://product-selection.grundfos.com/fr/products/nk-nke-nke-series-2000-nk-bare-shaft?tab=products" xr:uid="{76D3161D-F2DD-4CCA-AC1D-AD2E393D8694}"/>
+    <hyperlink ref="J25" r:id="rId15" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft?tab=products" xr:uid="{9CA4757F-439C-4161-8B60-7C14A9EDCA69}"/>
+    <hyperlink ref="J26" r:id="rId16" display="https://product-selection.grundfos.com/fr/products/tp-tpe?tab=products" xr:uid="{0C9A1473-1926-417A-947F-8561754B7D76}"/>
+    <hyperlink ref="N23" r:id="rId17" display="https://product-selection.grundfos.com/fr/products/tp-tpe?tab=products" xr:uid="{7D2D046F-1C95-42DD-8F35-90280675B9EA}"/>
+    <hyperlink ref="N21" r:id="rId18" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nbe?tab=models" xr:uid="{303D01A6-AC7B-42EE-AE09-2A10FBED3940}"/>
+    <hyperlink ref="N22" r:id="rId19" display="https://product-selection.grundfos.com/fr/products/nk-nke-nke-series-2000-nk-bare-shaft?tab=products" xr:uid="{A1442A3E-E286-4D87-BF5A-B52C00F11931}"/>
+    <hyperlink ref="N24" r:id="rId20" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft?tab=products" xr:uid="{91C811C0-E7C2-45CC-8C4A-41851188982F}"/>
+    <hyperlink ref="K21" r:id="rId21" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte?tab=products" xr:uid="{168A97AE-925F-4CB8-99FA-4D28B053F7CB}"/>
+    <hyperlink ref="L22" r:id="rId22" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte/cre?tab=models" xr:uid="{43E68B92-4EB3-4ECE-A299-C7DDCAFB1889}"/>
+    <hyperlink ref="L23" r:id="rId23" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte/crne?tab=models" xr:uid="{9DD9406E-F477-49F6-BA29-841ED00CE74B}"/>
+    <hyperlink ref="M21" r:id="rId24" display="https://product-selection.grundfos.com/fr/products/cm-cme/cme?tab=models" xr:uid="{CB210458-379C-4663-B0FD-73E843090C67}"/>
+    <hyperlink ref="M22" r:id="rId25" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nbe?tab=models" xr:uid="{3776F606-4CBE-49B1-912C-5B2BC9586206}"/>
+    <hyperlink ref="M23" r:id="rId26" display="https://product-selection.grundfos.com/fr/products/nk-nke-nke-series-2000-nk-bare-shaft?tab=products" xr:uid="{8731A9E7-9B51-450F-BCB5-013214A2B33F}"/>
+    <hyperlink ref="M24" r:id="rId27" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft?tab=products" xr:uid="{EDB8C821-F675-4CE1-B7B0-0FAF39DCEFD4}"/>
+    <hyperlink ref="L25" r:id="rId28" display="https://product-selection.grundfos.com/fr/products/hydro-multi-e?tab=models" xr:uid="{5995DFA3-65AE-4378-BD2E-CDA4F6FA5ED7}"/>
+    <hyperlink ref="L26" r:id="rId29" display="https://product-selection.grundfos.com/fr/products/hydro-mpc?tab=products" xr:uid="{2E37CE89-9B22-43AA-B967-C6F20A25613F}"/>
+    <hyperlink ref="L24" r:id="rId30" display="https://product-selection.grundfos.com/fr/products/hydro-solo-e?tab=models" xr:uid="{5A1F2584-1AA0-4C8B-A55D-39C825C8A3F8}"/>
+    <hyperlink ref="O21" r:id="rId31" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/sl1?tab=models" xr:uid="{9C7E88DB-59BA-4B5C-8769-45D64CC97D40}"/>
+    <hyperlink ref="O22" r:id="rId32" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/slv?tab=models" xr:uid="{00039B9D-B404-44A8-B557-BBF172D7CD31}"/>
+    <hyperlink ref="O23" r:id="rId33" display="https://product-selection.grundfos.com/fr/products/sesl-9-30-kw?tab=models" xr:uid="{C90FBAD5-7C9C-4429-9BAC-9BE027B562FD}"/>
+    <hyperlink ref="O25" r:id="rId34" display="https://product-selection.grundfos.com/fr/products/s?tab=products" xr:uid="{6F267867-1729-460E-9939-DEBA10D95429}"/>
+    <hyperlink ref="O24" r:id="rId35" display="https://product-selection.grundfos.com/fr/products/sesl-frame-size-56?tab=models" xr:uid="{541D6F69-2D4F-412B-91C7-A0B79C20C0CA}"/>
+    <hyperlink ref="P22" r:id="rId36" display="https://product-selection.grundfos.com/fr/products/unilift-ap/unilift-apg?tab=models" xr:uid="{CF6542DD-C411-4584-A2A2-ADD9BD336104}"/>
+    <hyperlink ref="P21" r:id="rId37" display="https://product-selection.grundfos.com/fr/products/seg?tab=models" xr:uid="{AF847B64-9B08-45DD-8487-57C6900B0D5F}"/>
+    <hyperlink ref="Q21" r:id="rId38" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/se1?tab=models" xr:uid="{D2271F27-967E-46DC-8195-E2EAFD3339EB}"/>
+    <hyperlink ref="Q22" r:id="rId39" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/sev?tab=models" xr:uid="{6D042873-5F32-4A50-8803-93F40528C6A1}"/>
+    <hyperlink ref="Q23" r:id="rId40" display="https://product-selection.grundfos.com/fr/products/sesl-9-30-kw?tab=models" xr:uid="{A344F5B5-8A97-456F-87D5-4C6EFCA52D3A}"/>
+    <hyperlink ref="Q24" r:id="rId41" display="https://product-selection.grundfos.com/fr/products/sesl-frame-size-56?tab=models" xr:uid="{BB0B40A3-A20A-44BC-9FC9-E9EE00FC9F45}"/>
+    <hyperlink ref="Q25" r:id="rId42" display="https://product-selection.grundfos.com/fr/products/s?tab=products" xr:uid="{2E26D22E-3FD7-4718-9B39-661D30AF938C}"/>
+    <hyperlink ref="Q26" r:id="rId43" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft/nkg-supervortex-impeller?tab=explore" xr:uid="{FA539854-B47D-4B47-9F9A-7CE595B28025}"/>
+    <hyperlink ref="S21" r:id="rId44" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/se1?tab=models" xr:uid="{66C50FE8-D6EA-4602-866A-7B3258A9261C}"/>
+    <hyperlink ref="S22" r:id="rId45" display="https://product-selection.grundfos.com/fr/products/sesl-range-48/sev?tab=models" xr:uid="{DEFE3A48-5152-4917-935D-8BAB7D40CDD7}"/>
+    <hyperlink ref="S23" r:id="rId46" display="https://product-selection.grundfos.com/fr/products/sesl-9-30-kw?tab=models" xr:uid="{62BA715F-3850-4F49-A593-7645C6C0C3CC}"/>
+    <hyperlink ref="S24" r:id="rId47" display="https://product-selection.grundfos.com/fr/products/sesl-frame-size-56?tab=models" xr:uid="{F0AA29DC-4DA5-4CA6-94B3-C22351F6904E}"/>
+    <hyperlink ref="S25" r:id="rId48" display="https://product-selection.grundfos.com/fr/products/s?tab=products" xr:uid="{96671AB9-9AEA-4A5F-B84F-E78888F9B311}"/>
+    <hyperlink ref="S26" r:id="rId49" display="https://product-selection.grundfos.com/fr/products/nkg-nkge-nkg-bare-shaft/nkg-supervortex-impeller?tab=explore" xr:uid="{8A1CF826-08F5-4AF2-B984-9AA020480952}"/>
+    <hyperlink ref="O26" r:id="rId50" display="https://product-selection.grundfos.com/fr/products/unilift-ap/unilift-ap50b?tab=models" xr:uid="{14E21A07-FF5F-4129-AE6E-260A1AA5098C}"/>
+    <hyperlink ref="W21" r:id="rId51" display="https://product-selection.grundfos.com/fr/products/unilift-ap?tab=products" xr:uid="{FF1F3D5A-16C1-4C5A-8F69-37BEB2C51657}"/>
+    <hyperlink ref="W22" r:id="rId52" display="https://product-selection.grundfos.com/fr/products/unilift-kp?tab=models" xr:uid="{D8B15CDE-A46F-4955-8CE5-B1F2491BDDEE}"/>
+    <hyperlink ref="W23" r:id="rId53" display="https://product-selection.grundfos.com/fr/products/unilift-cc?tab=models" xr:uid="{5DA16314-BD6C-4DB3-8EC0-A99C56D3006D}"/>
+    <hyperlink ref="W24" r:id="rId54" display="https://product-selection.grundfos.com/fr/products/dp?tab=models" xr:uid="{4D82ED98-3DD6-4697-9C9C-A060C7E06489}"/>
+    <hyperlink ref="W25" r:id="rId55" display="https://product-selection.grundfos.com/fr/products/ef?tab=models" xr:uid="{ABDE8970-72CB-4EB8-979F-99183A9FD9D3}"/>
+    <hyperlink ref="Y21" r:id="rId56" display="https://product-selection.grundfos.com/fr/products/mt-tank-mounted-pumps/mtr?tab=models" xr:uid="{D5799B15-EF87-41DF-88D8-05F25935D793}"/>
+    <hyperlink ref="Y22" r:id="rId57" display="https://product-selection.grundfos.com/fr/products/mt-tank-mounted-pumps/mtre?tab=models" xr:uid="{7E2DAAB5-3884-49DD-BF25-FA92C2CE9951}"/>
+    <hyperlink ref="Y23" r:id="rId58" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nb?tab=documentation" xr:uid="{92C19ACB-7462-4938-A66E-478979299908}"/>
+    <hyperlink ref="Y24" r:id="rId59" display="https://product-selection.grundfos.com/fr/products/nb-nbe-nbe-series-2000/nbe?tab=models" xr:uid="{D2CCE95F-A5DF-4715-B3CA-DB297F6DF5C8}"/>
+    <hyperlink ref="Y25" r:id="rId60" display="https://product-selection.grundfos.com/fr/products/nk-nke-nke-series-2000-nk-bare-shaft?tab=products" xr:uid="{EA080A36-FCEB-4D04-B389-F8ABE5514300}"/>
+    <hyperlink ref="Y26" r:id="rId61" display="https://product-selection.grundfos.com/fr/products/tp-tpe?tab=products" xr:uid="{2A2A6B6D-2CAA-4110-9FED-BCA8DC5F1709}"/>
+    <hyperlink ref="Y27" r:id="rId62" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte?tab=products" xr:uid="{D902984C-2BC5-48A4-BF49-DCE4C7E629F6}"/>
+    <hyperlink ref="Z21" r:id="rId63" display="https://product-selection.grundfos.com/fr/products/hydro-en?tab=models" xr:uid="{69CECDCF-71ED-40D6-A274-30663F73D3A6}"/>
+    <hyperlink ref="AD21" r:id="rId64" display="https://product-selection.grundfos.com/fr/products/poweradapt?tab=models" xr:uid="{CBB79406-3EE4-4CC7-BCD3-398882D58A96}"/>
+    <hyperlink ref="AD22" r:id="rId65" display="https://product-selection.grundfos.com/fr/products/rsi?tab=models" xr:uid="{2ECDD4BA-B757-4A11-9F78-EB235920F462}"/>
+    <hyperlink ref="AD23" r:id="rId66" display="https://product-selection.grundfos.com/fr/products/crflex?tab=models" xr:uid="{F1835770-C21F-4E8A-9EBF-7C701B0E9CF4}"/>
+    <hyperlink ref="AD24" r:id="rId67" display="https://product-selection.grundfos.com/fr/products/sqflex?tab=models" xr:uid="{2932EAA4-553E-42B6-AD4B-37D91C9B845C}"/>
+    <hyperlink ref="AD25" r:id="rId68" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/sp?tab=models" xr:uid="{25A70C6E-05E1-4E40-956B-50B78B088135}"/>
+    <hyperlink ref="AD26" r:id="rId69" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/spe?tab=models" xr:uid="{7C346AF6-2EEB-4DFC-A819-DAE2C3B09113}"/>
+    <hyperlink ref="AD27" r:id="rId70" display="https://product-selection.grundfos.com/fr/products/cr-cre-cri-crie-crn-crne-crt-crte?tab=products" xr:uid="{9F4AE584-6CDD-45BE-ABC9-5087AAD766B9}"/>
+    <hyperlink ref="AE21" r:id="rId71" display="https://product-selection.grundfos.com/fr/products/dosing-pumps-digital/dda?tab=models" xr:uid="{68600FE5-FDB0-4237-8B8A-45786462FE8A}"/>
+    <hyperlink ref="AE22" r:id="rId72" display="https://product-selection.grundfos.com/fr/products/dosing-pumps-digital/dme?tab=models" xr:uid="{41502941-2297-46B7-A840-2EF7A24064D7}"/>
+    <hyperlink ref="AE23" r:id="rId73" display="https://product-selection.grundfos.com/fr/products/dosing-pumps-mechanical/dmx?tab=models" xr:uid="{A892A826-C3E1-4B26-9529-8174E76C068D}"/>
+    <hyperlink ref="AE24" r:id="rId74" display="https://product-selection.grundfos.com/fr/products/dosing-pumps-mechanical/dmh?tab=models" xr:uid="{60926621-C7DA-4892-9ACA-4145E303C37B}"/>
+    <hyperlink ref="AE25" r:id="rId75" xr:uid="{EB339B7E-AAB0-4720-A5DC-B7E47BEFE888}"/>
+    <hyperlink ref="AF23" r:id="rId76" display="https://product-selection.grundfos.com/fr/products/disinfection-systems/oxiperm?tab=models" xr:uid="{D1CFBDC1-076A-4661-B343-B5087946D2BF}"/>
+    <hyperlink ref="AF21" r:id="rId77" display="https://product-selection.grundfos.com/fr/products/disinfection-systems/vaccuperm?tab=models" xr:uid="{0E5CA30E-D80E-4BC1-BE8D-5757C0E703F9}"/>
+    <hyperlink ref="AF22" r:id="rId78" display="https://product-selection.grundfos.com/fr/products/disinfection-systems/selcoperm?tab=models" xr:uid="{3FE337C4-03C2-4326-92F3-2ADF14429172}"/>
+    <hyperlink ref="C29" r:id="rId79" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-4" xr:uid="{7CECB146-2C6E-4D8C-8362-B574F0A0B1CD}"/>
+    <hyperlink ref="C30" r:id="rId80" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-6" xr:uid="{77066640-D437-4393-AE04-9291CA2EA2E2}"/>
+    <hyperlink ref="C31" r:id="rId81" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-8" xr:uid="{440D559C-9B55-46F7-B47D-809066594D8E}"/>
+    <hyperlink ref="C32" r:id="rId82" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-actun-zetos" xr:uid="{6B88B868-32F8-4635-8067-C4F8AA30A87A}"/>
+    <hyperlink ref="C33" r:id="rId83" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-14-24" xr:uid="{6AAEB27D-0CD4-409C-9175-B5DC81BA5B91}"/>
+    <hyperlink ref="D29" r:id="rId84" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-4" xr:uid="{70B5668C-6DE4-4721-BD0D-15695ACCFD10}"/>
+    <hyperlink ref="D30" r:id="rId85" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-6" xr:uid="{AB0F5528-0721-49E7-9EB4-443A836A5BE6}"/>
+    <hyperlink ref="D31" r:id="rId86" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-8" xr:uid="{CE5D4CF5-B9AD-4786-AF2A-5CBA0FB4461E}"/>
+    <hyperlink ref="D32" r:id="rId87" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-actun-zetos" xr:uid="{F3302311-60D3-4257-BE0E-8ADCE8FD3F26}"/>
+    <hyperlink ref="D33" r:id="rId88" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-14-24" xr:uid="{C714C692-05B2-43B9-83CE-06CDCF547DAA}"/>
+    <hyperlink ref="F29" r:id="rId89" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-scp" xr:uid="{7BEBF8BE-E457-43DD-A078-9A05C9712ED1}"/>
+    <hyperlink ref="F30" r:id="rId90" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-atmos-tera-sch" xr:uid="{8AC9B5FF-3554-4A3F-9A49-254FDDC1D679}"/>
+    <hyperlink ref="G29" r:id="rId91" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-4" xr:uid="{A6F45EEC-DFC1-4F41-A737-7D50D323F858}"/>
+    <hyperlink ref="G30" r:id="rId92" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-6" xr:uid="{E8092E13-22EC-4AA4-A0E2-CB8C894814DA}"/>
+    <hyperlink ref="G31" r:id="rId93" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-sub-twi-8" xr:uid="{06C47C82-BB6B-4167-9AFC-F87F629A6D2D}"/>
+    <hyperlink ref="G32" r:id="rId94" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-actun-zetos" xr:uid="{7F484481-A382-4AA7-BC6F-9F9E8E881F13}"/>
+    <hyperlink ref="G33" r:id="rId95" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-14-24" xr:uid="{145E082E-ACF5-4C03-95AA-D5FF287B68E9}"/>
+    <hyperlink ref="J29" r:id="rId96" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-medana-ch1-l" xr:uid="{CB6CAFF8-329E-47DC-8F46-39C8BB5E04DD}"/>
+    <hyperlink ref="J30" r:id="rId97" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-zeox-first-h" xr:uid="{2D403080-ECF0-434D-8570-2DCE4384BDB3}"/>
+    <hyperlink ref="K29" r:id="rId98" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-helix-v" xr:uid="{24EB14FB-8853-4DD9-BFF7-D08622F6269E}"/>
+    <hyperlink ref="K30" r:id="rId99" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-helix-first-v" xr:uid="{292648A6-CEF7-4F6A-B9E8-2C2D1935D493}"/>
+    <hyperlink ref="L29" r:id="rId100" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-helix-ve" xr:uid="{CB04A41A-2CE9-45EC-90FB-F63D1D7003E0}"/>
+    <hyperlink ref="L30" r:id="rId101" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-helix2-0-ve" xr:uid="{0D95BEE0-BF20-4117-86C3-9423999074AC}"/>
+    <hyperlink ref="M29" r:id="rId102" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-medana-ch3-le" xr:uid="{E61CDC21-E587-41FD-8720-AA95E8F2BCB8}"/>
+    <hyperlink ref="N29" r:id="rId103" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-isar-modh1-e-2-3" xr:uid="{2D23D0CC-B7DF-4FF1-ABE9-A9C38B0D675F}"/>
+    <hyperlink ref="N30" r:id="rId104" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-siboost2-0-smart-helix-ve" xr:uid="{FFEEE275-2C73-4EC4-B193-CB85762B0142}"/>
+    <hyperlink ref="O29" r:id="rId105" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-pro" xr:uid="{40187CA6-E027-4F57-B695-B124E41E9781}"/>
+    <hyperlink ref="O30" r:id="rId106" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-supra" xr:uid="{6510CD0A-CFE7-486C-91AF-7C7A655B4AFB}"/>
+    <hyperlink ref="O31" r:id="rId107" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-solid" xr:uid="{BDC567B5-AC65-4996-9A0B-1AF09DF2041A}"/>
+    <hyperlink ref="Q29" r:id="rId108" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-bloc" xr:uid="{3980AF89-63D6-4F8A-AA62-E67520B41458}"/>
+    <hyperlink ref="Q30" r:id="rId109" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-norm" xr:uid="{713EE9E0-CE07-4B5A-8098-8828FD7A2BE1}"/>
+    <hyperlink ref="P29" r:id="rId110" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-pro-s" xr:uid="{7EA67BA6-0CB9-4BC2-8D2F-2187D3E3EC87}"/>
+    <hyperlink ref="O32" r:id="rId111" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-fa-configure" xr:uid="{F271E929-C189-489C-95BA-44C8F95B9706}"/>
+    <hyperlink ref="S29" r:id="rId112" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-pro" xr:uid="{4E520461-D8CA-4714-95A3-4A07D979003B}"/>
+    <hyperlink ref="S30" r:id="rId113" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-supra" xr:uid="{7E747CBF-258D-4F97-AE71-AF52B950EDDE}"/>
+    <hyperlink ref="S31" r:id="rId114" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-solid" xr:uid="{90F21445-AD91-480E-9E60-99DEEB471A24}"/>
+    <hyperlink ref="S32" r:id="rId115" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-fa-configure" xr:uid="{CAC9CBDD-5033-4067-92F5-E1A89E7A10BF}"/>
+    <hyperlink ref="U29" r:id="rId116" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-pro" xr:uid="{DED143CB-BC81-4CC1-99AF-6D9EFDCA04A2}"/>
+    <hyperlink ref="U30" r:id="rId117" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-supra" xr:uid="{AD0F4A4E-82E3-443D-B5CE-BB1383456F96}"/>
+    <hyperlink ref="U31" r:id="rId118" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-rexa-solid" xr:uid="{F30C0BD2-ACC1-498E-B06C-26D556B514B6}"/>
+    <hyperlink ref="U32" r:id="rId119" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-emu-fa-configure" xr:uid="{FC92FF04-817E-49C9-B9E1-3FED19E3DBAA}"/>
+    <hyperlink ref="W29" r:id="rId120" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-drain-tm-tmw-tmr-32" xr:uid="{0F177732-3552-46D9-B2A1-0858315CC611}"/>
+    <hyperlink ref="W30" r:id="rId121" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-padus-uni" xr:uid="{31C21B43-5DBE-431A-A886-4FBC3A6BE491}"/>
+    <hyperlink ref="W31" r:id="rId122" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-padus-mini3" xr:uid="{D91894CF-CB16-4C43-980E-41E743666848}"/>
+    <hyperlink ref="W32" r:id="rId123" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-padus-pro" xr:uid="{79DE7E3B-A7A2-4098-B5DF-694F7F93640D}"/>
+    <hyperlink ref="Z29" r:id="rId124" display="https://wilo.com/fr/fr/Produits-Applications/fr/produits-applications/wilo-cof-helix" xr:uid="{2E5216D3-37DA-48CB-ABA0-7C21064BB2D3}"/>
   </hyperlinks>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="8" scale="83" orientation="landscape" r:id="rId125"/>
@@ -5905,7 +5832,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9695ECB-13A0-4CDA-8A65-46AFD650B789}">
   <dimension ref="F23"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
   <sheetData>
     <row r="23" spans="6:6">
       <c r="F23">
@@ -5919,6 +5846,22 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <FileHash xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
+    <nombre xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
+    <CloudMigratorVersion xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <CloudMigratorOriginId xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
+    <TaxCatchAll xmlns="c4b3ccb6-1a3d-47c8-9c28-87cc19c94359" xsi:nil="true"/>
+    <UniqueSourceRef xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101004976F38B5FA2A5428FEEC343358A0CB6" ma:contentTypeVersion="19" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="d78edfbf191a497d28ab4f4b405a2c3f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xmlns:ns3="c4b3ccb6-1a3d-47c8-9c28-87cc19c94359" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="79eaa508d83d12f280b303d7506ce0b5" ns2:_="" ns3:_="">
     <xsd:import namespace="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5"/>
@@ -6169,7 +6112,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -6178,32 +6121,16 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <FileHash xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
-    <nombre xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
-    <CloudMigratorVersion xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <CloudMigratorOriginId xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
-    <TaxCatchAll xmlns="c4b3ccb6-1a3d-47c8-9c28-87cc19c94359" xsi:nil="true"/>
-    <UniqueSourceRef xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DFA46023-FA4E-40CC-AE09-8D10AF59D952}"/>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2B67381A-06A2-445B-9B84-A17F50FAEFF2}"/>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CC74D80B-69A9-4194-90FE-61316E92C740}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DFA46023-FA4E-40CC-AE09-8D10AF59D952}"/>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Mise à jour depuis Excel — 2026-10-05T17:40:55.510Z
</commit_message>
<xml_diff>
--- a/comparatif.xlsx
+++ b/comparatif.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30602"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nge1.sharepoint.com/sites/FR_SADE_DAM/Documents partages/01 - Achats/Achats Production/Pompes &amp; Instrum/Pompes/ABAQUE POMPES/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7827D0F7-18B5-442C-A64F-98E374DE428A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E8BF0816-812B-4593-B51E-FBAB886C413A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{723C6001-552E-447F-BEBB-92F546F7738F}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="286">
   <si>
-    <t>Eau potable et irrigation</t>
+    <t>Eau potable et irrigation 123</t>
   </si>
   <si>
     <t>Eau chargée</t>
@@ -84,10 +84,10 @@
     <t>DESINFECTION</t>
   </si>
   <si>
-    <t>Pompes immergées</t>
-  </si>
-  <si>
-    <t>Surface</t>
+    <t>Pompes immergées  1</t>
+  </si>
+  <si>
+    <t>Surface 2</t>
   </si>
   <si>
     <t>Immergées</t>
@@ -1838,6 +1838,60 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="255" wrapText="1"/>
     </xf>
@@ -1867,60 +1921,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2288,104 +2288,104 @@
     <row r="2" spans="1:32" s="70" customFormat="1" ht="23.25" customHeight="1" thickBot="1">
       <c r="A2" s="68"/>
       <c r="B2" s="69"/>
-      <c r="C2" s="112" t="s">
+      <c r="C2" s="102" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="112"/>
-      <c r="E2" s="112"/>
-      <c r="F2" s="112"/>
-      <c r="G2" s="112"/>
-      <c r="H2" s="112"/>
-      <c r="I2" s="112"/>
-      <c r="J2" s="112"/>
-      <c r="K2" s="112"/>
-      <c r="L2" s="112"/>
-      <c r="M2" s="112"/>
-      <c r="N2" s="112"/>
-      <c r="O2" s="119" t="s">
+      <c r="D2" s="102"/>
+      <c r="E2" s="102"/>
+      <c r="F2" s="102"/>
+      <c r="G2" s="102"/>
+      <c r="H2" s="102"/>
+      <c r="I2" s="102"/>
+      <c r="J2" s="102"/>
+      <c r="K2" s="102"/>
+      <c r="L2" s="102"/>
+      <c r="M2" s="102"/>
+      <c r="N2" s="102"/>
+      <c r="O2" s="109" t="s">
         <v>1</v>
       </c>
-      <c r="P2" s="119"/>
-      <c r="Q2" s="119"/>
-      <c r="R2" s="119"/>
-      <c r="S2" s="119"/>
-      <c r="T2" s="119"/>
-      <c r="U2" s="113" t="s">
+      <c r="P2" s="109"/>
+      <c r="Q2" s="109"/>
+      <c r="R2" s="109"/>
+      <c r="S2" s="109"/>
+      <c r="T2" s="109"/>
+      <c r="U2" s="103" t="s">
         <v>2</v>
       </c>
-      <c r="V2" s="113"/>
-      <c r="W2" s="115" t="s">
+      <c r="V2" s="103"/>
+      <c r="W2" s="105" t="s">
         <v>3</v>
       </c>
-      <c r="X2" s="104" t="s">
+      <c r="X2" s="98" t="s">
         <v>4</v>
       </c>
-      <c r="Y2" s="104" t="s">
+      <c r="Y2" s="98" t="s">
         <v>5</v>
       </c>
-      <c r="Z2" s="104" t="s">
+      <c r="Z2" s="98" t="s">
         <v>6</v>
       </c>
-      <c r="AA2" s="104" t="s">
+      <c r="AA2" s="98" t="s">
         <v>7</v>
       </c>
-      <c r="AB2" s="104" t="s">
+      <c r="AB2" s="98" t="s">
         <v>8</v>
       </c>
-      <c r="AC2" s="104" t="s">
+      <c r="AC2" s="98" t="s">
         <v>9</v>
       </c>
-      <c r="AD2" s="102" t="s">
+      <c r="AD2" s="92" t="s">
         <v>10</v>
       </c>
-      <c r="AE2" s="102" t="s">
+      <c r="AE2" s="92" t="s">
         <v>11</v>
       </c>
-      <c r="AF2" s="102" t="s">
+      <c r="AF2" s="92" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:32" s="70" customFormat="1" ht="23.25" customHeight="1">
       <c r="A3" s="68"/>
       <c r="B3" s="71"/>
-      <c r="C3" s="110" t="s">
+      <c r="C3" s="100" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="111"/>
-      <c r="E3" s="111"/>
+      <c r="D3" s="101"/>
+      <c r="E3" s="101"/>
       <c r="F3" s="72"/>
-      <c r="G3" s="110" t="s">
+      <c r="G3" s="100" t="s">
         <v>14</v>
       </c>
-      <c r="H3" s="111"/>
-      <c r="I3" s="111"/>
-      <c r="J3" s="111"/>
-      <c r="K3" s="111"/>
-      <c r="L3" s="111"/>
+      <c r="H3" s="101"/>
+      <c r="I3" s="101"/>
+      <c r="J3" s="101"/>
+      <c r="K3" s="101"/>
+      <c r="L3" s="101"/>
       <c r="M3" s="72"/>
       <c r="N3" s="73"/>
-      <c r="O3" s="110" t="s">
+      <c r="O3" s="100" t="s">
         <v>15</v>
       </c>
-      <c r="P3" s="111"/>
-      <c r="Q3" s="110" t="s">
+      <c r="P3" s="101"/>
+      <c r="Q3" s="100" t="s">
         <v>16</v>
       </c>
-      <c r="R3" s="111"/>
-      <c r="S3" s="111"/>
-      <c r="T3" s="118"/>
-      <c r="U3" s="114"/>
-      <c r="V3" s="114"/>
-      <c r="W3" s="116"/>
-      <c r="X3" s="105"/>
-      <c r="Y3" s="105"/>
-      <c r="Z3" s="105"/>
-      <c r="AA3" s="105"/>
-      <c r="AB3" s="105"/>
-      <c r="AC3" s="105"/>
-      <c r="AD3" s="103"/>
-      <c r="AE3" s="103"/>
-      <c r="AF3" s="103"/>
+      <c r="R3" s="101"/>
+      <c r="S3" s="101"/>
+      <c r="T3" s="108"/>
+      <c r="U3" s="104"/>
+      <c r="V3" s="104"/>
+      <c r="W3" s="106"/>
+      <c r="X3" s="99"/>
+      <c r="Y3" s="99"/>
+      <c r="Z3" s="99"/>
+      <c r="AA3" s="99"/>
+      <c r="AB3" s="99"/>
+      <c r="AC3" s="99"/>
+      <c r="AD3" s="93"/>
+      <c r="AE3" s="93"/>
+      <c r="AF3" s="93"/>
     </row>
     <row r="4" spans="1:32" s="80" customFormat="1" ht="57.75" customHeight="1">
       <c r="B4" s="81" t="s">
@@ -2451,16 +2451,16 @@
       <c r="V4" s="83" t="s">
         <v>35</v>
       </c>
-      <c r="W4" s="117"/>
-      <c r="X4" s="105"/>
-      <c r="Y4" s="105"/>
-      <c r="Z4" s="105"/>
-      <c r="AA4" s="105"/>
-      <c r="AB4" s="105"/>
-      <c r="AC4" s="105"/>
-      <c r="AD4" s="103"/>
-      <c r="AE4" s="103"/>
-      <c r="AF4" s="106"/>
+      <c r="W4" s="107"/>
+      <c r="X4" s="99"/>
+      <c r="Y4" s="99"/>
+      <c r="Z4" s="99"/>
+      <c r="AA4" s="99"/>
+      <c r="AB4" s="99"/>
+      <c r="AC4" s="99"/>
+      <c r="AD4" s="93"/>
+      <c r="AE4" s="93"/>
+      <c r="AF4" s="94"/>
     </row>
     <row r="5" spans="1:32" s="80" customFormat="1" ht="10.15" customHeight="1" thickBot="1">
       <c r="B5" s="87"/>
@@ -2581,10 +2581,10 @@
       </c>
     </row>
     <row r="7" spans="1:32" s="1" customFormat="1" ht="18" customHeight="1">
-      <c r="A7" s="107" t="s">
+      <c r="A7" s="95" t="s">
         <v>49</v>
       </c>
-      <c r="B7" s="98" t="s">
+      <c r="B7" s="116" t="s">
         <v>50</v>
       </c>
       <c r="C7" s="11" t="s">
@@ -2641,8 +2641,8 @@
       <c r="AF7" s="76"/>
     </row>
     <row r="8" spans="1:32" s="1" customFormat="1" ht="18" customHeight="1">
-      <c r="A8" s="108"/>
-      <c r="B8" s="96"/>
+      <c r="A8" s="96"/>
+      <c r="B8" s="114"/>
       <c r="C8" s="11" t="s">
         <v>58</v>
       </c>
@@ -2705,8 +2705,8 @@
       <c r="AF8" s="76"/>
     </row>
     <row r="9" spans="1:32" s="1" customFormat="1" ht="18" customHeight="1">
-      <c r="A9" s="108"/>
-      <c r="B9" s="96"/>
+      <c r="A9" s="96"/>
+      <c r="B9" s="114"/>
       <c r="C9" s="11"/>
       <c r="D9" s="11"/>
       <c r="E9" s="11"/>
@@ -2753,8 +2753,8 @@
       <c r="AF9" s="76"/>
     </row>
     <row r="10" spans="1:32" s="1" customFormat="1" ht="18" customHeight="1">
-      <c r="A10" s="108"/>
-      <c r="B10" s="96"/>
+      <c r="A10" s="96"/>
+      <c r="B10" s="114"/>
       <c r="C10" s="11"/>
       <c r="D10" s="11"/>
       <c r="E10" s="11"/>
@@ -2793,8 +2793,8 @@
       <c r="AF10" s="76"/>
     </row>
     <row r="11" spans="1:32" s="1" customFormat="1" ht="18" customHeight="1">
-      <c r="A11" s="108"/>
-      <c r="B11" s="97"/>
+      <c r="A11" s="96"/>
+      <c r="B11" s="115"/>
       <c r="C11" s="52"/>
       <c r="D11" s="52"/>
       <c r="E11" s="52"/>
@@ -2835,8 +2835,8 @@
       <c r="AF11" s="76"/>
     </row>
     <row r="12" spans="1:32" ht="18" customHeight="1">
-      <c r="A12" s="108"/>
-      <c r="B12" s="95" t="s">
+      <c r="A12" s="96"/>
+      <c r="B12" s="113" t="s">
         <v>75</v>
       </c>
       <c r="C12" s="61" t="s">
@@ -2925,8 +2925,8 @@
       <c r="AF12" s="75"/>
     </row>
     <row r="13" spans="1:32" ht="18" customHeight="1">
-      <c r="A13" s="108"/>
-      <c r="B13" s="96"/>
+      <c r="A13" s="96"/>
+      <c r="B13" s="114"/>
       <c r="C13" s="11" t="s">
         <v>91</v>
       </c>
@@ -2997,8 +2997,8 @@
       <c r="AF13" s="40"/>
     </row>
     <row r="14" spans="1:32" ht="18" customHeight="1">
-      <c r="A14" s="108"/>
-      <c r="B14" s="96"/>
+      <c r="A14" s="96"/>
+      <c r="B14" s="114"/>
       <c r="C14" s="11" t="s">
         <v>102</v>
       </c>
@@ -3062,8 +3062,8 @@
       <c r="AF14" s="40"/>
     </row>
     <row r="15" spans="1:32" ht="18" customHeight="1">
-      <c r="A15" s="108"/>
-      <c r="B15" s="96"/>
+      <c r="A15" s="96"/>
+      <c r="B15" s="114"/>
       <c r="C15" s="11" t="s">
         <v>110</v>
       </c>
@@ -3122,8 +3122,8 @@
       <c r="AF15" s="40"/>
     </row>
     <row r="16" spans="1:32" ht="18" customHeight="1">
-      <c r="A16" s="108"/>
-      <c r="B16" s="96"/>
+      <c r="A16" s="96"/>
+      <c r="B16" s="114"/>
       <c r="C16" s="11" t="s">
         <v>116</v>
       </c>
@@ -3178,8 +3178,8 @@
       <c r="AF16" s="40"/>
     </row>
     <row r="17" spans="1:155" ht="18" customHeight="1">
-      <c r="A17" s="108"/>
-      <c r="B17" s="96"/>
+      <c r="A17" s="96"/>
+      <c r="B17" s="114"/>
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
@@ -3226,8 +3226,8 @@
       <c r="AF17" s="40"/>
     </row>
     <row r="18" spans="1:155" ht="18" customHeight="1">
-      <c r="A18" s="109"/>
-      <c r="B18" s="97"/>
+      <c r="A18" s="97"/>
+      <c r="B18" s="115"/>
       <c r="C18" s="32"/>
       <c r="D18" s="32"/>
       <c r="E18" s="32"/>
@@ -3349,7 +3349,7 @@
     </row>
     <row r="20" spans="1:155" s="1" customFormat="1" ht="36" customHeight="1">
       <c r="A20" s="21"/>
-      <c r="B20" s="92" t="s">
+      <c r="B20" s="110" t="s">
         <v>146</v>
       </c>
       <c r="C20" s="22" t="s">
@@ -3445,7 +3445,7 @@
     </row>
     <row r="21" spans="1:155" ht="18" customHeight="1">
       <c r="A21" s="24"/>
-      <c r="B21" s="93"/>
+      <c r="B21" s="111"/>
       <c r="C21" s="25" t="s">
         <v>168</v>
       </c>
@@ -3517,7 +3517,7 @@
     </row>
     <row r="22" spans="1:155" ht="18" customHeight="1">
       <c r="A22" s="24"/>
-      <c r="B22" s="93"/>
+      <c r="B22" s="111"/>
       <c r="C22" s="25" t="s">
         <v>186</v>
       </c>
@@ -3583,7 +3583,7 @@
     </row>
     <row r="23" spans="1:155" ht="18" customHeight="1">
       <c r="A23" s="24"/>
-      <c r="B23" s="93"/>
+      <c r="B23" s="111"/>
       <c r="C23" s="25" t="s">
         <v>200</v>
       </c>
@@ -3645,7 +3645,7 @@
     </row>
     <row r="24" spans="1:155" ht="18" customHeight="1">
       <c r="A24" s="24"/>
-      <c r="B24" s="93"/>
+      <c r="B24" s="111"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
       <c r="E24" s="4"/>
@@ -3701,7 +3701,7 @@
     </row>
     <row r="25" spans="1:155" ht="18" customHeight="1">
       <c r="A25" s="24"/>
-      <c r="B25" s="93"/>
+      <c r="B25" s="111"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
       <c r="E25" s="4"/>
@@ -3753,7 +3753,7 @@
     </row>
     <row r="26" spans="1:155" ht="18" customHeight="1">
       <c r="A26" s="28"/>
-      <c r="B26" s="93"/>
+      <c r="B26" s="111"/>
       <c r="C26" s="6"/>
       <c r="D26" s="6"/>
       <c r="E26" s="6"/>
@@ -3801,7 +3801,7 @@
     </row>
     <row r="27" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1">
       <c r="A27" s="30"/>
-      <c r="B27" s="94"/>
+      <c r="B27" s="112"/>
       <c r="C27" s="32"/>
       <c r="D27" s="32"/>
       <c r="E27" s="32"/>
@@ -3962,7 +3962,7 @@
     </row>
     <row r="28" spans="1:155" s="10" customFormat="1" ht="36" customHeight="1">
       <c r="A28" s="21"/>
-      <c r="B28" s="99" t="s">
+      <c r="B28" s="117" t="s">
         <v>222</v>
       </c>
       <c r="C28" s="36" t="s">
@@ -4161,7 +4161,7 @@
     </row>
     <row r="29" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1">
       <c r="A29" s="24"/>
-      <c r="B29" s="100"/>
+      <c r="B29" s="118"/>
       <c r="C29" s="13" t="s">
         <v>239</v>
       </c>
@@ -4348,7 +4348,7 @@
     </row>
     <row r="30" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1">
       <c r="A30" s="24"/>
-      <c r="B30" s="100"/>
+      <c r="B30" s="118"/>
       <c r="C30" s="13" t="s">
         <v>251</v>
       </c>
@@ -4529,7 +4529,7 @@
     </row>
     <row r="31" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1">
       <c r="A31" s="24"/>
-      <c r="B31" s="100"/>
+      <c r="B31" s="118"/>
       <c r="C31" s="13" t="s">
         <v>260</v>
       </c>
@@ -4698,7 +4698,7 @@
     </row>
     <row r="32" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1">
       <c r="A32" s="24"/>
-      <c r="B32" s="100"/>
+      <c r="B32" s="118"/>
       <c r="C32" s="13" t="s">
         <v>263</v>
       </c>
@@ -4867,7 +4867,7 @@
     </row>
     <row r="33" spans="1:155" s="10" customFormat="1" ht="18" customHeight="1">
       <c r="A33" s="30"/>
-      <c r="B33" s="101"/>
+      <c r="B33" s="119"/>
       <c r="C33" s="33" t="s">
         <v>266</v>
       </c>
@@ -5675,6 +5675,12 @@
     <filterColumn colId="20" showButton="0"/>
   </autoFilter>
   <mergeCells count="22">
+    <mergeCell ref="B20:B27"/>
+    <mergeCell ref="B12:B18"/>
+    <mergeCell ref="B7:B11"/>
+    <mergeCell ref="B28:B33"/>
+    <mergeCell ref="AD2:AD4"/>
+    <mergeCell ref="Z2:Z4"/>
     <mergeCell ref="AE2:AE4"/>
     <mergeCell ref="AF2:AF4"/>
     <mergeCell ref="A7:A18"/>
@@ -5691,12 +5697,6 @@
     <mergeCell ref="O2:T2"/>
     <mergeCell ref="O3:P3"/>
     <mergeCell ref="Y2:Y4"/>
-    <mergeCell ref="B20:B27"/>
-    <mergeCell ref="B12:B18"/>
-    <mergeCell ref="B7:B11"/>
-    <mergeCell ref="B28:B33"/>
-    <mergeCell ref="AD2:AD4"/>
-    <mergeCell ref="Z2:Z4"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C21" r:id="rId1" display="https://product-selection.grundfos.com/fr/products/sp-sp-g/sp?tab=models" xr:uid="{FE987DC0-578A-4A81-AB17-6E49D6983782}"/>
@@ -5846,19 +5846,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <FileHash xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
-    <nombre xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
-    <CloudMigratorVersion xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <CloudMigratorOriginId xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
-    <TaxCatchAll xmlns="c4b3ccb6-1a3d-47c8-9c28-87cc19c94359" xsi:nil="true"/>
-    <UniqueSourceRef xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6113,16 +6106,23 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <FileHash xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
+    <nombre xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
+    <CloudMigratorVersion xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <CloudMigratorOriginId xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
+    <TaxCatchAll xmlns="c4b3ccb6-1a3d-47c8-9c28-87cc19c94359" xsi:nil="true"/>
+    <UniqueSourceRef xmlns="2d8fbdb5-7e30-42e0-adda-e1c0c4f617c5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DFA46023-FA4E-40CC-AE09-8D10AF59D952}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CC74D80B-69A9-4194-90FE-61316E92C740}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6130,7 +6130,7 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CC74D80B-69A9-4194-90FE-61316E92C740}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DFA46023-FA4E-40CC-AE09-8D10AF59D952}"/>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Mise à jour depuis Excel — 2026-10-05T18:01:57.155Z
</commit_message>
<xml_diff>
--- a/comparatif.xlsx
+++ b/comparatif.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nge1.sharepoint.com/sites/FR_SADE_DAM/Documents partages/01 - Achats/Achats Production/Pompes &amp; Instrum/Pompes/ABAQUE POMPES/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E8BF0816-812B-4593-B51E-FBAB886C413A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{353CB3FE-3F89-4349-92FD-93874CD5C930}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{723C6001-552E-447F-BEBB-92F546F7738F}"/>
   </bookViews>
@@ -84,10 +84,10 @@
     <t>DESINFECTION</t>
   </si>
   <si>
-    <t>Pompes immergées  1</t>
-  </si>
-  <si>
-    <t>Surface 2</t>
+    <t>Pompes immergées  ESSAI</t>
+  </si>
+  <si>
+    <t>Surface JJJJJJ</t>
   </si>
   <si>
     <t>Immergées</t>

</xml_diff>

<commit_message>
Mise à jour depuis Excel — 2026-10-06T06:36:55.188Z
</commit_message>
<xml_diff>
--- a/comparatif.xlsx
+++ b/comparatif.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30602"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30601"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nge1.sharepoint.com/sites/FR_SADE_DAM/Documents partages/01 - Achats/Achats Production/Pompes &amp; Instrum/Pompes/ABAQUE POMPES/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{353CB3FE-3F89-4349-92FD-93874CD5C930}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{46210D3F-262D-4D5B-9E1D-44E7118764CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{723C6001-552E-447F-BEBB-92F546F7738F}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="286">
   <si>
-    <t>Eau potable et irrigation 123</t>
+    <t>Eau potable et irrigation Essai PV</t>
   </si>
   <si>
     <t>Eau chargée</t>
@@ -84,10 +84,10 @@
     <t>DESINFECTION</t>
   </si>
   <si>
-    <t>Pompes immergées  ESSAI</t>
-  </si>
-  <si>
-    <t>Surface JJJJJJ</t>
+    <t xml:space="preserve">Pompes immergées  </t>
+  </si>
+  <si>
+    <t>Surface</t>
   </si>
   <si>
     <t>Immergées</t>

</xml_diff>